<commit_message>
Update berita 2026-08-07 20:34 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-08.xlsx
+++ b/data/berita_2026-08-08.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$62</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I45"/>
+  <dimension ref="A1:I62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -2548,8 +2548,807 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Jalan Abdul Muis ditutup hingga pemadaman api selesai</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 03:22:38 +0700</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Kapolres Metro Jakarta Pusat Kombes Reynold EP Hutagalung menyatakan Jalan Abdul Muis yang menjadi lokasi kebakaran ...</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685257/jalan-abdul-muis-ditutup-hingga-pemadaman-api-selesai</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000472219.jpg</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Polda Metro Jaya siagakan 125 personil amankan kebakaran Bapenda</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 03:16:37 +0700</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Kepolisian Daerah (Polda) Metro Jaya menyiagakan 125 personil untuk mengamankan lingkungan di sekitar lokasi kebakaran ...</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685256/polda-metro-jaya-siagakan-125-personil-amankan-kebakaran-bapenda</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000472212.jpg</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Tiga unit "bronto skylift" dikerahkan untuk padamkan api di Abdul Muis</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 02:54:46 +0700</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Dinas Penanggulangan Kebakaran dan Penyelamatan (Gulkarmat) DKI Jakarta mengerahkan tiga unit bronto skylift untuk ...</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685252/tiga-unit-bronto-skylift-dikerahkan-untuk-padamkan-api-di-abdul-muis</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000472214.jpg</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Tujuh rekomendasi kegiatan akhir pekan di Jakarta</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 02:51:14 +0700</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Beragam kegiatan seni, budaya, film, hingga pasar kreatif dapat menjadi pilihan masyarakat untuk mengisi akhir pekan di ...</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685249/tujuh-rekomendasi-kegiatan-akhir-pekan-di-jakarta</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/16/Pertunjukan-kolosal-Tari-Ondel-Ondel-di-TMII-160526-Ada-2.jpg</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Yayasan sekolah bantah keterlibatan guru dalam penyimpanan senjata</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 02:48:17 +0700</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>ANTARA - Pihak yayasan sekolah swasta di Pondok Pinang, Kebayoran Lama, Jakarta Selatan, membantah keterlibatan guru ...</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5685247/yayasan-sekolah-bantah-keterlibatan-guru-dalam-penyimpanan-senjata</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/Screenshot-2026-08-08-023135.jpg</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Kencan singkat dengan Suzuki XL7 di GIIAS 2026</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 02:45:27 +0700</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Memanfaatkan pameran otomotif Gaikindo Indonesia International Auto Show (GIIAS) 2026, PT Suzuki Indomobil Sales (SIS) ...</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685248/kencan-singkat-dengan-suzuki-xl7-di-giias-2026</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/WhatsApp-Image-2026-08-07-at-19.53.52.jpeg</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Puslabfor Polri Diterjunkan Investigasi Penyebab Kebakaran Gedung Bapenda DKI</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 03:25:42 +0700</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Rolando Fransiscus Sihombing</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Puslabfor Polri ditugaskan menyelidiki kebakaran gedung Bapenda DKI Jakarta. Investigasi fokus pada titik awal api yang diduga berasal dari lantai 11.</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609394/puslabfor-polri-diterjunkan-investigasi-penyebab-kebakaran-gedung-bapenda-dki</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/reynold-elisa-partomuan-hutagalung-1786133934965_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Petugas Damkar Sisir Lantai 12 Gedung Bapenda DKI Cegah Api Berkobar Lagi</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 03:07:12 +0700</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Rolando Fransiscus Sihombing</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Petugas damkar mulai melakukan pendinginan kebakaran Gedung Bapenda DKI Jakarta di Gambir, Jakpus. Petugas damkar menyisir tiap lantai gedung.</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609393/petugas-damkar-sisir-lantai-12-gedung-bapenda-dki-cegah-api-berkobar-lagi</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/gedung-bapenda-dki-terbakar-rolandodetikcom-1786131098034_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Korban Kebakaran Gedung Bapenda DKI Dievakuasi dari Lantai 15, Ini Kondisinya</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 02:42:29 +0700</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Rolando Fransiscus Sihombing</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Petugas Damkar mengevakuasi satu orang dari Gedung Bapenda DKI Jakarta di Jakpus yang terbakar. Korban dievakuasi dari lantai 15.</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609390/korban-kebakaran-gedung-bapenda-dki-dievakuasi-dari-lantai-15-ini-kondisinya</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/korban-kebakaran-gedung-bapenda-dki-dievakuasi-rolandodetikcom-1786131724966_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Gedung Bapenda DKI yang Terbakar dari Lantai 11 sampai 16</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 02:35:31 +0700</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Rolando Fransiscus Sihombing</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Kebakaran melanda Gedung Bapenda DKI Jakarta dari lantai 11 hingga 16. Pemadaman berlangsung 4 jam, penyebab masih diselidiki. Satu korban selamat dievakuasi.</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609389/gedung-bapenda-dki-yang-terbakar-dari-lantai-11-sampai-16</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/gedung-bapenda-dki-jakarta-di-kawasan-gambir-jakarta-pusat-dilanda-kebakaran-1786122454211_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Kebakaran Gedung Bapenda DKI Sudah Terkendali, Damkar Mulai Pendinginan</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 02:31:51 +0700</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Rolando Fransiscus Sihombing</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Kebakaran Gedung Bapenda DKI Jakarta telah terkendali. Damkar melakukan pendinginan setelah evakuasi satu korban. Penyebab kebakaran masih diselidiki.</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609388/kebakaran-gedung-bapenda-dki-sudah-terkendali-damkar-mulai-pendinginan</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/gedung-bapenda-dki-terbakar-rolandodetikcom-1786131098034_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Satu Orang Dievakuasi dari Gedung Bapenda DKI Jakarta</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 01:49:08 +0700</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Rolando Fransiscus Sihombing</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Petugas damkar mengevakuasi seorang pria dari Gedung Bapenda DKI Jakarta yang terbakar. Korban selamat langsung ditangani petugas medis.</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609385/satu-orang-dievakuasi-dari-gedung-bapenda-dki-jakarta</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/satu-orang-dievakuasi-dari-gedung-bapenda-dki-rolandodetikcom-1786128511586_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Prabowo Berseloroh Rambut Sudaryono Semakin Memutih usai Jadi Kepala BGN</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 03:06:14 +0700</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Presiden Prabowo berseloroh rambut Kepala BGN Sudaryono semakin memutih setelah menjabat.</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865562/prabowo-berseloroh-rambut-sudaryono-semakin-memutih-usai-jadi-kepala-bgn</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/mY_BCOcBIvByqJjVK620aeEYGjg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/prabowo-di-peluncuran-buku-bahlil.jpg</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Maman Abdurrahman Masuk Staf Shin Tae-yong di Persija, Pilar Juara 2018 Kini Jadi Asisten Pelatih</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 03:02:42 +0700</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Maman Abdurrahman kembali ke Persija dengan peran baru. Mantan bek Macan Kemayoran itu kini menjadi asisten Shin Tae-yong.</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865561/maman-abdurrahman-masuk-staf-shin-tae-yong-di-persija-pilar-juara-2018-kini-jadi-asisten-pelatih</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ipPZ4xdDCUSrUF5gAFNtB-pTyvk=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/pemain-senior-persija-maman-abdurrahman-dan-tony-sucipto.jpg</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>LPSK Luncurkan Dana Bantuan Korban TPKS, Restitusi Tak Lagi Bergantung dari Pelaku</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 02:45:31 +0700</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LPSK meluncurkan Dana Bantuan Korban (DBK) untuk memastikan hak korban TPKS tetap terpenuhi ketika pelaku tidak mampu membayar restitusi.</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865560/lpsk-luncurkan-dana-bantuan-korban-tpks-restitusi-tak-lagi-bergantung-dari-pelaku</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/-4tIvMFBvV9gbVy3cv_p_789khs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/lpsk-sananta.jpg</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Polisi Selidiki Penyebab Kebakaran Gedung Bapenda DKI</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 03:27:11 +0700</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Penyebab kebakaran Gedung Bapenda DKI diselidiki, polisi periksa 10 saksi.</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8264780/polisi-selidiki-penyebab-kebakaran-gedung-bapenda-dki</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/k_D7d_4friV41UDO_xXn_9_yctY=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9318696/original/054455200_1786134424-IMG_3447.jpg</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Kebakaran Gedung Bapenda DKI Masuk Tahap Pendinginan</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 02:55:52 +0700</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Setelah hampir 5 jam berjibaku, Damkar mulai pendinginan kebakaran Bapenda DKI Jakarta.</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8264772/kebakaran-gedung-bapenda-dki-masuk-tahap-pendinginan</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/zfq5G_jONactwf5HoU4x7_ES33A=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9318688/original/051146900_1786132547-IMG_3450.jpg</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I45"/>
+  <autoFilter ref="A1:I62"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-07 21:33 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-08.xlsx
+++ b/data/berita_2026-08-08.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$66</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I62"/>
+  <dimension ref="A1:I66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -3347,8 +3347,196 @@
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Jl Abdul Muis Ditutup hingga Pemadaman Kebakaran Gedung Bapenda DKI Selesai</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 04:04:54 +0700</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Rolando Fransiscus Sihombing</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Polisi menutup Jalan Abdul Muis di Jakarta Pusat akibat kebakaran gedung Bapenda. Pendinginan masih berlangsung, satu korban selamat dievakuasi.</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609395/jl-abdul-muis-ditutup-hingga-pemadaman-kebakaran-gedung-bapenda-dki-selesai</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/kebakaran-gedung-bapenda-dki-1786136517063_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Nahdlatul Ulama Tangsel Diajak Adaptif Di Tengah Disrupsi Teknologi Ruang Digital</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 04:09:51 +0700</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>PCNU Tangerang Selatan menggelar diskusi bertema transformasi digital untuk mendorong organisasi keagamaan lebih adaptif di era teknologi.</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7865565/nahdlatul-ulama-tangsel-diajak-adaptif-di-tengah-disrupsi-teknologi-ruang-digital</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Z1j_VDutyqYH1LTuWqlJnhSg_54=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/kadiskominfo-tangsel.jpg</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Prabowo Puji Bahlil Berhasil Bikin Jokowi Tertawa: Orang Solo Itu Kalem</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 03:50:00 +0700</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Presiden Prabowo memuji Bahlil Lahadalia sebagai sosok yang mampu mencairkan suasana dan membuat orang lain tertawa.</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865564/prabowo-puji-bahlil-berhasil-bikin-jokowi-tertawa-orang-solo-itu-kalem</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/mY_BCOcBIvByqJjVK620aeEYGjg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/prabowo-di-peluncuran-buku-bahlil.jpg</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Lewat Telepon 10 Menit, Dasco Himpun Rp200 Miliar untuk Korban Kekerasan Seksual</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 03:31:32 +0700</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Dasco menyebut tingginya kasus TPKS pada 2023–2024 memerlukan perhatian serius dan dukungan pendanaan yang lebih kuat.</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865563/lewat-telepon-10-menit-dasco-himpun-rp200-miliar-untuk-korban-kekerasan-seksual</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/OL0wtYiQYXgawreb1rKnxCIrsXA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/dasco-di-acara-lpsk.jpg</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I62"/>
+  <autoFilter ref="A1:I66"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-07 22:30 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-08.xlsx
+++ b/data/berita_2026-08-08.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$81</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,13 +419,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I66"/>
+  <dimension ref="A1:I81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="33" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="43" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
@@ -3535,8 +3535,713 @@
         </is>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Persija Jakarta umumkan susunan tim kepelatihan untuk musim 2026/2027</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 05:15:04 +0700</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Klub BRI Super League Persija Jakarta mengumumkan susunan tim kepelatihan di bawah pelatih kepala Shin Tae-yong untuk ...</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685280/persija-jakarta-umumkan-susunan-tim-kepelatihan-untuk-musim-2026-2027</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/08/Shin-Tae-Yong-latih-Persija-Jakarta-080626-MRH-2_1.jpg</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>MBG: Investasi modal manusia sejak sebelum kelahiran</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 05:05:41 +0700</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Tengkes atau stunting selama ini lebih sering dipahami sebagai persoalan gizi. Padahal, dampaknya jauh lebih luas ...</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685276/mbg-investasi-modal-manusia-sejak-sebelum-kelahiran</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/30/distribusi-mbg-di-batam-2830447.jpg</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Ramalingom dapatkan kesan positif bersama Persita Tangerang</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 04:40:11 +0700</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Pemain anyar Alexandre Ramalingom mengatakan mendapatkan kesan positif setelah beberapa hari menjalani latihan bersama ...</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685272/ramalingom-dapatkan-kesan-positif-bersama-persita-tangerang</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/image-37.jpg</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Toyota Astra Motor hadirkan pilihan relevan bagi konsumen</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 04:39:31 +0700</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/antaranewsdotcom</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>PT Toyota Astra Motor (TAM) menegaskan bahwa melalui strategi multi platform, perusahaan menghadirkan pilihan yang luas ...</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/berita/5685268/toyota-astra-motor-hadirkan-pilihan-relevan-bagi-konsumen</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/IMG_3484.jpeg</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Ismael Bennacer dan AC Milan sepakat akhiri kerja sama lebih cepat</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 04:38:43 +0700</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Gelandang Ismael Bennacer dan klub Liga Italia AC Milan resmi sepakat untuk mengakhiri kerja sama mereka lebih cepat ...</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685265/ismael-bennacer-dan-ac-milan-sepakat-akhiri-kerja-sama-lebih-cepat</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/09/05/1000017795.jpg</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Fiorentina dapatkan Franco Mastantuono dari Real Madrid</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 04:36:44 +0700</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Klub Liga Italia Fiorentina mendapatkan gelandang Franco Mastantuono dari klub Liga Spanyol Real Madrid pada bursa ...</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685261/fiorentina-dapatkan-franco-mastantuono-dari-real-madrid</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/08/22/Madrid.jpg</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Pihak Richard Lee Nilai Keterangan Doktif Berubah-ubah dan Ada Kejanggalan</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 05:15:17 +0700</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Muhammad Ahsan Nurrijal</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Sidang dokter Richard Lee berlanjut di Pengadilan Negeri Tangerang. Kuasa hukum merasa janggal dan menilai keterangan Doktif berubah-ubah.</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8609370/pihak-richard-lee-nilai-keterangan-doktif-berubah-ubah-dan-ada-kejanggalan</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/14/richard-lee-1784023978045_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Mobil Tabrak Penitipan Anak saat Jam Tidur Siang</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 04:00:30 +0700</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Sebuah mobil menabrak tempat penitipan anak di Kanchanaburi, Thailand Barat, saat anak-anak tengah tidur siang pada Jumat (7/8).</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260807203826-110-1389950/mobil-tabrak-penitipan-anak-saat-jam-tidur-siang</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/07/mobil-tabrak-penitipan-anak-saat-jam-tidur-siang-15-anak-terluka-1786110131893_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Api Hanguskan Setengah Gedung Bapenda Jakarta, Proses Pemadaman Butuh Waktu 4,5 Jam</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 05:00:34 +0700</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Pemadaman api  yang melanda Gedung Badan Pendapatan Daerah (Bapenda) DKI Jakarta menghabiskan waktu 4,5 jam.</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7865570/api-hanguskan-setengah-gedung-bapenda-jakarta-proses-pemadaman-butuh-waktu-45-jam</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/W9SHOqGhp7bj-avPCZWsw2q4wt4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/api-membara-di-gedung-bapenda-dki-jakarta.jpg</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Febrie Adriansyah Bakal Hadirkan Ahli dan Saksi Meringankan saat Pemeriksaan Lanjutan Kasus TPPU</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 04:45:43 +0700</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Kuasa hukum Febrie Adriansyah akan menghadirkan ahli dan saksi meringankan pada pemeriksaan lanjutan kasus dugaan TPPU.</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865569/febrie-adriansyah-bakal-hadirkan-ahli-dan-saksi-meringankan-saat-pemeriksaan-lanjutan-kasus-tppu</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/IuLXlaOB2NJPHo-WUyVmbSFBJSE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Febri-Diansyah-bela-febrie.jpg</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Dasco: Penanganan Korban TPKS Selama 2023–2024 Tidak Maksimal akibat Keterbatasan Pendanaan</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 04:32:31 +0700</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LPSK meluncurkan Dana Bantuan Korban (DBK), disertai dukungan dana Rp200 miliar untuk pemulihan dan pemenuhan hak korban.</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865568/dasco-penanganan-korban-tpks-selama-20232024-tidak-maksimal-akibat-keterbatasan-pendanaan</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/OL0wtYiQYXgawreb1rKnxCIrsXA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/dasco-di-acara-lpsk.jpg</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Periksa Febrie Adriansyah dan Nurman Herin, Tim 9 Kejagung Dalami Bukti Hasil Penggeledahan</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 04:20:16 +0700</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Tim 9 Kejagung memeriksa tiga dari lima orang yang dipanggil, termasuk tersangka Febrie Adriansyah dan Nurman Herin, dalam kasus dugaan TPPU.</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865567/periksa-febrie-adriansyah-dan-nurman-herin-tim-9-kejagung-dalami-bukti-hasil-penggeledahan</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/-o2_dp0zLpm0GQ9xCCLM7G7Cu4g=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/kapuspenkum-anang-123.jpg</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Jadwal Piala AFF 2026: Filipina Ingin Pecahkan Rekor di Malaysia, Thailand Selangkah ke Semifinal</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 04:17:21 +0700</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Filipina berambisi memutus rekor 54 tahun tanpa kemenangan di Malaysia. Carles Cuadrat optimistis Azkals mampu membuat sejarah hari ini, Sabtu (8/8).</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865566/jadwal-piala-aff-2026-filipina-ingin-pecahkan-rekor-di-malaysia-thailand-selangkah-ke-semifinal</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/EwezIMpOWTUmrjr-bTougWOm6uU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Timnas-Malaysia-Haqimi-Azim.jpg</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Otomotif</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Kuota Awal 100 Unit Mobil Listrik Honda Super-ONE 2026 Habis dalam Sehari</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 05:08:00 +0700</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Israr Itah</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, TANGERANG -- PT Honda Prospect Motor (HPM) mencatat pemesanan Honda Super-ONE melampaui alokasi yang disiapkan untuk pasar Indonesia pada 2026. Dalam sehari sejak pemesanan dibuka pada 5 Agustus 2026,...</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjf175348/kuota-awal-100-unit-mobil-listrik-honda-superone-2026-habis-dalam-sehari</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/091114000-1785343459-830-556.jpg</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Otomotif</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Kesan Pengunjung GIIAS 2026 Setelah Test Drive Changan Deepal S05 dan Nevo Q05</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 04:53:00 +0700</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Israr Itah</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, TANGERANG -- Changan menghadirkan dua SUV terbarunya, Deepal S05 dan Nevo Q05, di area test drive GAIKINDO Indonesia International Auto Show (GIIAS) 2026. Melalui sesi uji coba tersebut, pengunjung...</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjf0z7348/kesan-pengunjung-giias-2026-setelah-test-drive-changan-deepal-s05-dan-nevo-q05</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/mobil-test-drive-changan-nevo_260808025912-907.jpeg</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I66"/>
+  <autoFilter ref="A1:I81"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-07 23:26 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-08.xlsx
+++ b/data/berita_2026-08-08.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$103</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I81"/>
+  <dimension ref="A1:I103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -4240,8 +4240,1042 @@
         </is>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Program Pink Changing Lives® Mary Kay Mengubah Tujuan Menjadi Dampak Terukur Bagi Perempuan di Seluruh Dunia</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 06:02:16 +0700</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>- Sebagai pendukung global terhadap pemberdayaan perempuan, Mary Kay Inc. dengan bangga kembali menegaskan komitmennya ...</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685288/program-pink-changing-lives-mary-kay-mengubah-tujuan-menjadi-dampak-terukur-bagi-perempuan-di-seluruh-dunia</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/WhatsApp-Image-2026-08-08-at-04.28.30.jpeg</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>SPHP jaga harga beras</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 06:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Penyaluran program Stabilisasi Pasokan dan Harga Pangan (SPHP) untuk menjaga stabilitas harga beras mendekati 600.000 ...</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/infografik/5685009/sphp-jaga-harga-beras</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/20260807-SPHP-jaga-harga-beras_1.jpg</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Kemarin, Febrie diperiksa hingga tersangka kasus Petral dilimpahkan</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 05:57:58 +0700</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Sejumlah peristiwa hukum telah diwartakan oleh pewarta Kantor Berita ANTARA pada Jumat (7/8). Berikut beberapa berita ...</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685284/kemarin-febrie-diperiksa-hingga-tersangka-kasus-petral-dilimpahkan</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/kejagung-periksa-febrie-adriansyah-2836449.jpg</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Kemarin, rumus bernegara Prabowo hingga pendaftaran upacara HUT RI</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 05:56:55 +0700</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Sejumlah peristiwa politik telah diwartakan oleh pewarta Kantor Berita ANTARA pada Jumat (7/8). Berikut beberapa berita ...</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685283/kemarin-rumus-bernegara-prabowo-hingga-pendaftaran-upacara-hut-ri</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1001561814.jpg</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Titik Awal Kebakaran Gedung Bapenda DKI Diduga di Lantai 11 yang Direnovasi</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 06:14:53 +0700</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Rolando Fransiscus Sihombing</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Kebakaran hebat melanda gedung Bapenda DKI Jakarta, diduga berasal dari lantai 11 yang sedang direnovasi. Tim Puslabfor Polri menyelidiki penyebabnya.</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609407/titik-awal-kebakaran-gedung-bapenda-dki-diduga-di-lantai-11-yang-direnovasi</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/kebakaran-gedung-bapenda-dki-1786136516980_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Akhir Pelarian 8 Orang yang Siksa dan Paksa Onani Pria di Tangerang</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 06:00:31 +0700</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Tim detikcom</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Pelaku penganiayaan pria PG di Tangerang ditangkap di Pemalang. Korban dipaksa onani dan disiksa oleh rekan kerja setelah ingin resign.</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609406/akhir-pelarian-8-orang-yang-siksa-dan-paksa-onani-pria-di-tangerang</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2024/12/03/ilustrasi-pelecehan_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Korban Kebakaran yang Dievakuasi dari Gedung Bapenda DKI Seorang Pekerja</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 05:20:12 +0700</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Rolando Fransiscus Sihombing</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Petugas damkar DKI Jakarta berhasil mengevakuasi seorang pekerja dari lantai 15 gedung Bapenda yang terbakar. Pekerja dibawa ke rumah sakit untuk perawatan.</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609402/korban-kebakaran-yang-dievakuasi-dari-gedung-bapenda-dki-seorang-pekerja</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/korban-kebakaran-gedung-bapenda-dki-dievakuasi-1786140604946_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Prabowo Sebut Swasembada Pangan Nyata: Periksa Semua Gudang!</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 05:55:00 +0700</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Ilyas Fadilah</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Presiden Prabowo Subianto menyatakan Indonesia berhasil mencapai swasembada pangan.</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8609337/prabowo-sebut-swasembada-pangan-nyata-periksa-semua-gudang</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/31/presiden-prabowo-subianto-saat-memberikan-taklimat-di-depan-para-pimpinan-kamar-dagang-dan-industri-indonesia-kadin-di-istana--1785493704621_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Ananta Rispo Pamer Motor Baru Hadiah Ultah ke-8 Nikah dengan Siti Rohmah</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 06:03:00 +0700</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Mauludi Rismoyo</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Artis Ananta Rispo lagi berbahagia. Ia telah menjalani 8 tahun pernikahan dengan Siti Rohmah.</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8606520/ananta-rispo-pamer-motor-baru-hadiah-ultah-ke-8-nikah-dengan-siti-rohmah</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/ananta-rispo-1785987182815_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Apel Kebangsaan Jaga Jakarta Digelar di Monas Hari Ini</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 06:00:09 +0700</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Apel Kebangsaan Jaga Jakarta digelar di Monas, diinisiasi Polda Metro Jaya dengan menggandeng Kodam Jaya, Pemprov DKI dan sejumlah elemen masyarakat.</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260807193505-20-1389922/apel-kebangsaan-jaga-jakarta-digelar-di-monas-hari-ini</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2025/10/05/atraksi-udara-peringatan-hut-ke-80-tni-1759651629093_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>FOTO: Dua Pekan Macet Panjang Jalintim Sumatra di Palembang-Jambi</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 05:20:19 +0700</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Antrean kendaraan mengular di Jalintim di Air Batu, Banyuasin, Sumsel, yang menyambungkan rute Palembang dan Jambi selama dua pekan terakhir.</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260807185059-22-1389882/foto-dua-pekan-macet-panjang-jalintim-sumatra-di-palembang-jambi</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2022/04/25/jalan-lintas-timur-palembang-jambi-macet-49km-4_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Polisi Periksa Bigmo soal Ajak Anak Promo Vape Senin Pekan Depan</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 05:13:10 +0700</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Polda Metro Jaya akan memeriksa Youtuber Bigmo terkait dugaan mengajak anak di bawah umur mempromosikan liquid vape. Bigmo telah meminta maaf atas aksinya.</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808001432-12-1389989/polisi-periksa-bigmo-soal-ajak-anak-promo-vape-senin-pekan-depan</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2019/11/16/a05eed0d-ca97-43c2-8af8-6051f205a1ac_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Selain Febrie, Kejagung Periksa Nurman Herin di Kasus TPPU Kemarin</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 04:45:54 +0700</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Mobil tahanan menjemput Eks Jampidsus Febrie Adriansyah, tersangka TPPU, untuk pemeriksaan di Kejaksaan Agung.</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260807151935-12-1389781/selain-febrie-kejagung-periksa-nurman-herin-di-kasus-tppu-kemarin</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/07/kejagung-periksa-febrie-adriansyah-1786091327929_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Basarnas Kerahkan Heli Sisir Lokasi Kebakaran KMP Mutiara Sentosa II</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 04:18:52 +0700</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Basarnas terus mencari korban KMP Mutiara Sentosa II yang terbakar di perairan Madura meskipun operasi SAR resmi ditutup.</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260807235305-20-1389987/basarnas-kerahkan-heli-sisir-lokasi-kebakaran-kmp-mutiara-sentosa-ii</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/03/evakuasi-korban-tewas-kebakaran-km-mutiara-sentosa-ii-di-sumenep-1785712804547_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Dinsos Sulsel: Rekening Bansos Dipakai Judol Terbanyak Ada di Makassar</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 03:45:39 +0700</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Kepala Dinas Sosial Sulsel, Abdul Malik, ungkap banyak rekening penerima bansos di Makassar terindikasi judi online.</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808002125-20-1389990/dinsos-sulsel-rekening-bansos-dipakai-judol-terbanyak-ada-di-makassar</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2024/06/15/ilustrasi-judi-online-8_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Momen Prabowo Tes Langsung Kekuatan Genteng Buatan BRIN</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 03:08:28 +0700</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Presiden RI Prabowo Subianto melakukan uji coba ketahanan genteng inovasi Badan Riset dan Inovasi Nasional (BRIN), Kamis (6/8).</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260807105859-24-1389626/momen-prabowo-tes-langsung-kekuatan-genteng-buatan-brin</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/07/thumbnail-video-1786075284912_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Terdakwa Ledakan Galangan Tewaskan Pekerja Dituntut 1-2 Tahun Penjara</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 02:14:16 +0700</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Tujuh terdakwa kasus ledakan galangan kapal MT Federal II di Batam dituntut ringan, satu hingga dua tahun penjara.</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808015028-12-1389992/terdakwa-ledakan-galangan-tewaskan-pekerja-dituntut-1-2-tahun-penjara</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/03/07/tugboat-dihimpit-kapal-kargo-dikawasan-galangan-pt-asl-3-tewas-1-selamat-dan-1-hilang-1772861051992_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>FOTO: Sodom dan Gomorra, Operasi Polisi Bongkar Prostitusi Lima</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 05:30:20 +0700</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Operasi Soddom dan Gomorra sudah digelar berulang di berbagai distrik sejak 2022 untuk memberantas jaringan trata de personas dan proxenetismo.</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260807164223-136-1389819/foto-sodom-dan-gomorra-operasi-polisi-bongkar-prostitusi-lima</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/07/sodoma-dan-gomorra-operasi-polisi-bongkar-bordil-prostitusi-di-lima-1786095664231_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Timnas Voli Putri Indonesia Putus Rekor 7 Tahun Tak Bisa Menang atas Vietnam</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 05:46:25 +0700</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Timnas voli putri Indonesia memutus rekor tujuh tahun tidak bisa menang atas Vietnam lewat laga SEA V Cup 2026 leg kedua, Jumat (7/8/2026).</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7865571/timnas-voli-putri-indonesia-putus-rekor-7-tahun-tak-bisa-menang-atas-vietnam</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ji5jh_awPmeoo7bKdWFIChFnymU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Pemain-Timnas-Voli-Putri-Indonesia-melakukan-perayaan-setelah-mencetak-poin-saat.jpg</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Kejagung Buka Suara Terkait Sosok Febrio Dalam Kasus Kematian Sutrimo</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 06:24:43 +0700</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Kematian Sutrimo, Karumga Febrie Adriansyah meninggal tanda tanya.</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8264799/kejagung-buka-suara-terkait-sosok-febrio-dalam-kasus-kematian-sutrimo</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/Y9TE7xG2JA6_i8rqt0nVTPtgvjE=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9318584/original/056702000_1786106661-IMG_3040.jpg</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Kejagung Dalami Tujuh Perusahaan Terkait TPPU Febrie Adriansyah</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 06:14:03 +0700</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Kejagung menggeledah sejumlah kantor di Jakarta Selatan.</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8264795/kejagung-dalami-tujuh-perusahaan-terkait-tppu-febrie-adriansyah</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/FWX7CtExPF_PSpp3N1NQ8JeXw4E=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9318067/original/070489600_1786085809-IMG_20260807_131157_324.jpg</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Sisi Pahit Kurir Paket, Terjerat Suspend hingga Ongkir Terpangkas</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 06:07:25 +0700</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Setiap paket punya tujuan dan batas waktu. Di tengah jalan, kurir harus berhadapan dengan macet, alamat yang meleset, hingga risiko order bermasalah.</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8264580/sisi-pahit-kurir-paket-terjerat-suspend-hingga-ongkir-terpangkas</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/AVvSi1_7wSvYIv0OvBXkq7BSFn4=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9318563/original/039261100_1786104390-unnamed__23_.jpg</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I81"/>
+  <autoFilter ref="A1:I103"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-08 00:48 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-08.xlsx
+++ b/data/berita_2026-08-08.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$103</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$124</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I103"/>
+  <dimension ref="A1:I124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -5274,8 +5274,995 @@
         </is>
       </c>
     </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Ketangguhan makroekonomi sebagai kunci menghadapi tekanan daya beli</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 07:34:58 +0700</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Ada optimisme sekaligus kewaspadaan ketika Produk Domestik Bruto (PDB) Indonesia pada Kuartal II-2026 dirilis ke ...</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685307/ketangguhan-makroekonomi-sebagai-kunci-menghadapi-tekanan-daya-beli</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/10/26/1000729380_1600x1063.jpg</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Operasi katarak gratis perluas akses layanan kesehatan mata</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 07:31:06 +0700</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>ANTARA - Kementerian Kesehatan bersama Noor Dubai Foundation dan Perhimpunan Dokter Spesialis Mata Indonesia (Perdami) ...</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5685212/operasi-katarak-gratis-perluas-akses-layanan-kesehatan-mata</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_OPERASI-KATARAK-GRATIS-PERLUAS-AKSES-LAYANAN-KESEHATAN-MATA.jpg</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>DKI kemarin, rumah subsidi di Kemayoran hingga risiko obligasi daerah</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 07:28:53 +0700</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Peristiwa penting dan menarik terjadi di Jakarta selama Jumat (7/8) mulai dari Perumnas mulai bangun rumah susun ...</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685304/dki-kemarin-rumah-subsidi-di-kemayoran-hingga-risiko-obligasi-daerah</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/50016df8-c542-46c1-a2d4-0b9080d9190d.jpeg</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Kemarin, pemberhentian kepala SPPG hingga pemadaman kebakaran di Bromo</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 07:25:21 +0700</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Sejumlah warta humaniora kemarin, Jumat (7/8), masih menarik dibaca hari ini, mulai dari Badan Gizi Nasional (BGN) ...</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685301/kemarin-pemberhentian-kepala-sppg-hingga-pemadaman-kebakaran-di-bromo</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/Penutupan-Wisata-Bromo-040826-IS-4.jpg</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>BMKG prakirakan cuaca di mayoritas wilayah RI berawan tebal pada Sabtu</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 07:20:32 +0700</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Badan Meteorologi, Klimatologi, dan Geofisika (BMKG) memprakirakan cuaca hari ini, Sabtu, di sebagian besar wilayah ...</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685300/bmkg-prakirakan-cuaca-di-mayoritas-wilayah-ri-berawan-tebal-pada-sabtu</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2024/10/22/Waspada-Cuaca-Ekstrim-021120-Ief-1.jpg</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Perdagangan menumbuhkan peradaban</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 07:08:52 +0700</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Pameran sering dipandang sebagai peristiwa yang datang lalu berlalu. Stan dibongkar, lampu dipadamkan, dan keramaian ...</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685297/perdagangan-menumbuhkan-peradaban</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/SGE-2026-25.jpg</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Festival Lembah Baliem di Papua Pegunungan</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 07:00:31 +0700</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Sejumlah warga menari dalam pembukaan Festival Budaya Lembah Baliem (FBLB) ke-34 di Kabupaten Jayawijaya, Papua ...</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5685296/festival-lembah-baliem-di-papua-pegunungan</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/Festival-Lembah-Baliem-070826-yef-1.jpg</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Kriminal kemarin, Polisi sita 132 kg ganja hingga korban mutilasi</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 07:00:13 +0700</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Peristiwa kriminal terjadi di wilayah hukum Polda Metro Jaya pada Jumat (7/8) mulai dari Polres Jakpus sita 132 ...</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685295/kriminal-kemarin-polisi-sita-132-kg-ganja-hingga-korban-mutilasi</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/20260807_103050.jpg</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Ekonomi kemarin, Tol Prosiwangi hingga Telkom pangkas 34 entitas</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 06:53:19 +0700</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Berbagai peristiwa ekonomi diberitakan Kantor Berita ANTARA pada Jumat (7/8), mulai dari kesiapan pengoperasian Tol ...</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685293/ekonomi-kemarin-tol-prosiwangi-hingga-telkom-pangkas-34-entitas</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/Tol-Prosiwngi-Dibuka-Fungsional-Lumajang-160326-IS-3A.jpg</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Kebakaran gedung Badan Pendapatan Daerah DKI Jakarta</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 06:24:36 +0700</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Petugas Dinas Penanggulangan Kebakaran dan Penyelamatan (Gulkarmat) Jakarta bersiap memadamkan kobaran api yang ...</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5685289/kebakaran-gedung-badan-pendapatan-daerah-dki-jakarta</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/Gedung-Bapenda-DKI-Jakarta-kebakaran-070826-Bay-3.jpg</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Kencan singkat dengan Suzuki XL7 di GIIAS 2026</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 02:45:27 +0700</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/antaranewsdotcom</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Memanfaatkan pameran otomotif Gaikindo Indonesia International Auto Show (GIIAS) 2026, PT Suzuki Indomobil Sales (SIS) ...</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/berita/5685248/kencan-singkat-dengan-suzuki-xl7-di-giias-2026</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/WhatsApp-Image-2026-08-07-at-19.53.52.jpeg</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>OJK dorong literasi keuangan seiring meningkatnya pembiayaan kendaraan</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 02:21:55 +0700</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/antaranewsdotcom</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Otoritas Jasa Keuangan (OJK) menilai masih perlu adanya peningkatan literasi keuangan agar keputusan finansial yang ...</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/berita/5685229/ojk-dorong-literasi-keuangan-seiring-meningkatnya-pembiayaan-kendaraan</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/FOTO-4.JPG.jpeg</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Polisi Periksa 10 Saksi Terkait Kebakaran 6 Lantai di Gedung Bapenda DKI</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 07:25:30 +0700</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Rolando Fransiscus Sihombing</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Polisi memeriksa 10 saksi terkait kebakaran gedung Bapenda DKI Jakarta yang melanda 6 lantai. Penyebab kebakaran masih dalam penyelidikan.</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609449/polisi-periksa-10-saksi-terkait-kebakaran-6-lantai-di-gedung-bapenda-dki</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/kebakaran-gedung-bapenda-dki-1786136517063_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Pencarian Kaki Korban Mutilasi Depok Setelah 3 Pekan Terlewati</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 07:08:24 +0700</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Tim detikcom</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Pencarian potongan kaki korban mutilasi K di Kali Licin, Depok, masih berlanjut. Polisi menggunakan anjing K-9 untuk membantu menemukan sisa tubuh korban.</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609441/pencarian-kaki-korban-mutilasi-depok-setelah-3-pekan-terlewati</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/polisi-lanjut-cari-potongan-kaki-korban-mutilasi-di-kali-licin-depok-devidetikcom-1786074971617_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Waka Komisi IX DPR Dorong BGN Investigasi Buntut Kasus Keracunan MBG</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 06:52:25 +0700</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Tim detikcom</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Wakil Ketua Komisi IX DPR Yahya Zaini menyarankan orang tua dapat menuntut jalur hukum jika anaknya sakit akibat keracunan MBG.</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609440/waka-komisi-ix-dpr-dorong-bgn-investigasi-buntut-kasus-keracunan-mbg</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/01/30/wakil-ketua-komisi-ix-dpr-yahya-zaini-1769785727227_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Sosok Pemilik Nyaris Seribu Senjata dalam Sekolah di Jaksel Terkuak</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 06:33:49 +0700</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Tim detikcom</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Sekolah swasta di Pondok Pinang, Jakarta Selatan bikin heboh karena ditemukan hampir seribu senjata di salah satu ruangan. Pemilik senjata itu akhirnya terkuak.</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609417/sosok-pemilik-nyaris-seribu-senjata-dalam-sekolah-di-jaksel-terkuak</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/ruangan-mantan-kepala-yayasan-ditemukannya-senjata-di-sekolah-swasta-jaksel-taufiqdetikcom-1786104460813_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Diah Permatasari-Cut Keke Awet 20 Tahun Bersahabat, Saling Hormati Privasi</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 07:07:41 +0700</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>wes</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Persabahatan Diah Permatasari dengan Cut Keke telah terjalin 20 tahun. Diah menuturkan sangat menghargai privasi masing-masing.</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8608282/diah-permatasari-cut-keke-awet-20-tahun-bersahabat-saling-hormati-privasi</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/diah-paramita-dan-cut-keke-1786077414535_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Kereta Trans Sumatra Dilirik KAI, China-Rusia Minati Trans Kalimantan</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 06:00:12 +0700</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Dudy mengungkap KAI berminat mengembangkan proyek Trans Sumatra, sementara investor China dan Rusia lebih tertarik menggarap Trans Kalimantan Railway.</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260807192607-92-1389918/kereta-trans-sumatra-dilirik-kai-china-rusia-minati-trans-kalimantan</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/02/19/menteri-perhubungan-ri-dudy-purwagandhi-menyebut-sejumlah-infrastruktur-perkeretaapian-di-sumatra-tak-memungkinkan-untuk-menun-1771482477996_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Chord Gitar dan Lirik Lagu Jangan Paksa Rindu (Beda) - Ifan Seventeen</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 07:34:00 +0700</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>TribunNews.com menyajikan berita dan video terkini dari regional, nasional dan internasional dengan sudut pandang dan nilai-nilai lokal</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>https://asset-2.tribunnews.com/tribunnews/foto/bank/images/logo-tribunnews1_20160901_101844.jpg</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Kuasa Hukum Febrie Adriansyah Persoalkan Sprindik hingga Penerapan Pasal</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 06:46:34 +0700</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Tim hukum eks Jampidsus Febrie menilai penyidikan dugaan TPPU cacat hukum.</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8264804/kuasa-hukum-febrie-adriansyah-persoalkan-sprindik-hingga-penerapan-pasal</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/0L8AdUORc9UC8IsqRUWD4-5dQKQ=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9318645/original/065692700_1786119340-IMG_3095.jpg</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Bantah Punya 74 Kg Emas, Kubu Febrie Soroti Hal yang Belum Terungkap</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 06:33:13 +0700</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Persoalan kepemililkan emas kembali ditanya penyidik ke Febrie</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8264800/bantah-punya-74-kg-emas-kubu-febrie-soroti-hal-yang-belum-terungkap</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/2WEvQ2hmLFTijz9iyBipOx1Njqg=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9318624/original/089072000_1786113401-IMG_3067.jpg</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I103"/>
+  <autoFilter ref="A1:I124"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-08 02:57 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-08.xlsx
+++ b/data/berita_2026-08-08.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$124</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$228</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I124"/>
+  <dimension ref="A1:I228"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -6261,8 +6261,4897 @@
         </is>
       </c>
     </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Wamenkomdigi: Kampus harus jaga sisi kritis mahasiswa hadapi Gen AI</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:46:43 +0700</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Wakil Menteri Komunikasi dan Digital (Wamenkomdigi) Nezar Patria meminta perguruan tinggi agar tetap dapat menjaga sisi ...</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685391/wamenkomdigi-kampus-harus-jaga-sisi-kritis-mahasiswa-hadapi-gen-ai</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/1000141205.jpg</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>BI Bali manfaatkan 400 ribu lembar limbah uang rusak jadi medali</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:45:05 +0700</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Kantor Perwakilan Bank Indonesia (BI) Provinsi Bali memanfaatkan sekitar 400 ribu lembar limbah uang tidak layak edar ...</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685389/bi-bali-manfaatkan-400-ribu-lembar-limbah-uang-rusak-jadi-medali</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG_20260808_093510.jpg</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Kemenkum Sulteng catat 84.374 layanan AHU hingga Juli 2026</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:40:22 +0700</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Kantor Wilayah Kementerian Hukum Sulawesi Tengah mencatat sebanyak 84.374 layanan Administrasi Hukum Umum (AHU) ...</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685387/kemenkum-sulteng-catat-84374-layanan-ahu-hingga-juli-2026</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG-20260802-WA0012-1.jpg</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>YIARI: Karhutla berulang di Ketapang picu konflik orangutan-warga</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:39:39 +0700</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Yayasan Inisiasi Alam Rehabilitasi Indonesia (YIARI) menyatakan kebakaran hutan dan lahan (karhutla) yang terus ...</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685384/yiari-karhutla-berulang-di-ketapang-picu-konflik-orangutan-warga</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG-20260807-WA0034.jpg</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Status kebakaran gedung Bapenda DKI masih dalam tahap pendinginan</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:36:54 +0700</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Suku Dinas Penanggulangan Kebakaran dan Penyelamatan (Gulkarmat) Jakarta Pusat menyatakan status kebakaran di gedung ...</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685383/status-kebakaran-gedung-bapenda-dki-masih-dalam-tahap-pendinginan</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001017459.jpg</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Polisi tangkap komplotan pencuri dan penadah motor curian di Jakut</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:33:01 +0700</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Unit Reskrim Polsek Metro Penjaringan berhasil membekuk pelaku pencurian sepeda motor berinisial HPP alias B bersama ...</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685379/polisi-tangkap-komplotan-pencuri-dan-penadah-motor-curian-di-jakut</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/dd4f5a8b-5746-4da3-8fc5-217509ef3fc1.jpeg</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Membangun kemandirian energi desa melalui penguatan kapasitas Local Hero</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:30:49 +0700</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Lokal Hero Pertamina Drilling Services Indonesia, Alfredo Nicholas Saputra Kolin berpose di sela-sela kegiatan ...</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5685375/membangun-kemandirian-energi-desa-melalui-penguatan-kapasitas-local-hero</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/WhatsApp-Image-2026-08-08-at-09.09.12-2.jpeg</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Xabi Alonso sebut skuad Chelsea seimbang sesuai kebutuhan Liga Inggris</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:30:30 +0700</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Manajer Chelsea Xabi Alonso menyebut skuad yang dimiliki Chelsea saat ini seimbang di semua lini sehingga sesuai dengan ...</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685372/xabi-alonso-sebut-skuad-chelsea-seimbang-sesuai-kebutuhan-liga-inggris</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/konferensi-pers-chelsea-jelang-melawan-ac-milan-2836872.jpg</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>BKSDA Kalbar evakuasi orangutan di Ketapang dari ancaman karhutla</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:29:25 +0700</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Balai Konservasi Sumber Daya Alam (BKSDA) Kalimantan Barat (Kalbar) mengevakuasi seekor orangutan (Pongo ...</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685369/bksda-kalbar-evakuasi-orangutan-di-ketapang-dari-ancaman-karhutla</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG-20260807-WA0030.jpg</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Jam operasional Transjakarta Blok M-Ancol diperpanpang pekan ini</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:23:20 +0700</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>PT Transportasi Jakarta (Transjakarta) memperpanjang jam operasional layanan rute 1W Blok M–Ancol hingga pukul ...</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685365/jam-operasional-transjakarta-blok-m-ancol-diperpanpang-pekan-ini</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/03/24/InShot_20260324_175339206.jpg</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>BMKG: Pesisir NTT berpotensi dilanda rob pada 8–11 Agustus</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:20:21 +0700</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Badan Meteorologi, Klimatologi, dan Geofisika (BMKG) memperingatkan potensi banjir pesisir atau rob di sejumlah wilayah ...</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685364/bmkg-pesisir-ntt-berpotensi-dilanda-rob-pada-8-11-agustus</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000001557.jpg</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>VDNI modernisasi alat produksi pasir kalsinasi terbesar di Indonesia</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:15:52 +0700</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>PT Virtue Dragon Nickel Industry (VDNI) mulai mengoperasikan dua lini produksi pasir kalsinasi (roasted ore) terbesar ...</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685363/vdni-modernisasi-alat-produksi-pasir-kalsinasi-terbesar-di-indonesia</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/NIKEL.jpg</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Alasan perlu bijak pilih pugasan untuk pelengkap yogurt</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:15:44 +0700</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Yoghurt sering digambarkan sebagai makanan sehat, karena perusahaan menyoroti sifat rendah lemak atau ...</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685361/alasan-perlu-bijak-pilih-pugasan-untuk-pelengkap-yogurt</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/12/pexels-haberdoedas-33757136.jpg</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>BPS tegaskan data individu dilindungi oleh undang-undang</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:12:46 +0700</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Badan Pusat Statistik (BPS) menegaskan data-data individu dari data responden BPS dilindungi oleh ...</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685357/bps-tegaskan-data-individu-dilindungi-oleh-undang-undang</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/WhatsApp-Image-2026-08-08-at-08.19.28.jpeg</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Kementerian UMKM: Manfaat ojol sebagai UMKM bisa mendapatkan KUR</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:11:16 +0700</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Kementerian Usaha Mikro, Kecil, dan Menengah (UMKM) mengungkapkan salah satu manfaat pengemudi ojek online atau ojol ...</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685353/kementerian-umkm-manfaat-ojol-sebagai-umkm-bisa-mendapatkan-kur</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/WhatsApp-Image-2026-08-08-at-08.45.30.jpeg</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Danantara perluas akses rumah pertama melalui pembiayaan terintegrasi</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:01:48 +0700</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Badan Pengelola Investasi Daya Anagata Nusantara (Danantara) memperluas akses kepemilikan rumah pertama melalui ...</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685352/danantara-perluas-akses-rumah-pertama-melalui-pembiayaan-terintegrasi</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/Image-07-08-26-at-00.35.jpeg</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Aldila Sutjiadi singkirkan juara Wimbledon untuk melaju di Toronto</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:00:34 +0700</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Petenis Indonesia Aldila Sutjiadi bersama pasangannya petenis Selandia Baru Erin Routliffe membuat kejutan dengan ...</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685348/aldila-sutjiadi-singkirkan-juara-wimbledon-untuk-melaju-di-toronto</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/02/18/WhatsApp-Image-2025-02-18-at-14.35.40.jpeg</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Bansos PKH dan BPNT triwulan III-2026 mulai disalurkan</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Kementerian Sosial (Kemensos) mulai menyalurkan bantuan sosial (bansos) Program Keluarga Harapan (PKH) dan Bantuan ...</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/infografik/5684996/bansos-pkh-dan-bpnt-triwulan-iii-2026-mulai-disalurkan</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/20260808-Bansos-PKH-dan-BPNT-triwulan-III-2026-mulai-disalurkan_1.jpg</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Populer, pemanggilan Bigmo hingga LPDP diminta biayai riset lingkungan</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:56:27 +0700</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Beragam berita di Antaranews.com mendapatkan sorotan dari publik pada Sabtu, di antaranya terkait rencana pemanggilan ...</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685344/populer-pemanggilan-bigmo-hingga-lpdp-diminta-biayai-riset-lingkungan</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/29/1001020636.jpg</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Psikolog: Media sosial bukan tempat tepat melampiaskan amarah</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:55:44 +0700</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Psikolog klinis lulusan Universitas Indonesia sekaligus Direktur Personal Growth, lembaga yang bergerak di bidang ...</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685341/psikolog-media-sosial-bukan-tempat-tepat-melampiaskan-amarah</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/11/06/IMG-20251106-WA0061.jpg</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Survei ungkap kenaikan biaya jadi kekhawatiran utama pelaku usaha di Singapura</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:50:23 +0700</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Meningkatnya biaya usaha menjadi kekhawatiran terbesar bagi perusahaan-perusahaan di Singapura seiring ketegangan ...</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685340/survei-ungkap-kenaikan-biaya-jadi-kekhawatiran-utama-pelaku-usaha-di-singapura</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/CjkinzN000011_20260807_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>DKI diminta siapkan pelayanan kesehatan untuk antisipasi ISPA</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:48:53 +0700</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Pemerintah Provinsi (Pemprov) DKI Jakarta diminta menyiapkan pelayanan kesehatan di berbagai tingkatan yang memadai dan ...</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685336/dki-diminta-siapkan-pelayanan-kesehatan-untuk-antisipasi-ispa</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/11/20/1000680100.jpg</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Sri Lanka luncurkan program pengelolaan sampah nasional</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:43:24 +0700</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Sri Lanka meluncurkan program pengelolaan sampah nasional. Program ini bertujuan untuk membangun sistem nasional ...</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685332/sri-lanka-luncurkan-program-pengelolaan-sampah-nasional</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/Pabrik-daur-ulang-untuk-mengatasi-sampah-botol-plastik-041124-fah-7.jpg</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Polda Jambi pecat lima personel terkait tewasnya anggota Polres</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:40:31 +0700</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Polda Jambi menjatuhkan sanksi pemberhentian tidak dengan hormat (PTDH) kepada lima personel Polri terkait kasus ...</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685329/polda-jambi-pecat-lima-personel-terkait-tewasnya-anggota-polres</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/373418.jpg</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Indonesia raih empat medali di olimpiade bidang AI IOAI 2026</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:25:39 +0700</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Kontingen Indonesia meraih satu medali emas, dua perak, dan satu perunggu dalam Olimpiade Internasional Kecerdasan ...</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685325/indonesia-raih-empat-medali-di-olimpiade-bidang-ai-ioai-2026</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2024/11/04/KBRI-Astana.jpg</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Sabtu, gerai Samsat Keliling tersedia di delapan wilayah Detabek</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:23:13 +0700</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Polda Metro Jaya menyediakan layanan Sistem Administrasi Manunggal Satu Atap (Samsat) Keliling untuk membantu para ...</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685323/sabtu-gerai-samsat-keliling-tersedia-di-delapan-wilayah-detabek</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/04/1000806217_1.jpg</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Psikolog: terapkan “pause before posting” saat emosi meningkat</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:21:19 +0700</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Psikolog klinis lulusan Universitas Indonesia Ratih Ibrahim, MM, Psikolog, menyarankan seseorang menerapkan ...</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685320/psikolog-terapkan-pause-before-posting-saat-emosi-meningkat</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2021/08/13/antarafoto-jumlah-koneksi-ponsel-di-indonesia-130821-ysw-4.jpg</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Bawaslu gandeng mahasiswa wujudkan demokrasi transparan di era digital</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:15:03 +0700</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>ANTARA - Badan Pengawas Pemilihan Umum (Bawaslu), menggandeng kalangan mahasiswa bertransformasi digital di ...</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5685225/bawaslu-gandeng-mahasiswa-wujudkan-demokrasi-transparan-di-era-digital</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/BAWASLU-GANDENG-MAHASISWA-WUJUDKAN-DEMOKRASI-TRANSPARAN-DI-ERA-DIGITAL.jpg</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Perbaikan sawah terdampak bencana di Aceh Barat capai 75 persen</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:11:57 +0700</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>ANTARA - Pemulihan area persawahan seluas 1.308 hektare yang terdampak bencana di Kabupaten Aceh Barat, Aceh, kini ...</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5685219/perbaikan-sawah-terdampak-bencana-di-aceh-barat-capai-75-persen</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/PERBAIKAN-SAWAH-TERDAMPAK-BENCANA-DI-ACEH-BARAT-CAPAI-75-PERSEN-rev_2.jpg</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Sabtu, SIM Keliling tersedia di lima lokasi Jakarta</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:11:34 +0700</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Direktorat Lalu Lintas Polda Metro Jaya menyediakan layanan surat izin mengemudi (SIM) Keliling di lima lokasi di ...</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685319/sabtu-sim-keliling-tersedia-di-lima-lokasi-jakarta</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/03/6988.jpg</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Ratusan migran terdampar di Pantai Ceuta tak dapat ajukan suaka</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:04:48 +0700</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Ratusan migran masih terdampar di Pantai Playa del Trampolín, di wilayah Ceuta, wilayah kantong Spanyol di ...</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685317/ratusan-migran-terdampar-di-pantai-ceuta-tak-dapat-ajukan-suaka</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/AA-20260731-42116094-42116077-MIGRANTS_ARRIVE_ON_SHORE_AFTER_ATTEMPTING_SEA_CROSSING_TO_CEUTA_FROM_MOROCCO.jpg</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Pasar Ambuwa: ruang edukasi zero waste dan pangan lokal Gorontalo</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 07:59:23 +0700</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Deretan tikar tergelar di bawah rindangnya pepohonan Pasar Kuliner Ambuwa di Desa Huntu Selatan, Bone Bolango, ...</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685313/pasar-ambuwa-ruang-edukasi-zero-waste-dan-pangan-lokal-gorontalo</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/IMG_2014.jpeg</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Dubes: Rwanda mau perluas kerja sama bidang hankam dengan Indonesia</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 07:57:36 +0700</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Duta Besar Rwanda untuk Indonesia Abdul Karim Harelimana menyoroti kemitraan dengan Indonesia di bidang pertahanan dan ...</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685311/dubes-rwanda-mau-perluas-kerja-sama-bidang-hankam-dengan-indonesia</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG_1952.jpg</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Rekomendasi K-drama romcom hingga BLACKPINK rayakan 10 tahun debut</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 07:55:53 +0700</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Ragam warta seperti rekomendasi K-drama bergenre komedi romantis, BLACKPINK hadir di perayaan 10 tahun debut, festival ...</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685308/rekomendasi-k-drama-romcom-hingga-blackpink-rayakan-10-tahun-debut</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/02/28/Pink.jpg</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Kapolda Metro-Pangdam Jaya Pimpin Apel Kebangsaan, Ajak Warga Jaga Jakarta</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:41:14 +0700</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Kapolda dan Pangdam Jaya pimpin Apel Kebangsaan Jaga Jakarta. Elemen masyarakat berkomitmen menjaga keamanan dan persatuan untuk Indonesia.</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609526/kapolda-metro-pangdam-jaya-pimpin-apel-kebangsaan-ajak-warga-jaga-jakarta</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/polda-metro-jaya-menggelar-apel-kebangsaan-menggandeng-ormas-untuk-menjaga-jakarta-1786156805660_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Pendinginan Kebakaran Gedung Bapenda DKI Masih Berlanjut Pagi Ini</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:03:43 +0700</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Brigitta Belia Permata Sari</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Gedung Bapenda DKI Jakarta di terbakar tadi malam. Petugas pemadam kebakaran masih melakukan pendinginan hingga pagi ini.</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609499/pendinginan-kebakaran-gedung-bapenda-dki-masih-berlanjut-pagi-ini</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/kondisi-gedung-bapenda-dki-usai-terbakar-1786154575590_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Kapolri Hadiri Apel Pembukaan Muktamar XVI Tapak Suci Putera Muhammadiyah</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:55:56 +0700</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Rolando Fransiscus Sihombing</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Kapolri Jenderal Listyo Sigit Prabowo menghadiri Muktamar XVI Tapak Suci di Semarang, menerima penganugerahan anggota kehormatan dari PP TSPM.</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609494/kapolri-hadiri-apel-pembukaan-muktamar-xvi-tapak-suci-putera-muhammadiyah</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/kapolri-hadiri-apel-pembukaan-muktamar-xvi-tapak-suci-putera-muhammadiyah-1786154090566_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Bercak Darah hingga Tulang Ditemukan di Konter Bos HP Ambarawa Tewas Dibunuh</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:48:07 +0700</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Ardian Dwi Kurnia</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>Polisi mengungkap ada bercak darah dan serpihan tulang yang ditemukan di konter ponsel korban.</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609490/bercak-darah-hingga-tulang-ditemukan-di-konter-bos-hp-ambarawa-tewas-dibunuh</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/konter-hp-royal-phone-di-ambarawa-tkp-pencurian-dengan-kekerasan-kamis-682026-1786034565707_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Muncul Harapan Stasiun Gunung Putri Aktif Lagi, KCI Colek Kemenhub</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:45:47 +0700</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Firda Cynthia Anggrainy</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>Warga Gunung Putri berharap Stasiun nonaktif di Bogor dapat diaktifkan kembali. KAI Commuter akan mendorong regulator untuk reaktivasi stasiun.</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609488/muncul-harapan-stasiun-gunung-putri-aktif-lagi-kci-colek-kemenhub</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/06/manajer-public-relations-kai-commuter-leza-arlan-1783322149409_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Polisi Tangkap Komplotan Pencuri 600 Besi Ulir di Cikande Serang</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:22:59 +0700</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Arief Ikhsanudin</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>Tim Opsnal Polsek Cikande menangkap pencuri 600 batang besi ulir dan satu penadah. Aksi mereka terencana menggunakan crane untuk menghindari kecurigaan.</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609477/polisi-tangkap-komplotan-pencuri-600-besi-ulir-di-cikande-serang</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2023/07/25/ilustrasi-penangkapan_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Kata 2 Pihak soal Konflik Yayasan Terkait Ratusan Senjata di Sekolah</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:04:48 +0700</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Tim detikcom</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>Ratusan senjata ditemukan di sekolah swasta Jakarta. Pihak eks yayasan mengklaim senjata milik perusahaan berizin, namun ada konflik internal yang terungkap.</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609466/kata-2-pihak-soal-konflik-yayasan-terkait-ratusan-senjata-di-sekolah</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/temuan-ratusan-pucuk-senjata-di-sekolah-swasta-di-pondok-pinang-jakarta-selatan-1786014363566_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Bisik-bisik Reshuffle Setelah Agustusan Mencuat Lagi</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 07:45:55 +0700</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Tim detikcom</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>Kabar reshuffle kabinet Prabowo Subianto mencuat setelah 17 Agustus. Petinggi parpol hingga Istana merespons isu tersebut.</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609459/bisik-bisik-reshuffle-setelah-agustusan-mencuat-lagi</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/12/15/presiden-prabowo-pimpin-sidang-kabinet-paripurna-1765806819431_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Dana Asing Rp 17 T Masuk Pinjol RI, Pertanda Apa?</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:00:03 +0700</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Andi Hidayat</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>Otoritas Jasa Keuangan (OJK) mencatat pendanaan industri pinjaman daring (pindar) dari lender luar negeri sebesar Rp 17,28 triliun.</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/moneter/d-8609446/dana-asing-rp-17-t-masuk-pinjol-ri-pertanda-apa</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2022/11/24/ilustrasi-pinjol_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Prabowo Sudah Panggil Calon-calon Bos BI, Destry Damayanti Masuk Radar</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:00:30 +0700</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Herdi Alif Al Hikam</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>Presiden Prabowo Subianto masih mencari sosok yang tepat untuk menjadi Gubernur Bank Indonesia (BI) definitif.</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/moneter/d-8609445/prabowo-sudah-panggil-calon-calon-bos-bi-destry-damayanti-masuk-radar</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2017/05/15/726a6b96-e680-467e-b116-7fbb4ac0e022_169.jpg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Prabowo Ungkap Hampir 2.500 Jembatan Dibangun di Desa-desa</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 06:55:00 +0700</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Ilyas Fadilah</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Presiden Prabowo Subianto menyatakan pemerintah terus mempercepat pembangunan jembatan di desa-desa.</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/infrastruktur/d-8609341/prabowo-ungkap-hampir-2-500-jembatan-dibangun-di-desa-desa</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/20/presiden-prabowo-subianto-dok-youtube-setpres-1784537467947_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Harapan Kembali Mekar dari Kebun Bugenvil</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 06:30:00 +0700</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Agung Pambudhy</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Pembudidaya bugenvil di Bireuen kembali bangkit usai banjir bandang 2025 dengan meningkatnya penjualan tanaman hias seiring pulihnya akses pasar.</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/foto-bisnis/d-8609131/harapan-kembali-mekar-dari-kebun-bugenvil</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/usaha-tanaman-hias-bugenvil-pascabencana-di-aceh-1786109934911_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Potret Sederhana nan Hangat, Luna Maya Bersama Kakak Rayakan Ultah Ibu Desa</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:09:34 +0700</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Desi Puspasari</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Desa Maya Waltraud Maiyer, ibunda Luna Maya, ulang tahun. Anak-anak kumpul dan rayakan ultah ibu dengan suasana sederhana nan hangat.</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8609374/potret-sederhana-nan-hangat-luna-maya-bersama-kakak-rayakan-ultah-ibu-desa</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/luna-maya-1786124535117_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Irish Bella Bahagia Banget Penantian Panjang Hamil Anak Haldy Sabri Terkabul</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:07:23 +0700</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>wes</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Irish Bella menumpahkan kebahagiaan usai mengumumkan hamil anak pertama dari Haldy Sabri.</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8608272/irish-bella-bahagia-banget-penantian-panjang-hamil-anak-haldy-sabri-terkabul</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/irish-bella-1786070405076_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Kapolri Terima Anugerah Anggota Kehormatan di Muktamar Tapak Suci</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:46:14 +0700</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>Muktamar XVI Tapak Suci Resmi Dibuka di Semarang. Dalam gelaran ini, Kapolri Listyo Sigit Prabowo menerima  Anugerah Anggota Kehormatan.</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808093739-20-1390030/kapolri-terima-anugerah-anggota-kehormatan-di-muktamar-tapak-suci</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/muktamar-xvi-tapak-suci-resmi-dibuka-di-semarang-kapolri-terima-anugerah-anggota-kehormatan-1786156847225_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Warga Padati Cek Kesehatan Gratis dan Sembako di Apel Jaga Jakarta</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:37:40 +0700</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>Warga berbondong memadati tenda cek kesehatan gratis dan pembagian sembako di Apel Kebangsaan Jaga Jakarta untuk Indonesia, Sabtu (8/8).</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808093205-20-1390028/warga-padati-cek-kesehatan-gratis-dan-sembako-di-apel-jaga-jakarta</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/apel-kebangsaan-jaga-jakarta-untuk-indonesia-1786155667431_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Damkar Sisir Titik Panas di Gedung Bapenda DKI Pagi Ini</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:35:09 +0700</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>Petugas pemadam kebakaran masih melakukan pendinginan di Gedung Bapenda DKI Jakarta, Jalan Abdul Muis, Jakarta, Sabtu (8/8) pagi.</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808091544-20-1390026/damkar-sisir-titik-panas-di-gedung-bapenda-dki-pagi-ini</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/gedung-bapenda-dki-jakarta-kebakaran-1786149523783_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Kapolda Metro-Pangdam Jaya Sapa Peserta Apel Kebangsaan Jaga Jakarta</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:53:40 +0700</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>Kapolda Metro Jaya Komjen Pol Asep Edi Suheri dan Pangdam Jaya Letjen TNI Deddy Suryadi menyapa peserta Apel Kebangsaan Jaga Jakarta untuk Indonesia di Monas.</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808085034-20-1390022/kapolda-metro-pangdam-jaya-sapa-peserta-apel-kebangsaan-jaga-jakarta</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/apel-kebangsaan-jaga-jakarta-1786153774792_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Kapolda Metro Jaya: Menjaga Jakarta Berarti Menjaga Indonesia</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:40:29 +0700</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>Kapolda Metro Jaya, Komjen Pol Asep Edi Suheri, serukan menjaga Jakarta dalam Apel Kebangsaan Jaga Jakarta untuk Indonesia yang berlangsung di Monas.</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808083110-20-1390018/kapolda-metro-jaya-menjaga-jakarta-berarti-menjaga-indonesia</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/apel-kebangsaan-jaga-jakarta-1786153342261_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Pangdam Jaya Gandeng Pelbagai Elemen untuk Jaga Jakarta dan RI</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:39:10 +0700</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>Pangdam Jaya Letjen TNI Deddy Suryadi membacakan pernyataan terkait dengan Apel Kebangsaan Jaga Jakarta di Monas pada Sabtu (8/8).</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808082712-20-1390019/pangdam-jaya-gandeng-pelbagai-elemen-untuk-jaga-jakarta-dan-ri</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/apel-kebangsaan-jaga-jakarta-1786153289776_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Apel Kebangsaan Jaga Jakarta Bacakan 5 Deklarasi, Ini Isinya</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:34:06 +0700</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>Apel Kebangsaan Jaga Jakarta untuk Indonesia di Monas dihadiri 11 ribu peserta. Deklarasi lima poin dibacakan untuk menjaga persatuan dan keamanan.</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808075803-20-1390016/apel-kebangsaan-jaga-jakarta-bacakan-5-deklarasi-ini-isinya</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/apel-kebangsaan-jaga-jakarta-1786152525568_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>11 Ribu Orang Ramaikan Apel Kebangsaan Jaga Jakarta Hari Ini</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:22:42 +0700</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>Sekitar 11 ribu orang yang berasal dari berbagai elemen masyarakat turut meramaikan Apel Kebangsaan Jaga Jakarta untuk Indonesia.</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808081826-20-1390017/11-ribu-orang-ramaikan-apel-kebangsaan-jaga-jakarta-hari-ini</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/apel-kebangsaan-jaga-jakarta-1786152525481_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>FOTO: Gedung Bapenda DKI Terbakar Hebat, Satu Korban Dievakuasi</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:15:56 +0700</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>ANTARA</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Gedung Bapenda DKI Jakarta dilalap si jago api pada Jumat (7/8) malam. Satu orang korban yang terjebak di dalam berhasil dievakuasi.</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808073900-22-1390004/foto-gedung-bapenda-dki-terbakar-hebat-satu-korban-dievakuasi</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/gedung-bapenda-dki-jakarta-kebakaran-1786149523867_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Polda Metro Jaya Bantu Amankan Lokasi Kebakaran Gedung Bapenda DKI</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:01:18 +0700</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>Direktorat Samapta Polda Metro Jaya mengerahkan 72 personel untuk membantu penanganan dan pengamanan kebakaran Gedung Bapenda DKI Jakarta.</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808075129-20-1390013/polda-metro-jaya-bantu-amankan-lokasi-kebakaran-gedung-bapenda-dki</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/dit-samapta-polda-metro-jaya-kerahkan-personel-bantu-tangani-kebakaran-gedung-bapenda-1786150184126_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Prabowo Bentuk Tim Gabungan Lonjakkan Mutu Buku SD-SMA</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 07:58:53 +0700</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Presiden Prabowo Subianto akan membentuk tim gabungan untuk meningkatkan kualitas buku ajar bagi siswa SD hingga SMA.</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808075534-20-1390015/prabowo-bentuk-tim-gabungan-lonjakkan-mutu-buku-sd-sma</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/06/istana-buka-suara-soal-pengambilalihan-saham-kereta-cepat-oleh-kemenkeu-1785997652333_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Kebakaran Gedung Bapenda DKI Berhasil Dipadamkan</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 07:25:31 +0700</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>Kebakaran Gedung Bapenda DKI Jakarta berhasil dipadamkan, Sabtu (8/8) dini hari. Titik awal kebakaran diduga berawal dari lantai 11 bangunan.</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808071258-20-1390002/kebakaran-gedung-bapenda-dki-berhasil-dipadamkan</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/gedung-bapenda-dki-jakarta-kebakaran-1786149523783_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Pemprov Jabar Buka Suara soal Yurizal Warga Bogor Dicibir Banyak Nakes</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 07:25:29 +0700</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>Gubernur Jabar merespons soal nakes--termasuk beberapa dari provinsi--mencibir curhatan pasien BPJS. Belakangan almarhum pasien BPJS itu diketahui warga Bogor.</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260807202523-20-1389949/pemprov-jabar-buka-suara-soal-yurizal-warga-bogor-dicibir-banyak-nakes</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2020/07/28/gedung-sate-bandung_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Polisi Ungkap Sosok DS Pemilik Senpi yang Ditemukan di Sekolah Jaksel</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 07:05:19 +0700</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>Polisi mengungkap sosok berinisial DS, pemilik senjata api di sekolah swasta di Jakarta Selatan, merupakan seorang direktur perusahaan impor airsoft gun.</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808063622-12-1389997/polisi-ungkap-sosok-ds-pemilik-senpi-yang-ditemukan-di-sekolah-jaksel</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/06/995-senjata-yang-ditemukan-di-ruang-mantan-ketua-yayasan-sekolah-jaksel-1786011308187_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Polda Jabar Pamer Ribuan Bandar Narkoba dan Pelaku Kejahatan Jalanan</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 06:58:01 +0700</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>Polda Jabar hadirkan ribuan bandar narkoba dan pelaku kejahatan jalanan yang berhasil diamankan sepanjang 2026 hingga pertengahan Juli lalu.</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808065111-12-1389999/polda-jabar-pamer-ribuan-bandar-narkoba-dan-pelaku-kejahatan-jalanan</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2023/05/30/ilustrasi-penangkapan_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Kasus Ratusan Senjata dan Dugaan Sengketa Yayasan Sekolah di Jaksel</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 06:30:11 +0700</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>Kasus ratusan senjata di sekolah swasta Pondok Pinang terkait sengketa yayasan. Kuasa hukum klaim senjata legal untuk ekstrakurikuler menembak.</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260807175104-12-1389853/kasus-ratusan-senjata-dan-dugaan-sengketa-yayasan-sekolah-di-jaksel</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/06/995-senjata-yang-ditemukan-di-ruang-mantan-ketua-yayasan-sekolah-jaksel-1786011308099_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Ekonomi RI Tumbuh 5,29 Persen, Saatnya Investasi atau Tahan Dulu?</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:05:33 +0700</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>Meski momentum ekonomi mulai membaik, investor ritel tetap diminta berhati-hati dan menghindari keputusan investasi yang terburu-buru.</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260808062909-83-1389998/ekonomi-ri-tumbuh-529-persen-saatnya-investasi-atau-tahan-dulu</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2022/04/23/ilustrasi-dompet-berisi-uang-rupiah_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Perajin Pohon Pinang di Tangerang Kebanjiran Pesanan Jelang HUT ke-81</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:35:24 +0700</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>Meningkatnya permintaan pohon pinang jelang HUT ke-81 RI membawa berkah bagi para perajin musiman pohon pinang di Kecamatan Pinang, Tangerang.</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260808065117-92-1390000/perajin-pohon-pinang-di-tangerang-kebanjiran-pesanan-jelang-hut-ke-81</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/07/jelang-hut-ke-81-ri-perajin-pohon-pinang-di-tangerang-kebanjiran-pesanan-1786109302493_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Toyota Klaim Penjualan Kendaraan Elektrifikasi Tumbuh Signifikan di Indonesia</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:37:28 +0700</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>Di semester I 2026, penjualan kendaraan elektrifikasi naik hampir 27 persen dengan volume penjualan 117.000 unit.</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/otomotif/7865613/toyota-klaim-penjualan-kendaraan-elektrifikasi-tumbuh-signifikan-di-indonesia</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/2jnNJmtFVpigwCyhYuIL4FFsnH8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Hiroyuki-Oide-dan-Toyota-bZ4X-BEV-di-GIIAS-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Kebakaran Gedung Bapenda DKI, Api Diduga dari Ruang Server Lantai 11</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:37:01 +0700</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>Dalam penanganan kebakaran tersebut, petugas mengerahkan sekitar 40 unit kendaraan dengan total 200 personel.</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7865612/kebakaran-gedung-bapenda-dki-api-diduga-dari-ruang-server-lantai-11</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/WEg6aNuIonboivDqai0AIN6RniU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Bapenda-1-08082026.jpg</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>KPK Segera Periksa Kepala Kantor Imigrasi Jakarta Selatan Terkait Temuan 8.500 Dolar Singapura</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:33:13 +0700</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>KPK akan memanggil Kepala Kantor Imigrasi Jaksel, Winarko untuk klarifikasi temuan uang tunai 8.500 dolar Singapura.</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865611/kpk-segera-periksa-kepala-kantor-imigrasi-jakarta-selatan-terkait-temuan-8500-dolar-singapura</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/k8nKXH37-FgbyRj3-UYj5SaQHHA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/logo-kpk-nih.jpg</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>8 Fakta Penembakan Sekolah Thailand, Pelaku Remaja 14 Tahun Dikenal Anak Baik, Diduga Dibully</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:25:09 +0700</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>Penembakan sekolah Thailand menewaskan 9 orang. Pelaku remaja 14 tahun dikenal anak baik, namun diduga tertekan dan dibully.</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7865610/8-fakta-penembakan-sekolah-thailand-pelaku-remaja-14-tahun-dikenal-anak-baik-diduga-dibully</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/EEK0q3rG-ePVrPFD67WwzdJ5rp8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Penembakan-di-sekolah-Thailand.jpg</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Sidang Praperadilan Eks Jampidsus Febrie Digelar 18 dan 19 Agustus 2026</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:12:01 +0700</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>Termohon dalam perkara tersebut adalah Jaksa Agung RI cq Jaksa Agung Muda Tipidsus Kejaksaan Agung RI.</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865609/sidang-praperadilan-eks-jampidsus-febrie-digelar-18-dan-19-agustus-2026</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/eQh7NUBPd1a5LZJ7hmRGe9FD4wA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Febrie-Adriansyah-Jalani-Pemeriksaan-Lanjutan-Kasus-TPPU_20260807_134205.jpg</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Luhut Soal Larangan Ekspor Bijih Nikel: Dulu Kami Dicibir, Ditekan</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:11:15 +0700</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>Selain cibiran, Indonesia juga digugat ke Organisasi Perdagangan Dunia (WTO) saat menerbitkan larangan ekspor nikel.</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/bisnis/7865608/luhut-soal-larangan-ekspor-bijih-nikel-dulu-kami-dicibir-ditekan</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/tdBaPhGkUP-QVa6VHpT03-JxDYw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Luhut-Binsar-Pandjaitan-soal-nikel-OK.jpg</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Soal Adanya Pembullyan terhadap Anak-anaknya, Sarwendah Tegaskan Bukan Terjadi di Lingkungan Sekolah</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:10:01 +0700</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>Artis Sarwendah tegaskan adanya pembullyan terhadap anak-anaknya bukan terjadi di lingkungan sekolah.</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7865607/soal-adanya-pembullyan-terhadap-anak-anaknya-sarwendah-tegaskan-bukan-terjadi-di-lingkungan-sekolah</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/hejjyutIHrD-Ze4ySSbS4hhh3cc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/sarwendah-komnas-perempuan.jpg</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Turki-Saudi-Pakistan Bentuk Pakta Pertahanan, Bagaimana Reaksi Iran dan Apa Artinya bagi Israel?</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:08:58 +0700</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>Turki, Saudi, dan Pakistan membentuk pakta pertahanan baru. Iran mengkritik, sementara Israel menghadapi perubahan peta keamanan regional.</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7865606/turki-saudi-pakistan-bentuk-pakta-pertahanan-bagaimana-reaksi-iran-dan-apa-artinya-bagi-israel</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/PvgbH-YBoiclVSPm4k--wF4AK44=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/pakistan-turki-arab-saudi-mbs-erdogan.jpg</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Situasi Terkini di Gedung Bapenda DKI Jakarta, Masih Tercium Bau Bangunan Terbakar</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:07:22 +0700</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>Bangunan Gedung Badan Pendapatan Daerah (Bapenda) DKI Jakarta, Jakarta Pusat, terlihat gosong usai terbakar pada Jumat (7/8/2026) malam.</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7865605/situasi-terkini-di-gedung-bapenda-dki-jakarta-masih-tercium-bau-bangunan-terbakar</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/rv51hiq3uSbhKBZMgl55gt0C_5g=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/kondisi-gedung-Bapenda-DKI-Jakarta-usai-kebakaran.jpg</t>
+        </is>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>5 Hal yang Perlu Diperhatikan saat Daftar TKA 2026 bagi Siswa SMA/SMK Sederajat</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:00:54 +0700</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>Beberapa hal yang perlu diperhatikan saat mendaftar TKA 2026 bagi sekolah dan murid SMA/SMK sederajat agar prosesnya berjalan dengan lancar.</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/pendidikan/7865604/5-hal-yang-perlu-diperhatikan-saat-daftar-tka-2026-bagi-siswa-smasmk-sederajat</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/F94ajPJx-p-EvEmiJMrwViRev8c=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/smk-n-4-kota-malang-pelatihan-pembuatan-aplikasi_20220928_140654.jpg</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Komentar Negatif Nakes pada Pasien BPJS, Menkes Kabinet Bayangan: Ada yang Salah di Sistem Kesehatan</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:00:48 +0700</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>Menteri Kesehatan Kabinet Bayangan Irma Hidayana menilai, viralnya komentar negatif oknum tenaga kesehatan menjadi refleksi bagi dunia kesehatan RI.</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865603/komentar-negatif-nakes-pada-pasien-bpjs-menkes-kabinet-bayangan-ada-yang-salah-di-sistem-kesehatan</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Nhv1FOGhfSQcOjn7TTxomsGyqrU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/celoteh-pasien-bpjs.jpg</t>
+        </is>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Polda Metro Jaya Kerahkan 72 Personel Bantu Tangani Kebakaran Gedung Bapenda DKI</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:54:12 +0700</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>Polda Metro Jaya mengerahkan 72 personel untuk membantu penanganan dan pengamanan kebakaran Gedung Bapenda DKI, Jumat (7/8/2026) malam.</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7865602/polda-metro-jaya-kerahkan-72-personel-bantu-tangani-kebakaran-gedung-bapenda-dki</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Kp-8LNeBplBGvLBymMmQrFKR_yw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/PMJ-bantu-pemadaman-jaya-65-gedung-bapenda-DKI.jpg</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>3 Ganda Putra Malaysia Reuni di Kejuaraan Dunia BWF 2026, Chia/Soh Tatap Memori Manis 4 Tahun Silam</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:50:58 +0700</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>Tiga pasangan ganda putra Malaysia kembali berduet di Kejuaraan Dunia BWF 2026 setelah menjalani perombakan, termasuk Aaron Chia/Soh Wooi Yik.</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7865601/3-ganda-putra-malaysia-reuni-di-kejuaraan-dunia-bwf-2026-chiasoh-tatap-memori-manis-4-tahun-silam</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/yoV87cuvFbibknPtbgk8pRanBAQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/aaron-chiasoh-wooi-yik-kalah_20240608_210449.jpg</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Gugatan Hak Asuh Anak Masih Bergulir, Pengacara Ruben Onsu Sampaikan Pesan untuk Pihak Sarwendah</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:43:31 +0700</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>Pengacara Ruben Onsu sampaikan pesan untuk pihak Sarwendah di tengah bergulirnya gugatan hak asuh anak di Pengadilan Negeri Jakarta Selatan.</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7865600/gugatan-hak-asuh-anak-masih-bergulir-pengacara-ruben-onsu-sampaikan-pesan-untuk-pihak-sarwendah</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/vxemmMAeJ6xXTgYKO3tDO16iMwc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Ruben-Onsu-2-31072025.jpg</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>IPW Ungkap Risiko Polisi Direkrut Sindikat Narkoba: Pimpinan Polri Harus Perkuat Regulasi</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:42:16 +0700</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>IPW menyoroti dugaan keterlibatan anggota Polri dalam sejumlah kasus narkoba sepanjang 2026.</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865599/ipw-ungkap-risiko-polisi-direkrut-sindikat-narkoba-pimpinan-polri-harus-perkuat-regulasi</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/QBhaUDQEU67Cx_9lrMfBuFTKP44=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Kasat-Narkoba-Polresta-Banda-Aceh-AKP-Muhammad-Jabir.jpg</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>20 Link Twibbon Hari Kucing Sedunia 2026, Lengkap dengan Cara Mudah Unggah di Sosial Media</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:31:33 +0700</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>Link Twibbon Hari Kucing Sedunia 2026, bingkai foto cocok dipakai sebagai foto profil dan diunggah di sosial media pada tanggal 8 Agustus 2026.</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865598/20-link-twibbon-hari-kucing-sedunia-2026-lengkap-dengan-cara-mudah-unggah-di-sosial-media</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/-ED9w7lb7EbWLU4JnXL0MbmFBgI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Link-Twibbon-Hari-Kucing-Sedunia-2026-bingkai-foto.jpg</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Cegah Jemaah Jadi Korban, Kemenhaj Operasikan Posko Pengawasan Umrah di Bandara Soekarno-Hatta</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:28:18 +0700</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>Kemenhaj RI mulai mengoperasikan Posko Pengawasan Penyelenggara Perjalanan Ibadah Umrah (PPIU) di Terminal 2F Bandara Internasional Soekarno-Hatta</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865597/cegah-jemaah-jadi-korban-kemenhaj-operasikan-posko-pengawasan-umrah-di-bandara-soekarno-hatta</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/_alNEFAU6_Y0bNYjFRofps9N5mg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/WAKTU-UMRAH-Sejumlah-jemaah-haji-berjalan-keluar-dari-Masjidil-Haram-menuju-Terminal-Syib-Amir.jpg</t>
+        </is>
+      </c>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Pakar Hukum Sebut Pengembangan Kasus Febrie Penting Dilakukan untuk Memunculkan Aktor Utama</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:27:10 +0700</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>Perkara yang menjerat eks Jampidsus Febrie Adriansyah diduga tidak hanya melibatkan satu orang.</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865596/pakar-hukum-sebut-pengembangan-kasus-febrie-penting-dilakukan-untuk-memunculkan-aktor-utama</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/eQh7NUBPd1a5LZJ7hmRGe9FD4wA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Febrie-Adriansyah-Jalani-Pemeriksaan-Lanjutan-Kasus-TPPU_20260807_134205.jpg</t>
+        </is>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Bangun Chemistry di Jakarta Undercover, Caitlin Halderman dan Baskara Mahendra Sering Jalan Bareng</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:21:35 +0700</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>Aktris Caitlin Halderman mengungkap pengalamannya saat beradu akting dengan Baskara Mahendra dalam serial Jakarta Undercover.</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7865595/bangun-chemistry-di-jakarta-undercover-caitlin-halderman-dan-baskara-mahendra-sering-jalan-bareng</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/gmHFUAOoXDrQtVo1agI808C0ppQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Caitlin-Haldeman-1-08082026.jpg</t>
+        </is>
+      </c>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Pelaku Penembakan Massal di Sekolah Thailand Dikenal Pendiam, Korban Tewas Naik Menjadi 9 Orang</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:19:22 +0700</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>Remaja 14 tahun tersangka penembakan sekolah Thailand disebut pendiam dan gemar bermain gim. Korban tewas naik menjadi 9 orang.</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7865594/pelaku-penembakan-massal-di-sekolah-thailand-dikenal-pendiam-korban-tewas-naik-menjadi-9-orang</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/WuDt6Wu4OotVgflffCRKclRVW1o=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/P1ENEMBAKAN-DI-T1HAILAND-Tangkap-layar-YouTube-The-Star-7-A.jpg</t>
+        </is>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Penampakan Lokasi yang Ditemukan 995 Airsoft Gun di Sekolah</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:15:00 +0700</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>Petugas menunjukkan ruangan yang telah dipasang garis polisi di sebuah sekolah swasta di kawasan Pondok Pinang, Jakarta Selatan.</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260807193635-7-757534/penampakan-lokasi-yang-ditemukan-995-airsoft-gun-di-sekolah</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/07/petugas-menunjukkan-ruangan-yang-telah-dipasang-garis-polisi-di-sebuah-sekolah-swasta-di-kawasan-pondok-pinang-jakarta-selatan-1786106178189_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Gedung Bapenda DKI Jakarta Terbakar Hebat Semalam, Apa Penyebabnya?</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 07:45:00 +0700</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>Puslabfor Bareskrim Polri diterjunkan untuk menginvestigasi penyebab kebakaran gedung Bapenda DKI Jakarta di Gambir</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260808061834-4-757566/gedung-bapenda-dki-jakarta-terbakar-hebat-semalam-apa-penyebabnya</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2024/01/20/ilustrasi-kebakaran_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Siswa 14 Tahun Tembak Mati 8 Orang, Alasannya Tak Terduga</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 07:30:00 +0700</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>Tim Redaksi</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>Pelaku siswa berusia 14 tahun menembak mati 8 orang di sekolah termasuk kakek dan neneknya</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260807213605-4-757565/siswa-14-tahun-tembak-mati-8-orang-alasannya-tak-terduga</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/07/para-siswa-berlari-saat-mengevakuasi-diri-dari-sekolah-debsirin-nonthaburilokasi-terjadinya-insiden-penembakandi-distrik-bang--1786084015262_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Jakarta Punya Tol Layang Baru di 2028, Anti Macet ke Bandara Soetta</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 07:15:00 +0700</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>Progres pembangunan Jalan Tol Layang baru ini mencapai 44,12% dan ditargetkan dapat beroperasi pada 2028. Ke Bandara Soetta anti macet.</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260807155818-7-757476/jakarta-punya-tol-layang-baru-di-2028-anti-macet-ke-bandara-soetta</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/07/suasana-pengerjaan-area-proyek-pembangunan-jalan-tol-harbour-road-ii-hbr-ii-di-kawasan-tanjung-priok-jakarta-jumat-782026-1786092785719_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Ada "Aliansi" Pertahanan Baru, Kekuatan Nuklir Asia Gabung Saudi-Turki</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 07:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>pgr</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>Arab Saudi, Turki dan Pakistan membentuk aliansi pertahanan baru</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260807212249-4-757556/ada-aliansi-pertahanan-baru-kekuatan-nuklir-asia-gabung-saudi-turki</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2023/07/18/saudi-arabia-turkey-erdogan-gulf-trip_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Siaga Perang, Negara Ini Latihan Tempur-Siapkan Militer Besar-besaran</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 06:45:00 +0700</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>Reuters</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>Taiwan mulai melaksanakan latihan militer tahunan terbesar bertajuk Han Kuang, Jumat (7/8/2026). L</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260807162621-7-757500/siaga-perang-negara-ini-latihan-tempur-siapkan-militer-besar-besaran</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/07/taiwan-mulai-melaksanakan-latihan-militer-tahunan-terbesar-bertajuk-han-kuang-jumat-782026-latihan-ini-bagian-dari-upaya-menin-1786095276407_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Bocah 14 Tahun Bawa Senjata Tembak Mati 8 Orang, Polisi Buka Suara</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 06:30:00 +0700</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>Terjadi penembakan brutal di sebuah sekolah di Thailand</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260807205641-4-757546/bocah-14-tahun-bawa-senjata-tembak-mati-8-orang-polisi-buka-suara</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/07/petugas-darurat-berkumpul-di-dalam-area-sekolah-debsirin-nonthaburi-menyusul-insiden-penembakan-di-sekolah-tersebut-di-distrik-1786084015598_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Tiba-Tiba Muncul Mobil Tahun 1885 di BSD, Begini Bentuknya</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 05:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz Indonesia hadirkan Benz Patent-Motorwagen, mobil pertama dunia yang menandai lahirnya industri otomotif modern.</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260807174139-4-757525/tiba-tiba-muncul-mobil-tahun-1885-di-bsd-begini-bentuknya</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/07/benz-patent-motorwagen-di-giias-2026-1786099514814_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Saldo Minimal Nasabah Prioritas Bank BRI-Mandiri-BNI per Agustus 2026</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:30:00 +0700</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>Saldo minimum Bank BRI-Mandiri dan BNI</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260808074643-17-757573/saldo-minimal-nasabah-prioritas-bank-bri-mandiri-bni-per-agustus-2026</t>
+        </is>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2021/05/24/intip-biaya-transaksi-di-atm-bni-1_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>Bisnis</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Transformasi BUMN, Telkom Pangkas 34 Entitas Usaha</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:36:20 +0700</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>Ahmad Fikri Noor</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- PT Telkom Indonesia memangkas 34 entitas dari 67 entitas usaha dalam proses transformasi BUMN untuk membangun organisasi yang lebih ramping, efisien, dan kompetitif.
+“Transformasi bukan soal mengubah struktur...</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjfj8k490/transformasi-bumn-telkom-pangkas-34-entitas-usaha</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/pt-telkom-indonesia-persero-tbk-telkom-menuntaskan-target-penyederhanaan_260706135419-792.jpeg</t>
+        </is>
+      </c>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>Energi</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>Pasokan Konsentrat dari Papua Kembali Masuk, Smelter Freeport Bersiap Produksi</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:29:36 +0700</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>Ahmad Fikri Noor</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- Presiden Direktur PT Freeport Indonesia Tony Wenas menyampaikan smelter katoda tembaga di kawasan industri Java Integrated Industrial and Port Estate (JIIPE), Manyar, Gresik, Jawa Timur, mulai kembali...</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjfixc490/pasokan-konsentrat-dari-papua-kembali-masuk-smelter-freeport-bersiap-produksi</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/pt-freeport-indonesia_260508190826-855.jpeg</t>
+        </is>
+      </c>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>Finansial</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>Pajak Marketplace Ditunda, Ekonom Soroti Dampaknya bagi UMKM</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:29:06 +0700</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>Ahmad Fikri Noor</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- Ekonom Center of Reform on Economics (CORE) Yusuf Rendy Manilet menilai penundaan pungutan Pajak Penghasilan (PPh) Pasal 22 atas transaksi di platform lokapasar (marketplace) memberikan ruang bagi...</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjfg4i490/pajak-marketplace-ditunda-ekonom-soroti-dampaknya-bagi-umkm</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/041080100-1739871490-830-556.jpg</t>
+        </is>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>10 Pengelola Akun Medsos Ditahan, 4 Modus Terungkap</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:46:59 +0700</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>Polisi mengungkap empat modus penyebaran konten provokatif dan hoaks.</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8264870/10-pengelola-akun-medsos-ditahan-4-modus-terungkap</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/mrLB6lWmQxjIO2nzD-595vAzeKI=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9308726/original/081906100_1785171837-IMG_0856.jpg</t>
+        </is>
+      </c>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Kebakaran Gedung Bapenda DKI, Titik Api Diduga dari Lantai 11</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:27:57 +0700</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>Petugas masih menyisir titik panas untuk mencegah api kembali menyala.</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8264855/kebakaran-gedung-bapenda-dki-titik-api-diduga-dari-lantai-11</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/42B01YC5FDkIDRmw2a58lHmRIzk=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9318747/original/067967000_1786155435-IMG_20260808_082643_127.jpg</t>
+        </is>
+      </c>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Alasan Prabowo Ingin Buku Pelajaran Diperbarui</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:26:30 +0700</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>Pemerintah terus mematangkan langkah pembaruan buku ajar nasional</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8264841/alasan-prabowo-ingin-buku-pelajaran-diperbarui</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/FoiefrwGe4QDCRwl2XNxoHsJAeY=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/5386433/original/064295900_1761008005-8.jpg</t>
+        </is>
+      </c>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Bangun Kemandirian Energi Desa, Pertamina Perkuat Kapasitas "Local Hero"</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:57:32 +0700</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>Melalui program DEB yang telah menjangkau 262 desa, Pertamina membina para local hero melalui edukasi, pelatihan, serta sertifikasi.</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/08/08/09561911/bangun-kemandirian-energi-desa-pertamina-perkuat-kapasitas-local-hero</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/WqUdKG_c-7l7WWu8FcpDGXRZ5hc=/0x0:1279x853/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/08/6a76963a4c74d.jpeg</t>
+        </is>
+      </c>
+      <c r="I226" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Boss Kidswear Hadir di Pacific Place, Usung Konsep Mini-Me</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:57:32 +0700</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>Bimbi Group hadirkan Boss Kidswear di Pacific Place, menjadikan pakaian anak sebagai medium bangun rasa percaya diri sejak dini.</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>https://lifestyle.kompas.com/read/2026/08/08/092200620/boss-kidswear-hadir-di-pacific-place-usung-konsep-mini-me</t>
+        </is>
+      </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/7sLKzZDhN9hylE1ECY-Dd4c3luk=/0x57:1280x910/1200x675/filters:watermark(data/photo/2026/01/30/697c817ed68bb.png,0,-0,1)/data/photo/2026/08/07/6a76032c9a9ce.jpeg</t>
+        </is>
+      </c>
+      <c r="I227" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>Money</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>BPS Pastikan Data Sensus Ekonomi 2026 Tak Dipakai untuk Tarik Pajak</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:57:32 +0700</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>BPS RI memastikan Sensus Ekonomi 2026 tidak akan digunakan untuk penarikan pajak. Data responden dilindungi UU, murni untuk statistik dan arah kebijakan ekonomi.</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>https://money.kompas.com/read/2026/08/08/090000726/bps-pastikan-data-sensus-ekonomi-2026-tak-dipakai-untuk-tarik-pajak</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/UdgmFkRjxw6kS-6QKaZykZNAl6I=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815e7ef28.png,0,-0,1)/data/photo/2026/08/07/6a7600005297a.jpg</t>
+        </is>
+      </c>
+      <c r="I228" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I124"/>
+  <autoFilter ref="A1:I228"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-08 04:08 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-08.xlsx
+++ b/data/berita_2026-08-08.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$228</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$293</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I228"/>
+  <dimension ref="A1:I293"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -11150,8 +11150,3063 @@
         </is>
       </c>
     </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Polisi bantah lamban tangani kasus temuan senjata di sekolah Jaksel</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:53:29 +0700</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>Polres Metro Jakarta Selatan membantah lamban dalam menangani kasus temuan senjata di sebuah sekolah swasta di wilayah ...</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685431/polisi-bantah-lamban-tangani-kasus-temuan-senjata-di-sekolah-jaksel</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001017729.jpg</t>
+        </is>
+      </c>
+      <c r="I229" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>PBB: Bantuan yang diizinkan masuk Gaza naik 33 persen pada Juli 2026</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:48:18 +0700</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>Jumlah pasokan penting yang diizinkan masuk ke Jalur Gaza meningkat 33 persen pada Juli tahun ini dibandingkan bulan ...</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685429/pbb-bantuan-yang-diizinkan-masuk-gaza-naik-33-persen-pada-juli-2026</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/CjkinzN000005_20260808_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>DKI pastikan data pajak dan aset daerah aman dari kebakaran Bapenda</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:46:49 +0700</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>Pemerintah Provinsi (Pemprov) DKI Jakarta memastikan data perpajakan dan aset daerah aman dari kebakaran di gedung ...</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685427/dki-pastikan-data-pajak-dan-aset-daerah-aman-dari-kebakaran-bapenda</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001017627.jpg</t>
+        </is>
+      </c>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Abelardo De La Espriella resmi dilantik sebagai Presiden baru Kolombia</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:45:01 +0700</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>Abelardo de la Espriella dilantik sebagai presiden baru Kolombia pada Jumat (7/8) waktu setempat di Kota Cali, Kolombia ...</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685425/abelardo-de-la-espriella-resmi-dilantik-sebagai-presiden-baru-kolombia</t>
+        </is>
+      </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/CjkinzN000007_20260808_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Korban kebakaran gedung Bapenda DKI dirawat di RSUD Tarakan</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:43:10 +0700</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>Suku Dinas Penanggulangan Kebakaran dan Penyelamatan (Gulkarmat) Jakarta Pusat menyebutkan korban yang berhasil ...</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685423/korban-kebakaran-gedung-bapenda-dki-dirawat-di-rsud-tarakan</t>
+        </is>
+      </c>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001017493.jpg</t>
+        </is>
+      </c>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Spanyol terapkan pemeriksaan perbatasan sementara ke pendatang Italia</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:42:08 +0700</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>Spanyol pada Jumat (7/8) mengumumkan untuk sementara waktu akan memberlakukan kembali pemeriksaan perbatasan dalam ...</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685419/spanyol-terapkan-pemeriksaan-perbatasan-sementara-ke-pendatang-italia</t>
+        </is>
+      </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/CjkinzN000008_20260808_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Mendag ajak BRICS perkuat kolaborasi hadapi ketidakpastian global</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:41:36 +0700</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>Menteri Perdagangan (Mendag) RI Budi Santoso mengajak negara-negara anggota BRICS untuk memperkuat kolaborasi dalam ...</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685415/mendag-ajak-brics-perkuat-kolaborasi-hadapi-ketidakpastian-global</t>
+        </is>
+      </c>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG_3700.jpeg</t>
+        </is>
+      </c>
+      <c r="I235" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Tim gabungan padamkan kebakaran lahan di kawasan Sembalun Rinjani</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:38:27 +0700</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>Tim gabungan Balai Taman Nasional Gunung Rinjani (TNGR) Provinsi Nusa Tenggara Barat (NTB) bergerak cepat melakukan ...</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685412/tim-gabungan-padamkan-kebakaran-lahan-di-kawasan-sembalun-rinjani</t>
+        </is>
+      </c>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1005746996.jpg</t>
+        </is>
+      </c>
+      <c r="I236" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Waketum MUI sebut pemimpin harus adaptif hadapi transformasi digital</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:27:01 +0700</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>Wakil Ketua Umum Majelis Ulama Indonesia (MUI) KH Marsudi Syuhud mengatakan pemimpin harus mampu beradaptasi dengan ...</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685409/waketum-mui-sebut-pemimpin-harus-adaptif-hadapi-transformasi-digital</t>
+        </is>
+      </c>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001224989.jpg</t>
+        </is>
+      </c>
+      <c r="I237" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Gulkarmat: Kebakaran gedung Bapenda DKI berasal dari lantai 11</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:19:23 +0700</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>Suku Dinas Penanggulangan Kebakaran dan Penyelamatan Jakarta Pusat (Gulkarmat Jakpus) menyatakan kebakaran gedung Badan ...</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685407/gulkarmat-kebakaran-gedung-bapenda-dki-berasal-dari-lantai-11</t>
+        </is>
+      </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001017532.jpg</t>
+        </is>
+      </c>
+      <c r="I238" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Dasco sebut komitmen bantuan untuk korban TPKS capai Rp200 miliar</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:18:58 +0700</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>Wakil Ketua DPR RI Sufmi Dasco Ahmad mengatakan komitmen bantuan untuk mendukung Dana Bantuan Korban (DBK) bagi ...</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685404/dasco-sebut-komitmen-bantuan-untuk-korban-tpks-capai-rp200-miliar</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001224189.jpg</t>
+        </is>
+      </c>
+      <c r="I239" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Harga emas Antam pada Sabtu meroket Rp40.000 jadi Rp2,690 juta/gr</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:09:08 +0700</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>Harga emas Antam yang dipantau dari laman Logam Mulia di Jakarta, Sabtu pukul 10.05 WIB melonjak Rp40.000 menjadi ...</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685401/harga-emas-antam-pada-sabtu-meroket-rp40000-jadi-rp2690-juta-gr</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/02/03/harga-emas-antam-naik-2717610.jpg</t>
+        </is>
+      </c>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Mendag dorong perdagangan berbasis aturan untuk UMKM di BRICS</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:05:17 +0700</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>Menteri Perdagangan Budi Santoso dalam Pertemuan Para Menteri Perdagangan BRICS (BRICS Trade Ministers' Meeting) di ...</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685399/mendag-dorong-perdagangan-berbasis-aturan-untuk-umkm-di-brics</t>
+        </is>
+      </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG_3698.jpeg</t>
+        </is>
+      </c>
+      <c r="I241" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>BGN tegaskan SLHS jadi syarat mutlak operasional SPPG</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:01:54 +0700</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>Kepala Badan Gizi Nasional (BGN) Sudaryono menegaskan Sertifikat Laik Higiene dan Sanitasi (SLHS) menjadi syarat mutlak ...</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685395/bgn-tegaskan-slhs-jadi-syarat-mutlak-operasional-sppg</t>
+        </is>
+      </c>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG-20260808-WA0006_edit_2211329196295903.jpg</t>
+        </is>
+      </c>
+      <c r="I242" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Lebih segar dan elegan! Wajah baru Geely EX2 tampil di GIIAS 2026</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/antaranewsdotcom</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>ANTARA - SUV Geely yang sempat rilis pada awal tahun 2026,Geely EX2, kembali hadir dengan wajah baru di GIIAS ...</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/video/5683967/lebih-segar-dan-elegan-wajah-baru-geely-ex2-tampil-di-giias-2026</t>
+        </is>
+      </c>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/LEBIH-SEGAR-DAN-ELEGAN-WAJAH-BARU-GEELY-EX2-TAMPIL-DI-GIIAS-2026_1.jpg</t>
+        </is>
+      </c>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Teknologi gamifikasi jadi media promosi produk kreatif dan wisataRI</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:52:34 +0700</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>Wakil Menteri Ekraf Irene Umar menilai pengembangan teknologi gamifikasi berpotensi menjadi media promosi yang mampu ...</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685392/teknologi-gamifikasi-jadi-media-promosi-produk-kreatif-dan-wisatari</t>
+        </is>
+      </c>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000455660.jpg</t>
+        </is>
+      </c>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Korban Kebakaran Gedung Bapenda DKI Masih Dirawat, Alami Sesak Nafas</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:59:47 +0700</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>Polda Metro Jaya mengungkapkan kondisi terkini korban kebakaran gedung Badan Pendapatan Daerah (Bapenda) DKI Jakarta.</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609611/korban-kebakaran-gedung-bapenda-dki-masih-dirawat-alami-sesak-nafas</t>
+        </is>
+      </c>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/potret-kobaran-api-mengamuk-di-gedung-bapenda-dki-1786160999327_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Kapolri Bicara Filosofi Pendekar: Bela Kebenaran, Lindungi yang Lemah</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:38:44 +0700</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>Lisye Sri Rahayu</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>Kapolri Jenderal Sigit menghadiri Muktamar XVI Tapak Suci Putera Muhammadiyah di Semarang, menekankan filosofi pendekar.</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609569/kapolri-bicara-filosofi-pendekar-bela-kebenaran-lindungi-yang-lemah</t>
+        </is>
+      </c>
+      <c r="H246" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/kapolri-jenderal-listyo-sigit-prabowo-1786157459837_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Mobil Putih Tabrak Lari Motor di Jakbar Berujung Diamuk Massa</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:29:12 +0700</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>Mei Amelia R</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>Sebuah mobil Honda Odyssey dirusak massa di Cengkareng setelah diduga melarikan diri usai menabrak pengendara motor. Kejadian viral ini menimbulkan kemacetan.</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609562/mobil-putih-tabrak-lari-motor-di-jakbar-berujung-diamuk-massa</t>
+        </is>
+      </c>
+      <c r="H247" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2023/05/15/ilustrasi-kecelakaan_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I247" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Hutama Karya Borong 3 Gold Bintang 4 di TJSL &amp;amp; CSR Award BUMN Track 2026</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:06:43 +0700</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>Inkana Putri</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>Hutama Karya meraih tiga penghargaan Gold #Star 4 dalam TJSL &amp; CSR BUMN Track Award 2026, berkat program yang berdampak sosial, ekonomi, dan lingkungan.</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609543/hutama-karya-borong-3-gold-bintang-4-di-tjsl-csr-award-bumn-track-2026</t>
+        </is>
+      </c>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/hutama-karya-borong-3-gold-bintang-4-di-tjsl-csr-award-bumn-track-2026-1786158354982.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I248" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Kapolri Dianugerahkan Jadi Anggota Kehormatan Tapak Suci Putera Muhammadiyah</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:54:36 +0700</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>Lisye Sri Rahayu</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>Kapolri Jenderal Sigit dianugerahi anggota kehormatan Tapak Suci Muhammadiyah. Dia berharap hubungan Polri dan Muhammadiyah semakin erat ke depannya.</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609538/kapolri-dianugerahkan-jadi-anggota-kehormatan-tapak-suci-putera-muhammadiyah</t>
+        </is>
+      </c>
+      <c r="H249" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/kapolri-jenderal-listyo-sigit-prabowo-1786157459631_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Said Abdullah: Soekarno Cup Jadi Ajang Bangun Pesepakbola Berkarakter</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:54:19 +0700</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>Inkana Putri</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>Soekarno Cup 2026 di Jawa Timur, 10-24 Agustus, diikuti 16 tim. Pembukaan dengan penyalaan obor, dihadiri DPP PDI Perjuangan dan legenda Timnas.</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609536/said-abdullah-soekarno-cup-jadi-ajang-bangun-pesepakbola-berkarakter</t>
+        </is>
+      </c>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/ketua-dpd-pdi-perjuangan-jawa-timur-said-abdullah-1786157476659_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>UGM Nonaktifkan Mahasiswi PPDS Buntut Komentar 'Orang Have' ke Pasien BPJS</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:46:49 +0700</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>Adji G Rinepta</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>UGM menonaktifkan Elda Putri Rahardini, mahasiswi PPDS. Penonaktifan dilakukan buntut komentar Elda di media sosial yang menyindir pasien BPJS.</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609530/ugm-nonaktifkan-mahasiswi-ppds-buntut-komentar-orang-have-ke-pasien-bpjs</t>
+        </is>
+      </c>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/01/15/ilustrasi-kamar-rumah-sakit_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I251" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Janji Manis Juncurryahn untuk Dita Karang</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:05:32 +0700</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>Desi Puspasari</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>Dita Karang dan YouTuber Juncurryahn atau Ahn Jun Sung mengunggah momen kebersamaan. Juncurryahn janji selalu mendampingi idol asal Indonesia itu.</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8609500/janji-manis-juncurryahn-untuk-dita-karang</t>
+        </is>
+      </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/dita-karang-1786154032316_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I252" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Kebakaran Bromo Diduga Berawal dari Perapian Pelintas Jalur</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:45:10 +0700</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>Kepala Balai Besar Taman Nasional Bromo Tengger Semeru duga penyebab kebakaran Bromo adalah ulah manusia.</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808103157-20-1390041/kebakaran-bromo-diduga-berawal-dari-perapian-pelintas-jalur</t>
+        </is>
+      </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/06/kebakaran-hutan-kawasan-gunung-bromo-1786018084811_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I253" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Detik-detik Kebakaran Hebat Lahap Gedung Bapenda DKI</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:21:06 +0700</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>Gedung Badan Pendapatan Daerah (Bapenda) DKI Jakarta mengalami kebakaran pada Jumat (7/8) malam.</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808100641-24-1390038/detik-detik-kebakaran-hebat-lahap-gedung-bapenda-dki</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/thumbnail-video-1786158515742_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>Kemenkes Ungkap Almarhum Yurizal Pasien BPJS Tunggu 8 Jam di IGD RSCM</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:15:50 +0700</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>Almarhum Yurizal sebelumnya curhat via threads soal menunggu dapat ruang hingga 8 jam, dan tak menyebut nama RS-nya. Dia kemudian dicibir banyak nakes.</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260807194229-20-1389926/kemenkes-ungkap-almarhum-yurizal-pasien-bpjs-tunggu-8-jam-di-igd-rscm</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2021/06/28/ilustrasi-pasien-dan-dokter_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Kapolda Metro Jaya Tegaskan TNI-Polri Sinergi Jaga Jakarta</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:08:05 +0700</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>Kapolda Metro Jaya Komjen Pol Asep Edi Suheri menyatakan TNI-Polri bersinergi dalam menjaga stabilitas dan keamanan Jakarta.</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808100344-20-1390037/kapolda-metro-jaya-tegaskan-tni-polri-sinergi-jaga-jakarta</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/apel-kebangsaan-jaga-jakarta-untuk-indonesia-1786161022487_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I256" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Said Abdullah: Soekarno Cup Ajang Membangun Pesepak Bola Berkarakter</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:03:47 +0700</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>Ketua DPD PDI Perjuangan Jawa Timur, Said Abdullah mengatakan, Soekarno Cup menandai keterlibatan PDI Perjuangan dalam membangun karakter bangsa.</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808100105-633-1390035/said-abdullah-soekarno-cup-ajang-membangun-pesepak-bola-berkarakter</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2025/08/21/said-abdullah-1755762616082_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I257" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Tanda-tanda Trump Mulai Kelimpungan Hadapi Iran</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:35:33 +0700</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>Presiden Amerika Serikat (AS) Donald Trump mulai menunjukkan tanda-tanda kelimpungan menghadapi Iran. Terlihat dari mana saja?</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260808085206-134-1390024/tanda-tanda-trump-mulai-kelimpungan-hadapi-iran</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/07/23/trump-kesulitan-lindungi-50-ribu-tentara-as-dari-serangan-iran-1784792922025_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Pengadilan Minta Proyek Ruang Dansa Gedung Putih Disetop, Trump Ngamuk</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:45:22 +0700</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>Pengadilan banding federal AS meminta pemerintahan Presiden Donald Trump menghentikan proyek pembangunan ballroom atau ruang dansa di Gedung Putih.</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260808083333-134-1390021/pengadilan-minta-proyek-ruang-dansa-gedung-putih-disetop-trump-ngamuk</t>
+        </is>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2025/10/01/us-government-shutdown-looms-as-house-and-senate-disagree-on-fun-1759301756561_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I259" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Presiden Iran Pezeshkian Diisukan Pernah Ajukan Resign Sampai 28 Kali</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:05:29 +0700</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>Presiden Iran Masoud Pezeshkian diisukan pernah mengajukan pengunduran diri sebanyak 28 kali kepada pemimpin Tertinggi Mojtaba Khamenei.</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260807180332-120-1389858/presiden-iran-pezeshkian-diisukan-pernah-ajukan-resign-sampai-28-kali</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/04/23/iran-politics-anniversary-1776923694179_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I260" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Fokus Lacak Aset Korupsi CSR BI-OJK, KPK Usut Kekayaan Anggota DPR Heri Gunawan dan Satori</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:53:55 +0700</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>Komisi Pemberantasan Korupsi terus menelusuri dan menyita aset milik dua anggota DPR RI, Heri Gunawan dan Satori.</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865639/fokus-lacak-aset-korupsi-csr-bi-ojk-kpk-usut-kekayaan-anggota-dpr-heri-gunawan-dan-satori</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/RkRQbB5ElLJeY6Ae04HB_PZDcXU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Heri-Gunawan-dan-Satori.jpg</t>
+        </is>
+      </c>
+      <c r="I261" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Kapolri Terima Gelar Anggota Kehormatan dari Tapak Suci: Jadikan Polri Keluarga Besar Muhammadiyah</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:51:10 +0700</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>Afnan Hadikusumo, menganugerahkan gelar Anggota Kehormatan kepada Kapolri Jenderal Listyo Sigit Prabowo.</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865638/kapolri-terima-gelar-anggota-kehormatan-dari-tapak-suci-jadikan-polri-keluarga-besar-muhammadiyah</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/xGw6xcKMF9zapi_NpxuewxXGxuM=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Kapolri-dapat-gelar-penghormatan.jpg</t>
+        </is>
+      </c>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Pentingnya Penguatan Ekosistem AI, Mahasiswa UNSIA Dibekali Kompetensi Masa Depan</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:49:09 +0700</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>UNSIA mempercepat transformasi menjadi AI Innovator University dengan memperkuat kompetensi AI bagi dosen dan mahasiswa.</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865637/pentingnya-penguatan-ekosistem-ai-mahasiswa-unsia-dibekali-kompetensi-masa-depan</t>
+        </is>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/0RszBwPlvAunutfkO_gS65KlBlE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/wa-pengembangan-kolaborasi-d-aran-AIHO-IST.jpg</t>
+        </is>
+      </c>
+      <c r="I263" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>Uban di Usia Muda, Normal atau Harus Diwaspadai? Ini Penjelasan Dokter</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:48:48 +0700</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>Uban di usia muda apakah normal atau justru harus di waspadai? menurut dokter estetika hal ini tergantung genetik dan jumlahnya, simak penjelasannya.</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7865636/uban-di-usia-muda-normal-atau-harus-diwaspadai-ini-penjelasan-dokter</t>
+        </is>
+      </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/JAmNymtILDvuIbFl2WWOG51-A9k=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/tren-terbaru-rambut-untuk-awal-tahun_20230213_200809.jpg</t>
+        </is>
+      </c>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Soal Peran Houthi di Timur Tengah, Pakar: Iran Terapkan Prinsip Plausible Deniability</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:46:45 +0700</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>Iran memanfaatkan hubungan dengan Houthi melalui prinsip plausible deniability, sehingga dapat mendukung tanpa terlihat terlibat langsung.</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7865635/soal-peran-houthi-di-timur-tengah-pakar-iran-terapkan-prinsip-plausible-deniability</t>
+        </is>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/N0SBKbaoBUBCyC1c32pCneWApqc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/anggota-kelompok-H1outhi-dalam-sebuah-a.jpg</t>
+        </is>
+      </c>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Update Top Skor Piala AFF 2026: Nguyen Dinh Bac Harumkan Vietnam, Mitchell Baker Tenggelam</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:43:55 +0700</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>Penyerang Vietnam, Nguyen Dinh Bac, kini berada di posisi teratas persaingan top skor setelah tampil tajam saat membantu timnya mengalahkan Kamboja.</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865634/update-top-skor-piala-aff-2026-nguyen-dinh-bac-harumkan-vietnam-mitchell-baker-tenggelam</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/UlEQdtd4869uQ1s7ZFox2LqSuYw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Vietnam-U23-Nguyen-Dinh-Bac.jpg</t>
+        </is>
+      </c>
+      <c r="I266" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Di Balik Tingginya Peminat SNBT 2026, Mengenal Prodi K3 UNS dan Peluang Kariernya</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:43:48 +0700</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>Prodi K3 UNS menjadi yang paling diminati di SNBT 2026. Kenali keunggulan pendidikan, fasilitas, dan peluang karier lulusannya.</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/pendidikan-go/7865633/di-balik-tingginya-peminat-snbt-2026-mengenal-prodi-k3-uns-dan-peluang-kariernya</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/o5Oz9MV2ZqMCkMDcPKensnnRs3c=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Prodi-K3-UNS.jpg</t>
+        </is>
+      </c>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Dukung Tumbuh Kembang Anak, BRI Peduli Bangun Posyandu Matahari di Sleman</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:42:58 +0700</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>BRI Peduli meresmikan Posyandu Matahari di Sleman melalui Program Desa Brilian 1000 HPK untuk mendukung kesehatan ibu dan anak.</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865632/dukung-tumbuh-kembang-anak-bri-peduli-bangun-posyandu-matahari-di-sleman</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/MPFq30XNSskMJiDCnzE1ysdEzl8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/BRI-Peduli-di-Sleman.jpg</t>
+        </is>
+      </c>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Setengah Gedung Bapenda Jakarta Hangus, Puslabfor Polri Selidiki Penyebab Kebakaran</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:42:32 +0700</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>Puslabfor Polri telah diterjunkan ke lokasi untuk melakukan pemeriksaan penyebab kebakaran Gedung Bapenda DKI Jakarta, Jumat (7/8/2026) malam.</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7865631/setengah-gedung-bapenda-jakarta-hangus-puslabfor-polri-selidiki-penyebab-kebakaran</t>
+        </is>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/WEg6aNuIonboivDqai0AIN6RniU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Bapenda-1-08082026.jpg</t>
+        </is>
+      </c>
+      <c r="I269" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>Venue Kejuaraan Dunia BWF 2026 Direnovasi Hampir Rp 40 Miliar, Libatkan Ahli Lighting dari Indonesia</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:42:25 +0700</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>Venue Kejuaraan Dunia BWF 2026 di Stadion Indoor Indira Gandhi, New Delhi, direnovasi dengan biaya hampir Rp40 miliar.</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7865630/venue-kejuaraan-dunia-bwf-2026-direnovasi-hampir-rp-40-miliar-libatkan-ahli-lighting-dari-indonesia</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/CMrL-RLSDBdJOaUbM3-J8h7L_9k=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Turnamen-Dunia-dan-Hiburan-di-Polytron-Indonesia-Open-2026_20260606_215422.jpg</t>
+        </is>
+      </c>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Kunci Jawaban Matematika Kelas 5 SD Halaman 175, 176: Mengukur dan Membandingkan Sudut Kipas Lipat</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:40:37 +0700</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>Simak kunci jawaban Matematika Kelas 5 SD halaman 175, 176 Kurikulum Merdeka Bab 6 tentang Sudut.</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/pendidikan/7865629/kunci-jawaban-matematika-kelas-5-sd-halaman-175-176-mengukur-dan-membandingkan-sudut-kipas-lipat</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/1JPKJGa96_InI21Y0aEE8NCU4z4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/SISWA-SD-BELAJAR-20.jpg</t>
+        </is>
+      </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Sosok Cesar Gastelum, Influencer Meksiko yang Tewas usai Ditembak OTK saat Live TikTok</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:40:20 +0700</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>Cesar Gastelum, influencer TikTok asal Meksiko berusia 24 tahun, tewas ditembak orang tak dikenal saat live TikTok.</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7865628/sosok-cesar-gastelum-influencer-meksiko-yang-tewas-usai-ditembak-otk-saat-live-tiktok</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/POX2Oltj6cNUFfiZ7jYShalFYbw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Influencer-Meksiko-Tewas.jpg</t>
+        </is>
+      </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Kunci Jawaban Bahasa Indonesia Kelas 9 Halaman 60, 61 Edisi Revisi Latihan 2: Jenis Pantun</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:36:51 +0700</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>Simak kunci jawaban Bahasa Indonesia kelas 9 SMP, MTs halaman 63, 64 Kurikulum Merdeka Edisi Revisi, Latihan 3: Jenis Pantun dan Penjelasannya</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/pendidikan/7865627/kunci-jawaban-bahasa-indonesia-kelas-9-halaman-60-61-edisi-revisi-latihan-2-jenis-pantun</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/fWfi9fXNkXNJ3yuHfDIa7EUPkOk=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/SISWA-SMP-BELAJAR-09.jpg</t>
+        </is>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>6 Informasi Terbaru Kebakaran Gedung Bapenda DKI yang Dirangkum Pagi Ini</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:33:06 +0700</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>Kebakaran melanda Gedung Bapenda DKI Jakarta di Jalan Abdul Muis, Gambir, Jumat (7/8/2026) malam.</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7865626/6-informasi-terbaru-kebakaran-gedung-bapenda-dki-yang-dirangkum-pagi-ini</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/rpCNy4Sg99M2QQ5G5Q_JAqVYzvw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/akarta-Pusat-dari-umat-782026-malam.jpg</t>
+        </is>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>Febrie Adriansyah Dicopot sebagai Jaksa, Eks Wakil Ketua KPK: Risiko Conflict of Interest Berkurang</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:30:56 +0700</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>Kata eks Wakil Ketua KPK Saut Situmorang, pencopotan sementara Febrie Adriansyah dari status jaksa hanya 'mengurangi' konflik kepentingan.</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865625/febrie-adriansyah-dicopot-sebagai-jaksa-eks-wakil-ketua-kpk-risiko-conflict-of-interest-berkurang</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/SZuHJrPGwtLaF-DkBoZ6ACX9xgA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Febrie-Adriansyah-Jalani-Pemeriksaan-Lanjutan-Kasus-TPPU_20260807_134300.jpg</t>
+        </is>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>Tembus 2.000 Kilometer, Drone Ukraina Hantam Gudang Wildberries Rusia hingga Terbakar</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:26:24 +0700</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>Drone Ukraina menembus lebih dari 2.000 km ke wilayah Rusia dan menghantam gudang Wildberries di Ekaterinburg hingga terbakar.</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7865624/tembus-2000-kilometer-drone-ukraina-hantam-gudang-wildberries-rusia-hingga-terbakar</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/pK9VwhktUvQjmrlgnL8OyXyNp9Y=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/gudang-Wildberries.jpg</t>
+        </is>
+      </c>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Kunci Jawaban Bahasa Indonesia Kelas 9 Halaman 60, 61 Edisi Revisi Latihan 2: Informasi dalam Pantun</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:20:41 +0700</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>Kunci jawaban Bahasa Indonesia kelas 9 halaman 60, 61 Kurikulum Merdeka Edisi Revisi, Latihan 2: Analisislah informasi yang terdapat dalam pantun.</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/pendidikan/7865623/kunci-jawaban-bahasa-indonesia-kelas-9-halaman-60-61-edisi-revisi-latihan-2-informasi-dalam-pantun</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/I26CNXmBVbp-YSqMKF_baAJSXHw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/SISWA-SMP-BELAJAR-11.jpg</t>
+        </is>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>Kapolda Metro-Pangdam Jaya Pimpin Apel Kebangsaan di Monas, Ajak Elemen Masyarakat Jaga Jakarta</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:19:05 +0700</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>Kapolda Metro Jaya bersama Pangdam Jaya/Jayakarta memimpin Apel Kebangsaan Jaga Jakarta untuk Indonesia di Monas, Jakarta Pusat, Sabtu (8/8/2026).</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7865622/kapolda-metro-pangdam-jaya-pimpin-apel-kebangsaan-di-monas-ajak-elemen-masyarakat-jaga-jakarta</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/X_dROEuYYkiN250ka00jWc-ZTPM=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/apel-kebangsaan-monas-sabtu-pagi.jpg</t>
+        </is>
+      </c>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>Pakar TPPU Beberkan Pola Dugaan Pencucian Uang dalam Perkara Eks Jampidsus Febrie</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:13:39 +0700</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>Yenti menjelaskan dalam perkara TPPU, penyidik terlebih dahulu harus membuktikan adanya tindak pidana asal.</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865621/pakar-tppu-beberkan-pola-dugaan-pencucian-uang-dalam-perkara-eks-jampidsus-febrie</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/3g8IxaDmEU6orh1QGuQQxWerECg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/rkara-Eks-Jampidsus-f.jpg</t>
+        </is>
+      </c>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Pedoman Sehat 10 Ribu Langkah Sehari Lahir dari Slogan Iklan, Bukan Riset Medis</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:10:44 +0700</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>Formulasi 10.000 langkah bermula usai Olimpiade Tokyo 1964. Perusahaan Jepang luncurkan alat pedometer Manpo-kei, harfiah berarti 10 ribu langkah.</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7865620/pedoman-sehat-10-ribu-langkah-sehari-lahir-dari-slogan-iklan-bukan-riset-medis</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/6zbmRRgX2wkII2g3sS_bJ4o0pf8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Suasana-CFD-di-Jalan-Rasuna-Said-Jakarta.jpg</t>
+        </is>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>Video: Gak Cuma Buat Kapal Perang, PT PAL Siap Pasok Kapal Penumpag</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:00:55 +0700</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>Gak Cuma Buat Kapal Perang, PT PAL Siap Pasok Kapal Penumpang - Kapal Selam</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260803171600-8-756191/video-gak-cuma-buat-kapal-perang-pt-pal-siap-pasok-kapal-penumpag</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/04/gak-cuma-buat-kapal-perang-pt-pal-siap-pasok-kapal-penumpang-kapal-selam-1785809170142_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>AS Ancam Serang Iran, Negara Teluk Bisa Gelap Gulita</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>Negara teluk siap-siap gelap gulita</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260808091103-4-757586/as-ancam-serang-iran-negara-teluk-bisa-gelap-gulita</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/07/30/iran-crisisegypt-tanker-1785374383042_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Bapenda DKI Membara Tengah Malam, Petugas Berjibaku Lebih dari 4 Jam</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:45:00 +0700</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>Kebakaran Gedung Bapenda DKI di Gambir melanda lantai 11-16. Api berhasil dikendalikan setelah lebih dari empat jam, sementara penyebabnya masih diselidiki.</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260808083251-7-757578/bapenda-dki-membara-tengah-malam-petugas-berjibaku-lebih-dari-4-jam</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/08/kebakaran-melanda-gedung-badan-pendapatan-daerah-bapenda-dki-jakarta-di-gambir-jakarta-pusat-sejak-jumat-782026-malam-1786152656237_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>Lewat Posyandu Matahari, BRI Perkuat Layanan Kesehatan Ibu dan Anak</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:38:57 +0700</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>dpu</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>BRI Peduli luncurkan Posyandu Matahari di Desa Hargobinangun untuk tingkatkan kesehatan ibu dan anak. Program ini fokus edukasi dan pemberdayaan masyarakat.</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260808103159-4-757592/lewat-posyandu-matahari-bri-perkuat-layanan-kesehatan-ibu-anak</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/08/bri-peduli-1786160335796_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Potret Eks Jampidsus Febrie Usai Diperiksa Tim 9 Kejagung</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:30:00 +0700</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>Mantan Jampidsus Febrie Adriansyah diperiksa selama kurang lebih 7 jam oleh tim sembilan Kejaksaan Agung.</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260807211358-7-757549/potret-eks-jampidsus-febrie-usai-diperiksa-tim-9-kejagung</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/07/tersangka-kasus-dugaan-tindak-pidana-pencucian-uang-tppu-yang-merupakan-mantan-jampidsus-febrie-adriansyah-berjalan-menuju-mob-1786112000027_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Polisi Ungkap Identitas Pemilik Senjata Api di Sekolah Jaksel</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:15:00 +0700</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>Plisi mengungkap siapa pemilik senjata api di sekolah Jakarta Selatan</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260808075845-4-757575/polisi-ungkap-identitas-pemilik-senjata-api-di-sekolah-jaksel</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/07/petugas-menunjukkan-ruangan-yang-telah-dipasang-garis-polisi-di-sebuah-sekolah-swasta-di-kawasan-pondok-pinang-jakarta-selatan-1786106178113_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Video: DPR Bocorkan Jurus RI Genjot Ekspor Lewat Proyek Danantara</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:00:44 +0700</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>DPR Bocorkan Jurus RI Genjot Ekspor - Buka Lapangan Kerja Lewat Proyek Danantara</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260806152631-8-757164/video-dpr-bocorkan-jurus-ri-genjot-ekspor-lewat-proyek-danantara</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/06/dpr-bocorkan-jurus-ri-genjot-ekspor-buka-lapangan-kerja-lewat-proyek-danantara-1786005977764_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>Bisnis</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Bank Jakarta Siapkan Talenta Digital Hadapi Perubahan Industri Perbankan</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Satria K Yudha</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA – Perkembangan teknologi membuat kebutuhan perbankan terhadap sumber daya manusia dengan kompetensi digital semakin meningkat. Bank Jakarta memperkuat kapasitas talenta teknologi melalui Officer Development Program (ODP) Information Technology...</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjflme416/bank-jakarta-siapkan-talenta-digital-hadapi-perubahan-industri-perbankan</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/bank_260607094015-894.jpeg</t>
+        </is>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Petugas Ungkap Kendala Padamkan Kebakaran Gedung Bapenda DKI</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:05:19 +0700</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>Hampir lima jam, petugas berjibaku memadamkan kebakaran Gedung Bapenda DKI.</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8264908/petugas-ungkap-kendala-padamkan-kebakaran-gedung-bapenda-dki</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/ipD3F85iLpsa-vf0KfNygf0oJa8=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9318678/original/083581200_1786128701-WhatsApp_Image_2026-08-08_at_01.35.55__1_.jpeg</t>
+        </is>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Said Abdullah: Soekarno Cup, Membangun Pesepak Bola Berkarakter</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:05:06 +0700</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>Pada tahun 2025, Tim Sepak Bola PDI Perjuangan Jawa Timur menjuarai kompetisi Soekarno Cup di Bali.</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8264907/said-abdullah-soekarno-cup-membangun-pesepak-bola-berkarakter</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/kgfOPnTlGQORU6JmUKn1dTCzVVc=/0x0:768x433/673x379/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9318802/original/089342000_1786161821-Ketua_DPD_PDIP_Jawa_Timur_Said_Abdullah.jpeg</t>
+        </is>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Rumah Terduga Pelaku Pembunuh Bos Royal Phone Ambarawa Digeruduk Massa</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:08:50 +0700</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>'Kami imbau agar semua tetap tenang dan mempercayakan penegakan hukum kepada kepolisian,' ungkapnya.</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/08/08/110844878/rumah-terduga-pelaku-pembunuh-bos-royal-phone-ambarawa-digeruduk-massa</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/2_Kp0AoEtATI61GzUZC2i1pQD24=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/08/6a76a0305b9b0.jpg</t>
+        </is>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Panas Ekstrem, Lansia di Korea Selatan Pilih Ngadem di Bandara Incheon</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:08:50 +0700</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>Bandara Internasional Incheon, Korea Selatan, dimanfaatkan sebagai tempat berlindung dari gelombang panas oleh sejumlah warga lansia.</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>https://travel.kompas.com/read/2026/08/08/104109927/panas-ekstrem-lansia-di-korea-selatan-pilih-ngadem-di-bandara-incheon</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/D8ap5HUxoeRgqMdtBmhfsoANMxE=/0x0:600x400/1200x675/filters:watermark(data/photo/2026/01/30/697c81889b5f6.png,0,-0,1)/data/photo/2024/11/21/673eab7166adc.png</t>
+        </is>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Ramai Tren Fiber Maxxing, Perlukah Serat Sebanyak Itu?</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:08:50 +0700</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>Tren fiber maxxing dorong konsumsi serat hingga 100 gram per hari. Pakar gizi IPB ingatkan kebutuhan sebenarnya jauh lebih rendah.</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>https://lifestyle.kompas.com/read/2026/08/08/100300120/ramai-tren-fiber-maxxing-perlukah-serat-sebanyak-itu-</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/zyYlqDza_nv3zDeSAv1jRHhmp58=/0x0:1266x844/1200x675/filters:watermark(data/photo/2026/01/30/697c817ed68bb.png,0,-0,1)/data/photo/2021/09/21/6149458c12e59.jpg</t>
+        </is>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I228"/>
+  <autoFilter ref="A1:I293"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-08 05:40 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-08.xlsx
+++ b/data/berita_2026-08-08.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$293</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$366</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I293"/>
+  <dimension ref="A1:I366"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -14205,8 +14205,3439 @@
         </is>
       </c>
     </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Eala, Rybakina, Gauff melaju ke 16 besar WTA 1000 Toronto</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:31:19 +0700</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>Petenis Filipina Alexandra Eala, Elena Rybakina, dan Coco Gauff melaju ke babak 16 besar turnamen WTA 1000 National ...</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685496/eala-rybakina-gauff-melaju-ke-16-besar-wta-1000-toronto</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG_0155.jpeg</t>
+        </is>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>11.000 personel perkuat sinergitas lewat apel kebangsaan sambut HUT RI</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:29:43 +0700</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>Sebanyak 11.000 personel gabungan memperkuat sinergitas lewat Apel Kebangsaan dalam rangka menyambut Hari Ulang Tahun ...</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685492/11000-personel-perkuat-sinergitas-lewat-apel-kebangsaan-sambut-hut-ri</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001017914.jpg</t>
+        </is>
+      </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Presiden Iran: Teheran dukung dialog, tetapi tak bisa dipaksa menyerah</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:28:30 +0700</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>Presiden Iran Masoud Pezeshkian menegaskan kembali komitmen negaranya untuk menempuh jalur dialog demi melindungi ...</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685488/presiden-iran-teheran-dukung-dialog-tetapi-tak-bisa-dipaksa-menyerah</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/CjkinzN000003_20260808_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Anggota DPR minta pengawasan sekolah diperkuat usai temuan senjata</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:24:03 +0700</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>Anggota Komisi X DPR RI Adde Rosi Khoerunnisa meminta pengawasan dan keamanan satuan pendidikan diperkuat menyusul ...</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685487/anggota-dpr-minta-pengawasan-sekolah-diperkuat-usai-temuan-senjata</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/Sterilisasi-sekolah-swasta-usai-temuan-senjata-api-070826-RIV-4.jpg</t>
+        </is>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>KemenHAM Babel dampingi warga miskin dapatkan kepesertaan JKN</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:14:09 +0700</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>Kantor Wilayah Kementerian Hak Asasi Manusia Kepulauan Bangka Belitung siap mendampingi warga miskin yang belum ...</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685485/kemenham-babel-dampingi-warga-miskin-dapatkan-kepesertaan-jkn</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/ham-bpjs.jpg</t>
+        </is>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>Hashim kukuhkan 20 ormas baru untuk kawal program pemerintah</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:11:56 +0700</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>Ketua Dewan Pembina Forum Masyarakat Indonesia Emas (FORMAS) Hashim Djojohadikusumo mengukuhkan 20 organisasi ...</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685484/hashim-kukuhkan-20-ormas-baru-untuk-kawal-program-pemerintah</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001225147.jpg</t>
+        </is>
+      </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>DPR serap aspirasi Papua dalam penyusunan RUU Masyarakat Adat</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:08:07 +0700</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>Badan Legislasi (Baleg) DPR RI menyerap aspirasi dari Papua sebagai bagian dari penyusunan Rancangan Undang-Undang ...</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685483/dpr-serap-aspirasi-papua-dalam-penyusunan-ruu-masyarakat-adat</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1002077731.jpg</t>
+        </is>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>Kelompok milisi Irak nyatakan "tunda" balasan terhadap pasukan AS</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:06:33 +0700</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>Perlawanan Islam di Irak (Islamic Resistance in Iraq), kelompok yang menaungi milisi-milisi pro-Iran di Irak, pada ...</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685480/kelompok-milisi-irak-nyatakan-tunda-balasan-terhadap-pasukan-as</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2017/12/20171229bendera-irak-002baru2.jpg</t>
+        </is>
+      </c>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>Efek baik ikan berlemak pada kesehatan jantung</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:06:02 +0700</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>Banyak makanan seperti buah, sayuran dan biji-bijian utuh yang kaya serat dianggap baik untuk membantu menjaga ...</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685476/efek-baik-ikan-berlemak-pada-kesehatan-jantung</t>
+        </is>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/01/25/stethoscope-4820535_1920.jpg</t>
+        </is>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>"Ayah, Persebaya juara yah"</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:52:39 +0700</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>Rachmat Irianto memilih menepi ketika rekan-rekannya larut dalam pesta juara Persebaya Surabaya setelah memenangi Piala ...</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685472/ayah-persebaya-juara-yah</t>
+        </is>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG_20260808_105949.jpg</t>
+        </is>
+      </c>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Sastra untuk penyadaran kebangsaan</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:51:34 +0700</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>Bulan Agustus adalah bulan "kenang juang" bagi bangsa Indonesia yang dapat dimanfaatkan untuk melipatgandakan ...</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685471/sastra-untuk-penyadaran-kebangsaan</t>
+        </is>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/ilustrasi_sastra_kebangsaan.jpg</t>
+        </is>
+      </c>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Chile, Venezuela pulihkan hubungan konsuler usai 2 tahun penangguhan</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:47:34 +0700</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>Chile pada Kamis (6/8) menyatakan telah secara resmi memulihkan hubungan konsuler dengan Venezuela setelah penangguhan ...</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685467/chile-venezuela-pulihkan-hubungan-konsuler-usai-2-tahun-penangguhan</t>
+        </is>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2011/03/20110313094314amerikalatin.jpg</t>
+        </is>
+      </c>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Guru Besar: Bahan pangan lokal jaga kualitas MBG, biaya terjangkau</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:46:32 +0700</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>Guru Besar Ilmu Gizi IPB University Prof Dr Hardinsyah menawarkan pemanfaatan bahan pangan lokal sebagai salah ...</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685464/guru-besar-bahan-pangan-lokal-jaga-kualitas-mbg-biaya-terjangkau</t>
+        </is>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/budi-daya-nila-untuk-kebutuhan-mbg-di-medan-2836715.jpg</t>
+        </is>
+      </c>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Menyelamatkan Si Miskin dari muslihat jahat bandar judol</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:46:24 +0700</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>Kemiskinan dan judi seolah menjalin persahabatan yang kian sulit dipisahkan. Di tengah tekanan ekonomi, penghasilan ...</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685460/menyelamatkan-si-miskin-dari-muslihat-jahat-bandar-judol</t>
+        </is>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/mensos-sampaikan-penyaluran-bansos-triwulan-iii-2834955.jpg</t>
+        </is>
+      </c>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>BMKG ingatkan potensi karhutla Sulteng pada 9-15 Agustus</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:37:27 +0700</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>Badan Meteorologi, Klimatologi, dan Geofisika (BMKG) mengingatkan potensi kebakaran hutan dan lahan (karhutla) di ...</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685457/bmkg-ingatkan-potensi-karhutla-sulteng-pada-9-15-agustus</t>
+        </is>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG-20260808-WA0026.jpg</t>
+        </is>
+      </c>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>Gibran minta sekolah terdampak banjir di Bireuen segera diperbaiki</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:30:53 +0700</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>Wakil Presiden Gibran Rakabuming meminta jajarannya untuk mengecek kondisi SD Negeri 11 Jangka di Kabupaten Bireuen, ...</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685456/gibran-minta-sekolah-terdampak-banjir-di-bireuen-segera-diperbaiki</t>
+        </is>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG_3704.jpeg</t>
+        </is>
+      </c>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>Kemenhut tangani kebakaran di Gunung Gede Pangrango, tutup pendakian</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:30:26 +0700</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>Kementerian Kehutanan (Kemenhut) bergerak cepat menanggulangi kebakaran lahan di Alun-Alun Barat Surya Kencana, kawasan ...</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685452/kemenhut-tangani-kebakaran-di-gunung-gede-pangrango-tutup-pendakian</t>
+        </is>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/WhatsApp-Image-2026-08-08-at-10.34.46-1.jpeg</t>
+        </is>
+      </c>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>PIHPS catat harga cabai rawit Rp59.650/kg, telur ayam Rp29.450/kg</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:21:58 +0700</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>Pusat Informasi Harga Pangan Strategis (PIHPS) Nasional, yang dikelola Bank Indonesia, mencatat harga komoditas cabai ...</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685451/pihps-catat-harga-cabai-rawit-rp59650-kg-telur-ayam-rp29450-kg</t>
+        </is>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/7A481E67-A1B9-4B04-B2BE-B1CB184356FD.jpeg</t>
+        </is>
+      </c>
+      <c r="I311" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Indef menilai penguatan sektor produktif kunci perluas lapangan kerja</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:18:33 +0700</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>Direktur Eksekutif Institute for Development of Economics and Finance (Indef) Esther Sri Astuti menilai penguatan ...</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685448/indef-menilai-penguatan-sektor-produktif-kunci-perluas-lapangan-kerja</t>
+        </is>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/pertumbuhan-ekonomi-sulawesi-tenggara-semester-i-2026-2836753.jpg</t>
+        </is>
+      </c>
+      <c r="I312" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>Forum warga kembali desak pemerintah terbitkan PP Cukai MBDK</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:14:00 +0700</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>‎‎Forum Warga Kota (Fakta) Indonesia kembali mendesak pemerintah segera menerbitkan Peraturan Pemerintah ...</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685445/forum-warga-kembali-desak-pemerintah-terbitkan-pp-cukai-mbdk</t>
+        </is>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/f0a7ce8e-3875-4182-b5cf-e96d61f43fb6.jpeg</t>
+        </is>
+      </c>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>Daftar harga emas di Pegadaian yang kompak naik Sabtu ini</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:08:20 +0700</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>Harga emas di laman Pegadaian dikutip dari Jakarta, Sabtu, pukul 11.01 WIB, menunjukkan harga emas jenama Galeri24, ...</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685443/daftar-harga-emas-di-pegadaian-yang-kompak-naik-sabtu-ini</t>
+        </is>
+      </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/29/harga-emas-antam-turun-2829991.jpg</t>
+        </is>
+      </c>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Wamenekraf dorong festival musik jadi ruang bertemu pelaku kreatif</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:04:52 +0700</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>Wakil Menteri Ekonomi Kreatif/Wakil Kepala Badan Ekonomi Kreatif, Irene Umar, mendorong festival musik tidak hanya ...</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685439/wamenekraf-dorong-festival-musik-jadi-ruang-bertemu-pelaku-kreatif</t>
+        </is>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/db824575-4720-40e2-b7f5-a622694f8b74.jpeg</t>
+        </is>
+      </c>
+      <c r="I315" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>Mendag dorong pertemuan kedua JTC RI-Mesir digelar tahun ini</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:02:19 +0700</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>Menteri Perdagangan (Mendag) Budi Santoso berharap pertemuan kedua Komite Perdagangan Bersama (Joint Trade ...</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685435/mendag-dorong-pertemuan-kedua-jtc-ri-mesir-digelar-tahun-ini</t>
+        </is>
+      </c>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG_3702_1.jpeg</t>
+        </is>
+      </c>
+      <c r="I316" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>Damkar Sisir Tumpukan Kertas di Gedung Bapenda DKI Cegah Api Muncul Lagi</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:18:18 +0700</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>Brigitta Belia Permata Sari</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>Petugas pemadam kebakaran masih melakukan penyisiran di Gedung Badan Pendapatan Daerah (Bapenda) DKI Jakarta yang terbakar.</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609703/damkar-sisir-tumpukan-kertas-di-gedung-bapenda-dki-cegah-api-muncul-lagi</t>
+        </is>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/kondisi-gedung-bapenda-dki-usai-terbakar-1786154514661_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>Polisi Ungkap Saepul Pelaku Mutilasi Pria di Depok Pedagang Piscok</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:17:03 +0700</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>Polda Metro Jaya mengungkap identitas Saepul, pelaku mutilasi pria K. Saepul, yang berdagang piscok.</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609702/polisi-ungkap-saepul-pelaku-mutilasi-pria-di-depok-pedagang-piscok</t>
+        </is>
+      </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/polisi-melakukan-penyisiran-di-kali-licin-depok-untuk-mencari-potongan-kaki-korban-mutilasi-1786008041635_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I318" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>Pakar Dorong Polri Tindak Tegas Penyebar Konten Provokatif di Medsos</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:07:38 +0700</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>Anggi Muliawati</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>Pakar Hukum Tata Negara Muhammad Rullyandi mendorong Polri menindak tegas penyebar konten manipulatif di media sosial yang menimbulkan kegaduhan publik.</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609698/pakar-dorong-polri-tindak-tegas-penyebar-konten-provokatif-di-medsos</t>
+        </is>
+      </c>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2023/10/25/pakar-hukum-tata-negara-muhammad-rullyandi_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I319" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>Biddokes Polda Metro Bantu Tangani Korban Kebakaran Gedung Bapenda</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:05:13 +0700</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>Mei Amelia R</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>Polda Metro Jaya kerahkan Tim Keslap dan DVI untuk tangani kebakaran Gedung Bapenda DKI Jakarta. Satu korban selamat dirawat akibat hipoksia.</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609696/biddokes-polda-metro-bantu-tangani-korban-kebakaran-gedung-bapenda</t>
+        </is>
+      </c>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/tim-dokkes-polda-metro-jaya-bantu-menangani-korban-kebakaran-gedung-bapenda-dki-1786165499467_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I320" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>Polisi Rinci Temuan di Sekolah Jaksel: 995 Senjata Angin dan 1 Senpi</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:55:23 +0700</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>Polda Metro Jaya mengonfirmasi 996 senjata ditemukan di sekolah swasta, mayoritas senjata angin. Senjata api hanya satu dan pemiliknya sudah diketahui.</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609676/polisi-rinci-temuan-di-sekolah-jaksel-995-senjata-angin-dan-1-senpi</t>
+        </is>
+      </c>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/temuan-ratusan-pucuk-senjata-di-sekolah-swasta-di-pondok-pinang-jakarta-selatan-1786014363566_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I321" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>Eks Ketua Yayasan Dipanggil Pekan Depan soal Temuan 995 Senjata di Sekolah</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:52:10 +0700</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>Polisi akan memanggil mantan Ketua Yayasan sekolah swasta IWD terkait temuan 995 senjata angin dan satu senjata api. Pemanggilan dilakukan pekan depan.</t>
+        </is>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609675/eks-ketua-yayasan-dipanggil-pekan-depan-soal-temuan-995-senjata-di-sekolah</t>
+        </is>
+      </c>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/temuan-ratusan-pucuk-senjata-di-sekolah-swasta-di-pondok-pinang-jakarta-selatan-1786014363566_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I322" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>Kecelakaan Kapal Tenggelam yang Disebut Lebih Mematikan daripada Titanic</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:46:06 +0700</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>Rakhmad Hidayatulloh Permana</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>Jumlah korban jiwa dari kecelakaan kapal ini melampaui tragedi tenggelamnya Kapal Titanic.</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609669/kecelakaan-kapal-tenggelam-yang-disebut-lebih-mematikan-daripada-titanic</t>
+        </is>
+      </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/peristiwa-tenggelamnya-mv-le-joola-milik-pemerintah-senegal-merupakan-sejarah-kelam-yang-sulit-dilupakan-1786100657631_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I323" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>Polda Metro Tegaskan Jakarta Aman dan Terkendali, Ekonomi Lancar</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:36:32 +0700</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>Polda Metro Jaya memastikan Jakarta aman dan terkendali. Kegiatan masyarakat dan kunjungan pejabat luar negeri menunjukkan situasi yang kondusif.</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609659/polda-metro-tegaskan-jakarta-aman-dan-terkendali-ekonomi-lancar</t>
+        </is>
+      </c>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/kabid-humas-polda-metro-jaya-kombes-budi-hermanto-menegaskan-jakarta-aman-dan-terkendali-1786163705322_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I324" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>Apel Kebangsaan di Monas, Ojol hingga Buruh Serukan Komitmen Jaga Persatuan</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:33:53 +0700</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>Polda Metro Jaya dan Kodam Jaya menggelar apel kebangsaan di Jakarta dengan 11 ribu peserta. Acara ini menekankan persatuan dan keamanan Ibu Kota.</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609656/apel-kebangsaan-di-monas-ojol-hingga-buruh-serukan-komitmen-jaga-persatuan</t>
+        </is>
+      </c>
+      <c r="H325" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/polda-metro-jaya-menggelar-apel-kebangsaan-menggandeng-ormas-untuk-menjaga-jakarta-1786156805660_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I325" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>Kapolri Ajak Tapak Suci Putera Muhammadiyah Kolaborasi Jaga Negeri</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:25:24 +0700</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>Lisye Sri Rahayu</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>Kapolri Jenderal Listyo Sigit Prabowo mengajak Tapak Suci Putera Muhammadiyah berkolaborasi menjaga keamanan dan melindungi generasi muda.</t>
+        </is>
+      </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G326" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609647/kapolri-ajak-tapak-suci-putera-muhammadiyah-kolaborasi-jaga-negeri</t>
+        </is>
+      </c>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/kapolri-jenderal-listyo-sigit-prabowo-1786157459700_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I326" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>1 Lagi Tersangka Kasus Dana Syariah Indonesia Segera Disidang, Aset Rp 425 Miliar Disita</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:22:04 +0700</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>Wilda Hayatun Nufus</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>Dittipideksus Bareskrim Polri telah merampungkan berkas perkara tersangka mantan Direktur PT Dana Syariah Indonesia (DSI) inisial AS kasus fraud PT DSI.</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G327" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609639/1-lagi-tersangka-kasus-dana-syariah-indonesia-segera-disidang-aset-rp-425-miliar-disita</t>
+        </is>
+      </c>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/dittipideksus-bareskrim-polri-telah-merampungkan-lagi-berkas-perkara-tersangka-mantan-direktur-pt-dana-syariah-indonesia-dsi-i-1786162798543_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I327" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>Puslabfor Dikerahkan Selidiki Penyebab Kebakaran Gedung Bapenda DKI</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:20:26 +0700</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>Brigitta Belia Permata Sari</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>Tim Puslabfor dikerahkan untuk mengusut penyebab kebakaran gedung Bapenda DKI. Polisi masih menunggu proses penyisiran gedung oleh damkar sebelum olah TKP.</t>
+        </is>
+      </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G328" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609638/puslabfor-dikerahkan-selidiki-penyebab-kebakaran-gedung-bapenda-dki</t>
+        </is>
+      </c>
+      <c r="H328" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/gedung-bapenda-dki-dipasangi-garis-polisi-1786162667826_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I328" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Kapolri Dukung Program Pemerintah Hadapi Situasi Global: Kita Harus Mandiri</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:01:50 +0700</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>Lisye Sri Rahayu</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>Kapolri Jenderal Sigit menekankan pentingnya kemandirian Indonesia di tengah ketidakpastian global.</t>
+        </is>
+      </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G329" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609614/kapolri-dukung-program-pemerintah-hadapi-situasi-global-kita-harus-mandiri</t>
+        </is>
+      </c>
+      <c r="H329" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/kapolri-jenderal-listyo-sigit-prabowo-1786157459771_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>Danantara Telah Pangkas 274 BUMN</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:00:07 +0700</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>Heri Purnomo</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>Kepala BP BUMN, Dony Oskaria, mengungkapkan pemangkasan 274 entitas BUMN sebagai bagian dari transformasi untuk efisiensi.</t>
+        </is>
+      </c>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G330" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8609450/danantara-telah-pangkas-274-bumn</t>
+        </is>
+      </c>
+      <c r="H330" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/07/01/wisma-danantara-indonesia-1751345662273_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I330" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>MSCI Umumkan Rebalancing Saham 12 Agustus</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:00:32 +0700</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>Andi Hidayat</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>Penyedia indeks saham global, MSCI, akan mengumumkan hasil Tinjauan Indeks Agustus 2026 (August 2026 Index Review) atau rebalancing indeks pada 12 Agustus 2026.</t>
+        </is>
+      </c>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G331" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8609448/msci-umumkan-rebalancing-saham-12-agustus</t>
+        </is>
+      </c>
+      <c r="H331" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/01/28/bei-terapkan-trading-halt-imbas-ihsg-anjlok-1769587531040_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I331" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>Jamkrindo Cetak Laba Rp 743 M, Naik 34%</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:30:16 +0700</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>Ignacio Geordi Oswaldo</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>PT Jaminan Kredit Indonesia (Persero) atau Jamkrindo mencatatkan laba sebelum pajak sebesar Rp 743,23 miliar pada semester I-2026.</t>
+        </is>
+      </c>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G332" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/moneter/d-8609455/jamkrindo-cetak-laba-rp-743-m-naik-34</t>
+        </is>
+      </c>
+      <c r="H332" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2023/04/27/jamkrindo_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I332" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>Harga Emas Antam Hari Ini Melambung Tinggi</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:00:25 +0700</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>Ignacio Geordi Oswaldo</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>Harga emas Antam 24 karat naik Rp 40.000 per gram lagi dan kini berada di level Rp 2.690.000 per gram.</t>
+        </is>
+      </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G333" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8609521/harga-emas-antam-hari-ini-melambung-tinggi</t>
+        </is>
+      </c>
+      <c r="H333" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/10/21/harga-emas-antam-meroket-hari-ini-nyaris-rp-25-juta-per-gram-1761021329895_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>Sambut Spin-Off Tahap 2, InfraNexia Topang Konektivitas Wholesale</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:56:08 +0700</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>Melalui langkah ini, Telkom mempertajam fokus pengelolaan aset infrastruktur digital, memperluas kolaborasi, serta menciptakan nilai untuk jangka panjang.</t>
+        </is>
+      </c>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G334" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260808095243-625-1390033/sambut-spin-off-tahap-2-infranexia-topang-konektivitas-wholesale</t>
+        </is>
+      </c>
+      <c r="H334" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/telkom-1786157702667_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I334" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>Bukan Cuma di Film, Pemain Operasi Pesta Copet Akui Karakter Terbawa hingga di Luar Syuting</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:17:59 +0700</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>Pemain film Operasi Pesta Copet mengaku peran sebagai pencopet ikut terbawa hingga di luar proses syuting.</t>
+        </is>
+      </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G335" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7865681/bukan-cuma-di-film-pemain-operasi-pesta-copet-akui-karakter-terbawa-hingga-di-luar-syuting</t>
+        </is>
+      </c>
+      <c r="H335" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/5Nc86OtURgN_lcoII6Oxk0hDSQU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Zulfa-dan-Kawai.jpg</t>
+        </is>
+      </c>
+      <c r="I335" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>Prakiraan Cuaca Papua Barat Minggu 9 Agustus 2026, BMKG: Teluk Wondama Hujan Ringan Siang Hari</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:17:30 +0700</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>Prakiraan Cuaca Papua Barat Minggu 9 Agustus 2026 berpotensi hujan ringan pada siang hingga sore hari, Teluk Wondama hujan ringan pada siang hari.</t>
+        </is>
+      </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G336" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865680/prakiraan-cuaca-papua-barat-minggu-9-agustus-2026-bmkg-teluk-wondama-hujan-ringan-siang-hari</t>
+        </is>
+      </c>
+      <c r="H336" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/jZpjwAFeM_hG9ZoYPopBuPzxiF4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/wisata-Papua-Barat-Pantai-Bori-Kampung-Nuni-Distrik-Manokwari-Utara-Kabupaten-Manokwari.jpg</t>
+        </is>
+      </c>
+      <c r="I336" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>4 Teks Doa Upacara Hari Pramuka 2026, Singkat dan Khidmat</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:16:28 +0700</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>4 teks doa upacara Hari Pramuka 2026 yang singkat, tetapi tetap khidmat dan dapat menjadi referensi. Teks doa sesuai dengan tema Hari Pramuka 2026.</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G337" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/pendidikan/7865679/4-teks-doa-upacara-hari-pramuka-2026-singkat-dan-khidmat</t>
+        </is>
+      </c>
+      <c r="H337" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/jo-cczR-g1VXqTpl5fVdiPXq8q0=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/pemkot-malang-gelar-peringatan-hari-pramuka_20230819_130208.jpg</t>
+        </is>
+      </c>
+      <c r="I337" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Kunci Gitar Lagu Februari - Rony Parulian: Ini Pertama Kali Ku Paksa Beranikan Hati</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:15:04 +0700</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>Kunci gitar lagu Februari - Rony Parulian chord dasar yang mudah dimainkan: ini pertama kali ku paksa beranikan hati dengan sedikit romansa bunga.</t>
+        </is>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G338" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/musik/7865678/kunci-gitar-lagu-februari-rony-parulian-ini-pertama-kali-ku-paksaberanikan-hati</t>
+        </is>
+      </c>
+      <c r="H338" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/eR3zla2C-eLuRKdct7nJlHf_pG0=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Potret-gitar-akustik-untuk-kunci-chord-dasar-mudah-dimainkan-ifan-main-gitar.jpg</t>
+        </is>
+      </c>
+      <c r="I338" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Kunci Gitar Lagu Kita Melawan Dunia - BAALE ‘Film Operasi Pesta Copet’: Hanya Kau yang Tahu Aku</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:13:50 +0700</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>Kunci gitar lagu Kita Melawan Dunia - BAALE chord dasar mudah dimainkan: meskipun kau jauh dari pintar bodohnya aku terus merasa benar.</t>
+        </is>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G339" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/musik/7865677/kunci-gitar-lagu-kita-melawan-dunia-baale-film-operasi-pesta-copet-hanya-kau-yang-tahu-aku</t>
+        </is>
+      </c>
+      <c r="H339" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/rczNxOofvn1NTDkof7pOK0Fsojo=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/iqbal-ramadhanjpoy.jpg</t>
+        </is>
+      </c>
+      <c r="I339" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>Jadwal Semifinal Piala AFF 2026: Vietnam Menunggu Lawan, Thailand Butuh Satu Poin Agar Tak Bertemu</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:09:54 +0700</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>Timnas Vietnam memastikan tiket semifinal Asean Championship atau Piala AFF 2026 setelah keluar sebagai juara Grup A. Sementara di Grup B masih ketat.</t>
+        </is>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G340" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865676/jadwal-semifinal-piala-aff-2026-vietnam-menunggu-lawan-thailand-butuh-satu-poin-agar-tak-bertemu</t>
+        </is>
+      </c>
+      <c r="H340" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/QePOadZQiN674FYqUm-_jul1gPY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Timnas-Indonesia-Hadapi-Vietnam-di-Laga-Penyisihan-Piala-AFF-2026-2.jpg</t>
+        </is>
+      </c>
+      <c r="I340" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>Sesumbar Bek Singapura Usai Redam Timnas Indonesia, Eks Madura United Ungkap Rahasia The Lions</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:07:44 +0700</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>Bek Singapura Jacob Mahler sesumbar usai The Lions meredam Timnas Indonesia. Ia mengungkap rahasia mentalitas timnya hingga lolos ke semifinal.</t>
+        </is>
+      </c>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G341" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865675/sesumbar-bek-singapura-usai-redam-timnas-indonesia-eks-madura-united-ungkap-rahasia-the-lions</t>
+        </is>
+      </c>
+      <c r="H341" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/YblviT31OLUhxAt9xDIKI94p0os=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Bek-Timnas-Indonesia-Mitchell-Baker-saat-melawan-Singapura-di-PIala-AFF-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I341" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Putri Anwar Ibrahim Mundur dari PKR, Masa Depan Politik PM Malaysia Dipertanyakan</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:06:42 +0700</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>Nurul Izzah Anwar, putri PM Malaysia Anwar Ibrahim, memilih cuti sementara dari jabatan wakil presiden PKR.</t>
+        </is>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G342" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7865674/putri-anwar-ibrahim-mundur-dari-pkr-masa-depan-politik-pm-malaysia-dipertanyakan</t>
+        </is>
+      </c>
+      <c r="H342" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/yyHdXUv47erUXNgy_X4ep5CZLEI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/POLITIK-MALAYSIA-Nurul-Izzah-Anwar-kanan-pu.jpg</t>
+        </is>
+      </c>
+      <c r="I342" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>Live TikTok Berujung Maut: Kronologi Influencer Meksiko Tewas Ditembak, 2 Pria Bermotor Jadi Sorotan</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:01:49 +0700</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>Influencer TikTok asal Meksiko, Cesar Gastelum, tewas ditembak saat tengah melakukan siaran langsung TikTok.</t>
+        </is>
+      </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G343" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865673/live-tiktok-berujung-maut-kronologi-influencer-meksiko-tewas-ditembak-2-pria-bermotor-jadi-sorotan</t>
+        </is>
+      </c>
+      <c r="H343" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/POX2Oltj6cNUFfiZ7jYShalFYbw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Influencer-Meksiko-Tewas.jpg</t>
+        </is>
+      </c>
+      <c r="I343" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>Perasaan Bangga Pelatih Singapura usai Singkirkan Timnas Indonesia dari Piala AFF 2026</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:01:44 +0700</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>Pelatih Singapura, Gavin Lee, mengaku bangga setelah anak asuhnya mampu menyingkirkan Timnas Indonesia sekaligus mengamankan tiket ke semifinal.</t>
+        </is>
+      </c>
+      <c r="F344" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G344" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865672/perasaan-bangga-pelatih-singapura-usai-singkirkan-timnas-indonesia-dari-piala-aff-2026</t>
+        </is>
+      </c>
+      <c r="H344" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/tZqFKgwVQ5eW_YBK_O5n7jSWMXA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Timnas-Indonesia-Dicukur-Timnas-Vietnam-3-0_20260804_065938.jpg</t>
+        </is>
+      </c>
+      <c r="I344" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>Kunci Jawaban Bahasa Indonesia Kelas 9 Halaman 68 Edisi Revisi: Belajar Menulis Pantun</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:57:46 +0700</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>Kunci jawaban Bahasa Indonesia kelas 9 halaman 68 SMP, MTs Kurikulum Merdeka Edisi Revisi, Belajar Menulis Pantun pada Bab 2 Belajar Berpantun</t>
+        </is>
+      </c>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G345" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/pendidikan/7865671/kunci-jawaban-bahasa-indonesia-kelas-9-halaman-68-edisi-revisi-belajar-menulis-pantun</t>
+        </is>
+      </c>
+      <c r="H345" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/jCJrUhYEs87eIWT8V7FFxnJwfHQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/SISWA-SMP-BELAJAR-03.jpg</t>
+        </is>
+      </c>
+      <c r="I345" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>Satu Korban Dievakuasi dari Lantai Paling Atas Gedung Bapenda DKI yang Terbakar</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:56:56 +0700</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>Satu korban yang selamat dari kebakaran gedung Bapenda DKI Jakarta, saat ini tengah di rawat di rumah sakit.</t>
+        </is>
+      </c>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G346" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7865670/satu-korban-dievakuasi-dari-lantai-paling-atas-gedung-bapenda-dki-yang-terbakar</t>
+        </is>
+      </c>
+      <c r="H346" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/WEg6aNuIonboivDqai0AIN6RniU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Bapenda-1-08082026.jpg</t>
+        </is>
+      </c>
+      <c r="I346" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>Kemensetneg Ingatkan Waspada Penipuan Pendaftaran Undangan Upacara HUT ke-81 RI, Hindari Modus Ini</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:55:01 +0700</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>Masyarakat diminta waspada penipuan pendaftaran undangan upacara HUT ke-81 RI di Istana Merdeka yang akan digelar pada 17 Agustus 2026.</t>
+        </is>
+      </c>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G347" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865669/kemensetneg-ingatkan-waspada-penipuan-pendaftaran-undangan-upacara-hut-ke-81-ri-hindari-modus-ini</t>
+        </is>
+      </c>
+      <c r="H347" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/o0_zlOyhi8b4L7YXj_iMlLMaHrQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Upacara-peringatan-Detik-detik-Proklamasi-di-Istana-Merdeka_20250817_165411.jpg</t>
+        </is>
+      </c>
+      <c r="I347" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Betrand Peto Disebut sebagai 'Pemegang Kartu' Konflik Ruben Onsu-Sarwendah</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:52:36 +0700</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>Betrand Peto disebut sebagai sosok 'pemegang kartu' atas konflik orang tua angkatnya, Ruben Onsu dan Sarwendah.</t>
+        </is>
+      </c>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G348" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7865668/betrand-peto-disebut-sebagai-pemegang-kartu-konflik-ruben-onsu-sarwendah</t>
+        </is>
+      </c>
+      <c r="H348" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/tenUH5P22L2cabOSMU5cvvx-9cs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Betrand-Peto-onyo2.jpg</t>
+        </is>
+      </c>
+      <c r="I348" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Kasus Temuan Senjata, Polisi Periksa Mantan Ketua Yayasan Sekolah di Pondok Pinang Pekan Depan</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:52:35 +0700</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>Polda Metro Jaya akan memanggil mantan ketua yayasan sekolah berinisial IWD terkait temuan ratusan senjata.</t>
+        </is>
+      </c>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G349" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865667/kasus-temuan-senjata-polisi-periksa-mantan-ketua-yayasan-sekolah-di-pondok-pinang-pekan-depan</t>
+        </is>
+      </c>
+      <c r="H349" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/C0lT2Y0zI_MxSjs7s2qkRNylM8s=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Benda-berbentuk-senjata-yang-ditemukan-di-sebuah-ruangan-321.jpg</t>
+        </is>
+      </c>
+      <c r="I349" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Smartphone Second Makin Diminati di Bali, Layanan Trade-in dan Service Jadi Andalan</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:49:04 +0700</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>Tren smartphone second meningkat di Bali. Rumah Gadget Bali hadirkan pilihan gawai berkualitas dengan layanan trade-in dan service.</t>
+        </is>
+      </c>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G350" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865666/smartphone-second-makin-diminati-di-bali-layanan-trade-in-dan-service-jadi-andalan</t>
+        </is>
+      </c>
+      <c r="H350" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/LCRwhDCMl3lzD6ryF1Optz70ENk=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Rumah-Gadget-Bali.jpg</t>
+        </is>
+      </c>
+      <c r="I350" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>AS Waspada, Putin Diprediksi Makin Berani Menguji Persatuan NATO</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:48:05 +0700</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>Intelijen AS menilai Vladimir Putin mungkin semakin berani melakukan aksi provokatif yang menyasar wilayah NATO.</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7865665/as-waspada-putin-diprediksi-makin-berani-menguji-persatuan-nato</t>
+        </is>
+      </c>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/YluflkzHOti6GRvPG5NTA8siVxs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Presiden-Rusia-Vladimir-Putin-menjawabsdsdd.jpg</t>
+        </is>
+      </c>
+      <c r="I351" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>Bertemu Shandy Purnamasari di Lapas, Isa Zega Menangis Peluk sang Pengusaha: Maafin Mami Ya Neng</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:47:30 +0700</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>Bertemu dengan Shandy Purnamasari di Lapas, Isa Zega menangis sambil memeluk sang pengusaha saat meminta maaf.</t>
+        </is>
+      </c>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G352" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7865664/bertemu-shandy-purnamasari-di-lapas-isa-zega-menangis-peluk-sang-pengusaha-maafin-mami-ya-neng</t>
+        </is>
+      </c>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/WN2_p6-4qWfzGn6pMmdhUKcCJyI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Shandy-Purnamasari-beri-kesaksian-dalam-persidangan-kasus-pencemaran-nama-baik-Isa-Zega.jpg</t>
+        </is>
+      </c>
+      <c r="I352" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>Polisi Jadwalkan Pemeriksaan Eks Ketua Yayasan IWD Soal Penemuan Ratusan Senjata di Sekolah Jaksel</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:47:06 +0700</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>Pemeriksaan terhadap IWD nantinya akan menjadi bagian dari pendalaman terkait proses impor senjata.</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G353" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7865663/polisi-jadwalkan-pemeriksaan-eks-ketua-yayasan-iwd-soal-penemuan-ratusan-senjata-di-sekolah-jaksel</t>
+        </is>
+      </c>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/enu60eSCVJ1ALLFEmi5pFfeMTg4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/996-senjata-di-sebuah-sekolah-kawasan-Pondok-Pinang-32010.jpg</t>
+        </is>
+      </c>
+      <c r="I353" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Wawancara Trump Memanas, Pewawancara Potong Pembahasannya soal Energi Angin</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:44:09 +0700</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>Donald Trump kesal setelah pembawa acara Jake Sherman memotong pembicaraannya soal energi angin yang disebutnya sebagai “bencana”.</t>
+        </is>
+      </c>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G354" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7865662/wawancara-trump-memanas-pewawancara-potong-pembahasannya-soal-energi-angin</t>
+        </is>
+      </c>
+      <c r="H354" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/GCmoWwgSOIPZubJ0CQDJsIWSy_Q=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Presiden-AS-Donald-T1rump-membuat-pengumuman-tentang-inovasi-nuklir-Amerika.jpg</t>
+        </is>
+      </c>
+      <c r="I354" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Bank-Bank Diminta Waspada Hadapi Petaka, Korbanya Sudah Bermunculan</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:30:00 +0700</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>Sejumlah bank di banyak negara diminta untuk waspada karena perkembangan AI</t>
+        </is>
+      </c>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G355" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260808063218-37-757568/bank-bank-diminta-waspada-hadapi-petaka-korbanya-sudah-bermunculan</t>
+        </is>
+      </c>
+      <c r="H355" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/05/person-doing-an-online-bank-transaction-1785901803723_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I355" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Bulan Terus Menjauhi Bumi, Dampaknya Mulai Terasa</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 08:15:00 +0700</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>Bulan ditemukan terus menjauhi bumi, jarak keduanya yang berkisar 384.400 km</t>
+        </is>
+      </c>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G356" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260808062319-37-757567/bulan-terus-menjauhi-bumi-dampaknya-mulai-terasa</t>
+        </is>
+      </c>
+      <c r="H356" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/04/08/matahari-tertutupi-sepenuhnya-oleh-bulan-selama-penerbangan-lintas-bulan-oleh-awak-artemis-ii-7-april-2026-1775622206743_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I356" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>Finansial</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>BPK Ungkap Tantangan Government 5.0, dari Data Terfragmentasi hingga Talenta AI</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>Satria K Yudha</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA – Badan Pemeriksa Keuangan (BPK) mengungkap sejumlah tantangan dalam transformasi menuju Government 5.0, mulai dari belum meratanya transformasi digital, data pemerintah yang terfragmentasi, hingga keterbatasan talenta kecerdasan buatan...</t>
+        </is>
+      </c>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G357" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjfmr0416/bpk-ungkap-tantangan-government-50-dari-data-terfragmentasi-hingga-talenta-ai</t>
+        </is>
+      </c>
+      <c r="H357" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/_260808105715-497.png</t>
+        </is>
+      </c>
+      <c r="I357" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>Bisnis</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>Incar Generasi Z, Danantara Perluas Akses Kepemilikan Rumah Pertama</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:55:04 +0700</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>Ahmad Fikri Noor</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA - Badan Pengelola Investasi Daya Anagata Nusantara (Danantara) memperluas akses kepemilikan rumah pertama melalui penyediaan pilihan hunian dan pembiayaan secara terintegrasi, termasuk bagi generasi muda. CEO Danantara Rosan Roeslani...</t>
+        </is>
+      </c>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G358" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjfpns490/incar-generasi-z-danantara-perluas-akses-kepemilikan-rumah-pertama</t>
+        </is>
+      </c>
+      <c r="H358" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/092241800-1778687390-830-556.jpg</t>
+        </is>
+      </c>
+      <c r="I358" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>Finansial</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>Harga Emas Antam dan Pegadaian Naik di Akhir Pekan, Ini Daftar Lengkapnya</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:39:42 +0700</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>Ahmad Fikri Noor</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA - Harga emas Antam yang dipantau dari laman Logam Mulia di Jakarta, Sabtu pukul 10.05 WIB melonjak Rp 40.000 menjadi Rp 2.690.000 dari semula Rp 2.650.000 per gram,...</t>
+        </is>
+      </c>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G359" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjfoty490/harga-emas-antam-dan-pegadaian-naik-di-akhir-pekan-ini-daftar-lengkapnya</t>
+        </is>
+      </c>
+      <c r="H359" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/karyawan-melayani-nasabah-yang-ingin-membeli-emas-di-gedung_260604140124-632.JPG</t>
+        </is>
+      </c>
+      <c r="I359" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>Pertanian</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>Hingga Agustus 2026, Kementan Terbitkan 889 Sertifikat Hak PVT untuk Benih Unggul</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:33:00 +0700</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>Dwi Murdaningsih</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA - Kementerian Pertanian (Kementan) kembali menerbitkan Sertifikat Hak Perlindungan Varietas Tanaman (PVT) sebagai komitmen menyediakan benih varietas unggul baru guna mengakselerasi terwujudnya swasembada pangan. Berdasarkan data Pusat Perlindungan...</t>
+        </is>
+      </c>
+      <c r="F360" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G360" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjfon0368/hingga-agustus-2026-kementan-terbitkan-889-sertifikat-hak-pvt-untuk-benih-unggul</t>
+        </is>
+      </c>
+      <c r="H360" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/petani-menanam-bibit-di-sawah-ilustrasi-_130108184912-472.jpg</t>
+        </is>
+      </c>
+      <c r="I360" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>Video Kerusuhan Agustus Viral, Awas Bisa Dipidana</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:10:26 +0700</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>Polisi menemukan konten lama yang kembali disebarkan menjelang Agustus.</t>
+        </is>
+      </c>
+      <c r="F361" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G361" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8264961/video-kerusuhan-agustus-viral-awas-bisa-dipidana</t>
+        </is>
+      </c>
+      <c r="H361" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/IuujafOaBM2iqKahHvnTZsEFoJ0=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/5332260/original/070333800_1756462138-WhatsApp_Image_2025-08-29_at_16.55.21.jpeg</t>
+        </is>
+      </c>
+      <c r="I361" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>Puslabfor Cari Titik Api Kebakaran Gedung Bapenda DKI</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:52:04 +0700</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>Puslabfor dikerahkan untuk mengungkap titik penyebab kebakaran.</t>
+        </is>
+      </c>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G362" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8264946/puslabfor-cari-titik-api-kebakaran-gedung-bapenda-dki</t>
+        </is>
+      </c>
+      <c r="H362" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/42B01YC5FDkIDRmw2a58lHmRIzk=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9318747/original/067967000_1786155435-IMG_20260808_082643_127.jpg</t>
+        </is>
+      </c>
+      <c r="I362" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>Polisi Ungkap 4 Modus Penyebaran Hoaks di Media Sosial</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:25:16 +0700</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>Pelaku tak hanya melakukan repost, tetapi juga memanipulasi dokumen.</t>
+        </is>
+      </c>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G363" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8264925/polisi-ungkap-4-modus-penyebaran-hoaks-di-media-sosial</t>
+        </is>
+      </c>
+      <c r="H363" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/_Uio_IQhHyansj9jLNGYpQoZVag=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9318822/original/044003300_1786163070-ChatGPT_Image_Aug_8__2026__11_21_46_AM.jpg</t>
+        </is>
+      </c>
+      <c r="I363" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>Money</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>Paradoks Sarjana: Mengapa Grafik Pengangguran Terdidik Terus Naik?</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:40:55 +0700</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>Kelompok yang diharapkan jadi motor penggerak pertumbuhan ekonomi berbasis pengetahuan jumlahnya makin banyak, tertahan di ruang tunggu pasar kerja.</t>
+        </is>
+      </c>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G364" t="inlineStr">
+        <is>
+          <t>https://money.kompas.com/read/2026/08/08/124000826/paradoks-sarjana--mengapa-grafik-pengangguran-terdidik-terus-naik-</t>
+        </is>
+      </c>
+      <c r="H364" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/M0Trs8fwJ84d5lkgbSmDzUN5cbU=/0x0:5489x3659/1200x675/filters:watermark(data/photo/2026/01/30/697c815e7ef28.png,0,-0,1)/data/photo/2026/07/26/6a6540468479a.jpg</t>
+        </is>
+      </c>
+      <c r="I364" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>Penumpang KMP Ambu-Ambu Melahirkan di Tengah Laut, Ibu dan Bayi Selamat</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:40:55 +0700</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>Penumpang KMP Ambu-Ambu terpaksa melahirkan bayinya di atas kapal setelah mengalami kontraksi hebat di tengah laut</t>
+        </is>
+      </c>
+      <c r="F365" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G365" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/08/08/120751478/penumpang-kmp-ambu-ambu-melahirkan-di-tengah-laut-ibu-dan-bayi-selamat</t>
+        </is>
+      </c>
+      <c r="H365" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/qzVxtG1iznGTnEJYb0lzWIP_0to=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/08/6a76b17f1f4e9.jpeg</t>
+        </is>
+      </c>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>Nepal Resmi Terapkan e-Visa Mulai 17 Agustus, Turis Makin Mudah Masuk</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:40:55 +0700</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>Nepal resmi menerapkan e-Visa mulai 17 Agustus 2026. Turis makin mudah masuk dengan mengurus dokumen secara online.</t>
+        </is>
+      </c>
+      <c r="F366" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G366" t="inlineStr">
+        <is>
+          <t>https://travel.kompas.com/read/2026/08/08/113000727/nepal-resmi-terapkan-e-visa-mulai-17-agustus-turis-makin-mudah-masuk</t>
+        </is>
+      </c>
+      <c r="H366" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/NjytJfQXfHIpsuNRZ-TL35V2JLo=/273x0:1893x1080/1200x675/filters:watermark(data/photo/2026/01/30/697c81889b5f6.png,0,-0,1)/data/photo/2026/08/08/6a76a96be742d.jpg</t>
+        </is>
+      </c>
+      <c r="I366" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I293"/>
+  <autoFilter ref="A1:I366"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-08 06:34 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-08.xlsx
+++ b/data/berita_2026-08-08.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$366</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$416</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I366"/>
+  <dimension ref="A1:I416"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -17636,8 +17636,2358 @@
         </is>
       </c>
     </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>Spanyol perketat pemeriksaan perbatasan bagi pelancong Italia</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:29:59 +0700</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>Pemerintah Spanyol akan memberlakukan pemeriksaan perbatasan di pelabuhan dan bandara terhadap pelancong dari Italia ...</t>
+        </is>
+      </c>
+      <c r="F367" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G367" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685545/spanyol-perketat-pemeriksaan-perbatasan-bagi-pelancong-italia</t>
+        </is>
+      </c>
+      <c r="H367" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/thumbs_b_c_163e90d67c855177fcf9553fd9012181.jpg</t>
+        </is>
+      </c>
+      <c r="I367" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>Gibran minta pemulihan pascabencana harus disertai mitigasi</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:27:40 +0700</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>Wakil Presiden (Wapres) Gibran Rakabuming Raka menekankan penanganan pascabencana tidak cukup hanya dengan ...</t>
+        </is>
+      </c>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G368" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685541/gibran-minta-pemulihan-pascabencana-harus-disertai-mitigasi</t>
+        </is>
+      </c>
+      <c r="H368" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG_3705.jpeg</t>
+        </is>
+      </c>
+      <c r="I368" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>MenPANRB apresiasi peran ASN muda dalam transformasi birokrasi</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:27:29 +0700</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>Menteri Pendayagunaan Aparatur Negara dan Reformasi Birokrasi (PANRB) Rini Widyantini mengapresiasi peran ASN muda ...</t>
+        </is>
+      </c>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G369" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685539/menpanrb-apresiasi-peran-asn-muda-dalam-transformasi-birokrasi</t>
+        </is>
+      </c>
+      <c r="H369" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000582403.jpg</t>
+        </is>
+      </c>
+      <c r="I369" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>Disdik Lampung: 140 SMA/SMK mendapatkan bantuan revitalisasi</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:27:01 +0700</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>Dinas Pendidikan (Disdik) Provinsi Lampung menyebutkan sebanyak 140 sekolah jenjang SMA dan SMK di provinsi ...</t>
+        </is>
+      </c>
+      <c r="F370" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G370" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685535/disdik-lampung-140-sma-smk-mendapatkan-bantuan-revitalisasi</t>
+        </is>
+      </c>
+      <c r="H370" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001140599.jpg</t>
+        </is>
+      </c>
+      <c r="I370" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>Serangan Houthi di Yaman Picu kekhawatiran eskalasi konflik</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:23:23 +0700</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>Serangan terbaru gerakan Ansar Allah, yang juga dikenal sebagai Houthi, terhadap posisi pasukan pemerintah Yaman ...</t>
+        </is>
+      </c>
+      <c r="F371" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G371" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685533/serangan-houthi-di-yaman-picu-kekhawatiran-eskalasi-konflik</t>
+        </is>
+      </c>
+      <c r="H371" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/26/thumbs_b_c_b33b499750060e31c2aa102c9311b388.jpg</t>
+        </is>
+      </c>
+      <c r="I371" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>AAJI: POJK 36/2025 perkuat ekosistem asuransi kesehatan lebih optimal</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:20:06 +0700</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>Asosiasi Asuransi Jiwa Indonesia (AAJI) menilai penerapan Peraturan Otoritas Jasa Keuangan (POJK) Nomor 36 Tahun 2025 ...</t>
+        </is>
+      </c>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G372" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685532/aaji-pojk-36-2025-perkuat-ekosistem-asuransi-kesehatan-lebih-optimal</t>
+        </is>
+      </c>
+      <c r="H372" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000455789.jpg</t>
+        </is>
+      </c>
+      <c r="I372" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>Dubes Rwanda optimistis PTA dengan Indonesia rampung tahun ini</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:17:15 +0700</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>Duta Besar Rwanda untuk Indonesia Abdul Karim Harelimana optimistis negaranya dapat merampungkan Perjanjian Perdagangan ...</t>
+        </is>
+      </c>
+      <c r="F373" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G373" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685527/dubes-rwanda-optimistis-pta-dengan-indonesia-rampung-tahun-ini</t>
+        </is>
+      </c>
+      <c r="H373" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG_1951.jpg</t>
+        </is>
+      </c>
+      <c r="I373" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>Lebanon: Kemajuan dalam perundingan perbatasan, tawanan dengan Israel</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:13:12 +0700</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>Presiden Lebanon Joseph Aoun pada Jumat (7/8) mengatakan bahwa kemajuan telah dicapai dalam perundingan terbaru di ...</t>
+        </is>
+      </c>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685524/lebanon-kemajuan-dalam-perundingan-perbatasan-tawanan-dengan-israel</t>
+        </is>
+      </c>
+      <c r="H374" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/25/Joseph-Aoun-Presiden-Lebanon.jpg</t>
+        </is>
+      </c>
+      <c r="I374" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>MenPANRB: Berdayakan perempuan untuk transformasi digital inklusif</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:13:06 +0700</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>Menteri Pendayagunaan Aparatur Negara dan Reformasi Birokrasi (PANRB) Rini Widyantini menilai pemberdayaan perempuan di ...</t>
+        </is>
+      </c>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G375" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685523/menpanrb-berdayakan-perempuan-untuk-transformasi-digital-inklusif</t>
+        </is>
+      </c>
+      <c r="H375" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000582382_1.jpg</t>
+        </is>
+      </c>
+      <c r="I375" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>Diaspora Rwanda di Indonesia rayakan Umuganura, momentum bersyukur</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:12:07 +0700</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>Diaspora Rwanda di Indonesia pada Jumat malam merayakan Umuganura, atau Hari Panen Nasional, sebagai ungkapan syukur ...</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G376" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685520/diaspora-rwanda-di-indonesia-rayakan-umuganura-momentum-bersyukur</t>
+        </is>
+      </c>
+      <c r="H376" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG_1960.jpg</t>
+        </is>
+      </c>
+      <c r="I376" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>Komisi III DPR desak Polda Sumut usut kematian mantan istri polisi</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:08:24 +0700</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>Ketua Komisi III DPR RI Habiburokhman mendesak Polda Sumatera Utara dan Polresta Medan mengusut secara transparan kasus ...</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G377" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685519/komisi-iii-dpr-desak-polda-sumut-usut-kematian-mantan-istri-polisi</t>
+        </is>
+      </c>
+      <c r="H377" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/06/1001228042.jpg</t>
+        </is>
+      </c>
+      <c r="I377" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>Jubir PBB: UNICEF tindak staf terkait dugaan spionase untuk Israel</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:01:08 +0700</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>Dana Anak Perserikatan Bangsa-Bangsa (UNICEF) mengambil tindakan terhadap seorang staf terkait tuduhan bahwa ia ...</t>
+        </is>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685509/jubir-pbb-unicef-tindak-staf-terkait-dugaan-spionase-untuk-israel</t>
+        </is>
+      </c>
+      <c r="H378" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2013/07/20130705spionase.jpg</t>
+        </is>
+      </c>
+      <c r="I378" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>Polda kerahkan Tim Keslap dan DVI tangani kebakaran gedung Bapenda DKI</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:00:49 +0700</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>Bidang Kedokteran dan Kesehatan (Biddokkes) Polda Metro Jaya mengerahkan Tim Kesehatan Lapangan (Keslap) dan Tim ...</t>
+        </is>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G379" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685508/polda-kerahkan-tim-keslap-dan-dvi-tangani-kebakaran-gedung-bapenda-dki</t>
+        </is>
+      </c>
+      <c r="H379" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001017913.jpg</t>
+        </is>
+      </c>
+      <c r="I379" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>BPIP bekali Paskibraka HUT Ke-81 RI untuk jadi pemimpin bangsa</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:54:44 +0700</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>Badan Pembinaan Ideologi Pancasila (BPIP) membekali calon anggota Pasukan Pengibar Bendera Pusaka (Paskibraka) HUT ...</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G380" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685504/bpip-bekali-paskibraka-hut-ke-81-ri-untuk-jadi-pemimpin-bangsa</t>
+        </is>
+      </c>
+      <c r="H380" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000035089_1.jpg</t>
+        </is>
+      </c>
+      <c r="I380" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>Gubernur Jateng: Pencak silat ikut berperan perkuat persatuan</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:48:14 +0700</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>Gubernur Jawa Tengah Ahmad Luthfi menyebut pencak silat sebagai warisan budaya bangsa yang ikut berperan penting dalam ...</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G381" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685501/gubernur-jateng-pencak-silat-ikut-berperan-perkuat-persatuan</t>
+        </is>
+      </c>
+      <c r="H381" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG_20260808_120355.jpg</t>
+        </is>
+      </c>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>Pertamina ciptakan dampak ekonomi lebih luas lewat pembinaan UMKM</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:43:02 +0700</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>Vice President Corporate Communication PT Pertamina (Persero) Muhammad Baron mengatakan beragam program pembinaan UMKM ...</t>
+        </is>
+      </c>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G382" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685499/pertamina-ciptakan-dampak-ekonomi-lebih-luas-lewat-pembinaan-umkm</t>
+        </is>
+      </c>
+      <c r="H382" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000405362.jpg</t>
+        </is>
+      </c>
+      <c r="I382" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>Hal-hal yang perlu disiapkan sebelum ikut lelang mobil bekas</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:40:23 +0700</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/antaranewsdotcom</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>Mereka yang hendak mengikuti lelang mobil bekas disarankan untuk lebih dulu menyiapkan anggaran guna menghindari ...</t>
+        </is>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G383" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/berita/5685497/hal-hal-yang-perlu-disiapkan-sebelum-ikut-lelang-mobil-bekas</t>
+        </is>
+      </c>
+      <c r="H383" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000035086.jpg</t>
+        </is>
+      </c>
+      <c r="I383" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>Kena Dampak Kebakaran Gedung Bapenda, Sistem Lampu Lalin DKI Diatur Manual</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:22:00 +0700</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>Brigitta Belia Permata Sari</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>Pramono Anung mengungkapkan sistem pengaturan lalu lintas ikut terdampak kebakaran gedung Bapenda. Pengaturan kini dilakukan manual dengan penambahan personel.</t>
+        </is>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G384" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609765/kena-dampak-kebakaran-gedung-bapenda-sistem-lampu-lalin-dki-diatur-manual</t>
+        </is>
+      </c>
+      <c r="H384" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/potret-kobaran-api-mengamuk-di-gedung-bapenda-dki-1786160999187_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I384" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>Polisi Periksa Dokter Tangani Jasad Sutrimo Pekan Depan, Ini yang Akan Digali</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:19:55 +0700</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>Polda Metro Jaya selidiki kematian Sutrimo di klinik kecantikan. Dokter yang menangani jasad Sutirmo akan dipanggil ulang untuk klarifikasi kondisi korban.</t>
+        </is>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G385" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609762/polisi-periksa-dokter-tangani-jasad-sutrimo-pekan-depan-ini-yang-akan-digali</t>
+        </is>
+      </c>
+      <c r="H385" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/24/polda-metro-jaya-menggelar-konferensi-pers-terkait-tindak-pidana-perdagangan-orang-tppo-pmi-ilegal-ke-libya-1784892641761_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I385" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>Gedung Bapenda Terbakar, Pramono: Data Pajak Aman dan Layanan Tetap Jalan</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:00:15 +0700</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>Brigitta Belia Permata Sari</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>Kebakaran melanda Gedung Dinas Teknis Bapenda DKI Jakarta. Gubernur Pramono pastikan pelayanan publik tetap berjalan.</t>
+        </is>
+      </c>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G386" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609736/gedung-bapenda-terbakar-pramono-data-pajak-aman-dan-layanan-tetap-jalan</t>
+        </is>
+      </c>
+      <c r="H386" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/kondisi-gedung-bapenda-dki-usai-terbakar-1786154575590_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I386" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>Mendes Ajak Lulusan UIN SMH Banten Ciptakan Lapangan Kerja di Desa</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:51:03 +0700</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>Inkana Putri</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>Menteri Yandri Susanto mengajak lulusan UIN Banten untuk ciptakan lapangan kerja di desa. Program desa ekspor dan wisata jadi fokus dalam pembangunan ekonomi.</t>
+        </is>
+      </c>
+      <c r="F387" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G387" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609725/mendes-ajak-lulusan-uin-smh-banten-ciptakan-lapangan-kerja-di-desa</t>
+        </is>
+      </c>
+      <c r="H387" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/menteri-desa-dan-pembangunan-daerah-tertinggal-mendes-pdt-yandri-susanto-1786168240782.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I387" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>Gedung Bapenda DKI Kebakaran, 1.000 ASN Bakal Diatur WFH Bergantian</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:34:24 +0700</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>Brigitta Belia Permata Sari</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>Pemprov DKI Jakarta menyiapkan skema bekerja dari rumah (WFH) untuk sementara secara bergantian bagi sekitar 1.000 ASN imbas Gedung Bapenda terbakar.</t>
+        </is>
+      </c>
+      <c r="F388" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G388" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609709/gedung-bapenda-dki-kebakaran-1-000-asn-bakal-diatur-wfh-bergantian</t>
+        </is>
+      </c>
+      <c r="H388" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/potret-kobaran-api-mengamuk-di-gedung-bapenda-dki-1786160999187_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I388" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>Kondisi Terkini Ibunda Aldi Taher yang Berjuang Sembuh dari Stroke</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:06:34 +0700</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>Muhammad Ahsan Nurrijal</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>Kondisi ibunda Aldi Taher, Rosita Ramlis, menunjukkan kemajuan positif setelah stroke. Aldi rela jual rumah demi biaya pengobatan dan perawatan ibunya.</t>
+        </is>
+      </c>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G389" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8609750/kondisi-terkini-ibunda-aldi-taher-yang-berjuang-sembuh-dari-stroke</t>
+        </is>
+      </c>
+      <c r="H389" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/06/26/aldi-taher-1782431307830_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I389" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>Momen Manis DJ Icha Kharoline Dampingi Arief Catur Rayakan Persebaya Juara</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:13:22 +0700</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>Mauludi Rismoyo</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>DJ Icha Kharoline mendampingi Arief Catur Pamungkas yang sukses mengantarkan Persebaya Surabaya menjadi juara Piala Presiden 2026. Begini momennya.</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G390" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8609626/momen-manis-dj-icha-kharoline-dampingi-arief-catur-rayakan-persebaya-juara</t>
+        </is>
+      </c>
+      <c r="H390" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/dj-icha-kharoline-1786145590979_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>Pemain Timnas Indonesia Cekcok dengan Suporter: Thom Haye Singgung Wasit, Pattynama Ditampar Raven</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:17:14 +0700</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>Gagal ke semifinal Piala AFF 2026, pemain Timnas Indonesia sempat cekcok dengan suporter. Thom Haye singgung wasit, Pattynama nyaris terpancing.</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G391" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865703/pemain-timnas-indonesia-cekcok-dengan-suporter-thom-haye-singgung-wasit-pattynama-ditampar-raven</t>
+        </is>
+      </c>
+      <c r="H391" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/1qiX77kti7ELszzDNbFWWTntpfE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Timnas-Indonesia-Hadapi-Vietnam-di-Laga-Penyisihan-Piala-AFF-2026-1.jpg</t>
+        </is>
+      </c>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>BTN Perluas Akses KPR ke Penyandang Disabilitas untuk Kepemilikan Hunian</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:17:09 +0700</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>BTN memperluas akses pembiayaan perumahan yang inklusif ke seluruh lapisan masyarakat, termasuk penyandang disabilitas.</t>
+        </is>
+      </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G392" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/bisnis/7865702/btn-perluas-akses-kpr-ke-penyandang-disabilitas-untuk-kepemilikan-hunian</t>
+        </is>
+      </c>
+      <c r="H392" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ALX3PXiLKXhGZjSq6lOZB8BLbHY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Akad-massal-KPR-subsidi-OK.jpg</t>
+        </is>
+      </c>
+      <c r="I392" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>Jakarta Bhayangkara Presisi Goes to Polandia! Venue Kejuaraan Dunia Voli Antarklub 2026 Dirilis</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:06:17 +0700</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>Jakarta Bhayangkara Presisi siap debut di Kejuaraan Dunia Voli Antarklub FIVB 2026 yang akan berlangsung di Polandia pada 15 hingga 20 Desember.</t>
+        </is>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G393" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7865701/jakarta-bhayangkara-presisi-goes-to-polandia-venue-kejuaraan-dunia-voli-antarklub-2026-dirilis</t>
+        </is>
+      </c>
+      <c r="H393" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/w7ii5f4loWbbpMY-gqlNQnbluoo=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Bhayangkara-Presisi-AVC-keita-simon.jpg</t>
+        </is>
+      </c>
+      <c r="I393" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>Reshuffle Kabinet, Rumor Norman Joesoef Jadi Wamenhan Dinilai Tidak Jelas Urgensinya</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:05:34 +0700</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>Isu perombakan jajaran menteri kabinet merah putih belakangan ini kembali menjadi sorotan publik.</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G394" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865700/reshuffle-kabinet-rumor-norman-joesoef-jadi-wamenhan-dinilai-tidak-jelas-urgensinya</t>
+        </is>
+      </c>
+      <c r="H394" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/R-TKuXmu5-Ke0WQxzfaTjMF3ZKQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Reshuffle-Kabinet-Jilid-III-2025.jpg</t>
+        </is>
+      </c>
+      <c r="I394" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>Prakiraan Cuaca Madura Jawa Timur Minggu, 9 Agustus 2026: Seluruh Wilayah Cerah Berawan</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:03:37 +0700</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>Data prakiraan cuaca di wilayah Pulau Madura, Jawa Timur, untuk Minggu (9/8/2026) langit cerah berawan waktu yang tepat untuk pergi berwisata</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G395" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865699/prakiraan-cuaca-madura-jawa-timur-minggu-9-agustus-2026-seluruh-wilayah-cerah-berawan</t>
+        </is>
+      </c>
+      <c r="H395" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/8UZZmSJ0D8lU7RT62SK6xrzwyv8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/gili-iyang-tempat-yang-memiliki-udara-paling-bersih-di-pulau-sumenep.jpg</t>
+        </is>
+      </c>
+      <c r="I395" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>Sempat Laporkan Isa Zega atas Kasus Pencemaran Nama Baik, Shandy Purnamasari: Maafkan dan Ikhlaskan</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:58:56 +0700</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>Sempat melaporkan Isa Zega atas kasus pencemaran nama baik, Shandy Purnamasari akui sudah maafkan sang selebgram.</t>
+        </is>
+      </c>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G396" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7865698/sempat-laporkan-isa-zega-atas-kasus-pencemaran-nama-baik-shandy-purnamasari-maafkan-dan-ikhlaskan</t>
+        </is>
+      </c>
+      <c r="H396" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/WN2_p6-4qWfzGn6pMmdhUKcCJyI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Shandy-Purnamasari-beri-kesaksian-dalam-persidangan-kasus-pencemaran-nama-baik-Isa-Zega.jpg</t>
+        </is>
+      </c>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>Ruben Onsu Disebut Adopsi Bayi, Obat Rindu Tak Bisa Kumpul dengan 2 Putrinya</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:56:53 +0700</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>Sahabat Ruben Onsu, Aditya Gumay mengungkapkan sang presenter kini telah mengadopsi bayi untuk obat rindu kangen anak.</t>
+        </is>
+      </c>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G397" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7865697/ruben-onsu-disebut-adopsi-bayi-obat-rindu-tak-bisa-kumpul-dengan-2-putrinya</t>
+        </is>
+      </c>
+      <c r="H397" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ZG3_PDED1CjlCCKn-J5WB8tswOA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Ruben-Onsu-KPAI.jpg</t>
+        </is>
+      </c>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>Marcos Tjung Satukan 8 Penyanyi Lintas Generasi dalam Video Klip Warna Warni Indonesia</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:54:26 +0700</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>Kehadiran delapan penyanyi lintas generasi dengan karakter masing-masing, menjadi salah satu kekuatan dalam karya tersebut.</t>
+        </is>
+      </c>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G398" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7865696/marcos-tjung-satukan-8-penyanyi-lintas-generasi-dalam-video-klip-warna-warni-indonesia</t>
+        </is>
+      </c>
+      <c r="H398" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ueocreIhMT5TYah22LHryMDEPT4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Marcos-Tjung-1-08082026.jpg</t>
+        </is>
+      </c>
+      <c r="I398" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>Wapres Gibran Tinjau Pasca-bencana di Aceh: Normalisasi Sungai Lebih Mahal dari Membangun Jembatan</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:52:30 +0700</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>Wapres Gibran tinjauan pasca bencana di Provinsi Aceh yakni pembangunan Jembatan Gantung Kendawi, Kabupaten Gayo Lues, Kamis (06/8/2026).</t>
+        </is>
+      </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G399" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865695/wapres-gibran-tinjau-pasca-bencana-di-aceh-normalisasi-sungai-lebih-mahal-dari-membangun-jembatan</t>
+        </is>
+      </c>
+      <c r="H399" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Ofg7oFVDORWWt-nzILuGJF0PyIg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/gibran-di-gayo-luwes.jpg</t>
+        </is>
+      </c>
+      <c r="I399" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>Hari Pramuka 2026 Jatuh pada Tanggal Berapa? Cek Jadwalnya di Sini</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:49:20 +0700</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>Hari Pramuka diperingati setiap 14 Agustus dan pada 2026 memasuki peringatan ke-65.</t>
+        </is>
+      </c>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G400" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865694/hari-pramuka-2026-jatuh-pada-tanggal-berapa-cek-jadwalnya-di-sini</t>
+        </is>
+      </c>
+      <c r="H400" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Anbh98FNk4CAGrKXCe1buHCDKaU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Logo-Hari-Pramuka-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I400" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>Kasus Fraud Dana Syariah Indonesia Dilimpahkan ke Kejaksaan, Bareskrim Sita Aset Rp 425 Miliar</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:48:22 +0700</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>Berkas perkara kedua dengan tersangka AS, eks Direktur PT DSI, telah dinyatakan lengkap atau P21 oleh Jaksa Penuntut Umum (JPU).</t>
+        </is>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G401" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865693/kasus-fraud-dana-syariah-indonesia-dilimpahkan-ke-kejaksaan-bareskrim-sita-aset-rp-425-miliar</t>
+        </is>
+      </c>
+      <c r="H401" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/-crZsm7zBOdBqsmI3pYpMRxgoug=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/fraud-dsi-nihhhhh.jpg</t>
+        </is>
+      </c>
+      <c r="I401" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>Timnas Indonesia Gagal Lolos Semifinal Piala AFF 2 Kali Beruntun, Ulangi Kisah Kelam 12 Tahun Silam</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:48:17 +0700</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>Gagal ke semifinal Piala AFF 2026, Timnas Indonesia mengulang kisah kelam 12 tahun silam saat juga tersingkir di fase grup dua edisi beruntun.</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G402" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865692/timnas-indonesia-gagal-lolos-semifinal-piala-aff-2-kali-beruntun-ulangi-kisah-kelam-12-tahun-silam</t>
+        </is>
+      </c>
+      <c r="H402" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/1a7ILPPDpySjbwe7SeQea4Z15Rg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Timnas-Indonesia-Dicukur-Timnas-Vietnam-3-0_20260804_065849.jpg</t>
+        </is>
+      </c>
+      <c r="I402" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>Perkuat Manajemen Risiko, Lembaga Penggerak Ekonomi MUI Gelar Pelatihan SDM</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:47:20 +0700</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>Tuntutan masyarakat terhadap transparansi dan akuntabilitas juga telah mengubah cara organisasi dikelola.</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865691/perkuat-manajemen-risiko-lembaga-penggerak-ekonomi-mui-gelar-pelatihan-sdm</t>
+        </is>
+      </c>
+      <c r="H403" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/i_QSfbkTGu1I0nCojuxmN6NdvO8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Risiko-Asosiasi-Energi-Indone.jpg</t>
+        </is>
+      </c>
+      <c r="I403" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>MGBKI Tak Setuju Wacana Cabut STR Dokter Usai Komentar Negatif Curhat Yurizal Viral</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:41:58 +0700</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>MGBKI menilai penyelesaian terhadap dugaan pelanggaran etika dokter harus dilakukan melalui mekanisme profesi yang berlaku, bukan penghakiman publik.</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G404" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865690/mgbki-tak-setuju-wacana-cabut-str-dokter-usai-komentar-negatif-curhat-yurizal-viral</t>
+        </is>
+      </c>
+      <c r="H404" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/mKiK7DSnd0Cxme8GVosRxLtbQdw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Sosok-Yurizal-Tri-Chaerawan.jpg</t>
+        </is>
+      </c>
+      <c r="I404" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>Terjemahan Lirik Lagu Proof - Paramore: It's Really Hard, I Can't Cry in Your Arms</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:35:06 +0700</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>Berikut ini merupakan terjemahan lirik lagu Proof yang dipopulerkan oleh grup band asal Franklin, Paramore.</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G405" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/musik/7865689/terjemahan-lirik-lagu-proof-paramore-its-really-hard-i-cant-cry-in-your-arms</t>
+        </is>
+      </c>
+      <c r="H405" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/zLN77GXG_MWcQ27NDqNvGgp-QJs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-musik-ilustrasi-lirik-ilustrasi-terjemahan-lirik-lagu.jpg</t>
+        </is>
+      </c>
+      <c r="I405" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>Toyota Sudah Kantongi SPK bZ4X Touring yang Mendebut di GIIAS 2026</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:33:32 +0700</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>Toyota sudah mengantongi surat pemesanan kendaraan (SPK) untuk mobil listrik baru Toyota bZ4X Touring yang pertama kali tampil di GIIAS 2026.</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G406" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/otomotif/7865688/toyota-sudah-kantongi-spk-bz4x-touring-yang-mendebut-di-giias-2026</t>
+        </is>
+      </c>
+      <c r="H406" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/2jnNJmtFVpigwCyhYuIL4FFsnH8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Hiroyuki-Oide-dan-Toyota-bZ4X-BEV-di-GIIAS-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I406" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>MBG Dipisah Paling Lambat 2028, Guru Besar UGM: MK Seperti Pemberi Nasehat, Bukan Lembaga Peradilan</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:31:06 +0700</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>Dosen Departemen Hukum Tata Negara di FH UGM ini mempertanyakan, mengapa MK tidak secara tegas memberlakukannya mulai APBN Tahun 2027 saja.</t>
+        </is>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G407" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865687/mbg-dipisah-paling-lambat-2028-guru-besar-ugm-mk-seperti-pemberi-nasehat-bukan-lembaga-peradilan</t>
+        </is>
+      </c>
+      <c r="H407" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Kxy0Y85qxTHxMbNcepFDroLjqqk=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/food-tray-mbg-2kf.jpg</t>
+        </is>
+      </c>
+      <c r="I407" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>Beasiswa BPI GTK 2026 Resmi Dibuka, Cek Kriteria Penerima, Cara Daftar dan Besaran Bantuan</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:28:57 +0700</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>BPI GTK 2026 resmi dibuka untuk calon guru dan guru jenjang D4/S1 dengan dua skema penerima.</t>
+        </is>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G408" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/pendidikan/7865686/beasiswa-bpi-gtk-2026-resmi-dibuka-cek-kriteria-penerima-cara-daftar-dan-besaran-bantuan</t>
+        </is>
+      </c>
+      <c r="H408" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Opo9c_38iz7LvELT4Bzv2snwTtk=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Beasiswa-BPI-GTK-2026-Resmi-Dibuka.jpg</t>
+        </is>
+      </c>
+      <c r="I408" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>Piala AFF 2026 Gagal Lagi, Penantian 30 Tahun Timnas Indonesia untuk Juara Kembali Berlanjut</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:28:12 +0700</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>Gagal di Piala AFF 2026 membuat penantian Timnas Indonesia untuk meraih gelar juara berlanjut. Skuad Garuda sudah 30 tahun belum pernah juara.</t>
+        </is>
+      </c>
+      <c r="F409" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G409" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865685/piala-aff-2026-gagal-lagi-penantian-30-tahun-timnas-indonesia-untuk-juara-kembali-berlanjut</t>
+        </is>
+      </c>
+      <c r="H409" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/XnwHrLgh_9fjfJVEBcVvY288K5U=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Skuad-Timnas-Indonesia-berdiskusi-bersama-sebelum-pertandingan-melawan-Vietnam.jpg</t>
+        </is>
+      </c>
+      <c r="I409" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>Naskah Ulang Janji Peringatan Hari Pramuka ke-65 Tahun 2026</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:27:33 +0700</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>Simak naskah ulang janji pada malam peringatan Hari Pramuka ke-65 tahun 2026 yang dilaksanakan pada Kamis, 13 Agustus 2026 malam.</t>
+        </is>
+      </c>
+      <c r="F410" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G410" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865684/naskah-ulang-janji-peringatan-hari-pramuka-ke-65-tahun-2026</t>
+        </is>
+      </c>
+      <c r="H410" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/K7Yjmd2gqaw9H9cqvw4s7ZyaXtc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Naskah-Ulang-Janji-Peringatan-Hari-Pramuka-ke-64-Tahun-2025.jpg</t>
+        </is>
+      </c>
+      <c r="I410" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>Pertanian</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>Danantara Tanam Investasi 2,5 Miliar Dolar AS ke Raksasa Produsen Daging Asal Brasil</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:15:00 +0700</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>Ahmad Fikri Noor</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA - Danantara Indonesia melalui Danantara Investment Management (DIM) menjalin kemitraan strategis jangka panjang dengan produsen daging global terkemuka asal Brasil, JBS Group. Hal ini sebagai upaya mendorong pengembangan...</t>
+        </is>
+      </c>
+      <c r="F411" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G411" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjfq79490/danantara-tanam-investasi-25-miliar-dolar-as-ke-raksasa-produsen-daging-asal-brasil</t>
+        </is>
+      </c>
+      <c r="H411" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/030113600-1763569982-830-556.jpg</t>
+        </is>
+      </c>
+      <c r="I411" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>Damkar Ungkap Pemadaman Gedung Bapenda Butuh Waktu Lama</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:11:15 +0700</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>Petugas ternyata masih menyisir lantai atas setelah api berhasil dipadamkan.</t>
+        </is>
+      </c>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G412" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8264992/damkar-ungkap-pemadaman-gedung-bapenda-butuh-waktu-lama</t>
+        </is>
+      </c>
+      <c r="H412" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/zfq5G_jONactwf5HoU4x7_ES33A=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9318688/original/051146900_1786132547-IMG_3450.jpg</t>
+        </is>
+      </c>
+      <c r="I412" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>Kebakaran Gedung Bapenda DKI, Petugas Sisir Lantai 11-16</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:50:59 +0700</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>Api sudah padam, tetapi petugas masih mencari titik panas tersisa.</t>
+        </is>
+      </c>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G413" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8264972/kebakaran-gedung-bapenda-dki-petugas-sisir-lantai-11-16</t>
+        </is>
+      </c>
+      <c r="H413" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/45x5fM3ErEdVhAno4tHEAYUUDR4=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9318748/original/078691900_1786155435-IMG_20260808_082636_225.jpg</t>
+        </is>
+      </c>
+      <c r="I413" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>Sejumlah Warga di Wonosobo Baru Terima ATM PKH, padahal Bantuan Telah Berjalan Sejak 2018</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:34:53 +0700</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>Sejumlah KPM di Wonosobo baru menerima atau menguasai kartu ATM PKH pada tahun 2026, padahal program tersebut telah berjalan sejak 2018</t>
+        </is>
+      </c>
+      <c r="F414" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G414" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/08/08/133035678/sejumlah-warga-di-wonosobo-baru-terima-atm-pkh-padahal-bantuan-telah</t>
+        </is>
+      </c>
+      <c r="H414" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/SsNXgPKRYi0yg_Ej14m1x_XHuNw=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/08/6a76964d5c2f8.jpg</t>
+        </is>
+      </c>
+      <c r="I414" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>Otomotif</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>Daihatsu Masih Pantau Pasar, Mobil Listrik Belum Prioritas?</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:34:53 +0700</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>Daihatsu saat ini masih melihat produk yang tersedia mampu memenuhi kebutuhan konsumen.</t>
+        </is>
+      </c>
+      <c r="F415" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G415" t="inlineStr">
+        <is>
+          <t>https://otomotif.kompas.com/read/2026/08/08/130200815/daihatsu-masih-pantau-pasar-mobil-listrik-belum-prioritas-</t>
+        </is>
+      </c>
+      <c r="H415" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/Hm8kS9aOliJ_oqYpBB0Cq3p_Qn8=/55x78:1229x861/1200x675/filters:watermark(data/photo/2026/01/30/697c81750a668.png,0,-0,1)/data/photo/2026/08/02/6a6e684716845.jpeg</t>
+        </is>
+      </c>
+      <c r="I415" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>Dua Dekade Pusat Grosir Solo: Dari Masa Keemasan, Badai Pandemi hingga Hantaman Pailit</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:34:53 +0700</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>Dua dekade lebih membersamai geliat perdagangan dan pariwisata Kota Solo, PGS kini resmi pamit menjadi bagian dari sejarah kota.</t>
+        </is>
+      </c>
+      <c r="F416" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G416" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/08/08/123300778/dua-dekade-pusat-grosir-solo--dari-masa-keemasan-badai-pandemi-hingga</t>
+        </is>
+      </c>
+      <c r="H416" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/hrl2qZ_usgI3UOG-bwiLIvJYRKg=/0x0:1280x853/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/05/6a730e210db76.jpg</t>
+        </is>
+      </c>
+      <c r="I416" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I366"/>
+  <autoFilter ref="A1:I416"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-08 07:44 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-08.xlsx
+++ b/data/berita_2026-08-08.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$416</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$489</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I416"/>
+  <dimension ref="A1:I489"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -19986,8 +19986,3440 @@
         </is>
       </c>
     </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>Akhir Agustus, 100 Sekolah Rakyat beroperasi di seluruh Indonesia</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:38:07 +0700</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>Sekretaris Kabinet Teddy Indra Wijaya mengungkapkan bahwa pada akhir Agustus 2026 atau setelah perayaan Hari ...</t>
+        </is>
+      </c>
+      <c r="F417" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G417" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685615/akhir-agustus-100-sekolah-rakyat-beroperasi-di-seluruh-indonesia</t>
+        </is>
+      </c>
+      <c r="H417" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000454906.jpg</t>
+        </is>
+      </c>
+      <c r="I417" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>BPK: Terapkan ESG-Government 5.0 perkuat tata kelola keuangan negara</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:32:47 +0700</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>Badan Pemeriksa Keuangan (BPK) mendorong penerapan prinsip Environmental, Social, and Governance (ESG) dan Government ...</t>
+        </is>
+      </c>
+      <c r="F418" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G418" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685612/bpk-terapkan-esg-government-50-perkuat-tata-kelola-keuangan-negara</t>
+        </is>
+      </c>
+      <c r="H418" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2024/06/20/1000062571.jpg</t>
+        </is>
+      </c>
+      <c r="I418" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>BMKG sebut penguatan monsun picu gelombang tinggi di NTB</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:31:23 +0700</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>Badan Meteorologi, Klimatologi, dan Geofisika (BMKG) menyebut monsun Australia yang membawa angin timuran menjadi salah ...</t>
+        </is>
+      </c>
+      <c r="F419" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G419" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685608/bmkg-sebut-penguatan-monsun-picu-gelombang-tinggi-di-ntb</t>
+        </is>
+      </c>
+      <c r="H419" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001442657.jpg</t>
+        </is>
+      </c>
+      <c r="I419" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>Pengukuhan Paskibraka di Istana dijadwalkan 15 Agustus</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:26:57 +0700</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>Badan Pembinaan Ideologi Pancasila (BPIP) menyebut pengukuhan Pasukan Pengibar Bendera Pusaka (Paskibraka) untuk ...</t>
+        </is>
+      </c>
+      <c r="F420" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G420" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685607/pengukuhan-paskibraka-di-istana-dijadwalkan-15-agustus</t>
+        </is>
+      </c>
+      <c r="H420" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000035101.jpg</t>
+        </is>
+      </c>
+      <c r="I420" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>Kemensos targetkan 150 ribu siswa masuk Sekolah Rakyat pada 2027</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:26:00 +0700</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>Pemerintah melalui Kementerian Sosial (Kemensos) menargetkan lebih dari 150 ribu siswa dari kota/kabupaten di Indonesia ...</t>
+        </is>
+      </c>
+      <c r="F421" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G421" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685604/kemensos-targetkan-150-ribu-siswa-masuk-sekolah-rakyat-pada-2027</t>
+        </is>
+      </c>
+      <c r="H421" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000454901.jpg</t>
+        </is>
+      </c>
+      <c r="I421" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>Pengamat: Relawan-parpol harus perkuat sosialisasi program Presiden</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:25:01 +0700</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>Pengamat politik Arfianto Purbolaksono menilai jaringan relawan dan partai politik pendukung Presiden Prabowo Subianto ...</t>
+        </is>
+      </c>
+      <c r="F422" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G422" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685600/pengamat-relawan-parpol-harus-perkuat-sosialisasi-program-presiden</t>
+        </is>
+      </c>
+      <c r="H422" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2024/11/15/WhatsApp-Image-2023-06-14-at-20.17.06-1_1.jpg</t>
+        </is>
+      </c>
+      <c r="I422" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>DK PBB kecam serangan Houthi dan pelanggaran wilayah Yaman</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:22:27 +0700</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>Dewan Keamanan Perserikatan Bangsa-Bangsa (DK PBB) mengecam serangan rudal kelompok Houthi Yaman terhadap Arab Saudi ...</t>
+        </is>
+      </c>
+      <c r="F423" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G423" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685596/dk-pbb-kecam-serangan-houthi-dan-pelanggaran-wilayah-yaman</t>
+        </is>
+      </c>
+      <c r="H423" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/24/ilustrasi-rapat-Dewan-Keamanan-PBB-DK-PBB_1.jpg</t>
+        </is>
+      </c>
+      <c r="I423" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>Muzani: Qanun Asasi NU jadi landasan menjaga keutuhan negara</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:21:47 +0700</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>Ketua MPR RI Ahmad Muzani menilai Qanun Asasi Nahdlatul Ulama (NU) menjadi landasan pemikiran organisasi dalam menjaga ...</t>
+        </is>
+      </c>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G424" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685593/muzani-qanun-asasi-nu-jadi-landasan-menjaga-keutuhan-negara</t>
+        </is>
+      </c>
+      <c r="H424" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001225255.jpg</t>
+        </is>
+      </c>
+      <c r="I424" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>Perawat Indonesia buka jalur baru karier di rumah sakit Malaysia</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:17:57 +0700</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>Konsulat Jenderal Republik Indonesia (KJRI) Johor Bahru menyampaikan bahwa 12 perawat asal Indonesia untuk pertama ...</t>
+        </is>
+      </c>
+      <c r="F425" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G425" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685589/perawat-indonesia-buka-jalur-baru-karier-di-rumah-sakit-malaysia</t>
+        </is>
+      </c>
+      <c r="H425" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001044869.jpg</t>
+        </is>
+      </c>
+      <c r="I425" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>Adang Daradjatun minta polisi transparan usut temuan ratusan senjata</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:17:04 +0700</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>Anggota Komisi III DPR RI Adang Daradjatun meminta Kepolisian mengusut secara transparan temuan ratusan senjata di ...</t>
+        </is>
+      </c>
+      <c r="F426" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G426" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685587/adang-daradjatun-minta-polisi-transparan-usut-temuan-ratusan-senjata</t>
+        </is>
+      </c>
+      <c r="H426" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001017729.jpg</t>
+        </is>
+      </c>
+      <c r="I426" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>ASN yang bertugas di gedung Bapenda boleh WFH secara bergantian</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:12:30 +0700</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>Pemerintah Provinsi DKI Jakarta menginstruksikan aparatur sipil negara (ASN) di gedung Badan Pendapatan Daerah ...</t>
+        </is>
+      </c>
+      <c r="F427" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G427" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685583/asn-yang-bertugas-di-gedung-bapenda-boleh-wfh-secara-bergantian</t>
+        </is>
+      </c>
+      <c r="H427" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001018108.jpg</t>
+        </is>
+      </c>
+      <c r="I427" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>Meksiko, Brasil pererat hubungan di tengah ketegangan Lula dan Trump</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:07:56 +0700</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>Meksiko dan Brasil sepakat memperdalam kerja sama di bidang perdagangan, energi, serta urusan multilateral dalam ...</t>
+        </is>
+      </c>
+      <c r="F428" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G428" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685576/meksiko-brasil-pererat-hubungan-di-tengah-ketegangan-lula-dan-trump</t>
+        </is>
+      </c>
+      <c r="H428" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/20/thumbs_b_c_0bbb35c4ff9cd2585c631f33a3b87a0a.jpg</t>
+        </is>
+      </c>
+      <c r="I428" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>BPIP tekankan pembentukan karakter dalam pendidikan Paskibraka</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:04:11 +0700</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>Badan Pembinaan Ideologi Pancasila (BPIP) menekankan pembentukan karakter dalam pendidikan Pasukan Pengibar Bendera ...</t>
+        </is>
+      </c>
+      <c r="F429" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G429" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685573/bpip-tekankan-pembentukan-karakter-dalam-pendidikan-paskibraka</t>
+        </is>
+      </c>
+      <c r="H429" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000035098.jpg</t>
+        </is>
+      </c>
+      <c r="I429" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>Itauma tanggapi status duel lawan Hrgovic jadi perebutan juara IBF</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:56:37 +0700</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>Petinju Moses Itauma menanggapi status duelnya melawan Filip Hrgovic dinaikkan menjadi perebutan gelar juara dunia ...</t>
+        </is>
+      </c>
+      <c r="F430" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G430" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685569/itauma-tanggapi-status-duel-lawan-hrgovic-jadi-perebutan-juara-ibf</t>
+        </is>
+      </c>
+      <c r="H430" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG_20260808_133429.jpg</t>
+        </is>
+      </c>
+      <c r="I430" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>Borneo Forum 2026 desak Pemerintah pangkas birokrasi replanting sawit</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:51:32 +0700</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>Borneo Forum 2026 mendesak pemerintah memangkas birokrasi Program Peremajaan Sawit Rakyat (PSR), menyusul sorotan tajam ...</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G431" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685568/borneo-forum-2026-desak-pemerintah-pangkas-birokrasi-replanting-sawit</t>
+        </is>
+      </c>
+      <c r="H431" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG_3678.jpeg</t>
+        </is>
+      </c>
+      <c r="I431" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>AS perkuat hubungan pertahanan dengan negara di Asia Tenggara</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:50:43 +0700</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>Wakil Menteri Perang AS untuk Kebijakan Elbridge Colby dan Asisten Menteri Perang AS untuk Keamanan Indo-Pasifik John ...</t>
+        </is>
+      </c>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G432" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685567/as-perkuat-hubungan-pertahanan-dengan-negara-di-asia-tenggara</t>
+        </is>
+      </c>
+      <c r="H432" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/30/AmerikaSerikatBenderaPixabay.jpg</t>
+        </is>
+      </c>
+      <c r="I432" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>Festival Lembutan jadi wadah memperluas pasar tembakau Temanggung</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:45:36 +0700</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>ANTARA -Festival Lembutan menjadi wadah untuk memperkenalkan, sekaligus memperluas pasar tembakau khas Temanggung, Jawa ...</t>
+        </is>
+      </c>
+      <c r="F433" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G433" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5685528/festival-lembutan-jadi-wadah-memperluas-pasar-tembakau-temanggung</t>
+        </is>
+      </c>
+      <c r="H433" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AYM_OKFESTIVAL-LEMBUTAN-JADI-WADAH-MEMPERLUAS-PASAR.jpg</t>
+        </is>
+      </c>
+      <c r="I433" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>AS nyatakan perang besar terhadap kartel, target pertama CJNG</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:43:37 +0700</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>Amerika Serikat perlu memulai perang besar melawan kartel dan target pertamanya adalah Kartel Jalisco New Generation ...</t>
+        </is>
+      </c>
+      <c r="F434" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G434" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685559/as-nyatakan-perang-besar-terhadap-kartel-target-pertama-cjng</t>
+        </is>
+      </c>
+      <c r="H434" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/16/XxjpbeE000336_20260615_PEPFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I434" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>Mendag dorong RI-India perkuat akses pasar dan investasi</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:41:00 +0700</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>Menteri Perdagangan (Mendag) RI Budi Santoso dan Menteri Perdagangan dan Industri India Piyush Goyal membahas penguatan ...</t>
+        </is>
+      </c>
+      <c r="F435" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G435" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685556/mendag-dorong-ri-india-perkuat-akses-pasar-dan-investasi</t>
+        </is>
+      </c>
+      <c r="H435" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG_3708.jpeg</t>
+        </is>
+      </c>
+      <c r="I435" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>Media preview Teater Nadirah</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:39:12 +0700</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>Seniman teater dari Alumni Kelas Aktor Salihara (AKSARA) mementaskan pertunjukan teater berjudul Nadirah saat media ...</t>
+        </is>
+      </c>
+      <c r="F436" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G436" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5685553/media-preview-teater-nadirah</t>
+        </is>
+      </c>
+      <c r="H436" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/Media-preview-teater-Nadirah-07082026-ab-3.jpg</t>
+        </is>
+      </c>
+      <c r="I436" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>Jenderal AS dorong Trump akhiri konflik dengan Iran</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:38:16 +0700</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>Ketua Kepala Staf Gabungan Amerika Serikat Jenderal Dan Caine selama beberapa pekan terakhir mendesak Gedung Putih ...</t>
+        </is>
+      </c>
+      <c r="F437" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G437" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685552/jenderal-as-dorong-trump-akhiri-konflik-dengan-iran</t>
+        </is>
+      </c>
+      <c r="H437" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/30/IranASBenderaAnadolu_py_am.jpg</t>
+        </is>
+      </c>
+      <c r="I437" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>OpenAI memperlambat pengembangan model Astra</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:34:32 +0700</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>Perusahaan kecerdasan artifisial OpenAI menangguhkan pengerjaan beberapa aspek dari model kecerdasan buatan ...</t>
+        </is>
+      </c>
+      <c r="F438" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G438" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685551/openai-memperlambat-pengembangan-model-astra</t>
+        </is>
+      </c>
+      <c r="H438" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2024/10/09/Clipboard_10-09-2024_04.jpg</t>
+        </is>
+      </c>
+      <c r="I438" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>AS dan Meksiko buru pemimpin kartel Jalisco New Generation</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:33:57 +0700</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>Amerika Serikat akan bekerja sama dengan Meksiko untuk memburu para pemimpin dan rekanan Kartel Jalisco New Generation ...</t>
+        </is>
+      </c>
+      <c r="F439" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G439" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685547/as-dan-meksiko-buru-pemimpin-kartel-jalisco-new-generation</t>
+        </is>
+      </c>
+      <c r="H439" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/02/23/2MOqhOqqHwXgUieJ_1.jpg</t>
+        </is>
+      </c>
+      <c r="I439" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>Kemenbud Raih Opini WTP dari BPK RI atas Laporan Keuangan TA 2025</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:31:13 +0700</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>Inkana Putri</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>Kemenbud RI meraih opini WTP dari BPK, menegaskan akuntabilitas keuangan yang baik. Menteri Fadli Zon berkomitmen untuk terus memperbaiki tata kelola.</t>
+        </is>
+      </c>
+      <c r="F440" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G440" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609837/kemenbud-raih-opini-wtp-dari-bpk-ri-atas-laporan-keuangan-ta-2025</t>
+        </is>
+      </c>
+      <c r="H440" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/kemenbud-raih-opini-wtp-dari-bpk-ri-atas-laporan-keuangan-ta-2025-1786174252253.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I440" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>Seskab Dorong Anak Putus Sekolah Berani Bermimpi Besar di Sekolah Rakyat</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:28:23 +0700</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>Fara Difa Alfeni</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>Sekretaris Kabinet Letkol Teddy mendorong anak putus sekolah untuk kembali belajar di Sekolah Rakyat. Program ini mendukung pendidikan bagi semua anak Indonesia</t>
+        </is>
+      </c>
+      <c r="F441" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G441" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609836/seskab-dorong-anak-putus-sekolah-berani-bermimpi-besar-di-sekolah-rakyat</t>
+        </is>
+      </c>
+      <c r="H441" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/seskab-teddy-dorong-anak-putus-sekolah-berani-bermimpi-besar-di-sekolah-rakyat-1786174078020.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I441" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>Bocah 10 Tahun di Lampung Tewas Diduga Tergantung Saat Main Ayunan</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:22:51 +0700</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>Tommy Saputra</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>Bocah 10 tahun di Lampung Utara ditemukan tewas tergantung di pohon saat bermain. Polisi menduga korban terjerat tali ayunan.</t>
+        </is>
+      </c>
+      <c r="F442" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G442" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609833/bocah-10-tahun-di-lampung-tewas-diduga-tergantung-saat-main-ayunan</t>
+        </is>
+      </c>
+      <c r="H442" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/polisi-mendatangi-olah-tkp-anak-10-tahun-tewas-tergantung-ayunan-1786162618411_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I442" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>Polda Metro-Kodam Jaya Gelar Bakti Kesehatan di Monas, Layani 1.876 Warga</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:22:16 +0700</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>Polda Metro Jaya dan Kodam Jaya menggelar Bakti Kesehatan di Monas, melayani 1.876 warga dengan berbagai layanan medis. Sinergi untuk masyarakat!</t>
+        </is>
+      </c>
+      <c r="F443" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G443" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609831/polda-metro-kodam-jaya-gelar-bakti-kesehatan-di-monas-layani-1-876-warga</t>
+        </is>
+      </c>
+      <c r="H443" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/polda-metro-dan-kasdam-jaya-menggelar-bakti-kesehatan-di-monas-1786173694248_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I443" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>KPK Bawa 3 Koper Usai Geledah Rumah Sekwan DPRD Kota Bengkulu</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:11:58 +0700</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>Heri Supandi</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>KPK menggeledah rumah Sekwan Kota Bengkulu, SF. Penyidik membawa tiga koper diduga berisi barang bukti.</t>
+        </is>
+      </c>
+      <c r="F444" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G444" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609823/kpk-bawa-3-koper-usai-geledah-rumah-sekwan-dprd-kota-bengkulu</t>
+        </is>
+      </c>
+      <c r="H444" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/kpk-bawa-koper-setelah-menggeledah-rumah-sekwan-dprd-kota-bengkulu-1786118577033_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I444" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>2 Hal Ini Diusut Polisi Terkait Temuan Senjata di Sekolah Jaksel</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:10:53 +0700</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>Polda Metro Jaya menyelidiki temuan 995 senjata angin di sekolah swasta Jakarta. Mantan ketua yayasan akan dipanggil untuk klarifikasi izin impor.</t>
+        </is>
+      </c>
+      <c r="F445" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G445" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609821/2-hal-ini-diusut-polisi-terkait-temuan-senjata-di-sekolah-jaksel</t>
+        </is>
+      </c>
+      <c r="H445" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/temuan-ratusan-pucuk-senjata-di-sekolah-swasta-di-pondok-pinang-jakarta-selatan-1786014363566_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I445" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>MPR Kirim Undangan Sidang Tahunan ke Presiden-Wapres Terdahulu Mulai Senin</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:41:45 +0700</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>Adrial akbar</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>MPR RI akan mengirimkan undangan sidang tahunan MPR serta sidang bersama DPR dan DPD RI kepada presiden dan wakil presiden terdahulu mulai Senin.</t>
+        </is>
+      </c>
+      <c r="F446" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G446" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609783/mpr-kirim-undangan-sidang-tahunan-ke-presiden-wapres-terdahulu-mulai-senin</t>
+        </is>
+      </c>
+      <c r="H446" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/ketua-mpr-ahmad-muzani-1786171279051_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I446" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>Truk Rem Blong Tabrak Motor di Nanggung Bogor, Pengemudi dan Penumpang Tewas</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:38:39 +0700</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>Rizky Adha Mahendra</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>Truk tabrak pengendara motor hingga masuk ke dalam jurang di Bogor. Pengemudi dan penumpang motor tewas.</t>
+        </is>
+      </c>
+      <c r="F447" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G447" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609780/truk-rem-blong-tabrak-motor-di-nanggung-bogor-pengemudi-dan-penumpang-tewas</t>
+        </is>
+      </c>
+      <c r="H447" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/05/02/ilustrasi-kecelakaan-1777698723734_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I447" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>MenterI LH Bakal Tindak Penebangan Pohon Depan Lapangan Padel Bandung: Barbar!</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:30:49 +0700</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>Rizky Adha Mahendra</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>Menteri LH Jumhur Hidayat mengecam penebangan 10 pohon ilegal di Bandung. Ia menegaskan tindakan tersebut tidak boleh dilakukan dan sedang diselidiki.</t>
+        </is>
+      </c>
+      <c r="F448" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G448" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609774/menteri-lh-bakal-tindak-penebangan-pohon-depan-lapangan-padel-bandung-barbar</t>
+        </is>
+      </c>
+      <c r="H448" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/07/menteri-lingkungan-hidup-jumhur-hidayat-seusai-melakukan-penanaman-mangrove-di-desa-labuhan-alas-kecamatan-alas-kabupaten-sumb-1783428053298_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I448" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>Ini Dugaan Sumber Kebakaran 176 Hektare Lahan di Gunung Bromo</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:29:57 +0700</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>M Rofiq</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>Kebakaran lahan di Gunung Bromo melanda 176 hektare, diduga akibat perapian warga.</t>
+        </is>
+      </c>
+      <c r="F449" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G449" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609773/ini-dugaan-sumber-kebakaran-176-hektare-lahan-di-gunung-bromo</t>
+        </is>
+      </c>
+      <c r="H449" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/drone-water-spray-turut-dikerahkan-untuk-memadamkan-api-kebakaran-hutan-di-bromo-1786098040220_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I449" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>Menteri LH hingga Wamendagri Hadiri Milangkala Majelis Musyawarah Sunda</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:28:33 +0700</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>Rizky Adha Mahendra</t>
+        </is>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t>Menteri LH Jumhur Hidayat menekankan pentingnya kearifan lokal dalam pembangunan saat menghadiri Milangkala MMS. Acara ini juga dihadiri tokoh masyarakat Sunda.</t>
+        </is>
+      </c>
+      <c r="F450" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G450" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609770/menteri-lh-hingga-wamendagri-hadiri-milangkala-majelis-musyawarah-sunda</t>
+        </is>
+      </c>
+      <c r="H450" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/milangkala-majelis-musyawarah-sunda-1786170471140_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I450" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>Jurus RI Bidik Pasar Karbon hingga Perdagangan Global dari Sektor Kehutanan</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:16:37 +0700</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>Fadhly Fauzi Rachman</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>Kemenhut memperkuat SDM untuk negosiasi internasional melalui pelatihan. Fokus pada perdagangan hasil hutan, pasar karbon, dan pengelolaan hutan global.</t>
+        </is>
+      </c>
+      <c r="F451" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G451" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/ekonomi-hijau/d-8609826/jurus-ri-bidik-pasar-karbon-hingga-perdagangan-global-dari-sektor-kehutanan</t>
+        </is>
+      </c>
+      <c r="H451" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2016/05/23/229dbf9d-4f13-411c-b23b-515bdafc0511_169.jpg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I451" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>Butuh Rp 150 M Benahi Gunungan Sampah Bantar Gebang</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:00:44 +0700</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>Aulia Damayanti</t>
+        </is>
+      </c>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t>Pemerintah menargetkan pembenahan TPST Bantar Gebang, Bekasi, termasuk mengakhiri praktik open dumping dapat dituntaskan pada 2027.</t>
+        </is>
+      </c>
+      <c r="F452" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G452" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8609518/butuh-rp-150-m-benahi-gunungan-sampah-bantar-gebang</t>
+        </is>
+      </c>
+      <c r="H452" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/butuh-rp-150-m-benahi-gunungan-sampah-bantar-gebang-1786155868410_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I452" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>AI hingga Ancaman Siber Jadi Tantangan Baru, Bank Siapkan Hal Ini</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:38:57 +0700</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>Fadhly Fauzi Rachman</t>
+        </is>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>Perbankan kini butuh talenta IT untuk menghadapi tantangan teknologi. Bank Jakarta luncurkan ODP IT untuk siapkan 17 peserta dalam transformasi digital.</t>
+        </is>
+      </c>
+      <c r="F453" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G453" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/moneter/d-8609818/ai-hingga-ancaman-siber-jadi-tantangan-baru-bank-siapkan-hal-ini</t>
+        </is>
+      </c>
+      <c r="H453" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2021/10/13/ilustrasi-it_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I453" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>Harga Batu Bara Acuan Turun Jadi US$ 124,4/Ton</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:00:54 +0700</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>Aulia Damayanti</t>
+        </is>
+      </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>Kementerian Energi dan Sumber Daya Mineral (ESDM) menetapkan Harga Batu bara Acuan (HBA) periode pertama Agustus 2026 sebesar US$ 124,44 per ton.</t>
+        </is>
+      </c>
+      <c r="F454" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G454" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8609483/harga-batu-bara-acuan-turun-jadi-us-124-4-ton</t>
+        </is>
+      </c>
+      <c r="H454" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/21/realisasi-devisa-ekspor-batu-bara-1784643932338_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I454" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>Terkait Insiden Kebakaran Kapal, Pelabuhan Dilengkapi X-Ray</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:26:42 +0700</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>Fadhly Fauzi Rachman</t>
+        </is>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>Insiden kebakaran kapal mendorong penguatan sistem keselamatan transportasi laut. MTI usulkan fasilitas X-Ray di pelabuhan untuk pemeriksaan lebih ketat.</t>
+        </is>
+      </c>
+      <c r="F455" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G455" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/infrastruktur/d-8609734/terkait-insiden-kebakaran-kapal-pelabuhan-dilengkapi-x-ray</t>
+        </is>
+      </c>
+      <c r="H455" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/02/km-mutiara-sentosa-2-terbakar-ratusan-penumpang-dievakuasi-dari-laut-madura-1785671535501_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I455" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>Ananda Omesh Ungkap Kondisi Terkini Dian Ayu usai Alami Saraf Kejepit</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:54:28 +0700</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>Muhammad Ahsan Nurrijal</t>
+        </is>
+      </c>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>Ananda Omesh mengungkap kondisi terkini istrinya, Dian Ayu, yang mengalami saraf kejepit. Ia menjalani perawatan intensif dan dukungan dari rekan selebritas.</t>
+        </is>
+      </c>
+      <c r="F456" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G456" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8609793/ananda-omesh-ungkap-kondisi-terkini-dian-ayu-usai-alami-saraf-kejepit</t>
+        </is>
+      </c>
+      <c r="H456" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/05/17/ananda-omesh-dian-ayu-1747484205917_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I456" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>Momen Horor Penembakan Massal di Idaho AS Terekam CCTV</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:50:43 +0700</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>REUTERS</t>
+        </is>
+      </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>Rekaman CCTV menunjukkan detik-detik penembakan massal yang terjadi di sebuah pusat perbelanjaan di Idaho, Amerika Serikat.</t>
+        </is>
+      </c>
+      <c r="F457" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G457" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260808125852-139-1390083/momen-horor-penembakan-massal-di-idaho-as-terekam-cctv</t>
+        </is>
+      </c>
+      <c r="H457" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/thumbnail-video-1786168850240_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I457" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>Viral Video Zelensky 'Langgar' Aturan UE soal Buka Tutup Botol</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:10:19 +0700</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>Video Presiden Ukraina Volodymyr Zelensky membuka tutup botol minuman viral di media sosial.</t>
+        </is>
+      </c>
+      <c r="F458" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G458" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260807203405-134-1389948/viral-video-zelensky-langgar-aturan-ue-soal-buka-tutup-botol</t>
+        </is>
+      </c>
+      <c r="H458" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2023/07/12/presiden-ukraina-volodymyr-zelensky_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I458" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>Jenderal Tertinggi AS Disebut Mulai Cari Cara Sudahi Perang Iran</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:00:13 +0700</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>Kepala Staf Gabungan Amerika Serikat (AS) Dan Caine dikabarkan sedang mencari cara untuk menyudahi perang AS vs Iran.</t>
+        </is>
+      </c>
+      <c r="F459" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G459" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260808122751-134-1390078/jenderal-tertinggi-as-disebut-mulai-cari-cara-sudahi-perang-iran</t>
+        </is>
+      </c>
+      <c r="H459" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/05/02/ketua-kepala-staf-gabungan-pentagon-dan-caine-1777696285799_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I459" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>Saudi, Pakistan dan Turki Teken Pakta Pertahanan Serupa NATO</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:15:37 +0700</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>Arab Saudi, Pakista, dan Turki meneken pakta pertahanan bersama yang menetapkan serangan terhadap salah satu akan dianggap sebagai serangan untuk semua.</t>
+        </is>
+      </c>
+      <c r="F460" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G460" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260808094942-120-1390031/saudi-pakistan-dan-turki-teken-pakta-pertahanan-serupa-nato</t>
+        </is>
+      </c>
+      <c r="H460" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/ilustrasi-bendera-arab-saudi-turki-dan-pakistan-1786159687128_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I460" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>Pengelolaan SDA Indonesia Dinilai Perlu Berorientasi Nilai Tambah</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:37:49 +0700</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>Indonesia memiliki kekayaan sumber daya alam (SDA) yang melimpah, mulai dari sumber daya terbarukan hingga yang tidak terbarukan</t>
+        </is>
+      </c>
+      <c r="F461" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G461" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/bisnis/7865732/pengelolaan-sda-indonesia-dinilai-perlu-berorientasi-nilai-tambah</t>
+        </is>
+      </c>
+      <c r="H461" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/zHr3jLvi9uhMGTXH8oJlukjkyuM=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/TATA-KELOLA-SDA-Ketua-Aliansi-Kebangsaan-Pontjo-Sutowo.jpg</t>
+        </is>
+      </c>
+      <c r="I461" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>Transfer Mengejutkan Liverpool, Dadakan Colek Barcelona demi Ronald Araujo</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:37:46 +0700</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>Liverpool disebut mencapai kesepakatan untuk mendatangkan bek Barcelona, Ronald Araujo, dengan status pinjaman dengan opsi pembelian</t>
+        </is>
+      </c>
+      <c r="F462" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G462" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865731/transfer-mengejutkan-liverpool-dadakan-colek-barcelona-demi-ronald-araujo</t>
+        </is>
+      </c>
+      <c r="H462" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/pa9IfbBgCJsjS_NmG9I05qdqqhE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/aksi-ronald-araujo-saat-dipercaya-tampil-bersama-barcelona.jpg</t>
+        </is>
+      </c>
+      <c r="I462" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>Ingin Punya Kartu Layanan Gratis? Daftar di 3 Lokasi CFD Minggu Ini</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:35:15 +0700</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>Pendaftaran Kartu Layanan Gratis (KLG) bagi pendaftar baru tersedia di tiga lokasi CFD pada Minggu, 9 Agustus 2026.</t>
+        </is>
+      </c>
+      <c r="F463" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G463" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7865730/ingin-punya-kartu-layanan-gratis-daftar-di-3-lokasi-cfd-minggu-ini</t>
+        </is>
+      </c>
+      <c r="H463" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/TZMbns9zQcnhSId7I9h_-CfO_nk=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Pendaftaran-Kartu-Layanan-Gratis-di-CFD-Minggu-9-Agustus-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I463" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>Kuasa Hukum Richard Lee Soroti Perbedaan BAP dan Keterangan Saksi dari Doktif di Sidang</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:29:51 +0700</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>Pihak Richard Lee masih memiliki puluhan pertanyaan yang akan diajukan di sidang lanjutan, guna menguji konsistensi keterangan saksi pelapor.</t>
+        </is>
+      </c>
+      <c r="F464" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G464" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7865729/kuasa-hukum-richard-lee-soroti-perbedaan-bap-dan-keterangan-saksi-dari-doktif-di-sidang</t>
+        </is>
+      </c>
+      <c r="H464" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Y3j_gfltl6GJQGxXiIRR13pYoPU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Richard-Lee-1-14072026.jpg</t>
+        </is>
+      </c>
+      <c r="I464" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>1.200 Personel Gabungan Amankan Duel Chelsea FC Vs AC Milan di GBK Malam Ini</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:28:56 +0700</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>Personel Pemprov DKI Jakarta yang dilibatkan berasal dari Satpol PP, Dinas Perhubungan, Dinas Kesehatan, hingga pemadam kebakaran.</t>
+        </is>
+      </c>
+      <c r="F465" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G465" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7865728/1200-personel-gabungan-amankan-duel-chelsea-fc-vs-ac-milan-di-gbk-malam-ini</t>
+        </is>
+      </c>
+      <c r="H465" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/NlyM_z3-Sb44LvyLLocpNMFhkr8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Kabid-Humas-Polda-Metro-Jaya-Kombes-Pol-Budi-Hermanto-343.jpg</t>
+        </is>
+      </c>
+      <c r="I465" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>Hino Beber 4 Kriteria Standarisasi Karoseri Truk dan Bus, Pre-delivery Sudah Terdigitalisasi</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:21:30 +0700</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>digitalisasi PDI membuat proses lebih cepat dan pencarian data lama juga lebih mudah dan cepat.</t>
+        </is>
+      </c>
+      <c r="F466" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G466" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/otomotif/7865727/hino-beber-4-kriteria-standarisasi-karoseri-truk-dan-bus-pre-delivery-sudah-terdigitalisasi</t>
+        </is>
+      </c>
+      <c r="H466" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/nMBu-d3nMPa7zH4tAkht28ShYJQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Diskusi-Panel-Hino-GIIAS-2026-OK.jpg</t>
+        </is>
+      </c>
+      <c r="I466" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>Cristiano Ronaldo Bikin Al Nassr Resah, Krisis 4 Tahun Lalu MU Kembali Terulang?</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:21:07 +0700</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>Cristiano Ronaldo kembali membuat Al Nassr berada dalam situasi penuh tanda tanya karena sudah 32 hari tak ikut berlatih bersama tim.</t>
+        </is>
+      </c>
+      <c r="F467" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G467" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865726/cristiano-ronaldo-bikin-al-nassr-resah-krisis-4-tahun-lalu-mu-kembali-terulang</t>
+        </is>
+      </c>
+      <c r="H467" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/oipdJGPr-njiPHTiWANSo_m_IGE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Selebrasi-Cristiano-Ronaldo-saat-cetak-gol-di-Al-Nassr.jpg</t>
+        </is>
+      </c>
+      <c r="I467" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>5 Tahun Pacaran, Dul Jaelani Minta Tissa Biani Menunggunya sampai Siap Menikah</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:19:19 +0700</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>Dul Jaelani mengaku belum siap menikah hingga meminta Tissa Biani menunggunya, meski keduanya sudah pacaran lima tahun.</t>
+        </is>
+      </c>
+      <c r="F468" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G468" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7865725/5-tahun-pacaran-dul-jaelani-minta-tissa-biani-menunggunya-sampai-siap-menikah</t>
+        </is>
+      </c>
+      <c r="H468" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/jEnS6KKNe_7AApb2tpTh62wfSsM=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Dul-Jaelani-dan-Tissa-Biani-di-cipete-jaksel-selasa.jpg</t>
+        </is>
+      </c>
+      <c r="I468" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>Gedung Bapenda Jakarta Kebakaran, Pramono Anung: Tidak Ada Korban Jiwa</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:17:59 +0700</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>Gubernur menegaskan bahwa data perpajakan DKI Jakarta aman karena sudah ter-back up secara digital, sehingga layanan perpajakan tidak terganggu.</t>
+        </is>
+      </c>
+      <c r="F469" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G469" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7865724/respons-pramono-anung-terkait-kebakaran-gedung-bapenda-jakarta-tidak-ada-korbn-jiwa</t>
+        </is>
+      </c>
+      <c r="H469" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/kn14NvzcN26yqxVmrx_J8CF8nEg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Bapenda-DKI-Jakarta.jpg</t>
+        </is>
+      </c>
+      <c r="I469" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>Penjelasan Gubernur Pramono Anung Terkait Kebakaran Gedung Bapenda DKI Jakarta</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:17:40 +0700</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>Gubernur telah menginstruksikan penebalan pasukan Dishub di lapangan agar pengaturan lalu lintas tetap lancar.</t>
+        </is>
+      </c>
+      <c r="F470" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G470" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7865723/penjelasan-gubernur-pramono-anung-terkait-kebakaran-gedung-bapenda-dki-jakarta</t>
+        </is>
+      </c>
+      <c r="H470" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/8oKD7KedTktuPKYPY4PG1DiYiQI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/GUBERNUR-DKI-JAKARTA-PRAMONO-ANUNG.jpg</t>
+        </is>
+      </c>
+      <c r="I470" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>Anak Terlihat Sehat Bikin Lega? Pakar Kesehatan Ingatkan Pentingnya Rawat Usus Tanpa Tunggu Sakit</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:16:32 +0700</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>Nutrisi yang tepat melalui pemanfaatan prebiotik, probiotik, maupun sinbiotik berbasis bukti ilmiah jadi pondasi penting kesehatan anak hingga dewasa.</t>
+        </is>
+      </c>
+      <c r="F471" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G471" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7865722/anak-terlihat-sehat-bikin-lega-pakar-kesehatan-ingatkan-pentingnya-rawat-usus-tanpa-tunggu-sakit</t>
+        </is>
+      </c>
+      <c r="H471" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/46M48-Yi7e21wB3MaYG8atHk4Uk=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Yvan-Vandenplas-1-08082026.jpg</t>
+        </is>
+      </c>
+      <c r="I471" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>Ungkap Kerinduan pada Mendiang Ayahnya, Sarwendah Dihujat, Posisi Ruben Onsu dan Anak Ikut Disorot</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:14:13 +0700</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>Ungkap kerinduan pada mendiang ayahnya, Sarwendah justu dihujat, posisi Ruben Onsu dan anak-anaknya ikut disorot.</t>
+        </is>
+      </c>
+      <c r="F472" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G472" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7865721/ungkap-kerinduan-pada-mendiang-ayahnya-sarwendah-dihujat-posisi-ruben-onsu-dan-anak-ikut-disorot</t>
+        </is>
+      </c>
+      <c r="H472" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/524gKIbyHp7cv9Q3X7b77bXKhSQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/sarwendah-sidang-hak-asuh.jpg</t>
+        </is>
+      </c>
+      <c r="I472" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>Jerawat Tak Kunjung Membaik? Dokter Sebut 3 Kesalahan Ini Sering Dilakukan</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:12:19 +0700</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>Dokter menyebut tiga kesalahan umum saat mengobati jerawat, yakni terlalu banyak memakai produk, sering berganti produk, dan over eksfoliasi.</t>
+        </is>
+      </c>
+      <c r="F473" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G473" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7865720/jerawat-tak-kunjung-membaik-dokter-sebut-3-kesalahan-ini-sering-dilakukan</t>
+        </is>
+      </c>
+      <c r="H473" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/p7q-bvySgC2zKUAF9ENNXztE1xg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Dokter-Spesialis-Dermatologi-Venereologi-dan-Estetika-RS-Hermina-Solo-dr-Arieffah-Sp-DVE.jpg</t>
+        </is>
+      </c>
+      <c r="I473" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>Sarwendah Luruskan Soal Perundungan Anak, Tegaskan Terjadi di Media Sosial Bukan Lingkungan Sekolah</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:11:29 +0700</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>Sarwendah menegaskan bahwa perundungan yang ia maksud tidak terjadi secara langsung di lingkungan sekolah anak-anaknya.</t>
+        </is>
+      </c>
+      <c r="F474" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G474" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7865719/sarwendah-luruskan-soal-perundungan-anak-tegaskan-terjadi-di-media-sosial-bukan-lingkungan-sekolah</t>
+        </is>
+      </c>
+      <c r="H474" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/yUEI0CAXSwNuRYvWOQ_aT_q189A=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Sarwendah-1-15072026.jpg</t>
+        </is>
+      </c>
+      <c r="I474" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>Jus Jambu Bantu Penderita DBD, Mitos atau Fakta? Ini Penjelasan Dokter</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:10:04 +0700</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>Apakah konsumsi jus jambu berkaitan dengan kondisi pasien DBD bahkan bisa mengobati mereka? Simak penjelasan dari dokter.</t>
+        </is>
+      </c>
+      <c r="F475" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G475" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7865718/jus-jambu-bantu-penderita-dbd-mitos-atau-fakta-ini-penjelasan-dokter</t>
+        </is>
+      </c>
+      <c r="H475" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Ojx5feawGtvJjokzvmGgwWiOVLs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/kasus-dbd-di-jakarta-terus-meningkat_20240417_183439.jpg</t>
+        </is>
+      </c>
+      <c r="I475" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>Kiai Marsudi Bersama Calon Ketua Umum PBNU Lainnya Hadiri Majelis Alumni IPNU</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:09:06 +0700</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>Kiai Marsudi telah terbiasa memanfaatkan berbagai instrumen teknologi modern berbasis Internet of Things (IoT).</t>
+        </is>
+      </c>
+      <c r="F476" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G476" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865717/kiai-marsudi-bersama-calon-ketua-umum-pbnu-lainnya-hadiri-majelis-alumni-ipnu</t>
+        </is>
+      </c>
+      <c r="H476" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/pqnRY9omczN3XEODQJ6hOasnJpM=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/juk-Kepemimpinan-NU-yang-Ad.jpg</t>
+        </is>
+      </c>
+      <c r="I476" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>Sprint Race MotoGP Inggris 2026: Marc Marquez Angkat Tangan,  Sadar Pilih 5 Besar di Silverstone</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:02:18 +0700</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>Marc Marquez tak membidik podium melainkan realistis lima besar pada sprint race MotoGP Inggris 2026 di Sirkuit Silverstone malam ini.</t>
+        </is>
+      </c>
+      <c r="F477" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G477" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7865716/sprint-race-motogp-inggris-2026-marc-marquez-angkat-tangan-sadar-pilih-5-besar-di-silverstone</t>
+        </is>
+      </c>
+      <c r="H477" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/qSS8KUXoBDjeiZ0CFKeNtyY3OpU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Marquez-vs-Bezzecchi-sprint-race-MotoGP-Jerman-2025.jpg</t>
+        </is>
+      </c>
+      <c r="I477" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>Terjemahan Lirik Lagu I Can See Clearly Now - Johnny Nash: I Can See All Obstacles in My Way</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:45:52 +0700</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>Simak terjemahan lirik lagu "I Can See Clearly Now" yang dibawakan oleh penyanyi dan penulis lagu asal Amerika Serikat (AS), Johnny Nash.</t>
+        </is>
+      </c>
+      <c r="F478" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G478" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/musik/7865715/terjemahan-lirik-lagu-i-can-see-clearly-now-johnny-nash-i-can-see-all-obstacles-in-my-way</t>
+        </is>
+      </c>
+      <c r="H478" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/dizVB9x6SK7BSsXjPU6kpy9COv4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/headset-vd-pink.jpg</t>
+        </is>
+      </c>
+      <c r="I478" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>Kebakaran Gedung Bapenda Jakarta, Gulkarmat Kerahkan 37 Mobil Damkar dan 180 Personel</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:45:20 +0700</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>Selang 10 menit kemudian, petugas tiba di lokasi dan langsung melakukan operasi pemadaman pada pukul 21.41 WIB.</t>
+        </is>
+      </c>
+      <c r="F479" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G479" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7865714/kebakaran-gedung-bapenda-jakarta-gulkarmat-kerahkan-37-mobil-damkar-dan-180-personel</t>
+        </is>
+      </c>
+      <c r="H479" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/kn14NvzcN26yqxVmrx_J8CF8nEg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Bapenda-DKI-Jakarta.jpg</t>
+        </is>
+      </c>
+      <c r="I479" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>Barang Mewah Dicuri, Tasyi Athasyia Singgung Trauma saat Berseteru hingga Difitnah Mantan Karyawan</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:44:56 +0700</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>Rumahnya mengalami pencurian, Tasyi Athasyia menyinggung soal trauma saat berseteru hingga difitnah eks karyawan.</t>
+        </is>
+      </c>
+      <c r="F480" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G480" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7865713/barang-mewah-dicuri-tasyi-athasyia-singgung-trauma-saat-berseteru-hingga-difitnah-mantan-karyawan</t>
+        </is>
+      </c>
+      <c r="H480" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/qa3hJrJieEFbvAcNsStLKCuUrUs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Tasyi-Athasyia-berikan-klarifikasi-usai-dituding-jatuhkan-produk-UMKM.jpg</t>
+        </is>
+      </c>
+      <c r="I480" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>Otomotif</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>5 Hal yang Perlu Disiapkan Sebelum Ikut Lelang Mobil Bekas</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:09:00 +0700</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>Ani Nursalikah</t>
+        </is>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- Mereka yang hendak mengikuti lelang mobil bekas disarankan untuk lebih dulu menyiapkan anggaran guna menghindari pengeluaran yang melebihi kemampuan finansial.
+Kepala Platform Lelang Kendaraan Bekas AUKSI Bady Qadarsyah menyampaikan...</t>
+        </is>
+      </c>
+      <c r="F481" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G481" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjfubi366/5-hal-yang-perlu-disiapkan-sebelum-ikut-lelang-mobil-bekas</t>
+        </is>
+      </c>
+      <c r="H481" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/028055400-1716973499-830-556.jpg</t>
+        </is>
+      </c>
+      <c r="I481" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>Pertanian</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>Aspirasi Mahasiswa Undip Bawa Mentan Amran Turun Langsung ke Alor</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:56:44 +0700</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>Dwi Murdaningsih</t>
+        </is>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, ALOR - Menteri Pertanian (Mentan) Andi Amran Sulaiman memberikan apresiasi khusus kepada Adriano Padama, mahasiswa Universitas Diponegoro (Undip) asal Kabupaten Alor, Nusa Tenggara Timur (NTT), yang berani menyuarakan persoalan...</t>
+        </is>
+      </c>
+      <c r="F482" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G482" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjfvak368/aspirasi-mahasiswa-undip-bawa-mentan-amran-turun-langsung-ke-alor</t>
+        </is>
+      </c>
+      <c r="H482" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/menteri-pertanian-mentan-andi-amran-sulaiman-saat-melakukan-kunjungan_260808135611-721.jpg</t>
+        </is>
+      </c>
+      <c r="I482" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>6 Fakta Kebakaran Gedung Bapenda DKI</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:40:00 +0700</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>Dua ledakan terdengar sebelum api melahap enam lantai Gedung Bapenda DKI.</t>
+        </is>
+      </c>
+      <c r="F483" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G483" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265045/6-fakta-kebakaran-gedung-bapenda-dki</t>
+        </is>
+      </c>
+      <c r="H483" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/42B01YC5FDkIDRmw2a58lHmRIzk=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9318747/original/067967000_1786155435-IMG_20260808_082643_127.jpg</t>
+        </is>
+      </c>
+      <c r="I483" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>Cahaya Senter Pandu Petugas Selamatkan Korban Terjebak Kebakaran Gedung Bapenda DKI</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:30:01 +0700</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>Kondisi korban cukup baik meski kini dirawat di RS karena sempat alami sesak napas.</t>
+        </is>
+      </c>
+      <c r="F484" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G484" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265042/cahaya-senter-pandu-petugas-selamatkan-korban-terjebak-kebakaran-gedung-bapenda-dki</t>
+        </is>
+      </c>
+      <c r="H484" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/n74q1Mlo7g6yuOG8j-VCXSZsSHY=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9318665/original/039881100_1786123337-IMG_3400.jpg</t>
+        </is>
+      </c>
+      <c r="I484" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>Penyebar Hoaks Bisa Kena UU Tipikor, Polisi Ungkap Syaratnya</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:07:33 +0700</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>Penyebar hoaks tak hanya terancam UU ITE. Ada jeratan lain yang menanti.</t>
+        </is>
+      </c>
+      <c r="F485" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G485" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265030/penyebar-hoaks-bisa-kena-uu-tipikor-polisi-ungkap-syaratnya</t>
+        </is>
+      </c>
+      <c r="H485" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/UGRokK_zhRbVoq1VYXPntbcjEYE=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9308725/original/048742000_1785171835-IMG_0875.jpg</t>
+        </is>
+      </c>
+      <c r="I485" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>Gedung Bapenda DKI Kebakaran, Data Perpajakan Dipastikan Aman</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:41:20 +0700</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>Kobaran api baru bisa dijinakkan 4,5 jam kemudian.</t>
+        </is>
+      </c>
+      <c r="F486" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G486" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265013/gedung-bapenda-dki-kebakaran-data-perpajakan-dipastikan-aman</t>
+        </is>
+      </c>
+      <c r="H486" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/LocynH8lNZ9lw7MI5JR6bBBSIRc=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9318664/original/080606200_1786123334-IMG_3392.jpg</t>
+        </is>
+      </c>
+      <c r="I486" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>Money</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>Harga Emas Pegadaian Naik Siang Ini, Antam Tembus Rp 2,79 Juta</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:44:50 +0700</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>Harga emas hari ini, Sabtu (8/8/2026) siang, di Pegadaian terpantau mengalami kenaikan dibandingkan pembaruan pada pagi hari.</t>
+        </is>
+      </c>
+      <c r="F487" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G487" t="inlineStr">
+        <is>
+          <t>https://money.kompas.com/read/2026/08/08/144321526/harga-emas-pegadaian-naik-siang-ini-antam-tembus-rp-279-juta</t>
+        </is>
+      </c>
+      <c r="H487" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/nZvJ-HtppZvkuppNYYgAbgAAzHw=/0x0:1200x800/1200x675/filters:watermark(data/photo/2026/01/30/697c815e7ef28.png,0,-0,1)/data/photo/2026/08/03/6a7004ba4e695.jpg</t>
+        </is>
+      </c>
+      <c r="I487" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>Pelaku Penembakan Sekolah Thailand Alami Stres, Sudah Rencanakan Aksi</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:44:50 +0700</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E488" t="inlineStr">
+        <is>
+          <t>Berdasarkan penyelidikan polisi Thailand, tersangka disebut sedang mengalami stres terkait dengan pendidikannya.</t>
+        </is>
+      </c>
+      <c r="F488" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G488" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/global/read/2026/08/08/141535470/pelaku-penembakan-sekolah-thailand-alami-stres-sudah-rencanakan-aksi</t>
+        </is>
+      </c>
+      <c r="H488" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/GaBqQTiD4TfK69wKS7RfeyCQaK0=/0x0:750x500/1200x675/filters:watermark(data/photo/2026/01/30/697c81ac46b81.png,0,-0,1)/data/photo/2023/07/02/64a0d820cb117.jpg</t>
+        </is>
+      </c>
+      <c r="I488" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>Harta Ludes Terbakar di KMP Mutiara Sentosa 2, Jadang Pasrah Hanya Terima Kompensasi Tiket Rp 2 Juta</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:44:50 +0700</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>Jadang mengungkapkan seluruh aset dan barang berharga hasil merantaunya di Jawa Barat telah dijual habis untuk modal kepindahan ke Makassar.</t>
+        </is>
+      </c>
+      <c r="F489" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G489" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/08/08/134225578/harta-ludes-terbakar-di-kmp-mutiara-sentosa-2-jadang-pasrah-hanya-terima</t>
+        </is>
+      </c>
+      <c r="H489" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/lqz_8k8mFiSCkiRpWTb9TNw9gdg=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/06/6a74515ca6d49.jpeg</t>
+        </is>
+      </c>
+      <c r="I489" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I416"/>
+  <autoFilter ref="A1:I489"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-08 08:30 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-08.xlsx
+++ b/data/berita_2026-08-08.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$489</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$551</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I489"/>
+  <dimension ref="A1:I551"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -23418,8 +23418,2923 @@
         </is>
       </c>
     </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>Redmi 17 4G dan 5G debut di pasar global</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:19:52 +0700</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E490" t="inlineStr">
+        <is>
+          <t>Setelah meluncurkan Redmi 17 5G di China, Redmi memperkenalkan Redmi 17 5G dan Redmi 17 4G ke pasar ...</t>
+        </is>
+      </c>
+      <c r="F490" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G490" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685652/redmi-17-4g-dan-5g-debut-di-pasar-global</t>
+        </is>
+      </c>
+      <c r="H490" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/InShot_20260808_141122050.jpg</t>
+        </is>
+      </c>
+      <c r="I490" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>Angkatan bersenjata Yaman melancarkan operasi terhadap kelompok Houthi</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:18:46 +0700</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E491" t="inlineStr">
+        <is>
+          <t>Tentara Yaman, Sabtu, mengumumkan bahwa mereka telah melancarkan operasi militer terhadap target dan peralatan militer ...</t>
+        </is>
+      </c>
+      <c r="F491" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G491" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685649/angkatan-bersenjata-yaman-melancarkan-operasi-terhadap-kelompok-houthi</t>
+        </is>
+      </c>
+      <c r="H491" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/Tentara-Yaman.jpg</t>
+        </is>
+      </c>
+      <c r="I491" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>DPRD DKI tawarkan Sekolah Rakyat bagi anak di Huntara Senen</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:12:48 +0700</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E492" t="inlineStr">
+        <is>
+          <t>Wakil Ketua DPRD DKI Jakarta Rani Mauliani menawarkan Sekolah Rakyat sebagai salah satu pilihan pendidikan bagi ...</t>
+        </is>
+      </c>
+      <c r="F492" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G492" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685648/dprd-dki-tawarkan-sekolah-rakyat-bagi-anak-di-huntara-senen</t>
+        </is>
+      </c>
+      <c r="H492" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001018175.jpg</t>
+        </is>
+      </c>
+      <c r="I492" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>Warga Huntara Senen usulkan fasilitas olahraga dan fogging</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:12:38 +0700</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>Warga Hunian Sementara (Huntara) Senen, Jakarta Pusat, meminta Pemerintah Provinsi DKI Jakarta membantu menyediakan ...</t>
+        </is>
+      </c>
+      <c r="F493" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G493" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685645/warga-huntara-senen-usulkan-fasilitas-olahraga-dan-fogging</t>
+        </is>
+      </c>
+      <c r="H493" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001018171.jpg</t>
+        </is>
+      </c>
+      <c r="I493" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>Jakut pangkas 5.157 pohon rawan tumbang antisipasi cuaca ekstrem</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:08:56 +0700</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E494" t="inlineStr">
+        <is>
+          <t>Pemerintah Kota Jakarta Utara melalui Suku Dinas Pertamanan dan Hutan Kota memangkas 5.157 pohon rawan tumbang di enam ...</t>
+        </is>
+      </c>
+      <c r="F494" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G494" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685644/jakut-pangkas-5157-pohon-rawan-tumbang-antisipasi-cuaca-ekstrem</t>
+        </is>
+      </c>
+      <c r="H494" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG_4451.jpeg</t>
+        </is>
+      </c>
+      <c r="I494" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>DPRD DKI dan KNPS dorong anak Huntara Senen tak putus sekolah</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:06:21 +0700</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>DPRD DKI Jakarta dan Komite Nasional Pencegahan Stunting (KNPS) Indonesia mendorong anak-anak di Hunian Sementara ...</t>
+        </is>
+      </c>
+      <c r="F495" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G495" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685643/dprd-dki-dan-knps-dorong-anak-huntara-senen-tak-putus-sekolah</t>
+        </is>
+      </c>
+      <c r="H495" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001018147.jpg</t>
+        </is>
+      </c>
+      <c r="I495" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>Sekjen ASEAN soroti pentingnya perkuat ketahanan, relevansi ASEAN</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:05:44 +0700</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t>Sekretaris Jenderal Perhimpunan Bangsa-Bangsa Asia Tenggara (ASEAN) Kao Kim Hourn menyoroti pentingnya memperkuat ...</t>
+        </is>
+      </c>
+      <c r="F496" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G496" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685641/sekjen-asean-soroti-pentingnya-perkuat-ketahanan-relevansi-asean</t>
+        </is>
+      </c>
+      <c r="H496" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000679936.jpg</t>
+        </is>
+      </c>
+      <c r="I496" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>Layanan haji Indonesia semakin memuaskan</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>Indeks kepuasan jamaah haji Indonesia 2026 naik, menandai layanan penyelenggaraan ibadah haji tahun ini dinilai lebih ...</t>
+        </is>
+      </c>
+      <c r="F497" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G497" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/infografik/5685517/layanan-haji-indonesia-semakin-memuaskan</t>
+        </is>
+      </c>
+      <c r="H497" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/20260808-Layanan-haji-Indonesia-semakin-memuaskan.jpg</t>
+        </is>
+      </c>
+      <c r="I497" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>Kevin Sibille ungkap misi bersama Bhayangkara FC</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:59:39 +0700</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>Bek asing anyar Kevin Sibille mengungkapkan misinya bersama klub Bhayangkara FC untuk mengarungi kompetisi musim ...</t>
+        </is>
+      </c>
+      <c r="F498" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G498" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685636/kevin-sibille-ungkap-misi-bersama-bhayangkara-fc</t>
+        </is>
+      </c>
+      <c r="H498" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/22/1250163.jpg</t>
+        </is>
+      </c>
+      <c r="I498" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>Persik Kediri perkuat lini pertahanan dengan daratkan dua bek impor</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:56:17 +0700</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>Klub BRI Super League Persik Kediri memperkuat lini pertahanan mereka dengan mendaratkan dua bek impor untuk mengarungi ...</t>
+        </is>
+      </c>
+      <c r="F499" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G499" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685633/persik-kediri-perkuat-lini-pertahanan-dengan-daratkan-dua-bek-impor</t>
+        </is>
+      </c>
+      <c r="H499" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/12/08/pelatih-baru-persik-kediri-2685844.jpg</t>
+        </is>
+      </c>
+      <c r="I499" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>Dirut ANTARA jadi narasumber di kegiatan Public Relations Talk di Makassar</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:52:58 +0700</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>Direktur Utama LKBN Antara Benny Siga Butarbutar (kiri) berbincang dengan peserta usai memberikan materi dalam kegiatan ...</t>
+        </is>
+      </c>
+      <c r="F500" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G500" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5685631/dirut-antara-jadi-narasumber-di-kegiatan-public-relations-talk-di-makassar</t>
+        </is>
+      </c>
+      <c r="H500" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/kegiatan-public-relations-talk-di-makassar-080826-ap-6.jpg</t>
+        </is>
+      </c>
+      <c r="I500" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>Lampaui HET, Bulog Kalbar upayakan stabilisasi harga beras premium</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:51:15 +0700</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>ANTARA - Lonjakan harga beras premium yang terjadi di Provinsi Kalimantan Barat, mendorong Perum Bulog Kantor Wilayah ...</t>
+        </is>
+      </c>
+      <c r="F501" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G501" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5685563/lampaui-het-bulog-kalbar-upayakan-stabilisasi-harga-beras-premium</t>
+        </is>
+      </c>
+      <c r="H501" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AYM_LAMPAUI-HET-BULOG-KALBAR-UPAYAKAN.jpg</t>
+        </is>
+      </c>
+      <c r="I501" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>Persija Jakarta dapatkan bekal berharga dari Piala Presiden 2026</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:49:15 +0700</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E502" t="inlineStr">
+        <is>
+          <t>Manajer klub Persija Jakarta Ardhi Tjahjoko menilai tim Macan Kemayoran mendapatkan bekal berharga dari turnamen ...</t>
+        </is>
+      </c>
+      <c r="F502" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G502" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685627/persija-jakarta-dapatkan-bekal-berharga-dari-piala-presiden-2026</t>
+        </is>
+      </c>
+      <c r="H502" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/persija-jakarta-raih-peringkat-tiga-piala-presiden-2026-2836020.jpg</t>
+        </is>
+      </c>
+      <c r="I502" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>Persib Bandung lanjutkan persiapan di Bali</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:44:05 +0700</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E503" t="inlineStr">
+        <is>
+          <t>Pelatih Persib Bandung Igor Tolic mengatakan tim asuhannya akan melanjutkan masa persiapan jelang kompetisi musim ...</t>
+        </is>
+      </c>
+      <c r="F503" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G503" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685623/persib-bandung-lanjutkan-persiapan-di-bali</t>
+        </is>
+      </c>
+      <c r="H503" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/persib-lolos-final-piala-presiden-2026-040826-nhw-2.jpg</t>
+        </is>
+      </c>
+      <c r="I503" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>BNPB dorong peninjauan Perda Pembakaran Lahan di Kalbar</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:41:55 +0700</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E504" t="inlineStr">
+        <is>
+          <t>Badan Nasional Penanggulangan Bencana (BNPB) mendorong Pemerintah Provinsi Kalimantan Barat meninjau penerapan ...</t>
+        </is>
+      </c>
+      <c r="F504" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G504" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685620/bnpb-dorong-peninjauan-perda-pembakaran-lahan-di-kalbar</t>
+        </is>
+      </c>
+      <c r="H504" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/Perda.jpg</t>
+        </is>
+      </c>
+      <c r="I504" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>BMW mulai memproduksi sedan listrik i3 di Munich</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:40:35 +0700</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/antaranewsdotcom</t>
+        </is>
+      </c>
+      <c r="E505" t="inlineStr">
+        <is>
+          <t>BMW sudah mulai memproduksi sedan listrik BMW i3 di pabrik milik perusahaan di Munich, Jerman.
+Menurut siaran Arena ...</t>
+        </is>
+      </c>
+      <c r="F505" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G505" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/berita/5685616/bmw-mulai-memproduksi-sedan-listrik-i3-di-munich</t>
+        </is>
+      </c>
+      <c r="H505" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/03/19/1000112229.jpg</t>
+        </is>
+      </c>
+      <c r="I505" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>Kecerobohan Sekian Detik, Puluhan Nyawa Melayang</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:13:05 +0700</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>Rakhmad Hidayatulloh Permana</t>
+        </is>
+      </c>
+      <c r="E506" t="inlineStr">
+        <is>
+          <t>Peristiwa kebakaran klub The Station menjadi salah satu tragedi paling mematikan di AS. Kecerobohan beberapa detik membuat puluhan nyawa melayang.</t>
+        </is>
+      </c>
+      <c r="F506" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G506" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609885/kecerobohan-sekian-detik-puluhan-nyawa-melayang</t>
+        </is>
+      </c>
+      <c r="H506" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/kebakaran-di-klub-malam-1786156620492_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I506" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>Penembakan Terjadi di Festival Budaya Lembah Baliem, Pengunjung Kocar-kacir</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:08:22 +0700</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>Paulus Pulo</t>
+        </is>
+      </c>
+      <c r="E507" t="inlineStr">
+        <is>
+          <t>Penembakan terjadi di Festival Budaya Lembah Baliem, Jayawijaya, Papua. Warga panik mencari tempat aman saat suara tembakan terdengar.</t>
+        </is>
+      </c>
+      <c r="F507" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G507" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609881/penembakan-terjadi-di-festival-budaya-lembah-baliem-pengunjung-kocar-kacir</t>
+        </is>
+      </c>
+      <c r="H507" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/penembakan-terjadi-lokasi-festival-budaya-lembah-baliem-jayawijaya-1786175421651_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I507" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>Pria di Sultra Open BO Sesama Jenis lalu Bawa Kabur Motor Teman Kencan</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:04:00 +0700</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>Reinhard Soplantila</t>
+        </is>
+      </c>
+      <c r="E508" t="inlineStr">
+        <is>
+          <t>Polisi menangkap pria berinisial AS (42) usai membawa kabur motor teman kencan sesama jenis inisial RN (19) usai open booking (BO) di sebuah hotel di Kolaka.</t>
+        </is>
+      </c>
+      <c r="F508" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G508" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609873/pria-di-sultra-open-bo-sesama-jenis-lalu-bawa-kabur-motor-teman-kencan</t>
+        </is>
+      </c>
+      <c r="H508" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2019/10/26/5b16224e-0123-430d-8a63-b1adb7dd4f9b_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I508" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>Kompolnas Wanti-wanti Propaganda Kekerasan di Ruang Digital Dilarang</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:02:32 +0700</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>Anggi Muliawati</t>
+        </is>
+      </c>
+      <c r="E509" t="inlineStr">
+        <is>
+          <t>Komisioner Kompolnas Choirul Anam mengatakan kebebasan berekspresi dilindungi konstitusi dan UU. Namun, dia mengingatkan kebebasan tetap memiliki batasan.</t>
+        </is>
+      </c>
+      <c r="F509" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G509" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609870/kompolnas-wanti-wanti-propaganda-kekerasan-di-ruang-digital-dilarang</t>
+        </is>
+      </c>
+      <c r="H509" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/07/09/komisioner-kompolnas-choirul-anam-rumondangdetikcom-1752074951783_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I509" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>Polda Metro Kerahkan 1.200 Personel Amankan Laga Chelsea Vs Milan di GBK</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:58:31 +0700</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E510" t="inlineStr">
+        <is>
+          <t>Dua raksasa Eropa, AC Milan dan Chelsea, bertanding di GBK Jakarta. Polda Metro Jaya siapkan 1.200 personel untuk pengamanan dan kelancaran acara.</t>
+        </is>
+      </c>
+      <c r="F510" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G510" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609868/polda-metro-kerahkan-1-200-personel-amankan-laga-chelsea-vs-milan-di-gbk</t>
+        </is>
+      </c>
+      <c r="H510" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2024/06/26/revitalisasi-rumput-sugbk-dimulai_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I510" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>Kisah Siti, Rela Anaknya Tinggal di Asrama demi Sekolah Rakyat</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:55:34 +0700</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>Inkana Putri</t>
+        </is>
+      </c>
+      <c r="E511" t="inlineStr">
+        <is>
+          <t>Ruang makan Politeknik Penerbangan Indonesia dipenuhi tawa saat MPLS di Sekolah Rakyat. Program ini bantu akses pendidikan bagi keluarga kurang mampu.</t>
+        </is>
+      </c>
+      <c r="F511" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G511" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609864/kisah-siti-rela-anaknya-tinggal-di-asrama-demi-sekolah-rakyat</t>
+        </is>
+      </c>
+      <c r="H511" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/di-hadapan-seskab-teddy-orang-tua-siswa-sekolah-rakyat-berbagi-kisah-haru-1786175663766.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I511" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>MPR Akan Undang Pakar hingga Akademisi Bahas PPHN Setelah 17 Agustus</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:47:30 +0700</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>Adrial akbar</t>
+        </is>
+      </c>
+      <c r="E512" t="inlineStr">
+        <is>
+          <t>Ketua MPR RI Ahmad Muzani akan bertemu pakar dan akademisi setelah 17 Agustus 2026 untuk membahas Pokok-Pokok Haluan Negara (PPHN).</t>
+        </is>
+      </c>
+      <c r="F512" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G512" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609855/mpr-akan-undang-pakar-hingga-akademisi-bahas-pphn-setelah-17-agustus</t>
+        </is>
+      </c>
+      <c r="H512" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/04/18/ketua-mpr-ahmad-muzani-1776504353935_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I512" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>Jatanras Polda Metro Tangkap Rampok Pembacok Pegawai Koperasi di Bekasi</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:45:59 +0700</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E513" t="inlineStr">
+        <is>
+          <t>Tim Jatanras Polda Metro menangkap 6 perampok bersenjata tajam di Cibitung. Korban, pegawai koperasi, terluka setelah diserang saat baru tiba di kantor.</t>
+        </is>
+      </c>
+      <c r="F513" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G513" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609854/jatanras-polda-metro-tangkap-rampok-pembacok-pegawai-koperasi-di-bekasi</t>
+        </is>
+      </c>
+      <c r="H513" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2023/07/25/ilustrasi-penangkapan_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I513" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>Kebakaran Gedung Bapenda DKI Padam, 2 Mobil Damkar Tetap Siaga di Lokasi</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:39:48 +0700</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>Brigitta Belia Permata Sari</t>
+        </is>
+      </c>
+      <c r="E514" t="inlineStr">
+        <is>
+          <t>Kebakaran yang melanda gedung Badan Pendapatan Daerah (Bapenda) DKI Jakarta sudah padam. Akan tetapi 2 mobil damkar masih disiagakan.</t>
+        </is>
+      </c>
+      <c r="F514" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G514" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609852/kebakaran-gedung-bapenda-dki-padam-2-mobil-damkar-tetap-siaga-di-lokasi</t>
+        </is>
+      </c>
+      <c r="H514" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/kondisi-gedung-bapenda-dki-usai-terbakar-1786154575590_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I514" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>BAZNAS Salurkan Rp 871 Juta untuk Zmart hingga Santripreneur di Gresik</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:38:05 +0700</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>Jemmi Purwodianto</t>
+        </is>
+      </c>
+      <c r="E515" t="inlineStr">
+        <is>
+          <t>BAZNAS dan Menko PM Abdul Muhaimin Iskandar salurkan bantuan Rp 871 juta untuk penguatan ekonomi umat di Gresik, melalui program Zmart dan BUMi Masjid.</t>
+        </is>
+      </c>
+      <c r="F515" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G515" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609850/baznas-salurkan-rp-871-juta-untuk-zmart-hingga-santripreneur-di-gresik</t>
+        </is>
+      </c>
+      <c r="H515" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/baznas-salurkan-zmart-bumi-dan-santripreneur-di-gresik-cak-imin-beri-apresiasi-1786174644219.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I515" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>Siasat Residivis Bobol 4 Kotak Amal di Bogor Hunting Masjid Sepi</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:34:44 +0700</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>Rizky Adha Mahendra</t>
+        </is>
+      </c>
+      <c r="E516" t="inlineStr">
+        <is>
+          <t>Polisi menangkap residivis berinisial R yang membobol empat kotak amal di Bogor. Pelaku memetakan masjid sepi untuk aksinya.</t>
+        </is>
+      </c>
+      <c r="F516" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G516" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609841/siasat-residivis-bobol-4-kotak-amal-di-bogor-hunting-masjid-sepi</t>
+        </is>
+      </c>
+      <c r="H516" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2022/12/14/pencurian-benda-sakral_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I516" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>Pembangunan Tol Jogja-Solo Hampir Rampung, Begini Progresnya</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:00:14 +0700</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>Aulia Damayanti</t>
+        </is>
+      </c>
+      <c r="E517" t="inlineStr">
+        <is>
+          <t>Pembangunan Tol Solo-Yogyakarta-NYIA Kulonprogo (Jogja-Solo) hampir rampung.</t>
+        </is>
+      </c>
+      <c r="F517" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G517" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/infrastruktur/d-8609632/pembangunan-tol-jogja-solo-hampir-rampung-begini-progresnya</t>
+        </is>
+      </c>
+      <c r="H517" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/pembangunan-tol-jogja-solo-hampir-rampung-begini-progresnya-1786162440374_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I517" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>Orang Tua Siswa Sekolah Rakyat Menangis Haru di Hadapan Seskab Teddy</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:25:08 +0700</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E518" t="inlineStr">
+        <is>
+          <t>Siti Yuliana, seorang ibu rumah tangga asal Jakarta Utara menangis di hadapan Sekretaris Kabinet Teddy Indra Wijaya, Menteri Sosial Saifullah Yusuf (Gus Ipul)</t>
+        </is>
+      </c>
+      <c r="F518" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G518" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808151335-20-1390115/orang-tua-siswa-sekolah-rakyat-menangis-haru-di-hadapan-seskab-teddy</t>
+        </is>
+      </c>
+      <c r="H518" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/sekretaris-kabinet-letkol-teddy-indra-wijaya-1786176733611_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I518" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>Terdampak Kebakaran Bapenda, Sistem Lampu Lalin DKI Diatur Manual</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:10:16 +0700</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E519" t="inlineStr">
+        <is>
+          <t>Gubernur DKI Pramono Anung mengungkapkan sistem pengendalian lalu lintas Dishub terdampak kebakaran Gedung Bapenda, pengaturan kini dilakukan manual.</t>
+        </is>
+      </c>
+      <c r="F519" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G519" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808141607-20-1390092/terdampak-kebakaran-bapenda-sistem-lampu-lalin-dki-diatur-manual</t>
+        </is>
+      </c>
+      <c r="H519" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2025/09/01/lalu-lintas-jakarta-lancar-1756692453337_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I519" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>Seskab Teddy: Anak Putus Sekolah Berani Mimpi Besar di Sekolah Rakyat</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:03:06 +0700</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E520" t="inlineStr">
+        <is>
+          <t>Sekretaris Kabinet Letkol Teddy Indra Wijaya mendorong anak-anak yang sempat putus sekolah maupun belum pernah mengenyam pendidikan untuk kembali bersekolah.</t>
+        </is>
+      </c>
+      <c r="F520" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G520" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808144718-20-1390101/seskab-teddy-anak-putus-sekolah-berani-mimpi-besar-di-sekolah-rakyat</t>
+        </is>
+      </c>
+      <c r="H520" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/sekretaris-kabinet-letkol-teddy-indra-wijaya-1786176091967_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I520" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>Wakapolri: Jangan Cuma Jadi Penonton, Jadilah Talenta Digital</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:46:30 +0700</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E521" t="inlineStr">
+        <is>
+          <t>Wakapolri Komjen Pol Dedi Prasetyo mengatakan Polri ingin hadir di ruang yang dekat dengan kehidupan generasi muda.</t>
+        </is>
+      </c>
+      <c r="F521" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G521" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808144137-20-1390099/wakapolri-jangan-cuma-jadi-penonton-jadilah-talenta-digital</t>
+        </is>
+      </c>
+      <c r="H521" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/35936-anak-muda-main-bareng-di-kapolri-cup-2026-1786174887891_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I521" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>Polda Metro Pastikan Kondisi Jakarta Aman Terkendali</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:40:42 +0700</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E522" t="inlineStr">
+        <is>
+          <t>Polda Metro Jaya menyatakan Jakarta aman dan terkendali. Kegiatan masyarakat dan perekonomian berjalan lancar.</t>
+        </is>
+      </c>
+      <c r="F522" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G522" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808125234-12-1390082/polda-metro-pastikan-kondisi-jakarta-aman-terkendali</t>
+        </is>
+      </c>
+      <c r="H522" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/apel-kebangsaan-jaga-jakarta-1786153774575_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I522" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>Hashim Djojohadikusumo Kukuhkan 20 Ormas Baru Kawal Program Pemerintah</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:32:43 +0700</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E523" t="inlineStr">
+        <is>
+          <t>Ketua Dewan Pembina FORMAS Hashim Djojohadikusumo mengukuhkan 20 ormas baru yang bergabung dalam FORMAS untuk mengawal program pemerintah.</t>
+        </is>
+      </c>
+      <c r="F523" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G523" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808123153-20-1390079/hashim-djojohadikusumo-kukuhkan-20-ormas-baru-kawal-program-pemerintah</t>
+        </is>
+      </c>
+      <c r="H523" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2025/10/31/hashim-djojohadikusumo-di-cnn-indonesia-awards-2025-1761904534643_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I523" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>Tak Terima Dimarahi Nakhoda, ABK Bakar Kapal di Perairan Aru Maluku</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:25:09 +0700</t>
+        </is>
+      </c>
+      <c r="D524" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E524" t="inlineStr">
+        <is>
+          <t>Seorang ABK membakar kapal penangkap cumi setelah dimarahi nakhoda di Perairan Aru. Dari 33 orang, 32 selamat, satu masih hilang.</t>
+        </is>
+      </c>
+      <c r="F524" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G524" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808123304-20-1390080/tak-terima-dimarahi-nakhoda-abk-bakar-kapal-di-perairan-aru-maluku</t>
+        </is>
+      </c>
+      <c r="H524" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/kapal-dibakar-di-perairan-aru-maluku-1786167433248_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I524" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>Sederet Fakta Terbaru Temuan Senjata di Sekolah Pondok Pinang Jaksel</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:19:04 +0700</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E525" t="inlineStr">
+        <is>
+          <t>Ratusan senjata ditemukan di sebuah sekolah swasta di Pondok Pinang, Kebayoran Lama, Jakarta Selatan. Berikut fakta-faktanya.</t>
+        </is>
+      </c>
+      <c r="F525" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G525" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808131623-12-1390086/sederet-fakta-terbaru-temuan-senjata-di-sekolah-pondok-pinang-jaksel</t>
+        </is>
+      </c>
+      <c r="H525" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/07/ratusan-senjata-di-yayasan-sekolah-jaksel-1786100090384_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I525" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>Kebakaran Gedung Bapenda, 1 Korban Dilarikan ke RS Tarakan</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:50:53 +0700</t>
+        </is>
+      </c>
+      <c r="D526" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E526" t="inlineStr">
+        <is>
+          <t>Kebakaran di Gedung Bapenda DKI Jakarta menyebabkan satu korban dilarikan di RSUD Tarakan. Tidak ada korban jiwa dalam insiden ini.</t>
+        </is>
+      </c>
+      <c r="F526" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G526" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808122017-20-1390077/kebakaran-gedung-bapenda-1-korban-dilarikan-ke-rs-tarakan</t>
+        </is>
+      </c>
+      <c r="H526" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/gedung-bapenda-dki-jakarta-kebakaran-1786149524124_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I526" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>FOTO: Sembako dan Cek Kesehatan Gratis di Apel Kebangsaan Jaga Jakarta</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:10:00 +0700</t>
+        </is>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E527" t="inlineStr">
+        <is>
+          <t>Warga berbondong memadati tenda cek kesehatan dan sembako gratis di Apel Kebangsaan Jaga Jakarta untuk Indonesia di Kawasan Monas, Jakarta, Sabtu (8/8).</t>
+        </is>
+      </c>
+      <c r="F527" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G527" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808115806-22-1390065/foto-sembako-dan-cek-kesehatan-gratis-di-apel-kebangsaan-jaga-jakarta</t>
+        </is>
+      </c>
+      <c r="H527" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/cek-kesehatan-dan-sembako-gratis-di-apel-kebangsaan-jaga-jakarta-1786165083968_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I527" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>FOTO: Semarak Apel Kebangsaan Jaga Jakarta untuk Indonesia</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:00:16 +0700</t>
+        </is>
+      </c>
+      <c r="D528" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E528" t="inlineStr">
+        <is>
+          <t>Apel Kebangsaan Jaga Jakarta untuk Indonesia digelar di Lapangan Monumen Nasional (Monas), Jakarta Pusat, Sabtu (8/8) pagi.</t>
+        </is>
+      </c>
+      <c r="F528" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G528" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808112625-22-1390050/foto-semarak-apel-kebangsaan-jaga-jakarta-untuk-indonesia</t>
+        </is>
+      </c>
+      <c r="H528" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/galfot-apel-kebangsaan-jaga-jakarta-untuk-indonesia-1786163179471_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I528" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>Puslabfor Diterjunkan Usut Penyebab Kebakaran Bapenda DKI</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:45:11 +0700</t>
+        </is>
+      </c>
+      <c r="D529" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E529" t="inlineStr">
+        <is>
+          <t>Puslabfor Polri diterjunkan guna mengusut pemicu kebakaran di Gedung Badan Pendapatan Daerah (Bapenda) DKI Jakarta pada Jumat (7/8).</t>
+        </is>
+      </c>
+      <c r="F529" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G529" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808113307-12-1390061/puslabfor-diterjunkan-usut-penyebab-kebakaran-bapenda-dki</t>
+        </is>
+      </c>
+      <c r="H529" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/gedung-bapenda-dki-jakarta-kebakaran-1786149524209_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I529" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>Pernyataan Pihak Keluarga Besar Almarhum Pasien BPJS Yurizal</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:17:15 +0700</t>
+        </is>
+      </c>
+      <c r="D530" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E530" t="inlineStr">
+        <is>
+          <t>Keluarga almarhum Yurizal mengucapkan terima kasih atas dukungan publik. Mereka pun berharap isu viral terkait pasien BPJS diselesaikan.</t>
+        </is>
+      </c>
+      <c r="F530" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G530" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808002722-20-1389991/pernyataan-pihak-keluarga-besar-almarhum-pasien-bpjs-yurizal</t>
+        </is>
+      </c>
+      <c r="H530" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2023/04/12/ilustrasi-berpegangan-tangan_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I530" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>Pangdam Jaya: Mari Bersatu Jaga Keamanan, Ketertiban dan Persatuan</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:14:03 +0700</t>
+        </is>
+      </c>
+      <c r="D531" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E531" t="inlineStr">
+        <is>
+          <t>Pangdam Jaya Letjen TNI Deddy Suryadi meminta semua elemen bangsa untuk bersatu dalam menjaga keamanan, ketertiban bangsa.</t>
+        </is>
+      </c>
+      <c r="F531" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G531" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808110654-20-1390048/pangdam-jaya-mari-bersatu-jaga-keamanan-ketertiban-dan-persatuan</t>
+        </is>
+      </c>
+      <c r="H531" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/apel-kebangsaan-jaga-jakarta-1786162153671_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I531" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>Kebakaran Melanda 30 Hektar Area Gunung Rinjani</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:06:06 +0700</t>
+        </is>
+      </c>
+      <c r="D532" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E532" t="inlineStr">
+        <is>
+          <t>Kebakaran kembali terjadi di kawasan Taman Nasional Gunung Rinjani (TNGR), Lombok, Nusa Tenggara Barat (NTB), pada Jumat (7/8).</t>
+        </is>
+      </c>
+      <c r="F532" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G532" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808110121-20-1390047/gunung-rinjani-kembali-dilalap-api</t>
+        </is>
+      </c>
+      <c r="H532" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2021/08/08/turkey-fire_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I532" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>Polda Metro Jaya Tegaskan TNI-Polri Sinergi Jaga Jakarta</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:08:05 +0700</t>
+        </is>
+      </c>
+      <c r="D533" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E533" t="inlineStr">
+        <is>
+          <t>Kabid Humas Polda Metro Jaya Kombes Budi Hermanto menyatakan TNI-Polri bersinergi dalam menjaga stabilitas dan keamanan Jakarta.</t>
+        </is>
+      </c>
+      <c r="F533" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G533" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808100344-20-1390037/polda-metro-jaya-tegaskan-tni-polri-sinergi-jaga-jakarta</t>
+        </is>
+      </c>
+      <c r="H533" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/apel-kebangsaan-jaga-jakarta-1786153774792_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I533" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>Isu Indonesia Punya 'Shadow Relationship' dengan Israel, FPN: Hentikan Seluruh Hubungan!</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:17:56 +0700</t>
+        </is>
+      </c>
+      <c r="D534" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E534" t="inlineStr">
+        <is>
+          <t>FPN menyoroti dugaan hubungan tersembunyi Indonesia-Israel melalui perdagangan, teknologi, pertahanan, dan kerja sama melalui negara ketiga.</t>
+        </is>
+      </c>
+      <c r="F534" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G534" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865743/isu-indonesia-punya-shadow-relationship-dengan-israel-fpn-hentikan-seluruh-hubungan</t>
+        </is>
+      </c>
+      <c r="H534" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/pDGO-yEFF4LNwjYVNjQW4nNdVFA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Furqan-AMC-FPN-124sdgsdhg.jpg</t>
+        </is>
+      </c>
+      <c r="I534" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>Tawaran Ngawur Barcelona untuk Rodri, Manchester City Auto Ngamuk</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:15:19 +0700</t>
+        </is>
+      </c>
+      <c r="D535" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E535" t="inlineStr">
+        <is>
+          <t>Barcelona melempar tawaran awal kepada Manchester City untuk Rodri di angka 45 juta Euro yang dianggap tak serius oleh The Citizens.</t>
+        </is>
+      </c>
+      <c r="F535" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G535" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865742/tawaran-ngawur-barcelona-untuk-rodri-manchester-city-auto-ngamuk</t>
+        </is>
+      </c>
+      <c r="H535" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/4dXj719Vm4nUfoswROCqzkHH19M=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Potret-duel-pertandingan-Manchester-City-vs-Arsenal-dalam-pekan-ke-33-Liga-Inggris.jpg</t>
+        </is>
+      </c>
+      <c r="I535" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>Ma’ruf Amin Ungkap Syarat Pemimpin NU: Harus Mampu Lakukan Islah</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:09:46 +0700</t>
+        </is>
+      </c>
+      <c r="D536" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E536" t="inlineStr">
+        <is>
+          <t>Jelang Muktamar Ke-35 NU, Ma’ruf Amin menyebut pemimpin organisasi ke depan harus mampu mendamaikan konflik dan menyatukan internal.</t>
+        </is>
+      </c>
+      <c r="F536" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G536" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865741/maruf-amin-ungkap-syarat-pemimpin-nu-harus-mampu-lakukan-ishlah</t>
+        </is>
+      </c>
+      <c r="H536" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ftM2eMpf0zZpnHxzfe99mRk-qbg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Maruf-Amin-dalam-Halaqah-Kebangsaan-dan-Qanun-Asasi-di-Gedung-MPR-RI-Jakarta.jpg</t>
+        </is>
+      </c>
+      <c r="I536" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>Manchester United Tolak Rafael Leao meski Cuma 50 Juta Euro, Marcus Rashford Jadi Penyebabnya</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:04:16 +0700</t>
+        </is>
+      </c>
+      <c r="D537" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E537" t="inlineStr">
+        <is>
+          <t>Rafael Leao dikabarkan ditawarkan AC Milan ke Manchester United hanya 50 juta euro, tetapi Setan Merah memilih mempertahankan Marcus Rashford.</t>
+        </is>
+      </c>
+      <c r="F537" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G537" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865740/manchester-united-tolak-rafael-leao-meski-cuma-50-juta-euro-marcus-rashford-jadi-penyebabnya</t>
+        </is>
+      </c>
+      <c r="H537" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/MTxcNKEgqzB7pj0bP-KkCFM9mfg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/pemain-depan-ac-milan-asal-portugal-rafael-leao-melihat-bola.jpg</t>
+        </is>
+      </c>
+      <c r="I537" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>Kunci Jawaban Bahasa Indonesia Kawan Seiring Kelas 3 Halaman 18 Kurikulum Merdeka: Aktivitas 2</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:51:08 +0700</t>
+        </is>
+      </c>
+      <c r="D538" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E538" t="inlineStr">
+        <is>
+          <t>Soal ini terdapat pada buku Bahasa Indonesia Kawan Seiring Kelas 3 Halaman 18 Kurikulum Merdeka, tepatnya pada Aktivitas 2.</t>
+        </is>
+      </c>
+      <c r="F538" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G538" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/pendidikan/7865739/kunci-jawaban-bahasa-indonesia-kawan-seiring-kelas-3-halaman-18-kurikulum-merdeka-aktivitas-2</t>
+        </is>
+      </c>
+      <c r="H538" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/k8J3TVJbmHA5o0uqsIdxfHLQwpg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/siswa-SD-belajar-di-sekolah-1.jpg</t>
+        </is>
+      </c>
+      <c r="I538" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>Terjemahan Lirik Lagu Maladie - Mauvais Djo, Viral TikTok: Elle a Les Cheveux Blonds</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:50:07 +0700</t>
+        </is>
+      </c>
+      <c r="D539" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E539" t="inlineStr">
+        <is>
+          <t>Simak lirik dan terjemahan lagu berbahasa Prancis yang  berjudul Maladie yang dinyanyikan oleh Mauvais Djo.</t>
+        </is>
+      </c>
+      <c r="F539" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G539" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/musik/7865738/terjemahan-lirik-lagu-maladie-mauvais-djo-viral-tiktok-elle-a-les-cheveux-blonds</t>
+        </is>
+      </c>
+      <c r="H539" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/8ofGbaRMpqu_gFPWYkenF6qEE2Y=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Potret-ilustrasi-lirik-lagu-terjemahan-musik-mendengarkan-musik.jpg</t>
+        </is>
+      </c>
+      <c r="I539" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>Eks Pelatih Timnas Tak Permasalahkan Rivan Nurmulki Mundur, Alasannya Disebut Bijak</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:44:59 +0700</t>
+        </is>
+      </c>
+      <c r="D540" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E540" t="inlineStr">
+        <is>
+          <t>Eks pelatih Timnas Voli Putra Indonesia Erwin Rusni tak mempermasalahkan mundurnya Rivan Nurmulki dari timnas untuk kepentingan regenerasi.</t>
+        </is>
+      </c>
+      <c r="F540" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G540" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7865737/eks-pelatih-timnas-tak-permasalahkan-rivan-nurmulki-mundur-alasannya-disebut-bijak</t>
+        </is>
+      </c>
+      <c r="H540" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/AMAreX8qhWr20BTc1PCBHjrAm-o=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Opposite-Timnas-Voli-Putra-Indonesia-Rivan-Nurmulki-kanan-saat.jpg</t>
+        </is>
+      </c>
+      <c r="I540" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>First Drive Changan Nevo Q05, SUV Listrik dengan Kabin Lega dan Nyaman</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:44:34 +0700</t>
+        </is>
+      </c>
+      <c r="D541" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E541" t="inlineStr">
+        <is>
+          <t>Tribunnews berkesempatan test drive Nevo Q05 di kawasan BSD, Tangerang, di sela penyelenggaraan GIIAS 2026.</t>
+        </is>
+      </c>
+      <c r="F541" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G541" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/otomotif/7865736/first-drive-changan-nevo-q05-suv-listrik-dengan-kabin-lega-dan-nyaman</t>
+        </is>
+      </c>
+      <c r="H541" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/V96rdtScpvAmS0OxikiwO8Hv8zE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Test-drive-Nevo-Q05.jpg</t>
+        </is>
+      </c>
+      <c r="I541" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>Ketua MPR Sebut Pembahasan PPHN Dibuka Lagi Setelah 17 Agustus, Masyarakat Akan Dilibatkan</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:40:50 +0700</t>
+        </is>
+      </c>
+      <c r="D542" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E542" t="inlineStr">
+        <is>
+          <t>Muzani mengatakan MPR sebelumnya telah menyerahkan rancangan PPHN kepada Presiden Prabowo Subianto.</t>
+        </is>
+      </c>
+      <c r="F542" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G542" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865735/ketua-mpr-sebut-pembahasan-pphn-dibuka-lagi-setelah-17-agustus-masyarakat-akan-dilibatkan</t>
+        </is>
+      </c>
+      <c r="H542" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/GaKXSByAQL1MLhGoRQVesYV6src=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Ketua-MPR-RI-Ahmad-Muza.jpg</t>
+        </is>
+      </c>
+      <c r="I542" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>Laporan The Geostrata Soroti Perbedaan Kashmir yang Dikelola India dan Pakistan</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:39:44 +0700</t>
+        </is>
+      </c>
+      <c r="D543" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E543" t="inlineStr">
+        <is>
+          <t>Model tata kelola berbeda disebut menjadi faktor utama yang membedakan perkembangan Jammu dan Kashmir.</t>
+        </is>
+      </c>
+      <c r="F543" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G543" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7865734/laporan-the-geostrata-soroti-perbedaan-kashmir-yang-dikelola-india-dan-pakistan</t>
+        </is>
+      </c>
+      <c r="H543" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/atBsW709-tYRJDxKaeCvQF1DmL8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Peta-interaktif-wilayah-Kashmir-yang-diakses-dari.jpg</t>
+        </is>
+      </c>
+      <c r="I543" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>Coco Sheet Produksi Lapas Purwokerto Tembus Pasar China</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:38:35 +0700</t>
+        </is>
+      </c>
+      <c r="D544" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E544" t="inlineStr">
+        <is>
+          <t>Sebanyak 400 lembar Coco Sheet produksi Lapas Kelas IIA Purwokerto diekspor perdana ke China untuk memasok industri kasur.</t>
+        </is>
+      </c>
+      <c r="F544" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G544" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/bisnis/7865733/coco-sheet-produksi-lapas-purwokerto-tembus-pasar-china</t>
+        </is>
+      </c>
+      <c r="H544" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/G1Onu-4upvmOMyW5rzjJ9OewaTA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Ekspor-Coco-Sheet-ke-China-OK.jpg</t>
+        </is>
+      </c>
+      <c r="I544" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>Pertanian</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>Amran Siapkan Strategi Pertanian Tiga Tahap untuk Atasi Kemiskinan Alor</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:15:52 +0700</t>
+        </is>
+      </c>
+      <c r="D545" t="inlineStr">
+        <is>
+          <t>Friska Yolandha</t>
+        </is>
+      </c>
+      <c r="E545" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- Menteri Pertanian (Mentan) Andi Amran Sulaiman menyiapkan strategi pertanian tiga tahap untuk mengatasi kemiskinan di Kabupaten Alor, Nusa Tenggara Timur (NTT). Strategi tersebut mencakup pemenuhan kebutuhan...</t>
+        </is>
+      </c>
+      <c r="F545" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G545" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjfyyg370/amran-siapkan-strategi-pertanian-tiga-tahap-untuk-atasi-kemiskinan-alor</t>
+        </is>
+      </c>
+      <c r="H545" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/_260808151509-185.png</t>
+        </is>
+      </c>
+      <c r="I545" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>Kondisi Gedung Bapenda DKI Setelah Kebakaran Padam</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:21:00 +0700</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E546" t="inlineStr">
+        <is>
+          <t>Petugas damkar mulai meninggalkan lokasi, kondisi Gedung Bapenda DKI terungkap.</t>
+        </is>
+      </c>
+      <c r="F546" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G546" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265077/kondisi-gedung-bapenda-dki-setelah-kebakaran-padam</t>
+        </is>
+      </c>
+      <c r="H546" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/xmPQOeE77DdyGBOCQpFd9KSe1VQ=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9319009/original/096630900_1786177236-IMG_20260808_123948_474.jpg</t>
+        </is>
+      </c>
+      <c r="I546" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>Ada Konser di Ancol, TransJakarta Perpanjang Operasional</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:58:17 +0700</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E547" t="inlineStr">
+        <is>
+          <t>Kabar baik bagi penonton konser Ancol, bus TransJakarta pulang lebih malam.</t>
+        </is>
+      </c>
+      <c r="F547" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G547" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265059/ada-konser-di-ancol-transjakarta-perpanjang-operasional</t>
+        </is>
+      </c>
+      <c r="H547" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/MMIPH39SWGGhu0j9JUXP5-xxLWc=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/5137785/original/055250800_1739961431-20250219-Penambahan_Jalur_Transjakarta-ANG_1.jpg</t>
+        </is>
+      </c>
+      <c r="I547" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>Polisi Buru Importir 995 Senjata yang Ditemukan di Sekolah Jaksel</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:55:17 +0700</t>
+        </is>
+      </c>
+      <c r="D548" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E548" t="inlineStr">
+        <is>
+          <t>Kuasa hukum mantan ketua yayasan mengklaim senjata itu untuk ekskul menembak.</t>
+        </is>
+      </c>
+      <c r="F548" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G548" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265057/polisi-buru-importir-995-senjata-yang-ditemukan-di-sekolah-jaksel</t>
+        </is>
+      </c>
+      <c r="H548" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/Fl_NzWIZKKZEWAlAQ_ZHoXsZU5g=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9317547/original/022307300_1786020542-WhatsApp_Image_2026-08-06_at_19.28.11.jpeg</t>
+        </is>
+      </c>
+      <c r="I548" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>Tren</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>2 Perempuan Ini Baru Tahu Tertukar Saat Lahir 37 Tahun Lalu, padahal Tinggal Berdekatan</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:30:53 +0700</t>
+        </is>
+      </c>
+      <c r="D549" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E549" t="inlineStr">
+        <is>
+          <t>Dua perempuan di China tertukar saat bayi dan baru ketahuan setelah 37 tahun lamanya. Ironisnya, rumah mereka cuma berjarak 4 kilometer saja.</t>
+        </is>
+      </c>
+      <c r="F549" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G549" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/tren/read/2026/08/08/153000765/2-perempuan-ini-baru-tahu-tertukar-saat-lahir-37-tahun-lalu-padahal-tinggal</t>
+        </is>
+      </c>
+      <c r="H549" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/TaAnG3l8yWfHc27eSu_LzkzssBo=/0x129:1493x1124/1200x675/filters:watermark(data/photo/2026/01/30/697c818d0ca91.png,0,-0,1)/data/photo/2026/07/30/6a6b1e8b5ce1c.jpg</t>
+        </is>
+      </c>
+      <c r="I549" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>Tren</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>Apakah di Indonesia Bisa Lihat Gerhana Matahari Tanggal 12 Agustus?</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:30:53 +0700</t>
+        </is>
+      </c>
+      <c r="D550" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E550" t="inlineStr">
+        <is>
+          <t>Pada tanggal 12 Agustus bakal ada gerhana matahari total yang diperkirakan sangat lama. Apakah di Indonesia bisa melihat fenomena ini?</t>
+        </is>
+      </c>
+      <c r="F550" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G550" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/tren/read/2026/08/08/150000665/apakah-di-indonesia-bisa-lihat-gerhana-matahari-tanggal-12-agustus-</t>
+        </is>
+      </c>
+      <c r="H550" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/SRTjpDo9rKieU5-cfZaxig9_zfI=/0x1:2000x1334/1200x675/filters:watermark(data/photo/2026/01/30/697c818d0ca91.png,0,-0,1)/data/photo/2026/04/09/69d76657605ba.webp</t>
+        </is>
+      </c>
+      <c r="I550" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>Tren</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>Jenderal AS Dorong Trump Akhiri Konflik Iran, Ini Risiko jika Perang Berlanjut</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:30:53 +0700</t>
+        </is>
+      </c>
+      <c r="D551" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E551" t="inlineStr">
+        <is>
+          <t>Jenderal AS mendorong pemerintahan Presiden Donald Trump mencari jalan keluar dari konflik dengan Iran yang terus berlarut.</t>
+        </is>
+      </c>
+      <c r="F551" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G551" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/tren/read/2026/08/08/143000065/jenderal-as-dorong-trump-akhiri-konflik-iran-ini-risiko-jika-perang</t>
+        </is>
+      </c>
+      <c r="H551" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/BxYI1c2ygW4K3JHL9_anU0SX97Q=/0x0:1964x1309/1200x675/filters:watermark(data/photo/2026/01/30/697c818d0ca91.png,0,-0,1)/data/photo/2026/08/07/6a75355247e5a.jpg</t>
+        </is>
+      </c>
+      <c r="I551" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I489"/>
+  <autoFilter ref="A1:I551"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-08 09:29 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-08.xlsx
+++ b/data/berita_2026-08-08.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$551</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$609</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I551"/>
+  <dimension ref="A1:I609"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -26333,8 +26333,2734 @@
         </is>
       </c>
     </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>OKI sambut baik perjanjian pertahanan antara Saudi, Turkiye, Pakistan</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:21:48 +0700</t>
+        </is>
+      </c>
+      <c r="D552" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E552" t="inlineStr">
+        <is>
+          <t>Organisasi Kerja Sama Islam (OKI), Jumat (7/8) menyambut baik penandatanganan Perjanjian Pertahanan Bersama Makkah ...</t>
+        </is>
+      </c>
+      <c r="F552" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G552" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685715/oki-sambut-baik-perjanjian-pertahanan-antara-saudi-turkiye-pakistan</t>
+        </is>
+      </c>
+      <c r="H552" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/Sekjen-OKI-Hissein-Brahim-Taha.jpg</t>
+        </is>
+      </c>
+      <c r="I552" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>Dinsos: Siswa SRMA 18 Blora mengalami peningkatan rasa percaya diri</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:17:07 +0700</t>
+        </is>
+      </c>
+      <c r="D553" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E553" t="inlineStr">
+        <is>
+          <t>Para siswa yang menempuh pendidikan di Sekolah Rakyat Menengah Atas (SRMA) 18 Blora, Jawa Tengah selama setahun ...</t>
+        </is>
+      </c>
+      <c r="F553" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G553" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685712/dinsos-siswa-srma-18-blora-mengalami-peningkatan-rasa-percayadiri</t>
+        </is>
+      </c>
+      <c r="H553" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/sekolah-rakyat-BLORA.jpg</t>
+        </is>
+      </c>
+      <c r="I553" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>Unhan: Industri pertahanan perlu sinergi kebijakan dan teknologi</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:13:42 +0700</t>
+        </is>
+      </c>
+      <c r="D554" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E554" t="inlineStr">
+        <is>
+          <t>Dosen Fakultas Teknologi Pertahanan Universitas Pertahanan (Unhan) Ade Muhammad menilai penguatan industri pertahanan ...</t>
+        </is>
+      </c>
+      <c r="F554" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G554" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685708/unhan-industri-pertahanan-perlu-sinergi-kebijakan-dan-teknologi</t>
+        </is>
+      </c>
+      <c r="H554" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/21-presidenri.go.id-Foto-BPMI-Setpres-Cahyo.jpeg</t>
+        </is>
+      </c>
+      <c r="I554" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>Bawaslu gandeng DPP LIRA siapkan 1.000 relawan pengawas Pemilu 2029</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:12:01 +0700</t>
+        </is>
+      </c>
+      <c r="D555" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E555" t="inlineStr">
+        <is>
+          <t>Badan Pengawas Pemilihan Umum (Bawaslu) RI menggandeng DPP Pemuda Lumbung Informasi Rakyat (LIRA) untuk memperkuat ...</t>
+        </is>
+      </c>
+      <c r="F555" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G555" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685707/bawaslu-gandeng-dpp-lira-siapkan-1000-relawan-pengawas-pemilu-2029</t>
+        </is>
+      </c>
+      <c r="H555" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001017587.jpg</t>
+        </is>
+      </c>
+      <c r="I555" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>ATR/BPN dorong musyawarah optimalkan penyelesaian sengketa tanah</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:10:09 +0700</t>
+        </is>
+      </c>
+      <c r="D556" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E556" t="inlineStr">
+        <is>
+          <t>Sekretaris Jenderal (Sekjen) Kementerian Agraria dan Tata Ruang/Badan Pertanahan Nasional (ATR/BPN) Dalu Agung Darmawan ...</t>
+        </is>
+      </c>
+      <c r="F556" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G556" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685705/atr-bpn-dorong-musyawarah-optimalkan-penyelesaian-sengketa-tanah</t>
+        </is>
+      </c>
+      <c r="H556" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/30/BPN-2_1.jpg</t>
+        </is>
+      </c>
+      <c r="I556" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>Buruh apresiasi Kapolri jembatani dialog terkait RUU Ketenagakerjaan</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:09:49 +0700</t>
+        </is>
+      </c>
+      <c r="D557" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E557" t="inlineStr">
+        <is>
+          <t>Koalisi Besar Perjuangan Buruh Indonesia (KBPBI) mengapresiasi Kapolri Jenderal Listyo Sigit Prabowo yang membuka ruang ...</t>
+        </is>
+      </c>
+      <c r="F557" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G557" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685704/buruh-apresiasi-kapolri-jembatani-dialog-terkait-ruu-ketenagakerjaan</t>
+        </is>
+      </c>
+      <c r="H557" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/WhatsApp-Image-2026-08-08-at-11.06.28-AM.jpeg</t>
+        </is>
+      </c>
+      <c r="I557" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>FBLB 2026 jadi ajang promosi budaya Papua Pegunungan</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:04:14 +0700</t>
+        </is>
+      </c>
+      <c r="D558" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E558" t="inlineStr">
+        <is>
+          <t>Wakil Menteri Pariwisata Ni Luh Puspa menyampaikan bahwa Festival Budaya Lembah Baliem (FBLB) 2026 merupakan ...</t>
+        </is>
+      </c>
+      <c r="F558" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G558" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685703/fblb-2026-jadi-ajang-promosi-budaya-papua-pegunungan</t>
+        </is>
+      </c>
+      <c r="H558" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/WhatsApp-Image-2026-08-08-at-13.01.24.jpeg</t>
+        </is>
+      </c>
+      <c r="I558" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>Manggala Agni tangani karhutla di Riau seluas 100 hektare lebih</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:59:56 +0700</t>
+        </is>
+      </c>
+      <c r="D559" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E559" t="inlineStr">
+        <is>
+          <t>Tim Manggala Agni Daerah Operasi Rengat masih menangani dua kebakaran hutan dan lahan (karhutla) di Kabupaten Pelalawan ...</t>
+        </is>
+      </c>
+      <c r="F559" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G559" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685701/manggala-agni-tangani-karhutla-di-riau-seluas-100-hektare-lebih</t>
+        </is>
+      </c>
+      <c r="H559" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000700950.jpg</t>
+        </is>
+      </c>
+      <c r="I559" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>Latih kedisiplinan siswa, Sekolah Rakyat Kupang libatkan Taruna Akmil</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:58:53 +0700</t>
+        </is>
+      </c>
+      <c r="D560" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E560" t="inlineStr">
+        <is>
+          <t>ANTARA - Ratusan siswa-siswi Sekolah Rakyat Terintegrasi I Kabupaten Kupang dari jenjang SD, SMP, hingga SMA, pada ...</t>
+        </is>
+      </c>
+      <c r="F560" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G560" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5685640/latih-kedisiplinan-siswa-sekolah-rakyat-kupang-libatkan-taruna-akmil</t>
+        </is>
+      </c>
+      <c r="H560" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/LATIH-KEDISIPLINAN-SISWA-SEKOLAH-RAKYAT-KUPANG-LIBATKAN-TARUNA-AKMIL.jpg</t>
+        </is>
+      </c>
+      <c r="I560" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>Rycko Menoza: Literasi politik harus dilakukan berkelanjutan</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:56:49 +0700</t>
+        </is>
+      </c>
+      <c r="D561" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E561" t="inlineStr">
+        <is>
+          <t>Anggota Komisi II DPR RI Rycko Menoza mendorong sosialisasi dan literasi politik dilakukan secara berkelanjutan untuk ...</t>
+        </is>
+      </c>
+      <c r="F561" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G561" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685697/rycko-menoza-literasi-politik-harus-dilakukan-berkelanjutan</t>
+        </is>
+      </c>
+      <c r="H561" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG-20260808-WA0007.jpg</t>
+        </is>
+      </c>
+      <c r="I561" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>Disdukcapil Batam beri 420 kuota KIA gratis dalam rangkaian HAN</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:53:22 +0700</t>
+        </is>
+      </c>
+      <c r="D562" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E562" t="inlineStr">
+        <is>
+          <t>ANTARA - Dinas Kependudukan dan Pencatatan Sipil (Disdukcapil) Kota Batam, Kepulauan Riau membuka 420 kuota Kartu ...</t>
+        </is>
+      </c>
+      <c r="F562" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G562" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5685580/disdukcapil-batam-beri-420-kuota-kia-gratis-dalam-rangkaian-han</t>
+        </is>
+      </c>
+      <c r="H562" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AYM_DISDUKCAPIL-BATAM-BERI-420-KUOTA.jpg</t>
+        </is>
+      </c>
+      <c r="I562" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>Rycko Menoza dorong edukasi politik di perkotaan diperluas</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:49:19 +0700</t>
+        </is>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E563" t="inlineStr">
+        <is>
+          <t>Anggota Komisi II DPR RI Rycko Menoza mendorong perluasan edukasi politik di kawasan perkotaan untuk meningkatkan ...</t>
+        </is>
+      </c>
+      <c r="F563" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G563" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685689/rycko-menoza-dorong-edukasi-politik-di-perkotaan-diperluas</t>
+        </is>
+      </c>
+      <c r="H563" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG-20260808-WA0009.jpg</t>
+        </is>
+      </c>
+      <c r="I563" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>Peneliti gunakan AI untuk merancang bakteriofag antibakteri</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:43:07 +0700</t>
+        </is>
+      </c>
+      <c r="D564" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E564" t="inlineStr">
+        <is>
+          <t>Kecerdasan Buatan (AI) telah digunakan oleh tim peneliti di Amerika Serikat untuk merancang genom lengkap untuk ...</t>
+        </is>
+      </c>
+      <c r="F564" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G564" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685688/peneliti-gunakan-ai-untuk-merancang-bakteriofag-antibakteri</t>
+        </is>
+      </c>
+      <c r="H564" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/CjkinzN000031_20260807_CBMFN0A001.jpeg</t>
+        </is>
+      </c>
+      <c r="I564" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>"Trio" produk teknologi dorong pertumbuhan ekspor China</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:37:57 +0700</t>
+        </is>
+      </c>
+      <c r="D565" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E565" t="inlineStr">
+        <is>
+          <t>Robot, produk terkait AI, dan obat-obatan inovatif muncul sebagai pendorong baru pertumbuhan ekspor China, seiring ...</t>
+        </is>
+      </c>
+      <c r="F565" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G565" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685687/trio-produk-teknologi-dorong-pertumbuhan-ekspor-china</t>
+        </is>
+      </c>
+      <c r="H565" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/17/Konferensi-Kecerdasan-Buatan-Dunia-di-Shanghai-170726-dln-9.jpg</t>
+        </is>
+      </c>
+      <c r="I565" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>Indonesia hadapi tuan rumah Jepang di voli putri Asian Games 2026</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:37:34 +0700</t>
+        </is>
+      </c>
+      <c r="D566" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E566" t="inlineStr">
+        <is>
+          <t>Tim nasional bola voli putri Indonesia akan menghadapi tuan rumah Jepang pada fase grup Asian Games Aichi-Nagoya 2026 ...</t>
+        </is>
+      </c>
+      <c r="F566" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G566" t="inlineStr">
+        <is>
+          <t>https://asiangames.antaranews.com/berita/5685684/indonesia-hadapi-tuan-rumah-jepang-di-voli-putri-asian-games-2026</t>
+        </is>
+      </c>
+      <c r="H566" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/12/15/indonesia-raih-medali-perunggu-volly-putri-sea-games-2025-2690821.jpg</t>
+        </is>
+      </c>
+      <c r="I566" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>Tabrak dua pemotor, mobil diamuk massa di Jakbar</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:34:26 +0700</t>
+        </is>
+      </c>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E567" t="inlineStr">
+        <is>
+          <t>Mobil bernomor polisi B-232-WL menjadi sasaran amuk massa usai menabrak dua pemotor di Jalan Wijaya I, Grogol ...</t>
+        </is>
+      </c>
+      <c r="F567" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G567" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685680/tabrak-dua-pemotor-mobil-diamuk-massa-di-jakbar</t>
+        </is>
+      </c>
+      <c r="H567" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2020/04/20/ilustrasi-kecelakaan-motor_copy_800x533.jpg</t>
+        </is>
+      </c>
+      <c r="I567" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>Film "Kuasa Gelap: Perjanjian Darah" akan hadir dalam format IMAX</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:34:24 +0700</t>
+        </is>
+      </c>
+      <c r="D568" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E568" t="inlineStr">
+        <is>
+          <t>Film horor "Kuasa Gelap: Perjanjian Darah" akan ditayangkan di bioskop mulai 8 Oktober 2026 dalam ...</t>
+        </is>
+      </c>
+      <c r="F568" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G568" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685676/film-kuasa-gelap-perjanjian-darah-akan-hadir-dalam-format-imax</t>
+        </is>
+      </c>
+      <c r="H568" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG_2168.jpeg</t>
+        </is>
+      </c>
+      <c r="I568" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>Mendukbangga: Program Genting bantu rumah layak huni keluarga stunting</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:34:12 +0700</t>
+        </is>
+      </c>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E569" t="inlineStr">
+        <is>
+          <t>Menteri Kependudukan dan Pembangunan Keluarga (Mendukbangga)/Kepala BKKBN Wihaji mengatakan Program Gerakan Orang Tua ...</t>
+        </is>
+      </c>
+      <c r="F569" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G569" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685672/mendukbangga-program-genting-bantu-rumah-layak-huni-keluarga-stunting</t>
+        </is>
+      </c>
+      <c r="H569" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/upscalemedia-transformed-9.jpeg</t>
+        </is>
+      </c>
+      <c r="I569" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>Voli putra Indonesia masuk grup berat bersama Iran di Asian Games 2026</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:31:25 +0700</t>
+        </is>
+      </c>
+      <c r="D570" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E570" t="inlineStr">
+        <is>
+          <t>Tim nasional bola voli putra Indonesia akan menghadapi juara bertahan Iran pada fase grup Asian Games Aichi-Nagoya 2026 ...</t>
+        </is>
+      </c>
+      <c r="F570" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G570" t="inlineStr">
+        <is>
+          <t>https://asiangames.antaranews.com/berita/5685668/voli-putra-indonesia-masuk-grup-berat-bersama-iran-di-asian-games-2026</t>
+        </is>
+      </c>
+      <c r="H570" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/26/sea-v-cup-2026-indonesia-kalahkan-kamboja-2828433.jpg</t>
+        </is>
+      </c>
+      <c r="I570" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>Sebanyak 65 personel damkar padamkan kebakaran rumah dekat Terminal UKI</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:30:39 +0700</t>
+        </is>
+      </c>
+      <c r="D571" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E571" t="inlineStr">
+        <is>
+          <t>Sebanyak 65 personel Suku Dinas Penanggulangan Kebakaran dan Penyelamatan (Gulkarmat) Jakarta Timur (Jaktim) masih ...</t>
+        </is>
+      </c>
+      <c r="F571" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G571" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685664/sebanyak-65-personel-damkar-padamkan-kebakaran-rumah-dekat-terminal-uki</t>
+        </is>
+      </c>
+      <c r="H571" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/InShot_20260808_151408040.jpg</t>
+        </is>
+      </c>
+      <c r="I571" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>Sekjen ATR/BPN: Pemetaan bidang tanah perkuat tata kelola pertanahan</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:28:33 +0700</t>
+        </is>
+      </c>
+      <c r="D572" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E572" t="inlineStr">
+        <is>
+          <t>Sekretaris Jenderal (Sekjen) Kementerian Agraria dan Tata Ruang/Badan Pertanahan Nasional (ATR/BPN) Dalu Agung Darmawan ...</t>
+        </is>
+      </c>
+      <c r="F572" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G572" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685660/sekjen-atr-bpn-pemetaan-bidang-tanah-perkuat-tata-kelola-pertanahan</t>
+        </is>
+      </c>
+      <c r="H572" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/30/WhatsApp-Image-2026-06-27-at-10.52.00.jpeg</t>
+        </is>
+      </c>
+      <c r="I572" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>BPIP: Satu siswa Sekolah Rakyat jadi calon Paskibraka nasional</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:26:40 +0700</t>
+        </is>
+      </c>
+      <c r="D573" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E573" t="inlineStr">
+        <is>
+          <t>Wakil Kepala Badan Pembinaan Ideologi Pancasila (BPIP) Rima Agristina mengatakan seorang siswa Sekolah Rakyat untuk ...</t>
+        </is>
+      </c>
+      <c r="F573" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G573" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685656/bpip-satu-siswa-sekolah-rakyat-jadi-calon-paskibraka-nasional</t>
+        </is>
+      </c>
+      <c r="H573" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000035106.jpg</t>
+        </is>
+      </c>
+      <c r="I573" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>Kapolres Metro Depok Ziarah ke Makam Jenderal Hoegeng dan Eyang Meri</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:16:58 +0700</t>
+        </is>
+      </c>
+      <c r="D574" t="inlineStr">
+        <is>
+          <t>Herianto Batubara</t>
+        </is>
+      </c>
+      <c r="E574" t="inlineStr">
+        <is>
+          <t>Kapolres Metro Depok, Kombes Rony, berziarah ke makam Jenderal Hoegeng. Ia berharap keteladanan Hoegeng jadi motivasi dalam tugasnya melayani masyarakat.</t>
+        </is>
+      </c>
+      <c r="F574" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G574" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609955/kapolres-metro-depok-ziarah-ke-makam-jenderal-hoegeng-dan-eyang-meri</t>
+        </is>
+      </c>
+      <c r="H574" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/kapolres-depok-1786180424720_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I574" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>Command Center Dishub Dipindah ke MT Haryono Imbas Kebakaran Gedung Bapenda</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:14:03 +0700</t>
+        </is>
+      </c>
+      <c r="D575" t="inlineStr">
+        <is>
+          <t>Brigitta Belia Permata Sari</t>
+        </is>
+      </c>
+      <c r="E575" t="inlineStr">
+        <is>
+          <t>Kebakaran di gedung Bapenda DKI Jakarta berdampak pada ruang pengendalian lalu lintas. Dishub DKI akan memindahkan Command Center ke Pusdatin MT Haryono.</t>
+        </is>
+      </c>
+      <c r="F575" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G575" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609940/command-center-dishub-dipindah-ke-mt-haryono-imbas-kebakaran-gedung-bapenda</t>
+        </is>
+      </c>
+      <c r="H575" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/gedung-bapenda-dki-dipasangi-garis-polisi-1786162667826_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I575" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>Kebakaran di Gedung Bapenda DKI Padam, Lalin Kembali Dibuka</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:12:57 +0700</t>
+        </is>
+      </c>
+      <c r="D576" t="inlineStr">
+        <is>
+          <t>Brigitta Belia Permata Sari</t>
+        </is>
+      </c>
+      <c r="E576" t="inlineStr">
+        <is>
+          <t>Kebakaran di Gedung Badan Pendapatan Daerah (Bapenda) DKI Jakarta padam. Lalu lintas (lalin) di Jalan Abdul Muis, Jakarta Pusat, kembali dibuka.</t>
+        </is>
+      </c>
+      <c r="F576" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G576" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609939/kebakaran-di-gedung-bapenda-dki-padam-lalin-kembali-dibuka</t>
+        </is>
+      </c>
+      <c r="H576" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/kebakaran-di-gedung-badan-pendapatan-daerah-bapenda-dki-jakarta-padam-lalu-lintas-lalin-di-jalan-abdul-muis-jakarta-pusat-kemb-1786180252639_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I576" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>E-Sports Kapolri Cup 2026 Digelar, Wakapolri Harap Anak Muda Jadi Talenta Digital</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:00:44 +0700</t>
+        </is>
+      </c>
+      <c r="D577" t="inlineStr">
+        <is>
+          <t>Wildan Noviansah</t>
+        </is>
+      </c>
+      <c r="E577" t="inlineStr">
+        <is>
+          <t>Kapolri Cup 2026 dibuka di Jakarta, diikuti 35.936 peserta. Kompetisi ini mendukung pengembangan talenta digital dan sportivitas di kalangan generasi muda.</t>
+        </is>
+      </c>
+      <c r="F577" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G577" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609922/e-sports-kapolri-cup-2026-digelar-wakapolri-harap-anak-muda-jadi-talenta-digital</t>
+        </is>
+      </c>
+      <c r="H577" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/kapolri-cup-2026-dibuka-di-jakarta-diikuti-35936-peserta-dokistimewa-1786179572532_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I577" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>Pengedar Obat Keras di Tangerang Diringkus, Ribuan Hexymer-Tramadol Disita</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:30:14 +0700</t>
+        </is>
+      </c>
+      <c r="D578" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E578" t="inlineStr">
+        <is>
+          <t>Polsek Neglasari membongkar peredaran obat keras ilegal di wilayah Neglasari, Kota Tangerang. Pengedar obat keras ilegal berinisial AF (26) ditangkap.</t>
+        </is>
+      </c>
+      <c r="F578" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G578" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609899/pengedar-obat-keras-di-tangerang-diringkus-ribuan-hexymer-tramadol-disita</t>
+        </is>
+      </c>
+      <c r="H578" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/polsek-neglasari-membongkar-peredaran-obat-keras-ilegal-di-wilayah-neglasari-kota-tangerang-pengedar-obat-keras-ilegal-berinis-1786177763977_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I578" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>Viral Mobil Diduga Tabrak Lari di Kemang Kabur ke Tol, Polisi Selidiki</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:26:14 +0700</t>
+        </is>
+      </c>
+      <c r="D579" t="inlineStr">
+        <is>
+          <t>Mulia Budi</t>
+        </is>
+      </c>
+      <c r="E579" t="inlineStr">
+        <is>
+          <t>Sebuah video viral menunjukkan mobil diduga tabrak lari di Kemang, Jakarta. Polisi selidiki kejadian ini setelah korban melapor dan mengalami luka ringan.</t>
+        </is>
+      </c>
+      <c r="F579" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G579" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609894/viral-mobil-diduga-tabrak-lari-di-kemang-kabur-ke-tol-polisi-selidiki</t>
+        </is>
+      </c>
+      <c r="H579" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2016/10/31/9fc3e56b-737f-44f3-b5a1-fe60c7308267_169.jpg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I579" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>Kompolnas Ingatkan Adanya Larangan Propaganda Kekerasan di Ruang Digital</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:02:32 +0700</t>
+        </is>
+      </c>
+      <c r="D580" t="inlineStr">
+        <is>
+          <t>Anggi Muliawati</t>
+        </is>
+      </c>
+      <c r="E580" t="inlineStr">
+        <is>
+          <t>Komisioner Kompolnas Choirul Anam mengatakan kebebasan berekspresi dilindungi konstitusi dan UU. Namun, dia mengingatkan kebebasan tetap memiliki batasan.</t>
+        </is>
+      </c>
+      <c r="F580" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G580" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609870/kompolnas-ingatkan-adanya-larangan-propaganda-kekerasan-di-ruang-digital</t>
+        </is>
+      </c>
+      <c r="H580" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/07/09/komisioner-kompolnas-choirul-anam-rumondangdetikcom-1752074951783_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I580" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>Korban Kebakaran Gedung Bapenda DKI Masih Dirawat, Alami Sesak Napas</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 10:59:47 +0700</t>
+        </is>
+      </c>
+      <c r="D581" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E581" t="inlineStr">
+        <is>
+          <t>Polda Metro Jaya mengungkapkan kondisi terkini korban kebakaran gedung Badan Pendapatan Daerah (Bapenda) DKI Jakarta.</t>
+        </is>
+      </c>
+      <c r="F581" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G581" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609611/korban-kebakaran-gedung-bapenda-dki-masih-dirawat-alami-sesak-napas</t>
+        </is>
+      </c>
+      <c r="H581" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/potret-kobaran-api-mengamuk-di-gedung-bapenda-dki-1786160999327_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I581" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>Mahasiswa Curhat Beras di Alor Tembus Rp 30.000/Kg, Mentan Turun Tangan</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:43:19 +0700</t>
+        </is>
+      </c>
+      <c r="D582" t="inlineStr">
+        <is>
+          <t>Heri Purnomo</t>
+        </is>
+      </c>
+      <c r="E582" t="inlineStr">
+        <is>
+          <t>Beras sudah aman, ada di gudang-gudang sekarang. Harga itu Rp 13.000, sama dengan harga Jakarta. Kita sekarang tidak akan kesulitan beras, ujar Amran.</t>
+        </is>
+      </c>
+      <c r="F582" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G582" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8609906/mahasiswa-curhat-beras-di-alor-tembus-rp-30-000-kg-mentan-turun-tangan</t>
+        </is>
+      </c>
+      <c r="H582" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/menteri-pertanian-mentan-andi-amran-sulaiman-1786178494091_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I582" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>Hadapi Kasasi Rizky Febian, Teddy Pardiyana Tetap Tenang dan Buka Pintu Mediasi</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:28:27 +0700</t>
+        </is>
+      </c>
+      <c r="D583" t="inlineStr">
+        <is>
+          <t>Febryantino Nur Pratama</t>
+        </is>
+      </c>
+      <c r="E583" t="inlineStr">
+        <is>
+          <t>Teddy Pardiyana tetap tenang menghadapi kasasi Rizky Febian dalam sengketa ahli waris Lina Jubaedah. Dia buka pintu mediasi untuk penyelesaian kekeluargaan.</t>
+        </is>
+      </c>
+      <c r="F583" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G583" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8609896/hadapi-kasasi-rizky-febian-teddy-pardiyana-tetap-tenang-dan-buka-pintu-mediasi</t>
+        </is>
+      </c>
+      <c r="H583" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/30/rizky-febian-1785413128625_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I583" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>Agenda Padat Chelsea di Indonesia dan Malaysia, The Blues 2 Hari 2 Pertandingan</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:17:22 +0700</t>
+        </is>
+      </c>
+      <c r="D584" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E584" t="inlineStr">
+        <is>
+          <t>Chelsea akan menjalani dua pertandingan dalam kurun waktu dua hari saja saat berada di Indonesia dan Malaysia pada akhir pekan ini.</t>
+        </is>
+      </c>
+      <c r="F584" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G584" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865762/agenda-padat-chelsea-di-indonesia-dan-malaysia-the-blues-2-hari-2-pertandingan</t>
+        </is>
+      </c>
+      <c r="H584" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/XMCQ777aoYfv890swQKzeDNaU1M=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Logo-klub-Liga-Inggris-Chelsea.jpg</t>
+        </is>
+      </c>
+      <c r="I584" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>Anggota Komisi III DPR Desak Pelaku Pembunuhan Bocah 6 Tahun di Tapsel Dihukum Maksimal</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:12:18 +0700</t>
+        </is>
+      </c>
+      <c r="D585" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E585" t="inlineStr">
+        <is>
+          <t>Anggota Komisi III DPR meminta tersangka pembunuhan bocah enam tahun di Tapsel dihukum maksimal, termasuk seumur hidup.</t>
+        </is>
+      </c>
+      <c r="F585" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G585" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865761/anggota-komisi-iii-dpr-desak-pelaku-pembunuhan-bocah-6-tahun-di-tapsel-dihukum-maksimal</t>
+        </is>
+      </c>
+      <c r="H585" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/UN6gcElZutWh6QRVeLvhSWcY7yU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Anggota-Komisi-III-DPR-RI-Soedeson-Tandra-dalam-rapat-di-Komisi-III-DPR-RI.jpg</t>
+        </is>
+      </c>
+      <c r="I585" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>Bukan Sekedar Mobil Listrik, MGS5 EV Hadir Sebagai SUV Keluarga yang Serba Bisa</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:11:56 +0700</t>
+        </is>
+      </c>
+      <c r="D586" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E586" t="inlineStr">
+        <is>
+          <t>Hadir sebagai SUV listrik, MGS5 EV tidak hanya menawarkan tenaga dan jarak tempuh, tetapi juga mengedepankan kenyamanan mobilitas sehari-hari.</t>
+        </is>
+      </c>
+      <c r="F586" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G586" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/otomotif/7865760/bukan-sekedar-mobil-listrik-mgs5-ev-hadir-sebagai-suv-keluarga-yang-serba-bisa</t>
+        </is>
+      </c>
+      <c r="H586" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/INKs-v1pvXHXbbx3basqKn0lv8Q=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/MGS5-EV-tampil-di-GIIAS-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I586" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>KH Ma’ruf Amin Ingatkan Warga NU Jangan Rebutan Tambang: Hati-hati Terjerat</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:06:39 +0700</t>
+        </is>
+      </c>
+      <c r="D587" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E587" t="inlineStr">
+        <is>
+          <t>KH Ma’ruf Amin meminta warga Nahdliyin untuk tidak berebut dalam pengelolaan tambang.</t>
+        </is>
+      </c>
+      <c r="F587" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G587" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865759/kh-maruf-amin-ingatkan-warga-nu-jangan-rebutan-tambang-hati-hati-terjerat</t>
+        </is>
+      </c>
+      <c r="H587" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ftM2eMpf0zZpnHxzfe99mRk-qbg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Maruf-Amin-dalam-Halaqah-Kebangsaan-dan-Qanun-Asasi-di-Gedung-MPR-RI-Jakarta.jpg</t>
+        </is>
+      </c>
+      <c r="I587" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>Jadwal Acara TV Minggu, 9 Agustus 2026: Upin dan Ipin di MNC TV,  Primetime News di Metro TV</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:05:04 +0700</t>
+        </is>
+      </c>
+      <c r="D588" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E588" t="inlineStr">
+        <is>
+          <t>Simak jadwal acara TV Minggu, 9 Agustus 2026, terdapat tayangan Upin &amp; Ipin di MNC TV,  dan Primetime News di Metro TV.</t>
+        </is>
+      </c>
+      <c r="F588" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G588" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7865758/jadwal-acara-tv-minggu-9-agustus-2026-upin-ipin-di-mnc-tv-primetime-news-di-metro-tv</t>
+        </is>
+      </c>
+      <c r="H588" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Fl8aETmbMmkOkLsjx-fRlfD8IZo=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Ilustrasi-Televisi-digital.jpg</t>
+        </is>
+      </c>
+      <c r="I588" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>Tak Ada Itikad Baik dari Karyawan soal Kasus Pencurian, Tasyi Athasyia Tegas Tempuh Langkah Hukum</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:04:17 +0700</t>
+        </is>
+      </c>
+      <c r="D589" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E589" t="inlineStr">
+        <is>
+          <t>Tak ada itikad baik dari karyawan soal kasus pencurian, Tasyi Athasyia tegas menempuh langkah hukum.</t>
+        </is>
+      </c>
+      <c r="F589" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G589" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7865757/tak-ada-itikad-baik-dari-karyawan-soal-kasus-pencurian-tasyi-athasyia-tegas-tempuh-langkah-hukum</t>
+        </is>
+      </c>
+      <c r="H589" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/qa3hJrJieEFbvAcNsStLKCuUrUs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Tasyi-Athasyia-berikan-klarifikasi-usai-dituding-jatuhkan-produk-UMKM.jpg</t>
+        </is>
+      </c>
+      <c r="I589" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>Perkuat Ketahanan Pesisir, 10.000 Mangrove Ditanam di Kawasan Konservasi Simbar Segara Bali</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:02:42 +0700</t>
+        </is>
+      </c>
+      <c r="D590" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E590" t="inlineStr">
+        <is>
+          <t>Program di Bali melanjutkan komitmen BTN dalam rehabilitasi ekosistem pesisir.</t>
+        </is>
+      </c>
+      <c r="F590" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G590" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865756/perkuat-ketahanan-pesisir-10000-mangrove-ditanam-di-kawasan-konservasi-simbar-segara-bali</t>
+        </is>
+      </c>
+      <c r="H590" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/zUKQhluZqRsWsgkhGe39F0uVs3U=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Kegiatan-ini-merupakan-upa-mberdayaan-masyarakat.jpg</t>
+        </is>
+      </c>
+      <c r="I590" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>APPI Dorong UMKM Sektor Pengelasan Naik Kelas dan Berdaya Saing</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:00:05 +0700</t>
+        </is>
+      </c>
+      <c r="D591" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E591" t="inlineStr">
+        <is>
+          <t>Asosiasi Pengusaha Pengelasan Indonesia (APPI) resmi dideklarasikan sebagai wadah pemersatu pengusaha pengelasan di Indonesia.</t>
+        </is>
+      </c>
+      <c r="F591" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G591" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/bisnis/7865755/appi-dorong-umkm-sektor-pengelasan-naik-kelas-dan-berdaya-saing</t>
+        </is>
+      </c>
+      <c r="H591" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/649-ZkOSiOFXM2r7cvzMoaaueRE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Deklarasi-APPI-di-Jakarta-OK.jpg</t>
+        </is>
+      </c>
+      <c r="I591" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>Sosok Candra Waskito, Bos Royal Phone Ambarawa Tewas Dirampok, Dikenal Dermawan Semasa Hidup</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:54:48 +0700</t>
+        </is>
+      </c>
+      <c r="D592" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E592" t="inlineStr">
+        <is>
+          <t>Bos Royal Phone Ambarawa Candra Waskito tewas dirampok, dikenal dermawan; polisi menangkap dua terduga pelaku.</t>
+        </is>
+      </c>
+      <c r="F592" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G592" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865754/sosok-candra-waskito-bos-royal-phone-ambarawa-tewas-dirampok-dikenal-dermawan-semasa-hidup</t>
+        </is>
+      </c>
+      <c r="H592" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/7ZZnVepqeCk6txc4fbmLp3oj0rQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Sosok-Candra-Waskito-Bos-Royal-Phone-Ambarawa-Tewas-Dirampok-Dikenal-Dermawan-Semasa-Hidup.jpg</t>
+        </is>
+      </c>
+      <c r="I592" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>Tanggal 9 Agustus 2026 Memperingati Hari Apa? Ada 2 Momen Penting, Ini Sejarahnya</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:52:40 +0700</t>
+        </is>
+      </c>
+      <c r="D593" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E593" t="inlineStr">
+        <is>
+          <t>Tanggal 9 Agustus 2026 memperingati 2 momen penting yaitu Hari Internasional Masyarakat Adat Sedunia dan International Coworking Day.</t>
+        </is>
+      </c>
+      <c r="F593" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G593" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865753/tanggal-9-agustus-2026-memperingati-hari-apa-ada-2-momen-penting-ini-sejarahnya</t>
+        </is>
+      </c>
+      <c r="H593" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/DMOWcyUjfqbjRs71IwHZ5k8wfdI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Kalender-Peringatan-9-Agustus-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I593" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>Prakiraan Cuaca Kota Ternate Minggu, 9 Agustus 2026: Mayoritas Berawan</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:50:03 +0700</t>
+        </is>
+      </c>
+      <c r="D594" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E594" t="inlineStr">
+        <is>
+          <t>Badan Meteorologi, Klimatologi, dan Geofisika (BMKG) merilis prakiraan cuaca wilayah Kota Ternate, Maluku Utara untuk Minggu (9/8/2026).</t>
+        </is>
+      </c>
+      <c r="F594" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G594" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865752/prakiraan-cuaca-kota-ternate-minggu-9-agustus-2026-mayoritas-berawan</t>
+        </is>
+      </c>
+      <c r="H594" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/rA2XTU7bmVbPNWwiiQweBmhopvE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/cuaca-ternate-ilustrasi.jpg</t>
+        </is>
+      </c>
+      <c r="I594" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>Menjajal MG ZS Hybrid+ Rp299 Jutaan: Tarikan Responsif, Nyaman Buat Harian</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:48:57 +0700</t>
+        </is>
+      </c>
+      <c r="D595" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E595" t="inlineStr">
+        <is>
+          <t>MG ZS Hybrid+ menawarkan kombinasi yang cukup menarik bagi konsumen yang mencari SUV hybrid untuk kebutuhan sehari-hari. Ini keunggulannya!</t>
+        </is>
+      </c>
+      <c r="F595" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G595" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/otomotif/7865751/menjajal-mg-zs-hybrid-rp299-jutaan-tarikan-responsif-nyaman-buat-harian</t>
+        </is>
+      </c>
+      <c r="H595" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/PyE-G-DxsONXczwStcuGUAEnQQM=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/MG-ZS-Hybrid.jpg</t>
+        </is>
+      </c>
+      <c r="I595" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>Eks Timnas: Skuad Voli Indonesia untuk Asian Games 2026 Sudah Oke, Sayangnya Tak Ada Doni</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:47:13 +0700</t>
+        </is>
+      </c>
+      <c r="D596" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E596" t="inlineStr">
+        <is>
+          <t>Eks Timnas Voli Putra Indonesia Erwin Rusni sayangkan Doni Haryono tidak masuk skuad Pelatnas Asian Games 2026 karena cedera.</t>
+        </is>
+      </c>
+      <c r="F596" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G596" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7865750/eks-timnas-skuad-voli-indonesia-untuk-asian-games-2026-sudah-oke-sayangnya-tak-ada-doni</t>
+        </is>
+      </c>
+      <c r="H596" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/TIEZk8S1BH2paU67L_kFfn2UGlo=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Timnas-Voli-Putra-Indonesia-foto-bersama-setelah-mengalahkan-Kamboja.jpg</t>
+        </is>
+      </c>
+      <c r="I596" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>MU Siap Tebus Klausul Bek Muda Timnas Spanyol Incaran Barcelona, Berpotensi Hijrah ke Old Trafford</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:46:35 +0700</t>
+        </is>
+      </c>
+      <c r="D597" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E597" t="inlineStr">
+        <is>
+          <t>MU siap menebus klausul 16 juta euro Jorge Salinas, sementara Barcelona keberatan membayar. Bek 19 tahun itu berpotensi hijrah ke Old Trafford.</t>
+        </is>
+      </c>
+      <c r="F597" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G597" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865749/mu-siap-tebus-klausul-bek-muda-timnas-spanyol-incaran-barcelona-berpotensi-hijrah-ke-old-trafford</t>
+        </is>
+      </c>
+      <c r="H597" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/zTibrEclfl4_bQZMLWSrNWRPlnc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Bek-muda-asal-Spanyol-Jorge-Salinas-diminati-oleh-Manchester-United.jpg</t>
+        </is>
+      </c>
+      <c r="I597" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>950 Dapur MBG Belum Penuhi Standar, BGN Beri Batas Waktu Hingga 10 Agustus</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:39:42 +0700</t>
+        </is>
+      </c>
+      <c r="D598" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E598" t="inlineStr">
+        <is>
+          <t>Sekitar 950 dapur MBG disebut belum memenuhi standar higiene dan sanitasi. BGN memberi waktu hingga 10 Agustus untuk berbenah.</t>
+        </is>
+      </c>
+      <c r="F598" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G598" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865748/950-dapur-mbg-belum-penuhi-standar-bgn-beri-batas-waktu-hingga-10-agustus</t>
+        </is>
+      </c>
+      <c r="H598" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/7awaG9H39EsF1vhf_ex71vxProQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Kepala-BGN-Sudaryono-dalam-konferensi-pers-di-kantor-BGN.jpg</t>
+        </is>
+      </c>
+      <c r="I598" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>Cerita Warga Detik-detik Kebakaran Gedung Bapenda DKI: Panik Evakuasi Anak, Takut SPBU Meledak</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:36:45 +0700</t>
+        </is>
+      </c>
+      <c r="D599" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E599" t="inlineStr">
+        <is>
+          <t>Fauzah mengaku panik dan langsung membawa anaknya menyelamatkan diri setelah melihat api membesar.</t>
+        </is>
+      </c>
+      <c r="F599" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G599" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7865747/cerita-warga-detik-detik-kebakaran-gedung-bapenda-dki-panik-evakuasi-anak-takut-spbu-meledak</t>
+        </is>
+      </c>
+      <c r="H599" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/kn14NvzcN26yqxVmrx_J8CF8nEg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Bapenda-DKI-Jakarta.jpg</t>
+        </is>
+      </c>
+      <c r="I599" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>Pimpinan MPR Ziarah ke Makam Bung Hatta, Ahmad Muzani: Momentum Mengenang Jasa Beliau</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:31:19 +0700</t>
+        </is>
+      </c>
+      <c r="D600" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E600" t="inlineStr">
+        <is>
+          <t>Pimpinan MPR RI melakukan ziarah ke makam Wakil Presiden pertama RI, Bung Hatta, sebagai momen untuk mereflesikan kemerdekaan Indonesia.</t>
+        </is>
+      </c>
+      <c r="F600" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G600" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kilas-kementerian/7865746/pimpinan-mpr-ziarah-ke-makam-bung-hatta-ahmad-muzani-momentum-mengenang-jasa-beliau</t>
+        </is>
+      </c>
+      <c r="H600" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/hZUzdBOG8pJwBa_yg-H7XkfhKiQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Pimpinan-MPR-ziarah-ke-makam-Bung-Hatta.jpg</t>
+        </is>
+      </c>
+      <c r="I600" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>Jelajah Bumi Sriwijaya, Presiden PKS Ngirup Cuko hingga Jajal Minisoccer di Palembang</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:27:33 +0700</t>
+        </is>
+      </c>
+      <c r="D601" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E601" t="inlineStr">
+        <is>
+          <t>Presiden PKS menjangkau warga Palembang lewat diskusi kebangsaan, laga minisoccer, hingga tradisi ngirup cuko di tepian Sungai Musi</t>
+        </is>
+      </c>
+      <c r="F601" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G601" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865745/jelajah-bumi-sriwijaya-presiden-pks-ngirup-cuko-hingga-jajal-minisoccer-di-palembang</t>
+        </is>
+      </c>
+      <c r="H601" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/tKe9wZjYdWAVZLQO-DfScKpYYys=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Almuzzammil-Yusuf-AMY.jpg</t>
+        </is>
+      </c>
+      <c r="I601" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>Prakiraan Cuaca Flores Besok Minggu, 9 Agustus 2026: Bajawa Diprediksi Cerah Berawan hingga Sejuk</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:20:43 +0700</t>
+        </is>
+      </c>
+      <c r="D602" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E602" t="inlineStr">
+        <is>
+          <t>Berikut detail prakiraan cuaca di beberapa kota terkenal di Flores untuk Minggu (9/8/2026)</t>
+        </is>
+      </c>
+      <c r="F602" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G602" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865744/prakiraan-cuaca-flores-besok-minggu-9-agustus-2026-bajawa-diprediksi-cerah-berawan-hingga-sejuk</t>
+        </is>
+      </c>
+      <c r="H602" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/O75JEKcTby2l9d_rvWB1HpXkxLY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Bukit-Avatar-di-Bajawa-Kabupaten-Ngada-Pulau-Flores-Nusa-Tenggara-Timur.jpg</t>
+        </is>
+      </c>
+      <c r="I602" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>Pertanian</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>Mentan Batalkan Rapat di Jakarta demi Tindaklanjuti Aspirasi Mahasiswa Alor</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:10:00 +0700</t>
+        </is>
+      </c>
+      <c r="D603" t="inlineStr">
+        <is>
+          <t>Friska Yolandha</t>
+        </is>
+      </c>
+      <c r="E603" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- Menteri Pertanian (Mentan) Andi Amran Sulaiman membatalkan agenda rapat pimpinan di Jakarta untuk langsung terbang ke Kabupaten Alor, Nusa Tenggara Timur (NTT), pada akhir pekan ini....</t>
+        </is>
+      </c>
+      <c r="F603" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G603" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjg0ee370/mentan-batalkan-rapat-di-jakarta-demi-tindaklanjuti-aspirasi-mahasiswa-alor</t>
+        </is>
+      </c>
+      <c r="H603" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/_260808151509-185.png</t>
+        </is>
+      </c>
+      <c r="I603" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>Kebakaran di Kebon Pala, 65 Personel Damkar Dikerahkan</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:12:05 +0700</t>
+        </is>
+      </c>
+      <c r="D604" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E604" t="inlineStr">
+        <is>
+          <t>13 mobil damkar dikerahkan, api akhirnya berhasil dikendalikan petugas.</t>
+        </is>
+      </c>
+      <c r="F604" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G604" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265125/kebakaran-di-kebon-pala-65-personel-damkar-dikerahkan</t>
+        </is>
+      </c>
+      <c r="H604" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/dBi8dsGTvJvDoh5-AzAAl374JMM=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9319075/original/022034900_1786180300-kebakaran.JPG</t>
+        </is>
+      </c>
+      <c r="I604" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>Prahara Pulau Emas Menyusuri Jejak Bencana Sumatera Lewat Foto</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:56:35 +0700</t>
+        </is>
+      </c>
+      <c r="D605" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E605" t="inlineStr">
+        <is>
+          <t>Pengunjung melihat karya dalam pameran foto jurnalistik Prahara Pulau Emas di Museum Tsunami Aceh, Banda Aceh, Sabtu, 8 Agustus 2026. Pameran tersebut menjadi ruang dokumentasi visual atas bencana hidrometeorologi yang terjadi di Aceh, Sumatera Utara, dan Sumatera Barat pada akhir November 2025. Sebanyak 68 karya dari 38 pewarta foto se-Indonesia ditampilkan dalam rangkaian pameran dan peluncuran buku foto jurnalistik yang berlangsung 3 hingga 8 Agustus 2026. Roadshow sebelumnya digelar di Padang dan dijadwalkan berlanjut ke Medan.</t>
+        </is>
+      </c>
+      <c r="F605" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G605" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/photo/read/8265103/prahara-pulau-emas-menyusuri-jejak-bencana-sumatera-lewat-foto</t>
+        </is>
+      </c>
+      <c r="H605" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/H4q-wVHEoDwPLKITftwXEd-VofE=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9319050/original/085404500_1786179369-ace1.jpg</t>
+        </is>
+      </c>
+      <c r="I605" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>Ruang Kontrol Dishub Terdampak Kebakaran Bapenda DKI, Lampu Lalu Lintas Diatur Manual</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:37:39 +0700</t>
+        </is>
+      </c>
+      <c r="D606" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E606" t="inlineStr">
+        <is>
+          <t>Pramono menginstruksikan penebalan pasukan Dishub di lapangan agar pengaturan lalu lintas tetap lancar.</t>
+        </is>
+      </c>
+      <c r="F606" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G606" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265092/ruang-kontrol-dishub-terdampak-kebakaran-bapenda-dki-lampu-lalu-lintas-diatur-manual</t>
+        </is>
+      </c>
+      <c r="H606" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/ipD3F85iLpsa-vf0KfNygf0oJa8=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9318678/original/083581200_1786128701-WhatsApp_Image_2026-08-08_at_01.35.55__1_.jpeg</t>
+        </is>
+      </c>
+      <c r="I606" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>Cahaya</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>Buka Muktamar Tapak Suci XIV, Ahmad Luthfi Soroti Peran Pencak Silat dalam Membangun Karakter dan Persatuan</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:29:32 +0700</t>
+        </is>
+      </c>
+      <c r="D607" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E607" t="inlineStr">
+        <is>
+          <t>Gubernur Jateng Ahmad Luthfi menyebut pencak silat berperan dalam membangun karakter, kebersamaan, kesehatan, dan persatuan bangsa.</t>
+        </is>
+      </c>
+      <c r="F607" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G607" t="inlineStr">
+        <is>
+          <t>https://cahaya.kompas.com/aktual/26H08162608090/buka-muktamar-tapak-suci-xiv-ahmad-luthfi-soroti-peran-pencak-silat-dalam</t>
+        </is>
+      </c>
+      <c r="H607" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/bDMkm9Tm9X_wNaUUoUd2r3KI_4s=/0x0:1200x800/1200x675/data/photo/2026/08/08/6a76f1c2b46b4.webp</t>
+        </is>
+      </c>
+      <c r="I607" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>Donald Trump Perketat Syarat Jadi Warga Negara AS, Wisata Kelahiran Jadi Sasaran</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:29:32 +0700</t>
+        </is>
+      </c>
+      <c r="D608" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E608" t="inlineStr">
+        <is>
+          <t>Donald Trump menandatangani perintah yang menargetkan praktik birth tourism (wisata kelahiran) sekaligus perketat syarat kewarganegaraan AS.</t>
+        </is>
+      </c>
+      <c r="F608" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G608" t="inlineStr">
+        <is>
+          <t>https://travel.kompas.com/read/2026/08/08/160013927/donald-trump-perketat-syarat-jadi-warga-negara-as-wisata-kelahiran-jadi</t>
+        </is>
+      </c>
+      <c r="H608" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/lnO7h2_5Zb05cH6DuqgfCsswxOo=/0x0:1998x1332/1200x675/filters:watermark(data/photo/2026/01/30/697c81889b5f6.png,0,-0,1)/data/photo/2026/07/24/6a635b23d5c70.jpg</t>
+        </is>
+      </c>
+      <c r="I608" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>Api Muncul Lagi di Kawasan B29 Gunung Bromo, 2 Helikopter Lakukan Pemadaman</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:29:32 +0700</t>
+        </is>
+      </c>
+      <c r="D609" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E609" t="inlineStr">
+        <is>
+          <t>Titik api kembali muncul di kawasan B29, TNBTS, pada Sabtu (8/8/2026). Dua unit helikopter melakukan pemadaman</t>
+        </is>
+      </c>
+      <c r="F609" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G609" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/08/08/152349778/api-muncul-lagi-di-kawasan-b29-gunung-bromo-2-helikopter-lakukan-pemadaman</t>
+        </is>
+      </c>
+      <c r="H609" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/1HEaXJSN7L65Z5s4-veqKtRQFCg=/140x0:1475x890/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/08/6a76e386ab63b.jpeg</t>
+        </is>
+      </c>
+      <c r="I609" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I551"/>
+  <autoFilter ref="A1:I609"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-08 10:25 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-08.xlsx
+++ b/data/berita_2026-08-08.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$609</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$677</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I609"/>
+  <dimension ref="A1:I677"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -29059,8 +29059,3204 @@
         </is>
       </c>
     </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>Hari Kucing Sedunia, kucing kampung dapat vaksin rabies gratis</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:13:35 +0700</t>
+        </is>
+      </c>
+      <c r="D610" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E610" t="inlineStr">
+        <is>
+          <t>Dokter hewan menyiapkan vaksin rabies untuk kucing saat peringatan Hari Kucing Sedunia 2026 di Plaza Aceh, Banda Aceh, ...</t>
+        </is>
+      </c>
+      <c r="F610" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G610" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5685763/hari-kucing-sedunia-kucing-kampung-dapat-vaksin-rabies-gratis</t>
+        </is>
+      </c>
+      <c r="H610" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/Vaksinasi-rabies-kucing-kampung-080826-Irp-2A.jpg</t>
+        </is>
+      </c>
+      <c r="I610" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>Ma'ruf Amin dorong NU perkuat pendidikan dan kemandirian ekonomi</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:11:49 +0700</t>
+        </is>
+      </c>
+      <c r="D611" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E611" t="inlineStr">
+        <is>
+          <t>Wakil Presiden Ke-13 RI Ma'ruf Amin mendorong Nahdlatul Ulama (NU) memperkuat umat dan memakmurkan negara melalui ...</t>
+        </is>
+      </c>
+      <c r="F611" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G611" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685760/maruf-amin-dorong-nu-perkuat-pendidikan-dan-kemandirian-ekonomi</t>
+        </is>
+      </c>
+      <c r="H611" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001225648.jpg</t>
+        </is>
+      </c>
+      <c r="I611" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>Polresta Bandung sita 90 kendaraan dari pengungkapan kejahatan jalanan</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:11:03 +0700</t>
+        </is>
+      </c>
+      <c r="D612" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E612" t="inlineStr">
+        <is>
+          <t>Polresta Bandung, Jawa Barat, mengamankan sekitar 90 unit sepeda motor sebagai barang bukti dari pengungkapan 29 kasus ...</t>
+        </is>
+      </c>
+      <c r="F612" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G612" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685756/polresta-bandung-sita-90-kendaraan-dari-pengungkapan-kejahatan-jalanan</t>
+        </is>
+      </c>
+      <c r="H612" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/487133.jpg</t>
+        </is>
+      </c>
+      <c r="I612" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>Utusan Khusus PBB peringatkan potensi konflik pasca serangan Houthi</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:09:33 +0700</t>
+        </is>
+      </c>
+      <c r="D613" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>Utusan Khusus PBB untuk Yaman Hans Grundberg memperingatkan potensi konflik berskala besar di tengah serangan yang ...</t>
+        </is>
+      </c>
+      <c r="F613" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G613" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685752/utusan-khusus-pbb-peringatkan-potensi-konflik-pasca-serangan-houthi</t>
+        </is>
+      </c>
+      <c r="H613" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/CjkinzN000011_20260808_CBMFN0A001.jpeg</t>
+        </is>
+      </c>
+      <c r="I613" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>Pakar dorong inovasi kemitraan untuk perkuat jaringan bisnis</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:54:51 +0700</t>
+        </is>
+      </c>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E614" t="inlineStr">
+        <is>
+          <t>Pakar Waralaba dan Kemitraan Tommy Andri Wardhana mendorong pelaku usaha untuk menerapkan inovasi kemitraan untuk ...</t>
+        </is>
+      </c>
+      <c r="F614" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G614" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685749/pakar-dorong-inovasi-kemitraan-untuk-perkuat-jaringan-bisnis</t>
+        </is>
+      </c>
+      <c r="H614" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000302143.jpg</t>
+        </is>
+      </c>
+      <c r="I614" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>UNIFIL laporkan aktivitas militer di Lebanon Selatan menurun</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:51:32 +0700</t>
+        </is>
+      </c>
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E615" t="inlineStr">
+        <is>
+          <t>Pasukan Interim PBB di Lebanon (UNIFIL), Jumat, melaporkan penurunan signifikan aktivitas militer di Lebanon ...</t>
+        </is>
+      </c>
+      <c r="F615" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G615" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685747/unifil-laporkan-aktivitas-militer-di-lebanon-selatan-menurun</t>
+        </is>
+      </c>
+      <c r="H615" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/13/Damai.jpg</t>
+        </is>
+      </c>
+      <c r="I615" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>Pengamat: Perkara eks Jampidsus ujian penting tegakkan supremasi hukum</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:43:46 +0700</t>
+        </is>
+      </c>
+      <c r="D616" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E616" t="inlineStr">
+        <is>
+          <t>Pengamat politik dari Universitas Nasional (Unas) Firdaus Syam menilai perkara eks Jampidsus Febrie Adriansyah menjadi ...</t>
+        </is>
+      </c>
+      <c r="F616" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G616" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685744/pengamat-perkara-eks-jampidsus-ujian-penting-tegakkan-supremasi-hukum</t>
+        </is>
+      </c>
+      <c r="H616" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1000087435.jpg</t>
+        </is>
+      </c>
+      <c r="I616" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>Caine dan pejabat AS nilai serangan udara tak cukup paksa Iran tunduk</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:41:09 +0700</t>
+        </is>
+      </c>
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E617" t="inlineStr">
+        <is>
+          <t>Ketua Kepala Staf Gabungan Amerika Serikat, Jenderal Dan Caine dan sejumlah pejabat lainnya meyakini bahwa penggunaan ...</t>
+        </is>
+      </c>
+      <c r="F617" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G617" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685743/caine-dan-pejabat-as-nilai-serangan-udara-tak-cukup-paksa-iran-tunduk</t>
+        </is>
+      </c>
+      <c r="H617" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/thumbs_b_c_d0b26d1916563e3561b4dec5516ff731.jpg</t>
+        </is>
+      </c>
+      <c r="I617" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>Dokter: Obesitas dapat meningkatkan risiko diabetes melitus tipe 2</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:39:57 +0700</t>
+        </is>
+      </c>
+      <c r="D618" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E618" t="inlineStr">
+        <is>
+          <t>Konsultan Endokrin Metabolik dan Diabetes Prof. Sidartawan Soegondo mengatakan penumpukan lemak berlebih khususnya di ...</t>
+        </is>
+      </c>
+      <c r="F618" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G618" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685740/dokter-obesitas-dapat-meningkatkan-risiko-diabetes-melitus-tipe-2</t>
+        </is>
+      </c>
+      <c r="H618" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001375514.jpg</t>
+        </is>
+      </c>
+      <c r="I618" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>DKI siap hadirkan bus rute Bunderan Senayan-Ancol saat "car free day"</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:39:33 +0700</t>
+        </is>
+      </c>
+      <c r="D619" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E619" t="inlineStr">
+        <is>
+          <t>Pemerintah Provinsi DKI Jakarta menghadirkan layanan shuttle bus Transjakarta rute Bunderan Senayan-Bunderan ...</t>
+        </is>
+      </c>
+      <c r="F619" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G619" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685736/dki-siap-hadirkan-bus-rute-bunderan-senayan-ancol-saat-car-free-day</t>
+        </is>
+      </c>
+      <c r="H619" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/12/1000303145_1.jpg</t>
+        </is>
+      </c>
+      <c r="I619" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>Menlu soroti perlunya perkuat ketahahan lewat keamanan pangan, energi</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:35:03 +0700</t>
+        </is>
+      </c>
+      <c r="D620" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E620" t="inlineStr">
+        <is>
+          <t>Menteri Luar Negeri Republik Indonesia (Menlu RI) Sugiono menyoroti perlunya memperkuat ketahanan di kawasan Asia ...</t>
+        </is>
+      </c>
+      <c r="F620" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G620" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685733/menlu-soroti-perlunya-perkuat-ketahahan-lewat-keamanan-pangan-energi</t>
+        </is>
+      </c>
+      <c r="H620" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000679879.jpg</t>
+        </is>
+      </c>
+      <c r="I620" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>Pengamat: Skuad Garuda harus bangun hadapi Piala Asia</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:34:23 +0700</t>
+        </is>
+      </c>
+      <c r="D621" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E621" t="inlineStr">
+        <is>
+          <t>Kegagalan tim nasional Indonesia dalam Piala AFF 2026 merupakan ujian membangun skuad menghadapi Piala Asia 2027, ...</t>
+        </is>
+      </c>
+      <c r="F621" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G621" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685731/pengamat-skuad-garuda-harus-bangun-hadapi-piala-asia</t>
+        </is>
+      </c>
+      <c r="H621" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/Timnas-Indonesia-lawan-Vietnam-030826-Bay-11b.jpg</t>
+        </is>
+      </c>
+      <c r="I621" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>Jelang upacara 17 Agustus, Paskibraka Nasional jalani latihan gabungan</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:31:16 +0700</t>
+        </is>
+      </c>
+      <c r="D622" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E622" t="inlineStr">
+        <is>
+          <t>Calon anggota Pasukan Pengibar Bendera Pusaka (Paskibraka) Nasional mengikuti latihan gabungan di Lapangan PPSDM ...</t>
+        </is>
+      </c>
+      <c r="F622" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G622" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5685728/jelang-upacara-17-agustus-paskibraka-nasional-jalani-latihan-gabungan</t>
+        </is>
+      </c>
+      <c r="H622" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/Latihan-gabungan-Paskibraka-Nasional-2026-080826-Bay-1A.jpg</t>
+        </is>
+      </c>
+      <c r="I622" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>KPHD dorong APBD berbasis ketahanan lingkungan</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:29:13 +0700</t>
+        </is>
+      </c>
+      <c r="D623" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E623" t="inlineStr">
+        <is>
+          <t>Kaukus Parlemen Hijau Daerah (KPHD) mendorong pemerintah daerah menyusun Anggaran Pendapatan dan Belanja Daerah (APBD) ...</t>
+        </is>
+      </c>
+      <c r="F623" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G623" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685724/kphd-dorong-apbd-berbasis-ketahanan-lingkungan</t>
+        </is>
+      </c>
+      <c r="H623" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/Anggota-DPRD-se-Indonesia.jpg</t>
+        </is>
+      </c>
+      <c r="I623" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>Gelombang panas melanda sebagian besar Korea Selatan</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:28:46 +0700</t>
+        </is>
+      </c>
+      <c r="D624" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>Sebagian besar wilayah Korea Selatan dilanda gelombang panas yang intens, dengan suhu pada siang hari diperkirakan ...</t>
+        </is>
+      </c>
+      <c r="F624" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G624" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685721/gelombang-panas-melanda-sebagian-besar-korea-selatan</t>
+        </is>
+      </c>
+      <c r="H624" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2024/08/04/ilustrasi-panas-ekstrem-China-dan-Jepang_1.jpg</t>
+        </is>
+      </c>
+      <c r="I624" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>Gedung Bapenda DKI terbakar, Pemprov pastikan data pajak aman, layanan tetap berjalan</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:27:28 +0700</t>
+        </is>
+      </c>
+      <c r="D625" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E625" t="inlineStr">
+        <is>
+          <t>Petugas Dinas Perhubungan (Dishub) DKI Jakarta berjaga pascakebakaran Gedung Badan Pendapatan Daerah (Bapenda) DKI ...</t>
+        </is>
+      </c>
+      <c r="F625" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G625" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5685719/gedung-bapenda-dki-terbakar-pemprov-pastikan-data-pajak-aman-layanan-tetap-berjalan</t>
+        </is>
+      </c>
+      <c r="H625" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/Pascakebakaran-Gedung-Bapenda-DKI-Jakarta-080826-RRY-1A.jpg</t>
+        </is>
+      </c>
+      <c r="I625" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>Pegawai Bank Emok Dipaksa Onani karena Dikira Mau Rebut Nasabah Bos</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:59:57 +0700</t>
+        </is>
+      </c>
+      <c r="D626" t="inlineStr">
+        <is>
+          <t>Arief Ikhsanudin</t>
+        </is>
+      </c>
+      <c r="E626" t="inlineStr">
+        <is>
+          <t>Polisi ungkap motif pria PG dianiaya dan dipaksa onani oleh bos dan rekan kerja. Lima tersangka ditangkap, termasuk bos 'bank emok'.</t>
+        </is>
+      </c>
+      <c r="F626" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G626" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610000/pegawai-bank-emok-dipaksa-onani-karena-dikira-mau-rebut-nasabah-bos</t>
+        </is>
+      </c>
+      <c r="H626" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2015/12/08/3fc3b526-7901-496f-a246-3044f7c11820_169.jpg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I626" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>2 Warga Sipil Luka Akibat Penembakan di Festival Lembah Baliem Jayawijaya</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:59:44 +0700</t>
+        </is>
+      </c>
+      <c r="D627" t="inlineStr">
+        <is>
+          <t>Syachrul Arsyad</t>
+        </is>
+      </c>
+      <c r="E627" t="inlineStr">
+        <is>
+          <t>Penembakan terjadi di Festival Budaya Lembah Baliem, Jayawijaya, mengakibatkan dua warga sipil luka. Situasi kini kondusif, evakuasi pengunjung dilakukan.</t>
+        </is>
+      </c>
+      <c r="F627" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G627" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609999/2-warga-sipil-luka-akibat-penembakan-di-festival-lembah-baliem-jayawijaya</t>
+        </is>
+      </c>
+      <c r="H627" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/penembakan-terjadi-di-festival-budaya-lembah-baliem-kabupaten-jayawijaya-1786181589666_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I627" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>Dishub DKI Siaga di Titik Macet Usai Sistem Lalin Terdampak Kebakaran Bapenda</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:41:50 +0700</t>
+        </is>
+      </c>
+      <c r="D628" t="inlineStr">
+        <is>
+          <t>Brigitta Belia Permata Sari</t>
+        </is>
+      </c>
+      <c r="E628" t="inlineStr">
+        <is>
+          <t>Dishub DKI akan mengerahkan petugas untuk mengatur lalin secara manual. Hal itu dilakukan usai ruang SPLL di gedung Bapenda DKI ikut terdampak kebakaran.</t>
+        </is>
+      </c>
+      <c r="F628" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G628" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609983/dishub-dki-siaga-di-titik-macet-usai-sistem-lalin-terdampak-kebakaran-bapenda</t>
+        </is>
+      </c>
+      <c r="H628" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2024/09/23/kepala-dinas-dukcapil-dki-jakarta-budi-awaluddin_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I628" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>Ibu dan Balita Ditemukan Tewas Terikat di Hutan Kalbar</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:41:16 +0700</t>
+        </is>
+      </c>
+      <c r="D629" t="inlineStr">
+        <is>
+          <t>Ocsya Ade CP</t>
+        </is>
+      </c>
+      <c r="E629" t="inlineStr">
+        <is>
+          <t>Warga Landak digegerkan penemuan jasad ibu dan anak terikat di hutan. Polisi selidiki dugaan pembunuhan terkait perampokan. Kasus ini mengundang perhatian.</t>
+        </is>
+      </c>
+      <c r="F629" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G629" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609982/ibu-dan-balita-ditemukan-tewas-terikat-di-hutan-kalbar</t>
+        </is>
+      </c>
+      <c r="H629" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/jenazah-ibu-dan-balitanya-yang-tewas-terikat-di-hutan-landak-1786178167460_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I629" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>HGB Ruko STC Tak Bisa Diperpanjang, DPRD Nilai Pemko Pekanbaru Sudah Tepat</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:35:52 +0700</t>
+        </is>
+      </c>
+      <c r="D630" t="inlineStr">
+        <is>
+          <t>Raja Adil Siregar</t>
+        </is>
+      </c>
+      <c r="E630" t="inlineStr">
+        <is>
+          <t>DPRD Pekanbaru minta kepastian hukum terkait kebijakan Pemko yang tidak perpanjang HGB ruko STC. Kemendagri tegaskan keputusan sesuai aturan.</t>
+        </is>
+      </c>
+      <c r="F630" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G630" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609976/hgb-ruko-stc-tak-bisa-diperpanjang-dprd-nilai-pemko-pekanbaru-sudah-tepat</t>
+        </is>
+      </c>
+      <c r="H630" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2021/10/27/gedung-dprd-pekanbaru_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I630" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>Termasuk Bos Bank Emok, 5 Orang Jadi Tersangka Kasus Pria Dipaksa Onani</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:35:21 +0700</t>
+        </is>
+      </c>
+      <c r="D631" t="inlineStr">
+        <is>
+          <t>Arief Ikhsanudin</t>
+        </is>
+      </c>
+      <c r="E631" t="inlineStr">
+        <is>
+          <t>Polisi amankan delapan orang terkait penganiayaan pegawai bank keliling di Tangerang. Lima tersangka, termasuk bos, dijerat dengan pasal kekerasan.</t>
+        </is>
+      </c>
+      <c r="F631" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G631" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609975/termasuk-bos-bank-emok-5-orang-jadi-tersangka-kasus-pria-dipaksa-onani</t>
+        </is>
+      </c>
+      <c r="H631" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2021/08/04/kekerasan-penganiayaan_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I631" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>Doli Kurnia Sebut Partisipasi Warga Dibutuhkan untuk Pembangunan Nasional</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:33:30 +0700</t>
+        </is>
+      </c>
+      <c r="D632" t="inlineStr">
+        <is>
+          <t>Dea Duta Aulia</t>
+        </is>
+      </c>
+      <c r="E632" t="inlineStr">
+        <is>
+          <t>DPP LPM RI periode 2025-2030 dilantik, fokus pada pemberdayaan masyarakat. LPM berperan strategis dalam pembangunan nasional dan sinergi dengan pemerintah.</t>
+        </is>
+      </c>
+      <c r="F632" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G632" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609974/doli-kurnia-sebut-partisipasi-warga-dibutuhkan-untuk-pembangunan-nasional</t>
+        </is>
+      </c>
+      <c r="H632" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/doli-kurnia-sebut-partisipasi-warga-dibutuhkan-untuk-pembangunan-nasional-1786181553090_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I632" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>Kapolri Dianugerahi Jadi Anggota Kehormatan Tapak Suci Putera Muhammadiyah</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 09:54:36 +0700</t>
+        </is>
+      </c>
+      <c r="D633" t="inlineStr">
+        <is>
+          <t>Lisye Sri Rahayu</t>
+        </is>
+      </c>
+      <c r="E633" t="inlineStr">
+        <is>
+          <t>Kapolri Jenderal Sigit dianugerahi anggota kehormatan Tapak Suci Muhammadiyah. Dia berharap hubungan Polri dan Muhammadiyah semakin erat ke depannya.</t>
+        </is>
+      </c>
+      <c r="F633" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G633" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8609538/kapolri-dianugerahi-jadi-anggota-kehormatan-tapak-suci-putera-muhammadiyah</t>
+        </is>
+      </c>
+      <c r="H633" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/kapolri-jenderal-listyo-sigit-prabowo-1786157459631_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I633" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>BI Buka Lowongan PCPM Angkatan 41, Ini Syarat Lengkapnya</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:00:46 +0700</t>
+        </is>
+      </c>
+      <c r="D634" t="inlineStr">
+        <is>
+          <t>Ignacio Geordi Oswaldo</t>
+        </is>
+      </c>
+      <c r="E634" t="inlineStr">
+        <is>
+          <t>Bank Indonesia (BI) akan membuka lowongan kerja melalui program Pendidikan Calon Pegawai Asisten Manajer (PCPM) angkatan 41 mulai besok, Minggu (9/8).</t>
+        </is>
+      </c>
+      <c r="F634" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G634" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/lainnya/d-8609934/bi-buka-lowongan-pcpm-angkatan-41-ini-syarat-lengkapnya</t>
+        </is>
+      </c>
+      <c r="H634" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2021/10/29/ilustrasi-bank-indonesia-4_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I634" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>Mentan Buka-bukaan Cara Dongkrak Pertanian dan Tekan Kemiskinan di Alor</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:30:58 +0700</t>
+        </is>
+      </c>
+      <c r="D635" t="inlineStr">
+        <is>
+          <t>Heri Purnomo</t>
+        </is>
+      </c>
+      <c r="E635" t="inlineStr">
+        <is>
+          <t>Menteri Pertanian Andi Amran Sulaiman mengunjungi Alor untuk mengatasi masalah pangan.</t>
+        </is>
+      </c>
+      <c r="F635" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G635" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8609952/mentan-buka-bukaan-cara-dongkrak-pertanian-dan-tekan-kemiskinan-di-alor</t>
+        </is>
+      </c>
+      <c r="H635" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/menteri-pertanian-mentan-andi-amran-sulaiman-1786178494016_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I635" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>Resmikan Pusat Persemaian Kemampo Banyuasin, Menhut Sampaikan Salam Prabowo</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:17:22 +0700</t>
+        </is>
+      </c>
+      <c r="D636" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E636" t="inlineStr">
+        <is>
+          <t>Menteri Kehutanan meresmikan Pusat Persemaian Sriwijaya Kemampo di Kawasan Hutan Dengan Tujuan Khusus (KHDTK) Kemampo, Kabupaten Banyuasin, Sumsel.</t>
+        </is>
+      </c>
+      <c r="F636" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G636" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865784/resmikan-pusat-persemaian-kemampo-banyuasin-menhut-sampaikan-salam-prabowo</t>
+        </is>
+      </c>
+      <c r="H636" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/9NdLPO-StURcWBuO2qScMZfhNKk=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Banyuasin-Persemaian-12314dgfa.jpg</t>
+        </is>
+      </c>
+      <c r="I636" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>Soal Penyegelan SDN di Bandung, Pemkot Disebut Gagal hingga Siswa Jadi Korban</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:13:08 +0700</t>
+        </is>
+      </c>
+      <c r="D637" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E637" t="inlineStr">
+        <is>
+          <t>SDN 026 Bojongloa Bandung digembok ahli waris akibat sengketa lahan. JPPI mengkritik kelalaian Pemkot Bandung dalam mengelola aset pendidikan.</t>
+        </is>
+      </c>
+      <c r="F637" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G637" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865783/soal-penyegelan-sdn-di-bandung-pemkot-disebut-gagal-hingga-siswa-jadi-korban</t>
+        </is>
+      </c>
+      <c r="H637" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/l1P32TLy3X8cEM76a_dW_v3Vqg4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/SD-Negeri-026-Bojongloa-disegel-asdf.jpg</t>
+        </is>
+      </c>
+      <c r="I637" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>Prakiraan Cuaca Pontianak Besok, Minggu 9 Agustus 2026: Didominasi Berawan</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:04:13 +0700</t>
+        </is>
+      </c>
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>Simak prakiraan cuaca Kota Pontianak  besok, Minggu 9 Agustus 2026, didominasi oleh cuaca berawan.</t>
+        </is>
+      </c>
+      <c r="F638" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G638" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865782/prakiraan-cuaca-pontianak-besok-minggu-9-agustus-2026-didominasi-berawan</t>
+        </is>
+      </c>
+      <c r="H638" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Eh-VM9JugL-I8mSjMBMU42UQpy0=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/TRIBUN-PONTIANAK-Ni-Made-Gunarsih.jpg</t>
+        </is>
+      </c>
+      <c r="I638" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>Hasil Indonesia vs Thailand SEA V Cup 2026: Sugiyama Mainkan Skuad Pelapis, Kalah 25-18 Set I</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:04:08 +0700</t>
+        </is>
+      </c>
+      <c r="D639" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E639" t="inlineStr">
+        <is>
+          <t>Timnas voli putri Indonesia kalah 25-18 pada set pertama atas Thailand pada SEA V Cup 2026 Leg 2.</t>
+        </is>
+      </c>
+      <c r="F639" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G639" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7865781/hasil-indonesia-vs-thailand-sea-v-cup-2026-sugiyama-mainkan-skuad-pelapis-kalah-25-18-set-i</t>
+        </is>
+      </c>
+      <c r="H639" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ji5jh_awPmeoo7bKdWFIChFnymU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Pemain-Timnas-Voli-Putri-Indonesia-melakukan-perayaan-setelah-mencetak-poin-saat.jpg</t>
+        </is>
+      </c>
+      <c r="I639" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>Jose Mourinho Bawa Aturan Ketat ke Real Madrid, Disiplin Pemain El Real Perhatian Utama</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:03:53 +0700</t>
+        </is>
+      </c>
+      <c r="D640" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E640" t="inlineStr">
+        <is>
+          <t>Jose Mourinho akan menerapkan beragam aturan ketat untuk menambah disiplin para pemain Real Madrid menjelang musim 2026/2027.</t>
+        </is>
+      </c>
+      <c r="F640" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G640" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865780/jose-mourinho-bawa-aturan-ketat-ke-real-madrid-disiplin-pemain-el-real-perhatian-utama</t>
+        </is>
+      </c>
+      <c r="H640" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/WsuDiHKzmIOtt3Kcg9LFZmyeXqI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Pelatih-anyar-Real-Madrid-Jose-Mourinho-dalam-pertandingan-uji-coba-pramusim.jpg</t>
+        </is>
+      </c>
+      <c r="I640" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>Christopher dan Rara Jadi Paskibraka di Istana, Keluarga Siapkan Nobar</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:58:47 +0700</t>
+        </is>
+      </c>
+      <c r="D641" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E641" t="inlineStr">
+        <is>
+          <t>Christopher dan Rara bersiap bertugas sebagai Paskibraka di Istana pada 17 Agustus, sementara keluarga menyiapkan cara menyaksikan.</t>
+        </is>
+      </c>
+      <c r="F641" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G641" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865779/christopher-dan-rara-jadi-paskibraka-di-istana-keluarga-siapkan-nobar</t>
+        </is>
+      </c>
+      <c r="H641" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/EWHbUEdMD1Ec8BkzGfywykMUXHY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Paskibraka-Christopher-Leon-Bringga-Tabuni-Papua-dan-Raudah-Mabrura-Riau.jpg</t>
+        </is>
+      </c>
+      <c r="I641" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>Update Penembakan Sekolah di Thailand: Ayah Pelaku Minta Maaf, Polisi Telusuri Asal Amunisi</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:58:22 +0700</t>
+        </is>
+      </c>
+      <c r="D642" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E642" t="inlineStr">
+        <is>
+          <t>Ayah pelaku penembakan massal di Nothanburi tampak sangat terpukul dan sempat menyampaikan pernyataan singkat kepada para awak media.</t>
+        </is>
+      </c>
+      <c r="F642" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G642" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7865778/update-penembakan-sekolah-di-thailand-ayah-pelaku-minta-maaf-polisi-telusuri-asal-amunisi</t>
+        </is>
+      </c>
+      <c r="H642" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/VTTQO-NJFdFtr3pzNQPnEL_m8tQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Siswa-di-Thailand-berlari-saat-penembakan.jpg</t>
+        </is>
+      </c>
+      <c r="I642" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>Jadi Tersangka, Mantan Ketua DPRD Ponorogo Jatim Perintahkan Mark Up Tunjangan Perumahan  15 Persen</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:52:56 +0700</t>
+        </is>
+      </c>
+      <c r="D643" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E643" t="inlineStr">
+        <is>
+          <t>Kejaksaan Negeri Ponorogo menetapkan SN, Ketua DPRD Ponorogo periode 2019-2024 sebagai tersangka.</t>
+        </is>
+      </c>
+      <c r="F643" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G643" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865777/jadi-tersangka-mantan-ketua-dprd-ponorogo-jatim-perintahkan-mark-up-tunjangan-perumahan-15-persen</t>
+        </is>
+      </c>
+      <c r="H643" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/9iBPkz-OjcF5Wqdlpipaysb1KzM=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/DITAHAN-SN-Ketua-DPRD-Ponorogo.jpg</t>
+        </is>
+      </c>
+      <c r="I643" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>Tanggapan Dinas PUTR soal Viral ASN di Bandung Barat yang Live di Medsos Minta Fee Proyek</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:50:19 +0700</t>
+        </is>
+      </c>
+      <c r="D644" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E644" t="inlineStr">
+        <is>
+          <t>Plt Kadis PUTR Bandung Barat peringatkan jajarannya agar bijak bermedsos usai viral oknum ASN live minta fee proyek di jam kerja.</t>
+        </is>
+      </c>
+      <c r="F644" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G644" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865776/tanggapan-dinas-putr-soal-viral-asn-di-bandung-barat-yang-live-di-medsos-minta-fee-proyek</t>
+        </is>
+      </c>
+      <c r="H644" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/6nxLjIYGCVemyZJLmJOvq3Lt6cI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ASN-live-minta-persenan-asdf-q2w3er-2qr.jpg</t>
+        </is>
+      </c>
+      <c r="I644" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>Cerita Korban Selamat dari Kecelakaan di Bandung saat Truk Pengangkut Batu Bara Patah As Roda</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:46:11 +0700</t>
+        </is>
+      </c>
+      <c r="D645" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E645" t="inlineStr">
+        <is>
+          <t>Truk pengangkut batu bara alami patah as roda dan tabrak enam kendaraan di Rancabali Bandung. Beruntung tidak ada korban jiwa dalam insiden ini.</t>
+        </is>
+      </c>
+      <c r="F645" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G645" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865775/cerita-korban-selamat-dari-kecelakaan-di-bandung-saat-truk-pengangkut-batu-bara-patah-as-roda</t>
+        </is>
+      </c>
+      <c r="H645" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/aLZEvc_ZJpGz8lU-gPIsVKd4lj0=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/kecelakaan-di-ciwidey-asdfv-awef.jpg</t>
+        </is>
+      </c>
+      <c r="I645" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>Merawat Syiar Islam Berkemajuan: Peringatan 666 Tahun Islam Masuk Papua di Fakfak</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:43:34 +0700</t>
+        </is>
+      </c>
+      <c r="D646" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E646" t="inlineStr">
+        <is>
+          <t>Peringatan 666 tahun masuknya Islam ke Papua menjadi momentum memperkuat tradisi, toleransi, dan dakwah berkemajuan di Bumi Cenderawasih.</t>
+        </is>
+      </c>
+      <c r="F646" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G646" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865774/merawat-syiar-islam-berkemajuan-peringatan-666-tahun-islam-masuk-papua-di-fakfak</t>
+        </is>
+      </c>
+      <c r="H646" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/rqpgLETnAieiRCdmT-thb-KF_T8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/BAITUL-ARQAM-di-Fakfak.jpg</t>
+        </is>
+      </c>
+      <c r="I646" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>Move On dari Piala AFF, John Herdman Fokus Incar Trofi Timnas Indonesia di FIFA ASEAN Cup 2026</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:41:36 +0700</t>
+        </is>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>Gagal di Piala AFF 2026, John Herdman langsung move on. Pelatih Timnas Indonesia membidik trofi pertama di FIFA ASEAN Cup 2026.</t>
+        </is>
+      </c>
+      <c r="F647" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G647" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865773/move-on-dari-piala-aff-john-herdman-fokus-incar-trofi-timnas-indonesia-di-fifa-asean-cup-2026</t>
+        </is>
+      </c>
+      <c r="H647" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/MSs3EL7n9e678yVL0iol34xKGjg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Gaya-John-Herdman-Debut-Melatih-Timnas-Indonesia_20260328_003813.jpg</t>
+        </is>
+      </c>
+      <c r="I647" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>Prakiraan Cuaca Sulawesi Barat Minggu, 9 Agustus 2026: Cek Wilayah Berpotensi Hujan</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:41:16 +0700</t>
+        </is>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>BMKG melaporkan prakiraan cuaca untuk wilayah Sulawesi Barat (Sulbar), Minggu (9/8/2026). Cek wilayah berpotensi hujan.</t>
+        </is>
+      </c>
+      <c r="F648" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G648" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865772/prakiraan-cuaca-sulawesi-barat-minggu-9-agustus-2026-cek-wilayah-berpotensi-hujan</t>
+        </is>
+      </c>
+      <c r="H648" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/zuUaADQ8yitcRX5Zk0F6srdEnKw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Prakiraan-Cuaca-Sulawesi-Barat-Selasa-10-Maret-2026Waspada-Hujan-Lebat-di-Wilayah-Ini.jpg</t>
+        </is>
+      </c>
+      <c r="I648" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>Terjemahan Lirik Lagu Call Me Maybe - Carly Rae Jepsen: I Looked to You As It Fell</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:40:44 +0700</t>
+        </is>
+      </c>
+      <c r="D649" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr">
+        <is>
+          <t>Simak terjemahan lirik lagu Call Me Maybe yang dipopulerkan oleh  Carly Rae Jepsen dalam artikel berikut ini.</t>
+        </is>
+      </c>
+      <c r="F649" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G649" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/musik/7865771/terjemahan-lirik-lagu-call-me-maybe-carly-rae-jepsen-i-looked-to-you-as-it-fell</t>
+        </is>
+      </c>
+      <c r="H649" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/CL9ms16FPIIxTCUp0D3p9YN4Z0w=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-musik-upgrade-fm.jpg</t>
+        </is>
+      </c>
+      <c r="I649" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>Masuk Bursa Ketum PBNU, Gus Kikin Sebut Gus Yahya dan 5 Nama Lain</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:38:20 +0700</t>
+        </is>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr">
+        <is>
+          <t>Gus Kikin mengonfirmasi namanya masuk bursa Ketum PBNU dan menyebut lima nama lain yang muncul menjelang Muktamar NU. Siapa saja?</t>
+        </is>
+      </c>
+      <c r="F650" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G650" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865770/masuk-bursa-ketum-pbnu-gus-kikin-sebut-gus-yahya-dan-5-nama-lain</t>
+        </is>
+      </c>
+      <c r="H650" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/FuvzATk_mb-cItCZkx0aM7ZK27w=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/KH-Abdul-Hakim-Mahfudz-atau-Gus-Kikin-Ketua-PWNU-Jawa-Timur-Pengasuh-Pesantren-Tebuireng.jpg</t>
+        </is>
+      </c>
+      <c r="I650" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>Filosofi Desain Jetour T2 i-DM, Desain Boxy Jadi Tren Dunia: Lampu Belakang Ternspirasi Lampion</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:37:15 +0700</t>
+        </is>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>Saat ini SUV dengan desain boxy seperti terdapat pada Jetour T2 series dan T1 serius yang diniagakan di Indonesia sedang digandrungi dunia.</t>
+        </is>
+      </c>
+      <c r="F651" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G651" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/otomotif/7865769/filosofi-desain-jetour-t2-i-dm-desain-boxy-jadi-tren-dunia-lampu-belakang-ternspirasi-lampion</t>
+        </is>
+      </c>
+      <c r="H651" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/hXS_-yg3_wAHd-mc6PPADwWSGQU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Jetour-T2-di-GIIAS-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I651" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>Dokter Tifa Tak Terima Disebut Pengecut dan Mundur dari Kasus Ijazah Jokowi</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:35:17 +0700</t>
+        </is>
+      </c>
+      <c r="D652" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E652" t="inlineStr">
+        <is>
+          <t>Dokter Tifa membantah mundur atau takut dalam polemik ijazah Jokowi dan menyebut keputusannya sebagai bentuk hijrah, bukan menyerah.</t>
+        </is>
+      </c>
+      <c r="F652" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G652" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865768/dokter-tifa-tak-terima-disebut-pengecut-dan-mundur-dari-kasus-ijazah-jokowi</t>
+        </is>
+      </c>
+      <c r="H652" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/gfX7VUL0OmUJ35AYFZFbd_QxdvM=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Pelimpahan-Berkas-Roy-Suryo-dan-Dokter-Tifa-Ke-Kejari-Jaksel_20260622_154323.jpg</t>
+        </is>
+      </c>
+      <c r="I652" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>Update Kasus Pilot Selundupkan Narkoba, Kepolisian Malaysia Amankan 2 Pegawai AVSEC Bandara KLIA</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:34:59 +0700</t>
+        </is>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E653" t="inlineStr">
+        <is>
+          <t>Dua petugas Aviation Security (AVSEC) telah diamankan Kepolisian Malaysia guna dimintai keterangan resmi terkait peristiwa tersebut</t>
+        </is>
+      </c>
+      <c r="F653" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G653" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7865767/update-kasus-pilot-selundupkan-narkoba-kepolisian-malaysia-amankan-2-pegawai-avsec-bandara-klia</t>
+        </is>
+      </c>
+      <c r="H653" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/91mQS1Ln7-ye69r2v_mXy_65KUA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Seorang-pilot-asal-Malaysia-berinisial-MSO-di.jpg</t>
+        </is>
+      </c>
+      <c r="I653" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>Jelang Intimate Concert, Sandhy Sondoro Jatuh Hati pada Kota Solo: Tentram, Kulinernya Best</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:27:32 +0700</t>
+        </is>
+      </c>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E654" t="inlineStr">
+        <is>
+          <t>Jelang Intimate Konser, Sandhy Sondoro jatuh hati pada Kota Solo: Tentram, Kulinernya The Best</t>
+        </is>
+      </c>
+      <c r="F654" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G654" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7865766/jelang-intimate-concert-sandhy-sondoro-jatuh-hati-pada-kota-solo-tentram-kulinernya-best</t>
+        </is>
+      </c>
+      <c r="H654" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/uyyHX7_ufaGmAtUxQud4zKsjaz8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Penyanyi-Sandhy-Sondoro-saat-berkunjung-ke-Kota-Solo.jpg</t>
+        </is>
+      </c>
+      <c r="I654" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>Piala Presiden 2026: Laboratorium Bernardo Tavares Buka Pintu Prestasi Persebaya</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:27:28 +0700</t>
+        </is>
+      </c>
+      <c r="D655" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E655" t="inlineStr">
+        <is>
+          <t>Bernardo Tavares menjadikan Piala Presiden 2026 sebagai laboratorium. Eksperimennya berbuah trofi sekaligus fondasi baru Persebaya.</t>
+        </is>
+      </c>
+      <c r="F655" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G655" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865765/piala-presiden-2026-laboratorium-bernardo-tavares-buka-pintu-prestasi-persebaya</t>
+        </is>
+      </c>
+      <c r="H655" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/MPB2YdqCga64l6eVCSxNIx_4k8M=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Persebaya-Surabaya-sukses-keluar-sebagai-juara-Piala-Presiden-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I655" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>Perang Iran Makin Rumit, Jenderal Top AS Diam-Diam Cari Jalan Keluar</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:15:01 +0700</t>
+        </is>
+      </c>
+      <c r="D656" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E656" t="inlineStr">
+        <is>
+          <t>Perang AS-Iran semakin rumit. Jenderal Caine mencari jalan keluar dari konflik, menilai opsi militer berisiko. Fokus kini pada strategi diplomasi dan simbolis.</t>
+        </is>
+      </c>
+      <c r="F656" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G656" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260808144001-4-757622/perang-iran-makin-rumit-jenderal-top-as-diam-diam-cari-jalan-keluar</t>
+        </is>
+      </c>
+      <c r="H656" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/07/09/iran-crisisusa-strikes-1783560096096_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I656" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>PHE Dorong Inovasi Pengeboran di Wilayah New Frontier</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:38:55 +0700</t>
+        </is>
+      </c>
+      <c r="D657" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr">
+        <is>
+          <t>Pertamina Hulu Energi memperluas eksplorasi ke new frontier dengan fokus pada migas non-konvensional dan teknologi modern untuk efisiensi dan keberlanjutan.</t>
+        </is>
+      </c>
+      <c r="F657" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G657" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260808163525-4-757632/phe-dorong-inovasi-pengeboran-di-wilayah-new-frontier</t>
+        </is>
+      </c>
+      <c r="H657" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/08/pertamina-hulu-energi-1786181922941_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I657" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>Mumpung Tanggal Muda, Transmart Kasih Diskon ke Pelanggan 50%+20%</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:30:49 +0700</t>
+        </is>
+      </c>
+      <c r="D658" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr">
+        <is>
+          <t>Transmart Full Day Sale hadir dengan diskon hingga 50% + 20% pada 9 Agustus 2026. Promo berlaku untuk pelanggan kartu kredit tertentu di seluruh Indonesia.</t>
+        </is>
+      </c>
+      <c r="F658" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G658" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260808104701-4-757594/mumpung-tanggal-muda-transmart-kasih-diskon-ke-pelanggan-50-20</t>
+        </is>
+      </c>
+      <c r="H658" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2025/03/23/transmart-full-day-sale-1742701562218_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I658" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>AS Salah Tembak Pesawat Penumpang Iran, 290 Orang Tewas</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:15:19 +0700</t>
+        </is>
+      </c>
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>Tragedi penerbangan Iran Air 655 terjadi pada 3 Juli 1988, saat USS Vincennes menembak jatuh pesawat komersial, menewaskan 290 orang.</t>
+        </is>
+      </c>
+      <c r="F659" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G659" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260808140519-4-757618/as-salah-tembak-pesawat-penumpang-iran-290-orang-tewas</t>
+        </is>
+      </c>
+      <c r="H659" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2025/06/20/iran-air-iran-guidebooktravel-blog-by-nelia-shidfar-1750411949253_169.webp?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I659" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>Video: PR Pengusaha Jaga Kelangsungan Produk Alkes Made In Indonesia</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:00:39 +0700</t>
+        </is>
+      </c>
+      <c r="D660" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E660" t="inlineStr">
+        <is>
+          <t>Pertahankan Kelangsungan Produk Alkes Made In Indonesia, Pengusaha Minta Keberpihakan Pemerintah</t>
+        </is>
+      </c>
+      <c r="F660" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G660" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260804162944-8-756522/video-pr-pengusaha-jaga-kelangsungan-produk-alkes-made-in-indonesia</t>
+        </is>
+      </c>
+      <c r="H660" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/04/rtahankan-kelangsungan-produk-alkes-made-in-indonesia-pengusaha-minta-keberpihakan-pemerintah-1785837679491_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I660" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>Begini Penampakan Gedung Bapenda DKI Hangus Usai Dilalap Api</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:45:37 +0700</t>
+        </is>
+      </c>
+      <c r="D661" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E661" t="inlineStr">
+        <is>
+          <t>Gedung Bapenda DKI hangus usai kebakaran. Pendinginan telah selesai, sementara penyelidikan masih berlangsung penyebab api dan satu korban telah dievakuasi.</t>
+        </is>
+      </c>
+      <c r="F661" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G661" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260808132435-7-757606/begini-penampakan-gedung-bapenda-dki-hangus-usai-dilalap-api</t>
+        </is>
+      </c>
+      <c r="H661" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/08/petugas-penanggulangan-kebakaran-dan-penyelamatan-gulkarmat-memasuki-gedung-badan-pendapatan-daerah-bapenda-dki-jakarta-setela-1786171326510_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I661" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>Video: Hidrogen Jadi Energi Hijau, Bisa Untuk Bus - Alat Berat Tambang</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:00:42 +0700</t>
+        </is>
+      </c>
+      <c r="D662" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia TV</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>Hidrogen Jadi Sumber Energi Hijau, Bisa Untuk Bus Umum - Alat Berat Tambang</t>
+        </is>
+      </c>
+      <c r="F662" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G662" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260805113602-8-756708/video-hidrogen-jadi-energi-hijau-bisa-untuk-bus--alat-berat-tambang</t>
+        </is>
+      </c>
+      <c r="H662" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/05/hidrogen-jadi-sumber-energi-hijau-bisa-untuk-bus-umum-alat-berat-tambang-1785907827648_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I662" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>Bikin Heboh, Sungai Hilang Jadi Hamparan Pasir dan Muncul Pulau</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D663" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>Polandia terancam mengalami kekeringan terburuk</t>
+        </is>
+      </c>
+      <c r="F663" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G663" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260808113611-4-757601/bikin-heboh-sungai-hilang-jadi-hamparan-pasir-dan-muncul-pulau</t>
+        </is>
+      </c>
+      <c r="H663" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/05/sebuah-pemandangan-dari-drone-memperlihatkan-cakrawala-warsawa-di-balik-hamparan-pasir-yang-muncul-ke-permukaan-di-sungai-vist-1785897303716_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I663" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>Pemerintah Bakal Kasih Rp26 Juta Jika Berhasil Tangkap Lele Jumbo Ini</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:45:00 +0700</t>
+        </is>
+      </c>
+      <c r="D664" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr">
+        <is>
+          <t>Departemen Sumber Daya Alam Maryland, Amerika Serikat, meluncurkan program pengendalian lele biru</t>
+        </is>
+      </c>
+      <c r="F664" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G664" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260808112725-4-757599/pemerintah-bakal-kasih-rp26-juta-jika-berhasil-tangkap-lele-jumbo-ini</t>
+        </is>
+      </c>
+      <c r="H664" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/07/01/ilustrasi-ikan-lele-biru-1782895305415_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I664" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>Respon Curhatan Adriano, Mentan Amran: Aspirasi Riil untuk Rakyat Alor</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:45:58 +0700</t>
+        </is>
+      </c>
+      <c r="D665" t="inlineStr">
+        <is>
+          <t>dpu</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr">
+        <is>
+          <t>Mentan Amran apresiasi Adriano, mahasiswa UNDIP, yang suarakan masalah pangan di Alor. Kunjungan langsung untuk tindaklanjuti aspirasi masyarakat.</t>
+        </is>
+      </c>
+      <c r="F665" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G665" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260808133731-4-757605/respon-curhatan-adriano-mentan-amran-aspirasi-riil-untuk-rakyat-alor</t>
+        </is>
+      </c>
+      <c r="H665" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/08/kementan-1786171453519_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I665" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>Proyek Ruang Dansa Gedung Putih Diminta Disetop, Trump Naik Pitam!</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:40:00 +0700</t>
+        </is>
+      </c>
+      <c r="D666" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>Pengadilan Banding Federal AS melayangkan surat teguran ke Presiden AS Donald Trump</t>
+        </is>
+      </c>
+      <c r="F666" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G666" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260808104508-4-757593/proyek-ruang-dansa-gedung-putih-diminta-disetop-trump-naik-pitam</t>
+        </is>
+      </c>
+      <c r="H666" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/04/presiden-as-donald-trump-menari-saat-menyampaikan-pidato-tentang-perekonomian-di-general-motors-proving-ground-di-milford-mich-1785832321413_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I666" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>Narita Shibori dan Perjalanan Menjadi UMKM Inklusif Binaan Pertamina</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:04:47 +0700</t>
+        </is>
+      </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E667" t="inlineStr">
+        <is>
+          <t>UMKM binaan Pertamina berhasil menembus pasar luas</t>
+        </is>
+      </c>
+      <c r="F667" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G667" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260808125945-4-757603/narita-shibori-dan-perjalanan-menjadi-umkm-inklusif-binaan-pertamina</t>
+        </is>
+      </c>
+      <c r="H667" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/08/pertamina-umkm-1786169063887_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I667" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>Video: Inovasi Bikin Benih Sayur Tahan Hama-Cuaca Ekstrem, Petani Cuan</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 13:00:29 +0700</t>
+        </is>
+      </c>
+      <c r="D668" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr">
+        <is>
+          <t>Inovasi Hasilkan Benih Sayur Tahan Hama dan Perubahan Cuaca, Petani Makin Cuan</t>
+        </is>
+      </c>
+      <c r="F668" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G668" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260804140328-8-756453/video-inovasi-bikin-benih-sayur-tahan-hama-cuaca-ekstrem-petani-cuan</t>
+        </is>
+      </c>
+      <c r="H668" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/04/inovasi-hasilkan-benih-sayur-tahan-hama-perubahan-cuaca-petani-makin-cuan-1785827396437_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I668" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>RI Bakal Punya Pabrik Baterai EV Raksasa, Ini Pemiliknya</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:20:00 +0700</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>Indonesia sebentar lagi akan memiliki pabrik baterai ev terbesar se Asia Tenggara</t>
+        </is>
+      </c>
+      <c r="F669" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G669" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260808093139-4-757588/ri-bakal-punya-pabrik-baterai-ev-raksasa-ini-pemiliknya</t>
+        </is>
+      </c>
+      <c r="H669" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/04/11/jac-motors-menghadirkan-urbanmover-n90-ev-cnbc-indonesiatias-budiarto-1775908116224_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I669" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>Video: Bikin Percaya Diri, Intip Cara Raditya Dika Pilih Pasta Gigi</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:00:37 +0700</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E670" t="inlineStr">
+        <is>
+          <t>Bikin Percaya Diri, Intip Cara Raditya Dika Pilih Pasta Gigi</t>
+        </is>
+      </c>
+      <c r="F670" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G670" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260804114737-8-756364/video-bikin-percaya-diri-intip-cara-raditya-dika-pilih-pasta-gigi</t>
+        </is>
+      </c>
+      <c r="H670" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/04/inovasi-pasta-gigi-atasi-masalah-gigi-berlubang-gigi-sensitif-1785822995159_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I670" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>Telkom Rampungkan Spin-Off InfraCo Tahap 2, Transaksi Capai Rp49,9 T</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:13:37 +0700</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>dpu</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr">
+        <is>
+          <t>Telkom melakukan Spin-Off InfraCo Tahap 2 untuk memperkuat infrastruktur digital. Langkah ini mendukung pertumbuhan dan efisiensi layanan konektivitas.</t>
+        </is>
+      </c>
+      <c r="F671" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G671" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260808140846-37-757619/telkom-rampungkan-spin-off-infraco-tahap-2-transaksi-capai-rp499-t</t>
+        </is>
+      </c>
+      <c r="H671" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/08/telkom-1786173187593_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I671" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>Finansial</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>Nilai Transaksi QRIS Capai Rp 600,69 Triliun hingga Juni 2026</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:10:00 +0700</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>Friska Yolandha</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA — Bank Indonesia (BI) mencatat volume transaksi digital Quick Response Code Indonesian Standard atau QRIS menembus 12,55 miliar di tanah air sepanjang paruh pertama 2026. Nilai ini...</t>
+        </is>
+      </c>
+      <c r="F672" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G672" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjg2yp370/nilai-transaksi-qris-capai-rp-60069-triliun-hingga-juni-2026</t>
+        </is>
+      </c>
+      <c r="H672" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/000552000-1769000525-830-556.jpg</t>
+        </is>
+      </c>
+      <c r="I672" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>Polda Metro Tegaskan Kondisi Jakarta Aman dan Terkendali</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:22:01 +0700</t>
+        </is>
+      </c>
+      <c r="D673" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr">
+        <is>
+          <t>Menurut Budi, kondisi Jakarta yang aman terlihat dari aktivitas warga yang tetap berjalan.</t>
+        </is>
+      </c>
+      <c r="F673" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G673" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265170/polda-metro-tegaskan-kondisi-jakarta-aman-dan-terkendali</t>
+        </is>
+      </c>
+      <c r="H673" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/5Yh44dykVy3wGV-hz5GCImLG2Gs=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/5424247/original/074560000_1764137623-Tes_DNA.jpeg</t>
+        </is>
+      </c>
+      <c r="I673" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>Kabar Terbaru Penyelidikan Kematian Sutrimo</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:31:25 +0700</t>
+        </is>
+      </c>
+      <c r="D674" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>Ada dugaan kematian Sutrimo tak wajar.</t>
+        </is>
+      </c>
+      <c r="F674" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G674" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265137/kabar-terbaru-penyelidikan-kematian-sutrimo</t>
+        </is>
+      </c>
+      <c r="H674" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/vQOZUdDZgZjxCauRoos9OZyE238=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9308043/original/073508400_1785126922-WhatsApp_Image_2026-07-27_at_11.26.57.jpeg</t>
+        </is>
+      </c>
+      <c r="I674" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>Otomotif</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>Fuso Telah Kirim 7.800 Unit Canter buat Koperasi Merah Putih</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:25:37 +0700</t>
+        </is>
+      </c>
+      <c r="D675" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr">
+        <is>
+          <t>Mitsubishi Fuso berkesempatan untuk men-supply sebanyak 20.600 unit Canter, itu sampai Desember 2026.</t>
+        </is>
+      </c>
+      <c r="F675" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G675" t="inlineStr">
+        <is>
+          <t>https://otomotif.kompas.com/read/2026/08/08/172100415/fuso-telah-kirim-7.800-unit-canter-buat-koperasi-merah-putih</t>
+        </is>
+      </c>
+      <c r="H675" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/Wbqobp94J1jJAPytzfsE-pFh5zA=/277x0:3661x2256/1200x675/filters:watermark(data/photo/2026/01/30/697c81750a668.png,0,-0,1)/data/photo/2026/07/31/6a6b8f328c609.jpg</t>
+        </is>
+      </c>
+      <c r="I675" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>Bola</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>Timnas Indonesia Tersingkir dari Piala AFF, John Herdman Yakin Juara di ASEAN Cup</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:25:37 +0700</t>
+        </is>
+      </c>
+      <c r="D676" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>Pelatih John Herdman yakin Timnas Indonesia dapat meraih trofi FIFA ASEAN Cup 2026.</t>
+        </is>
+      </c>
+      <c r="F676" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G676" t="inlineStr">
+        <is>
+          <t>https://bola.kompas.com/read/2026/08/08/16540128/timnas-indonesia-tersingkir-dari-piala-aff-john-herdman-yakin-juara-di-asean-cup</t>
+        </is>
+      </c>
+      <c r="H676" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/xzNQPrLMJtS2ZrJbYs0hChS0VNo=/1x0:1600x1066/1200x675/filters:watermark(data/photo/2026/01/30/697c8163c3944.png,0,-0,1)/data/photo/2026/08/05/6a726ecc87626.jpeg</t>
+        </is>
+      </c>
+      <c r="I676" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>Otomotif</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>Aira EV dan Air ev Beda Kelas? Ini Penjelasan Wuling</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:25:37 +0700</t>
+        </is>
+      </c>
+      <c r="D677" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>Wuling menegaskan Aira EV dan Air ev merupakan dua model berbeda dengan pendekatan desain yang tidak sama.</t>
+        </is>
+      </c>
+      <c r="F677" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G677" t="inlineStr">
+        <is>
+          <t>https://otomotif.kompas.com/read/2026/08/08/161826415/aira-ev-dan-air-ev-beda-kelas-ini-penjelasan-wuling</t>
+        </is>
+      </c>
+      <c r="H677" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/9Nh2k0FCi3Sa9ybQqP02orNgR5E=/134x0:1286x768/1200x675/filters:watermark(data/photo/2026/01/30/697c81750a668.png,0,-0,1)/data/photo/2026/08/08/6a76e475b38ca.png</t>
+        </is>
+      </c>
+      <c r="I677" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I609"/>
+  <autoFilter ref="A1:I677"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-08 11:23 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-08.xlsx
+++ b/data/berita_2026-08-08.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$677</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$716</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I677"/>
+  <dimension ref="A1:I716"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -32255,8 +32255,1841 @@
         </is>
       </c>
     </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>Top News</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>John Herdman janji benahi skuad Garuda seusai Piala AFF</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:56:08 +0700</t>
+        </is>
+      </c>
+      <c r="D678" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr">
+        <is>
+          <t>Pelatih tim nasional Indonesia John Herdman berjanji membenahi skuad Garuda demi punya semangat baru setelah gagal ...</t>
+        </is>
+      </c>
+      <c r="F678" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G678" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685799/john-herdman-janji-benahi-skuad-garuda-seusai-piala-aff</t>
+        </is>
+      </c>
+      <c r="H678" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/timnas-indonesia-dikalahkan-vietnam-di-piala-aff-2833619.jpg</t>
+        </is>
+      </c>
+      <c r="I678" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>Top News</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>Gunung Lewotobi Laki-laki erupsi empat kali, abu capai 500 meter</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:40:12 +0700</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr">
+        <is>
+          <t>Gunung Lewotobi Laki-laki di Kabupaten Flores Timur, Nusa Tenggara Timur dilaporkan mengalami empat kali erupsi pada ...</t>
+        </is>
+      </c>
+      <c r="F679" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G679" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685788/gunung-lewotobi-laki-laki-erupsi-empat-kali-abu-capai-500-meter</t>
+        </is>
+      </c>
+      <c r="H679" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG_20260808_181510_1.jpg</t>
+        </is>
+      </c>
+      <c r="I679" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>Mendag Dorong Pembahasan Perluasan Akses Pembiayaan UMKM di BRICS TMM</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:45:30 +0700</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>Dea Duta Aulia</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>Mendag Budi Santoso tekankan pentingnya sistem perdagangan berbasis aturan untuk mendukung UMKM, meningkatkan daya saing, dan akses pembiayaan di pasar global.</t>
+        </is>
+      </c>
+      <c r="F680" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G680" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610046/mendag-dorong-pembahasan-perluasan-akses-pembiayaan-umkm-di-brics-tmm</t>
+        </is>
+      </c>
+      <c r="H680" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/mendag-dorong-pembahasan-perluasan-akses-pembiayaan-umkm-di-brics-tmm-1786185844158_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I680" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>Depan Seskab Teddy, Siswa SR Bacakan Puisi 'Dari Jalanan Menuju Harapan'</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:38:35 +0700</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>Dea Duta Aulia</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr">
+        <is>
+          <t>Siswa Sekolah Rakyat tampil percaya diri di MPLS, menunjukkan kemajuan pendidikan. Program ini dukung akses pendidikan berkualitas bagi anak-anak kurang mampu.</t>
+        </is>
+      </c>
+      <c r="F681" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G681" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610041/depan-seskab-teddy-siswa-sr-bacakan-puisi-dari-jalanan-menuju-harapan</t>
+        </is>
+      </c>
+      <c r="H681" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/depan-seskab-teddy-siswa-sr-bacakan-puisi-dari-jalanan-menuju-harapan-1786185469892_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I681" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>Gagal Nyalip, Pemotor di Klapanunggal Bogor Tewas Usai Terlindas Truk</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:31:34 +0700</t>
+        </is>
+      </c>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>Rizky Adha Mahendra</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr">
+        <is>
+          <t>Kecelakaan lalu lintas sebuah truk dan sepeda motor terjadi di Desa Cikahuripan, Kecamatan Klapanunggal, Bogor, Jawa Barat. Pengendara motor meninggal dunia.</t>
+        </is>
+      </c>
+      <c r="F682" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G682" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610036/gagal-nyalip-pemotor-di-klapanunggal-bogor-tewas-usai-terlindas-truk</t>
+        </is>
+      </c>
+      <c r="H682" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2023/05/15/ilustrasi-kecelakaan_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I682" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>Raih Penghargaan detiktimur Awards, Harris Arthur Genjot Profesi Advokat</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:15:06 +0700</t>
+        </is>
+      </c>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>Fara Difa Alfeni</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr">
+        <is>
+          <t>Peradi Profesional, organisasi advokat baru, perkuat pendidikan hukum dengan kerja sama perguruan tinggi. Dapatkan penghargaan atas kemajuan pendidikan advokat.</t>
+        </is>
+      </c>
+      <c r="F683" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G683" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610025/raih-penghargaan-detiktimur-awards-harris-arthur-genjot-profesi-advokat</t>
+        </is>
+      </c>
+      <c r="H683" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/raih-penghargaan-detiktimur-awards-harris-arthur-genjot-profesi-advokat-1786184071737_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I683" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>Besok Serbu Transmart Full Day Sale! Diskon Melimpah 50% + 20%</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:55:32 +0700</t>
+        </is>
+      </c>
+      <c r="D684" t="inlineStr">
+        <is>
+          <t>Ignacio Geordi Oswaldo</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>Transmart Full Day Sale hadir lagi besok, Minggu 9 Agustus 2026.</t>
+        </is>
+      </c>
+      <c r="F684" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G684" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8609344/besok-serbu-transmart-full-day-sale-diskon-melimpah-50-20</t>
+        </is>
+      </c>
+      <c r="H684" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/transmart-full-day-sale-9-agustus-2026-1786121298154_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I684" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>Aisyah Aqilah Ungkap Sisi Introvert, Cuma Berisik di Depan Orang Terpercaya</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:15:10 +0700</t>
+        </is>
+      </c>
+      <c r="D685" t="inlineStr">
+        <is>
+          <t>Muhammad Ahsan Nurrijal</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr">
+        <is>
+          <t>Aisyah Aqilah ungkap sisi introvertnya, hanya berisik di depan orang terpercaya. Ia ingin terus berkembang dan menjadi pribadi yang lebih baik.</t>
+        </is>
+      </c>
+      <c r="F685" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G685" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8610081/aisyah-aqilah-ungkap-sisi-introvert-cuma-berisik-di-depan-orang-terpercaya</t>
+        </is>
+      </c>
+      <c r="H685" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/20/aisyah-aqilah-1784538909078_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I685" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>Anggi Rantika Wujudkan Mimpi Keliling Eropa, Terima Kasih ke Oki Rengga</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:11:48 +0700</t>
+        </is>
+      </c>
+      <c r="D686" t="inlineStr">
+        <is>
+          <t>Mauludi Rismoyo</t>
+        </is>
+      </c>
+      <c r="E686" t="inlineStr">
+        <is>
+          <t>Anggi Rantika lagi keliling Eropa. Beberapa negara disinggahinya untuk mewujudkan impian.</t>
+        </is>
+      </c>
+      <c r="F686" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G686" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8610018/anggi-rantika-wujudkan-mimpi-keliling-eropa-terima-kasih-ke-oki-rengga</t>
+        </is>
+      </c>
+      <c r="H686" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/anggi-rantika-1786179323662_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I686" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>Kecewa dan Malu, La Grande Indonesia Murka Timnas Tersingkir dari Piala AFF 2026</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:17:50 +0700</t>
+        </is>
+      </c>
+      <c r="D687" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr">
+        <is>
+          <t>Kelompok suporter tersebut mengunggah gambar Ketua Umum PSSI Erick Thohir yang tengah bersandar di dinding.</t>
+        </is>
+      </c>
+      <c r="F687" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G687" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865801/kecewa-dan-malu-la-grande-indonesia-murka-timnas-tersingkir-dari-piala-aff-2026</t>
+        </is>
+      </c>
+      <c r="H687" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/c0nSoWRrfQLO1x_KKweK-kGi8Jw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/La-Grande-Indonesia-LGI-suporter-Timnas.jpg</t>
+        </is>
+      </c>
+      <c r="I687" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>Alasan John Herdman Mainkan Cahya Supriadi di Laga Kontra Singapura, Hukuman Buat Nadeo?</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:15:48 +0700</t>
+        </is>
+      </c>
+      <c r="D688" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr">
+        <is>
+          <t>John Herdman sengaja memberikan kesempatan kepada Nadeo dan Cahya untuk bersaing memperebutkan posisi</t>
+        </is>
+      </c>
+      <c r="F688" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G688" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865800/alasan-john-herdman-mainkan-cahya-supriadi-di-laga-kontra-singapura-hukuman-buat-nadeo</t>
+        </is>
+      </c>
+      <c r="H688" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/iboht6amQhsYVg3hY7SU_axQqZo=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Aksi-kiper-Timnas-Indonesia-Cahya-Supriadi-dan-Beckham-Putra-berusaha-meredam-pemain-Singapura.jpg</t>
+        </is>
+      </c>
+      <c r="I688" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>Dominan Tapi Gagal Menang, John Herdman Bongkar Masalah Timnas Indonesia: Gegara Wasit?</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:13:17 +0700</t>
+        </is>
+      </c>
+      <c r="D689" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E689" t="inlineStr">
+        <is>
+          <t>Usai pertandingan, John Herdman mengakui timnya sebenarnya memiliki cukup banyak peluang untuk memenangkan pertandingan.</t>
+        </is>
+      </c>
+      <c r="F689" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G689" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865799/dominan-tapi-gagal-menang-john-herdman-bongkar-masalah-timnas-indonesia-gegara-wasit</t>
+        </is>
+      </c>
+      <c r="H689" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/iP_P_SP0LLpWUqXvqwDcAe20vcY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/TELAN-KEKALAHAN-Pelatih-TImnas-Indonesia-John-Herdman-bersama-sang-kapten-Rizky-Ridho.jpg</t>
+        </is>
+      </c>
+      <c r="I689" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>Hasil SEA V Cup 2026 Hari Ini: Indonesia Ajek Ketiga usai Kalah, Thailand Solid di Puncak Klasemen</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:12:59 +0700</t>
+        </is>
+      </c>
+      <c r="D690" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E690" t="inlineStr">
+        <is>
+          <t>Indonesia tak beranjak dari posisi ketiga klasemen SEA V Cup 2026 seusai kalah 3-0 dari Thailand sebagai tim peringkat pertama.</t>
+        </is>
+      </c>
+      <c r="F690" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G690" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7865798/hasil-sea-v-cup-2026-hari-ini-indonesia-ajek-ketiga-usai-kalah-thailand-solid-di-puncak-klasemen</t>
+        </is>
+      </c>
+      <c r="H690" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/LAwHs6XeRlKtxkdALLGPxJSPCrQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Pemain-Timnas-Voli-Putri-Indonesia-berselebrasi-setelah-mencetak.jpg</t>
+        </is>
+      </c>
+      <c r="I690" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>Xabi Alonso Terkejut Lihat Antusiasme Fans Indonesia, Chelsea Siap Tampil Maksimal Lawan AC Milan</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:11:23 +0700</t>
+        </is>
+      </c>
+      <c r="D691" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr">
+        <is>
+          <t>Chelsea dijadwalkan menghadapi AC Milan dalam pertandingan pramusim di Stadion Utama Gelora Bung Karno (SUGBK), Jakarta, Sabtu (8/8/2026).</t>
+        </is>
+      </c>
+      <c r="F691" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G691" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865797/xabi-alonso-terkejut-lihat-antusiasme-fans-indonesia-chelsea-siap-tampil-maksimal-lawan-ac-milan</t>
+        </is>
+      </c>
+      <c r="H691" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/d0YkIVb0C4q9ACj03o8AIfElBBc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/PERSIAPAN-JELANG-LAGA-Pelatih-Chelsea-Xabi-Alonso.jpg</t>
+        </is>
+      </c>
+      <c r="I691" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>Pasrahnya Orang Tua Siswa SDN di Bandung yang Sekolahnya Digembok Ahli Waris, Eva: Masih Khawatir</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:11:01 +0700</t>
+        </is>
+      </c>
+      <c r="D692" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr">
+        <is>
+          <t>Gerbang SDN 026 Bojongloa Bandung digembok ahli waris usai menang sengketa lahan. Orang tua murid khawatir insiden serupa terulang kembali.</t>
+        </is>
+      </c>
+      <c r="F692" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G692" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865796/pasrahnya-orang-tua-siswa-sdn-di-bandung-yang-sekolahnya-digembok-ahli-waris-eva-masih-khawatir</t>
+        </is>
+      </c>
+      <c r="H692" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/hu_L0--7BOaW0gxFkPPXPGh7Xjg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/sdn-026-bojongloa-disegel-asdf-wef.jpg</t>
+        </is>
+      </c>
+      <c r="I692" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>Indonesia Gagal di Piala AFF 2026, John Herdman Sudah Siapkan Target Trofi Berikutnya</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:08:47 +0700</t>
+        </is>
+      </c>
+      <c r="D693" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr">
+        <is>
+          <t>Menurut Herdman, Piala AFF 2026 juga menjadi kesempatan untuk melihat perkembangan sejumlah pemain domestik</t>
+        </is>
+      </c>
+      <c r="F693" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G693" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865795/indonesia-gagal-di-piala-aff-2026-john-herdman-sudah-siapkan-target-trofi-berikutnya</t>
+        </is>
+      </c>
+      <c r="H693" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/5--Pv7tebNEyl0mxHHmRV8UW3WE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Pelatih-Timnas-Indonesia-John-Herdman-saat-diwawancarai.jpg</t>
+        </is>
+      </c>
+      <c r="I693" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>Industri Pertambangan Terus Tingkatkan Kesiapsiagaan Hadapi Keadaan Darurat</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:06:38 +0700</t>
+        </is>
+      </c>
+      <c r="D694" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E694" t="inlineStr">
+        <is>
+          <t>Keikutsertaan puluhan tim ERT menjadi ajang untuk menguji kemampuan dalam menghadapi berbagai skenario keadaan darurat.</t>
+        </is>
+      </c>
+      <c r="F694" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G694" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865794/industri-pertambangan-terus-tingkatkan-kesiapsiagaan-hadapi-keadaan-darurat</t>
+        </is>
+      </c>
+      <c r="H694" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/_iZmI2SqvE1DJSCAJJC0cDHDVWQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/2026-sebagai-ajang-menguji-ko-ndisi-darurat.jpg</t>
+        </is>
+      </c>
+      <c r="I694" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>Harta Destry Damayanti yang Masuk Nominasi Calon Gubernur BI, Lebih Banyak dari Perry Warjiyo</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:48:01 +0700</t>
+        </is>
+      </c>
+      <c r="D695" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr">
+        <is>
+          <t>Berikut ini adalah harta kekayaan dari Destry Damayanti yang namanya masuk nominasi sebagai calon Gubernur Bank Indonesia (BI).</t>
+        </is>
+      </c>
+      <c r="F695" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G695" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865793/harta-destry-damayanti-yang-masuk-nominasi-calon-gubernur-bi-lebih-banyak-dari-perry-warjiyo</t>
+        </is>
+      </c>
+      <c r="H695" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/RlcDz-yUShtNNTSESrAD7JTmZV4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/INFOGRAFIS-Profil-PJS-Gubernur-BI-Destry-Damayanti.jpg</t>
+        </is>
+      </c>
+      <c r="I695" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>Spesifikasi ADVAN V11, Tablet Rp2,49 Juta Sudah Dibekali Gemini AI</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:47:24 +0700</t>
+        </is>
+      </c>
+      <c r="D696" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>ADVAN V11 meluncur dengan harga Rp2,49 juta, membawa Gemini AI, layar 11 inci FHD+, keyboard, dan RAM hingga 12 GB.</t>
+        </is>
+      </c>
+      <c r="F696" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G696" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/techno/7865792/spesifikasi-advan-v11-tablet-rp249-juta-sudah-dibekali-gemini-ai</t>
+        </is>
+      </c>
+      <c r="H696" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/J00MPdnMv05OTdzyq4i0e-IAvQg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ADVAN-V11.jpg</t>
+        </is>
+      </c>
+      <c r="I696" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>Perkuat Pendidikan Vokasi, Kelas Hino di SMK Lahirkan Ratusan Mekanik Handal</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:46:15 +0700</t>
+        </is>
+      </c>
+      <c r="D697" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>Saat ini sebanyak 350 lebih lulusan SMK bergabung dan bekerja di jaringan bengkel resmi Hino di  berbagai kota.</t>
+        </is>
+      </c>
+      <c r="F697" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G697" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/otomotif/7865791/perkuat-pendidikan-vokasi-kelas-hino-di-smk-lahirkan-ratusan-mekanik-handal</t>
+        </is>
+      </c>
+      <c r="H697" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/X9VqgsvklrT6IueRZOxEs5WSSp4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Diskusi-pendidikan-vokasi-Hino-GiIAS-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I697" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>Kasus Siswi SMP Dibunuh Mantan Pacar di Nabire, Psikolog Soroti Peran Sekolah dan Orang Tua</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:41:27 +0700</t>
+        </is>
+      </c>
+      <c r="D698" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E698" t="inlineStr">
+        <is>
+          <t>Psikolog UMM mendorong kolaborasi sekolah dan orang tua untuk mencegah kekerasan remaja dengan memperkuat regulasi emosi.</t>
+        </is>
+      </c>
+      <c r="F698" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G698" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865790/kasus-siswi-smp-dibunuh-mantan-pacar-di-nabire-psikolog-soroti-peran-sekolah-dan-orang-tua</t>
+        </is>
+      </c>
+      <c r="H698" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/rmbnvOgjCJYELl7JTwXVpirg4a8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Siswi-SMP-Dibunuh-Mantan-Pacar-di-Nabire-Kenapa-Anak-Bisa-Berbuat-Sadis-Ini-Penjelasan-Psikolog.jpg</t>
+        </is>
+      </c>
+      <c r="I698" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>Leapmotor Mulai Rakit Lokal B10 dan C10 di National Assemblers Purwakarta</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:38:41 +0700</t>
+        </is>
+      </c>
+      <c r="D699" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E699" t="inlineStr">
+        <is>
+          <t>Leapmotor resmi memulai perakitan lokal kendaraan listrik B10 dan C10 secara lokal di Purwakarta.</t>
+        </is>
+      </c>
+      <c r="F699" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G699" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/otomotif/7865789/leapmotor-mulai-rakit-lokal-b10-dan-c10-di-national-assemblers-purwakarta</t>
+        </is>
+      </c>
+      <c r="H699" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/FaJ8n4VvVjGnLUMJ_iQkEQfSHuA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Perakitan-Leapmotor-Purwakarta-OK.jpg</t>
+        </is>
+      </c>
+      <c r="I699" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>Persib Resmi Datangkan Bek Kroasia Danijel Loncar, Jadi Rekrutan Kedelapan Maung Bandung</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:31:13 +0700</t>
+        </is>
+      </c>
+      <c r="D700" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E700" t="inlineStr">
+        <is>
+          <t>Persib Bandung resmi mendatangkan bek Kroasia Danijel Loncar dengan kontrak dua musim. Menjadi rekrutan kedelapan Maung Bandung untuk musim 2026/2027.</t>
+        </is>
+      </c>
+      <c r="F700" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G700" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865788/persib-resmi-datangkan-bek-kroasia-danijel-loncar-jadi-rekrutan-kedelapan-maung-bandung</t>
+        </is>
+      </c>
+      <c r="H700" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/9jN0aVX-k0u2RyRpkd85Sy1x-9c=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Persib-Bandung-resmi-mendatangkan-bek-tengah-asal-Kroasia-Danijel-Loncar.jpg</t>
+        </is>
+      </c>
+      <c r="I700" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>Panggung Penuh Ancaman bagi Lionel Messi, La Pulga Paling Sering Diteror di Piala Dunia</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:29:54 +0700</t>
+        </is>
+      </c>
+      <c r="D701" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E701" t="inlineStr">
+        <is>
+          <t>Menurut sebuah laporan kepolisan Amerika Serikat, Lionel Messi menjadi pemain yang paling sering mendapatkan ancaman pembunuhan selama Piala Dunia</t>
+        </is>
+      </c>
+      <c r="F701" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G701" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865787/panggung-penuh-ancaman-bagi-lionel-messi-la-pulga-paling-sering-diteror-di-piala-dunia</t>
+        </is>
+      </c>
+      <c r="H701" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/CcGdnR2E68FXvD_gId03BzCbeRg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Lionel-Messi-vs-Angola.jpg</t>
+        </is>
+      </c>
+      <c r="I701" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>5 Polisi Dipecat Kasus Kematian Brigadir Eko di Jambi, Korban Awalnya Disebut Jatuh</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:24:11 +0700</t>
+        </is>
+      </c>
+      <c r="D702" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E702" t="inlineStr">
+        <is>
+          <t>Brigadir Eko, anggota polisi di Kabupaten Tanjung Jabung Timur ditemukan meninggal di kos-kosan miliknya di Desa Talang Babat</t>
+        </is>
+      </c>
+      <c r="F702" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G702" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865786/5-polisi-dipecat-kasus-kematian-brigadir-eko-di-jambi-korban-awalnya-disebut-jatuh</t>
+        </is>
+      </c>
+      <c r="H702" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/BBgBU-67z4h-pvl8VwqwvCWCNXs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Penampakan-rumah-indekos-milik-Brigpol-Eko-Winarto-Saputra.jpg</t>
+        </is>
+      </c>
+      <c r="I702" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>PM Thailand Revisi UU Senjata Api: Pemilik Senpi Ikut Dijerat Jika Barangnya Dicuri untuk Penembakan</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:20:28 +0700</t>
+        </is>
+      </c>
+      <c r="D703" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E703" t="inlineStr">
+        <is>
+          <t>Jika sebuah senpii digunakan oleh pihak lain untuk melakukan aksi penembakan di Nothanburi, maka pemilik senjata juga akan dihukum berat</t>
+        </is>
+      </c>
+      <c r="F703" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G703" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7865785/pm-thailand-revisi-uu-senjata-api-pemilik-senpi-ikut-dijerat-jika-barangnya-dicuri-untuk-penembakan</t>
+        </is>
+      </c>
+      <c r="H703" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/eaPRWuU-Atqx4rz6_Ay0D7pj2V4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Anutin-Charnvirakul-bersama-Partai-Bhumjaithai.jpg</t>
+        </is>
+      </c>
+      <c r="I703" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>Video: Jurus Bank Jatim Agar Sinergi KUB Saling Menguntungkan BPD</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:00:48 +0700</t>
+        </is>
+      </c>
+      <c r="D704" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E704" t="inlineStr">
+        <is>
+          <t>Agar Sinergi KUB Saling Menguntungkan BPD, Dirut Bank Jatim Ungkap Strateginya</t>
+        </is>
+      </c>
+      <c r="F704" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G704" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260805161846-19-756845/video-jurus-bank-jatim-agar-sinergi-kub-saling-menguntungkan-bpd</t>
+        </is>
+      </c>
+      <c r="H704" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/05/agar-sinergi-kub-saling-menguntungkan-bpd-dirut-bank-jatim-ungkap-strateginya-1785923045436_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I704" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>Setelah Resign dan Bantu Ibu Jaga Warung, Kini Pemilik 23.000 Toko</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:45:16 +0700</t>
+        </is>
+      </c>
+      <c r="D705" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E705" t="inlineStr">
+        <is>
+          <t>Djoko Susanto, pendiri Alfamart, memulai karier dari warung kelontong.</t>
+        </is>
+      </c>
+      <c r="F705" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G705" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260808141939-17-757620/setelah-resign-dan-bantu-ibu-jaga-warung-kini-pemilik-23000-toko</t>
+        </is>
+      </c>
+      <c r="H705" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2025/10/28/djoko-susanto-dokumen-alfa-groupyoutube-momentum-talk-1761616161938_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I705" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>Danantara Siapkan Rp44,5 Triliun untuk Garap Bisnis Daging Asia</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:00:07 +0700</t>
+        </is>
+      </c>
+      <c r="D706" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E706" t="inlineStr">
+        <is>
+          <t>BPI Danantara dan JBS NV sepakat investasi US$2,5 miliar untuk joint venture di pasar protein Asia Tenggara, Australia, dan Selandia Baru.</t>
+        </is>
+      </c>
+      <c r="F706" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G706" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260808140107-17-757617/danantara-siapkan-rp445-triliun-untuk-garap-bisnis-daging-asia</t>
+        </is>
+      </c>
+      <c r="H706" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2025/06/30/danantara-indonesia-cnbc-indonesiamuhammad-sabki-1751266532126_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I706" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>Ingin Anak Seperti Warren Buffett, Orang Tua China Siapkan Rp34 Juta</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:30:00 +0700</t>
+        </is>
+      </c>
+      <c r="D707" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E707" t="inlineStr">
+        <is>
+          <t>Muncul fenomena orang tua yang ingin anaknya seperti Wareen Buffett</t>
+        </is>
+      </c>
+      <c r="F707" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G707" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260808131101-17-757604/ingin-anak-seperti-warren-buffett-orang-tua-china-siapkan-rp34-juta</t>
+        </is>
+      </c>
+      <c r="H707" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2022/11/03/jurus-hemat-ala-warren-buffet-amin-ikut-kaya-raya_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I707" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>Dulu Raja Sawit Dunia, Negara Ini Sekarang Belajar dari Malaysia</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:15:00 +0700</t>
+        </is>
+      </c>
+      <c r="D708" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E708" t="inlineStr">
+        <is>
+          <t>Nigeria dahulunya adalah pemimpin sawit di dunia, kenapa sekarang belajar ke Malaysia?</t>
+        </is>
+      </c>
+      <c r="F708" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G708" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260808105502-17-757595/dulu-raja-sawit-dunia-negara-ini-sekarang-belajar-dari-malaysia</t>
+        </is>
+      </c>
+      <c r="H708" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/04/16/ilustrasi-lahan-sawit-1776312558427_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I708" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>Pendatang China Ini Jualan Kopi, Berubah Jadi Orang Terkaya RI</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:40:00 +0700</t>
+        </is>
+      </c>
+      <c r="D709" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E709" t="inlineStr">
+        <is>
+          <t>Seorang perantau China yang memulai kehidupannya dengan beradagang kopi</t>
+        </is>
+      </c>
+      <c r="F709" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G709" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260808085842-17-757585/pendatang-china-ini-jualan-kopi-berubah-jadi-orang-terkaya-ri</t>
+        </is>
+      </c>
+      <c r="H709" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2023/04/11/kapal-api_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I709" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>Konglomerat RI Ini Rutin Bolak-Balik Gunung Kawi, Begini Kisahnya</t>
+        </is>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 11:20:00 +0700</t>
+        </is>
+      </c>
+      <c r="D710" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E710" t="inlineStr">
+        <is>
+          <t>Kisah konglomerat RI yang rajin bolak balik ke Gunung Kawi</t>
+        </is>
+      </c>
+      <c r="F710" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G710" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260808091812-17-757587/konglomerat-ri-ini-rutin-bolak-balik-gunung-kawi-begini-kisahnya</t>
+        </is>
+      </c>
+      <c r="H710" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/07/06/gunung-kawi-1783311497189_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I710" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>Wamenpar Sempat Datang ke Festival Lembah Baliem Sebelum Insiden Penembakan</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:17:36 +0700</t>
+        </is>
+      </c>
+      <c r="D711" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E711" t="inlineStr">
+        <is>
+          <t>2 Orang warga luka-luka dalam insiden penembakan tersebut.</t>
+        </is>
+      </c>
+      <c r="F711" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G711" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265195/wamenpar-sempat-datang-ke-festival-lembah-baliem-sebelum-insiden-penembakan</t>
+        </is>
+      </c>
+      <c r="H711" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/Zeqr_43rDDsDTyil8vw3JLT4MeM=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9319148/original/061652600_1786187853-Screenshot_2026-08-08_181224.jpg</t>
+        </is>
+      </c>
+      <c r="I711" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>Festival Lembah Baliem Disetop Sementara Imbas Penembakan 2 Warga</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:54:32 +0700</t>
+        </is>
+      </c>
+      <c r="D712" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E712" t="inlineStr">
+        <is>
+          <t>Penghentian festival dilakukan agar aparat gabungan leluasa menangani lokasi kejadian dan memastikan keamanan di sekitar area festival.</t>
+        </is>
+      </c>
+      <c r="F712" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G712" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265181/festival-lembah-baliem-disetop-sementara-imbas-penembakan-2-warga</t>
+        </is>
+      </c>
+      <c r="H712" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/M3B9_cWxi66XWpa0o5RT2jolXaM=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9319133/original/085617400_1786186466-650b990f-554b-4466-addf-456a9511335d.jpg</t>
+        </is>
+      </c>
+      <c r="I712" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>Tembakan Meletus di Gerbang Festival Lembah Baliem, 2 Warga Luka</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:24:10 +0700</t>
+        </is>
+      </c>
+      <c r="D713" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E713" t="inlineStr">
+        <is>
+          <t>Pelaku dalam pengejaran petugas.</t>
+        </is>
+      </c>
+      <c r="F713" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G713" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265151/tembakan-meletus-di-gerbang-festival-lembah-baliem-2-warga-luka</t>
+        </is>
+      </c>
+      <c r="H713" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/uAVXqunR4fQGb6MFdwT8B7C1lAQ=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/1700256/original/092497000_1504586298-Tembak-Senjata-Api6.jpg</t>
+        </is>
+      </c>
+      <c r="I713" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>Hype</t>
+        </is>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>Saling Tulis Pesan Manis di Instagram, Dita Karang dan YouTuber Jun Curry Ahn Pacaran?</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:23:00 +0700</t>
+        </is>
+      </c>
+      <c r="D714" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E714" t="inlineStr">
+        <is>
+          <t>Dita Karang dan YouTuber Jun Curry Ahn dikabarkan berpacaran setelah unggah momen bersama</t>
+        </is>
+      </c>
+      <c r="F714" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G714" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/hype/read/2026/08/08/182209266/saling-tulis-pesan-manis-di-instagram-dita-karang-dan-youtuber-jun-curry</t>
+        </is>
+      </c>
+      <c r="H714" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/3wVtkyPKOl4JAnbwNGZCIJy8e7Q=/0x129:1199x929/1200x675/filters:watermark(data/photo/2026/01/30/697c8191ee571.png,0,-0,1)/data/photo/2026/08/08/6a77100729d30.jpg</t>
+        </is>
+      </c>
+      <c r="I714" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>5 Pastry Indonesia Terbaik Versi TasteAtlas, Mana Favoritmu?</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:23:00 +0700</t>
+        </is>
+      </c>
+      <c r="D715" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E715" t="inlineStr">
+        <is>
+          <t>5 pastry Indonesia terbaik versi TasteAtlas hadir dengan cita rasa khas. Odading, cireng, bakpia, kue bulan, dan panada jadi favorit.</t>
+        </is>
+      </c>
+      <c r="F715" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G715" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/food/read/2026/08/08/173100875/5-pastry-indonesia-terbaik-versi-tasteatlas-mana-favoritmu-</t>
+        </is>
+      </c>
+      <c r="H715" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/mGvuMU6CU4HV_Wd-CmFWXJ4r7kw=/0x0:1056x704/1200x675/filters:watermark(data/photo/2026/01/30/697c81a417f45.png,0,-0,1)/data/photo/2025/07/02/686506638d9f1.jpg</t>
+        </is>
+      </c>
+      <c r="I715" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>Eks Pengacara Pribadi Trump Resmi Jadi Jaksa Agung AS</t>
+        </is>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:23:00 +0700</t>
+        </is>
+      </c>
+      <c r="D716" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E716" t="inlineStr">
+        <is>
+          <t>Mantan pengacara pribadi Presiden Donald Trump, Todd Blanche resmi dikukuhkan sebagai Jaksa Agung Amerika Serikat, Sabtu (8/8/2026).</t>
+        </is>
+      </c>
+      <c r="F716" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G716" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/global/read/2026/08/08/170000670/eks-pengacara-pribadi-trump-resmi-jadi-jaksa-agung-as</t>
+        </is>
+      </c>
+      <c r="H716" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/_orJtuU0iJJ_hFvUrRLGxWhFrCY=/0x0:1200x800/1200x675/filters:watermark(data/photo/2026/01/30/697c81ac46b81.png,0,-0,1)/data/photo/2026/08/08/6a76fd484a811.jpg</t>
+        </is>
+      </c>
+      <c r="I716" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I677"/>
+  <autoFilter ref="A1:I716"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-08 12:29 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-08.xlsx
+++ b/data/berita_2026-08-08.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$716</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$784</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I716"/>
+  <dimension ref="A1:I784"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -34088,8 +34088,3204 @@
         </is>
       </c>
     </row>
+    <row r="717">
+      <c r="A717" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>Seskab Teddy tempati posisi kedua kinerja kabinet versi IPO</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:20:51 +0700</t>
+        </is>
+      </c>
+      <c r="D717" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E717" t="inlineStr">
+        <is>
+          <t>Sekretaris Kabinet RI Teddy Indra Wijaya menempati posisi kedua dalam penilaian positif publik terhadap kinerja jajaran ...</t>
+        </is>
+      </c>
+      <c r="F717" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G717" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685856/seskab-teddy-tempati-posisi-kedua-kinerja-kabinet-versi-ipo</t>
+        </is>
+      </c>
+      <c r="H717" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000454906.jpg</t>
+        </is>
+      </c>
+      <c r="I717" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>Bukan Sekadar Titik Transit, Stasiun Dukuh Atas Hubungkan Berbagai Pusat Aktivitas di Jabodebek</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:14:39 +0700</t>
+        </is>
+      </c>
+      <c r="D718" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E718" t="inlineStr">
+        <is>
+          <t>Setiap pagi, ribuan orang memulai aktivitasnya dari berbagai penjuru Jabodebek menggunakan LRT Jabodebek. Ada yang ...</t>
+        </is>
+      </c>
+      <c r="F718" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G718" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685853/bukan-sekadar-titik-transit-stasiun-dukuh-atas-hubungkan-berbagai-pusat-aktivitas-di-jabodebek</t>
+        </is>
+      </c>
+      <c r="H718" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000079087.jpg</t>
+        </is>
+      </c>
+      <c r="I718" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>DePA-RI dorong advokat bersatu wujudkan kepastian hukum</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:12:59 +0700</t>
+        </is>
+      </c>
+      <c r="D719" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E719" t="inlineStr">
+        <is>
+          <t>Ketua Umum Dewan Pergerakan Advokat Republik Indonesia (DePA-RI) TM Luthfi Yazid mendorong advokat dan organisasi ...</t>
+        </is>
+      </c>
+      <c r="F719" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G719" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685852/depa-ri-dorong-advokat-bersatu-wujudkan-kepastian-hukum</t>
+        </is>
+      </c>
+      <c r="H719" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000087507.jpg</t>
+        </is>
+      </c>
+      <c r="I719" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>Bruno Guimaraes gabung Arsenal dari Newcastle United</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:09:02 +0700</t>
+        </is>
+      </c>
+      <c r="D720" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E720" t="inlineStr">
+        <is>
+          <t>Gelandang asal Brasil, Bruno Guimaraes resmi bergabung Arsenal dari Newcastle United pada bursa transfer musim ...</t>
+        </is>
+      </c>
+      <c r="F720" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G720" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685848/bruno-guimaraes-gabung-arsenal-dari-newcastle-united</t>
+        </is>
+      </c>
+      <c r="H720" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000043103.jpg</t>
+        </is>
+      </c>
+      <c r="I720" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>Polda Metro-Kodam Jaya beri layanan kesehatan 1.876 warga di Monas</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:08:49 +0700</t>
+        </is>
+      </c>
+      <c r="D721" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E721" t="inlineStr">
+        <is>
+          <t>Polda Metro Jaya bersama Kodam Jaya memberi layanan kesehatan terhadap 1.876 warga dalam rangkaian Apel Kebangsaan ...</t>
+        </is>
+      </c>
+      <c r="F721" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G721" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685845/polda-metro-kodam-jaya-beri-layanan-kesehatan-1876-warga-di-monas</t>
+        </is>
+      </c>
+      <c r="H721" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001018558.jpg</t>
+        </is>
+      </c>
+      <c r="I721" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>Balai Karantina Kalbar amankan 1.286 telur Penyu dari Sambas</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:07:23 +0700</t>
+        </is>
+      </c>
+      <c r="D722" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E722" t="inlineStr">
+        <is>
+          <t>Balai Karantina Kalbar dan Satgas Pamtas TNI AD Gabma Temajuk mengamankan 1.286 telur penyu hasil temuan di dua lokasi ...</t>
+        </is>
+      </c>
+      <c r="F722" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G722" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685843/balai-karantina-kalbar-amankan-1286-telur-penyu-dari-sambas</t>
+        </is>
+      </c>
+      <c r="H722" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2012/08/20120806telur-penyu-edit.jpg</t>
+        </is>
+      </c>
+      <c r="I722" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>AGI: Hari Game Indonesia momentum untuk merayakan kreator gim lokal</t>
+        </is>
+      </c>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:04:34 +0700</t>
+        </is>
+      </c>
+      <c r="D723" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E723" t="inlineStr">
+        <is>
+          <t>Ketua Asosiasi Game Indonesia (AGI) Shafiq Husein mengatakan bahwa Hari Game Indonesia (HARGAI) 2026 merupakan momentum ...</t>
+        </is>
+      </c>
+      <c r="F723" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G723" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685841/agi-hari-game-indonesia-momentum-untuk-merayakan-kreator-gim-lokal</t>
+        </is>
+      </c>
+      <c r="H723" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000864447.jpg</t>
+        </is>
+      </c>
+      <c r="I723" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>Polda Metro kerahkan 1.200 personel amankan Chelsea vs AC Milan di GBK</t>
+        </is>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:03:09 +0700</t>
+        </is>
+      </c>
+      <c r="D724" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E724" t="inlineStr">
+        <is>
+          <t>Polda Metro Jaya mengerahkan 1.200 personel gabungan untuk mengamankan pertandingan Chelsea FC melawan AC Milan di ...</t>
+        </is>
+      </c>
+      <c r="F724" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G724" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685840/polda-metro-kerahkan-1200-personel-amankan-chelsea-vs-ac-milan-di-gbk</t>
+        </is>
+      </c>
+      <c r="H724" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001018566.jpg</t>
+        </is>
+      </c>
+      <c r="I724" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>Kemerdekaan di ruang digital</t>
+        </is>
+      </c>
+      <c r="C725" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:02:42 +0700</t>
+        </is>
+      </c>
+      <c r="D725" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E725" t="inlineStr">
+        <is>
+          <t>Menjelang 17 Agustus, kita biasanya kembali berbicara tentang kemerdekaan dengan bahasa yang klise: bebas dari ...</t>
+        </is>
+      </c>
+      <c r="F725" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G725" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685839/kemerdekaan-di-ruang-digital</t>
+        </is>
+      </c>
+      <c r="H725" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000555287.png</t>
+        </is>
+      </c>
+      <c r="I725" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>Gim lokal unjuk gigi di Hargai Playday 2026</t>
+        </is>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:02:13 +0700</t>
+        </is>
+      </c>
+      <c r="D726" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E726" t="inlineStr">
+        <is>
+          <t>Menteri Ekonomi Kreatif Teuku Riefky Harsya (kiri) mencoba gim karya pengembang lokal saat menghadiri Hari Game ...</t>
+        </is>
+      </c>
+      <c r="F726" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G726" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5685837/gim-lokal-unjuk-gigi-di-hargai-playday-2026</t>
+        </is>
+      </c>
+      <c r="H726" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/Hari-Game-Nasional-080826-IES-1A.jpg</t>
+        </is>
+      </c>
+      <c r="I726" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>Boston Celtics perkenalkan Mitchell Robinson sebagai rekrutan terbaru</t>
+        </is>
+      </c>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:50:41 +0700</t>
+        </is>
+      </c>
+      <c r="D727" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E727" t="inlineStr">
+        <is>
+          <t>Boston Celtics memperkenalkan Mitchell Robinson sebagai rekrutan terbaru untuk memperkuat posisi center dalam tim ...</t>
+        </is>
+      </c>
+      <c r="F727" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G727" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685835/boston-celtics-perkenalkan-mitchell-robinson-sebagai-rekrutan-terbaru</t>
+        </is>
+      </c>
+      <c r="H727" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000476629.jpg</t>
+        </is>
+      </c>
+      <c r="I727" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>Persib Bandung datangkan bek asal Kroasia Danijel Loncar</t>
+        </is>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:46:53 +0700</t>
+        </is>
+      </c>
+      <c r="D728" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E728" t="inlineStr">
+        <is>
+          <t>Persib Bandung mendatangkan bek tengah asal Kroasia Danijel Loncar untuk memperkuat lini pertahanan menghadapi ...</t>
+        </is>
+      </c>
+      <c r="F728" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G728" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685832/persib-bandung-datangkan-bek-asal-kroasia-danijel-loncar</t>
+        </is>
+      </c>
+      <c r="H728" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG_9303.jpeg</t>
+        </is>
+      </c>
+      <c r="I728" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>Marcos: Visi Komunitas ASEAN 2045 jadi panduan hadapi tantangan global</t>
+        </is>
+      </c>
+      <c r="C729" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:43:25 +0700</t>
+        </is>
+      </c>
+      <c r="D729" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E729" t="inlineStr">
+        <is>
+          <t>Filipina, sebagai Ketua ASEAN 2026, menegaskan penghormatannya terhadap Visi Komunitas ASEAN 2045 saat merayakan Hari ...</t>
+        </is>
+      </c>
+      <c r="F729" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G729" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685829/marcos-visi-komunitas-asean-2045-jadi-panduan-hadapi-tantangan-global</t>
+        </is>
+      </c>
+      <c r="H729" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000679895.jpg</t>
+        </is>
+      </c>
+      <c r="I729" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>Trackhouse enggan bicara gelar MotoGP meski Ogura di posisi kedua</t>
+        </is>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:42:38 +0700</t>
+        </is>
+      </c>
+      <c r="D730" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E730" t="inlineStr">
+        <is>
+          <t>Pemilik Trackhouse MotoGP Justin Marks menegaskan timnya belum memikirkan perebutan gelar juara dunia MotoGP 2026 ...</t>
+        </is>
+      </c>
+      <c r="F730" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G730" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685827/trackhouse-enggan-bicara-gelar-motogp-meski-ogura-di-posisi-kedua</t>
+        </is>
+      </c>
+      <c r="H730" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/29/ogura.jpg</t>
+        </is>
+      </c>
+      <c r="I730" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>IDAI promosikan kampanye rantai dukungan hangat bagi ibu menyusui</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:41:45 +0700</t>
+        </is>
+      </c>
+      <c r="D731" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E731" t="inlineStr">
+        <is>
+          <t>Ikatan Dokter Anak Indonesia (IDAI) mempromosikan kampanye rantai dukungan yang hangat bagi ibu menyusui guna ...</t>
+        </is>
+      </c>
+      <c r="F731" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G731" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685825/idai-promosikan-kampanye-rantai-dukungan-hangat-bagi-ibu-menyusui</t>
+        </is>
+      </c>
+      <c r="H731" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/03/11/persiapan-terminal-tirtonadi-jelang-mudik-lebaran-2748675.jpg</t>
+        </is>
+      </c>
+      <c r="I731" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>Pemkot Bandarlampung bagikan 10 ribu bendera Merah Putih sambut HUT RI</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:37:46 +0700</t>
+        </is>
+      </c>
+      <c r="D732" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E732" t="inlineStr">
+        <is>
+          <t>Pemerintah Kota (Pemkot) Bandarlampung membagikan sebanyak 10 ribu bendera Merah Putih kepada masyarakat dalam rangka ...</t>
+        </is>
+      </c>
+      <c r="F732" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G732" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685824/pemkot-bandarlampung-bagikan-10-ribu-bendera-merah-putih-sambut-hut-ri</t>
+        </is>
+      </c>
+      <c r="H732" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001141435.jpg</t>
+        </is>
+      </c>
+      <c r="I732" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>Polres Semarang ungkap pencurian ponsel disertai pembunuhan</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:31:43 +0700</t>
+        </is>
+      </c>
+      <c r="D733" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E733" t="inlineStr">
+        <is>
+          <t>Polres Semarang, Jawa Tengah, mengungkap kasus pencurian di toko telepon seluler di Ambarawa yang disertai pembunuhan ...</t>
+        </is>
+      </c>
+      <c r="F733" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G733" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685823/polres-semarang-ungkap-pencurian-ponsel-disertai-pembunuhan</t>
+        </is>
+      </c>
+      <c r="H733" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG_20260808_181914.jpg</t>
+        </is>
+      </c>
+      <c r="I733" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>Polres amankan lokasi FBLB ke-34 di Walesi Jayawijaya</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:30:30 +0700</t>
+        </is>
+      </c>
+      <c r="D734" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E734" t="inlineStr">
+        <is>
+          <t>Kepolisian Resor (Polres) Jayawijaya, Papua Pegunungan mengamankan lokasi penyelenggaraan Festival Budaya Lembah Baliem ...</t>
+        </is>
+      </c>
+      <c r="F734" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G734" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685821/polres-amankan-lokasi-fblb-ke-34-di-walesi-jayawijaya</t>
+        </is>
+      </c>
+      <c r="H734" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/WhatsApp-Image-2026-08-08-at-18.14.19.jpeg</t>
+        </is>
+      </c>
+      <c r="I734" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>Bukit Rhema, ketika wisata bertemu ruang doa dan pesan perdamaian</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:22:57 +0700</t>
+        </is>
+      </c>
+      <c r="D735" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E735" t="inlineStr">
+        <is>
+          <t>Udara sejuk menyambut langkah pengunjung yang menapaki jalan menuju sebuah bangunan berbentuk unik di atas perbukitan ...</t>
+        </is>
+      </c>
+      <c r="F735" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G735" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685819/bukit-rhema-ketika-wisata-bertemu-ruang-doa-dan-pesan-perdamaian</t>
+        </is>
+      </c>
+      <c r="H735" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG-20260808-WA0008.jpg</t>
+        </is>
+      </c>
+      <c r="I735" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>Pelatih timnas soroti potensi Mitchell Baker</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:22:18 +0700</t>
+        </is>
+      </c>
+      <c r="D736" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E736" t="inlineStr">
+        <is>
+          <t>Pelatih Timnas Indonesia John Herdman melihat sejumlah sisi positif, seperti penampilan penyerang muda Mitchell ...</t>
+        </is>
+      </c>
+      <c r="F736" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G736" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685817/pelatih-timnas-soroti-potensi-mitchell-baker</t>
+        </is>
+      </c>
+      <c r="H736" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/1003298738.jpg</t>
+        </is>
+      </c>
+      <c r="I736" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>Bapanas-Bulog salurkan bantuan pangan kepada 37.338 warga Alor-NTT</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:20:14 +0700</t>
+        </is>
+      </c>
+      <c r="D737" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E737" t="inlineStr">
+        <is>
+          <t>Perum Bulog bersama Badan Pangan Nasional (Bapanas) menyalurkan bantuan pangan perdana kepada 37.338 warga Kabupaten ...</t>
+        </is>
+      </c>
+      <c r="F737" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G737" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685816/bapanas-bulog-salurkan-bantuan-pangan-kepada-37338-warga-alor-ntt</t>
+        </is>
+      </c>
+      <c r="H737" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001665220.jpg</t>
+        </is>
+      </c>
+      <c r="I737" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>Polres Malang nyatakan Jemplang kondusif usai kebakaran Bromo</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:18:42 +0700</t>
+        </is>
+      </c>
+      <c r="D738" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E738" t="inlineStr">
+        <is>
+          <t>Kepolisian Resor Malang, Jawa Timur, menyatakan situasi di Jemplang, Desa Ngadas, Kecamatan Poncokusumo, Kabupaten ...</t>
+        </is>
+      </c>
+      <c r="F738" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G738" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685813/polres-malang-nyatakan-jemplang-kondusif-usai-kebakaran-bromo</t>
+        </is>
+      </c>
+      <c r="H738" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001407643.jpg</t>
+        </is>
+      </c>
+      <c r="I738" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>FIBA 3x3 Challenger kembali ke AS lewat FISE Birmingham 2026</t>
+        </is>
+      </c>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:15:39 +0700</t>
+        </is>
+      </c>
+      <c r="D739" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E739" t="inlineStr">
+        <is>
+          <t>Federasi Bola Basket Internasional (FIBA) 3x3 Challenger kembali lagi ke Amerika Serikat lewat seri FISE Birmingham ...</t>
+        </is>
+      </c>
+      <c r="F739" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G739" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685812/fiba-3x3-challenger-kembali-ke-as-lewat-fise-birmingham-2026</t>
+        </is>
+      </c>
+      <c r="H739" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/24/1000459387_1.jpg</t>
+        </is>
+      </c>
+      <c r="I739" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>Dishut Kalteng optimalkan patroli drone pantau titik api</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:06:07 +0700</t>
+        </is>
+      </c>
+      <c r="D740" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E740" t="inlineStr">
+        <is>
+          <t>Dinas Kehutanan (Dishut) Kalimantan Tengah mengintensifkan pemantauan potensi kebakaran hutan dan lahan (karhutla) ...</t>
+        </is>
+      </c>
+      <c r="F740" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G740" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685809/dishut-kalteng-optimalkan-patroli-drone-pantau-titik-api</t>
+        </is>
+      </c>
+      <c r="H740" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001732700.jpg</t>
+        </is>
+      </c>
+      <c r="I740" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>Pakar: Pengungkapan TPPU eks Jampidsus harus buktikan pidana asal</t>
+        </is>
+      </c>
+      <c r="C741" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:05:41 +0700</t>
+        </is>
+      </c>
+      <c r="D741" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E741" t="inlineStr">
+        <is>
+          <t>Pakar tindak pidana pencucian uang (TPPU) Yenti Garnasih mengatakan pengungkapan kasus TPPU mantan Jampidsus Febrie ...</t>
+        </is>
+      </c>
+      <c r="F741" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G741" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685807/pakar-pengungkapan-tppu-eks-jampidsus-harus-buktikan-pidana-asal</t>
+        </is>
+      </c>
+      <c r="H741" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2021/05/17/RDPU-Komisi-III-Dengan-Pansel-Capim-KPK-090919-RIV-2.jpg</t>
+        </is>
+      </c>
+      <c r="I741" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>9 amalan sunnah hari Jumat, dari mandi hingga baca Al-Kahfi</t>
+        </is>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:59:23 +0700</t>
+        </is>
+      </c>
+      <c r="D742" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E742" t="inlineStr">
+        <is>
+          <t>Hari Jumat memiliki keistimewaan bagi umat Islam karena menjadi hari yang penuh keberkahan. Selain melaksanakan shalat ...</t>
+        </is>
+      </c>
+      <c r="F742" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G742" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685803/9-amalan-sunnah-hari-jumat-dari-mandi-hingga-baca-al-kahfi</t>
+        </is>
+      </c>
+      <c r="H742" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2024/11/15/Penyintas-erupsi-Lewotobi-Jumatan-di-Mushola-darurat-151124-MT-6.jpg</t>
+        </is>
+      </c>
+      <c r="I742" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>GAPKI: Peningkatan produktivitas jaga posisi RI pimpin sawit dunia</t>
+        </is>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:56:30 +0700</t>
+        </is>
+      </c>
+      <c r="D743" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E743" t="inlineStr">
+        <is>
+          <t>Gabungan Pengusaha Kelapa Sawit Indonesia (GAPKI) menyampaikan peningkatan produktivitas petani plasma maupun ...</t>
+        </is>
+      </c>
+      <c r="F743" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G743" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685801/gapki-peningkatan-produktivitas-jaga-posisi-ri-pimpin-sawit-dunia</t>
+        </is>
+      </c>
+      <c r="H743" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/WhatsApp-Image-2026-08-08-at-14.51.38.jpeg</t>
+        </is>
+      </c>
+      <c r="I743" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>8 keutamaan membaca sholawat di hari Jumat, banyak pahalanya</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:55:51 +0700</t>
+        </is>
+      </c>
+      <c r="D744" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E744" t="inlineStr">
+        <is>
+          <t>Membaca sholawat kepada Nabi Muhammad SAW menjadi salah satu amalan yang dianjurkan bagi umat Islam, terutama pada hari ...</t>
+        </is>
+      </c>
+      <c r="F744" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G744" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685797/8-keutamaan-membaca-sholawat-di-hari-jumat-banyak-pahalanya</t>
+        </is>
+      </c>
+      <c r="H744" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/12/30/dzikir-dan-doa-akhir-tahun-2698471.jpg</t>
+        </is>
+      </c>
+      <c r="I744" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>Gula semut Banjarnegara tembus pasar Amerika, omzet capai ratusan juta</t>
+        </is>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:54:28 +0700</t>
+        </is>
+      </c>
+      <c r="D745" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E745" t="inlineStr">
+        <is>
+          <t>ANTARA - Gula semut Desa Gumelem Kulon, Kecamatan Susukan, Kabupaten Banjarnegara, Jawa Tengah, berhasil menembus ...</t>
+        </is>
+      </c>
+      <c r="F745" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G745" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5685765/gula-semut-banjarnegara-tembus-pasar-amerika-omzet-capai-ratusan-juta</t>
+        </is>
+      </c>
+      <c r="H745" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/GULA-SEMUT-BANJARNEGARA-TEMBUS-PASAR-AMERIKA-OMZET-CAPAI-RATUSAN-JUTA_1.jpg</t>
+        </is>
+      </c>
+      <c r="I745" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>Bolehkah ibu menyusui minum matcha? Ini batas aman kafeinnya</t>
+        </is>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:51:07 +0700</t>
+        </is>
+      </c>
+      <c r="D746" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E746" t="inlineStr">
+        <is>
+          <t>Matcha kini menjadi salah satu minuman favorit banyak orang. Rasanya yang khas, kandungan antioksidannya yang tinggi, ...</t>
+        </is>
+      </c>
+      <c r="F746" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G746" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685793/bolehkah-ibu-menyusui-minum-matcha-ini-batas-aman-kafeinnya</t>
+        </is>
+      </c>
+      <c r="H746" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/10/12/XxjpbeE007239_20250517_PEPFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I746" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>Contoh teks MC malam tirakatan 17 Agustus 2026, lengkap dan sopan</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:47:58 +0700</t>
+        </is>
+      </c>
+      <c r="D747" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E747" t="inlineStr">
+        <is>
+          <t>Malam tirakatan 17 Agustus menjadi salah satu tradisi masyarakat Indonesia dalam menyambut Hari Ulang Tahun Kemerdekaan ...</t>
+        </is>
+      </c>
+      <c r="F747" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G747" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685791/contoh-teks-mc-malam-tirakatan-17-agustus-2026-lengkap-dan-sopan</t>
+        </is>
+      </c>
+      <c r="H747" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2020/08/17/pawai-2.jpg</t>
+        </is>
+      </c>
+      <c r="I747" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>Humas didorong naik kelas hadapi krisis komunikasi dan multikrisis</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:46:44 +0700</t>
+        </is>
+      </c>
+      <c r="D748" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E748" t="inlineStr">
+        <is>
+          <t>ANTARA - Perhimpunan Hubungan Masyarakat Indonesia (Perhumas) menilai tantangan komunikasi publik semakin kompleks ...</t>
+        </is>
+      </c>
+      <c r="F748" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G748" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5685693/humas-didorong-naik-kelas-hadapi-krisis-komunikasi-dan-multikrisis</t>
+        </is>
+      </c>
+      <c r="H748" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/HUMAS-DIDORONG-NAIK-KELAS-HADAPI-KRISIS-KOMUNIKASI-DAN-MULTIKRISIS.jpg</t>
+        </is>
+      </c>
+      <c r="I748" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>Malam tirakatan 17 Agustus: Pengertian, makna, dan susunan acara</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:43:24 +0700</t>
+        </is>
+      </c>
+      <c r="D749" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E749" t="inlineStr">
+        <is>
+          <t>Malam tirakatan menjadi salah satu tradisi masyarakat Indonesia dalam menyambut Hari Ulang Tahun (HUT) Kemerdekaan ...</t>
+        </is>
+      </c>
+      <c r="F749" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G749" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685789/malam-tirakatan-17-agustus-pengertian-makna-dan-susunan-acara</t>
+        </is>
+      </c>
+      <c r="H749" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/latihan-gabungan-paskibraka-nasional-2026-2837235.jpg</t>
+        </is>
+      </c>
+      <c r="I749" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>Polresta Bandung menyita 6.624 botol miras berpita cukai palsu</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:36:33 +0700</t>
+        </is>
+      </c>
+      <c r="D750" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E750" t="inlineStr">
+        <is>
+          <t>Polresta Bandung, Jawa Barat, menyita 6.624 botol minuman keras (miras) berbagai merek yang diduga menggunakan pita ...</t>
+        </is>
+      </c>
+      <c r="F750" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G750" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685785/polresta-bandung-menyita-6624-botol-miras-berpita-cukai-palsu</t>
+        </is>
+      </c>
+      <c r="H750" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/487153.jpg</t>
+        </is>
+      </c>
+      <c r="I750" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>WIKA REKON Bangun Berbagai Infrastruktur Penunjang Food Estate di Wanam Papua dengan Berbagai Inovasi Engineering</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:28:28 +0700</t>
+        </is>
+      </c>
+      <c r="D751" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E751" t="inlineStr">
+        <is>
+          <t>Jakarta (ANTARA) – PT Wijaya Karya Rekayasa Konstruksi (WIKA REKON) terus berkontribusi dalam mendukung ...</t>
+        </is>
+      </c>
+      <c r="F751" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G751" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685781/wika-rekon-bangun-berbagai-infrastruktur-penunjang-food-estate-di-wanam-papua-dengan-berbagai-inovasi-engineering</t>
+        </is>
+      </c>
+      <c r="H751" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000079037.jpg</t>
+        </is>
+      </c>
+      <c r="I751" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>Afsel repatriasi lebih dari 77 ribu WNA tak berdokumen</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:28:10 +0700</t>
+        </is>
+      </c>
+      <c r="D752" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E752" t="inlineStr">
+        <is>
+          <t>Pemerintah Afrika Selatan merepatriasi sedikitnya 77.184 warga negara asing (WNA) tanpa dokumen hingga 3 Agustus 2026, ...</t>
+        </is>
+      </c>
+      <c r="F752" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G752" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685779/afsel-repatriasi-lebih-dari-77-ribu-wna-tak-berdokumen</t>
+        </is>
+      </c>
+      <c r="H752" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/CjkinzN000014_20260808_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I752" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>Empat produsen mobil tarik 512.000 lebih kendaraan di Korea Selatan</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:23:51 +0700</t>
+        </is>
+      </c>
+      <c r="D753" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/antaranewsdotcom</t>
+        </is>
+      </c>
+      <c r="E753" t="inlineStr">
+        <is>
+          <t>Produsen mobil Hyundai Motor Co., Kia Corp., Stellantis, dan Honda akan secara sukarela menarik kembali lebih dari ...</t>
+        </is>
+      </c>
+      <c r="F753" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G753" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/berita/5685776/empat-produsen-mobil-tarik-512000-lebih-kendaraan-di-korea-selatan</t>
+        </is>
+      </c>
+      <c r="H753" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/05/02/IMG_0041.jpeg</t>
+        </is>
+      </c>
+      <c r="I753" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>Gubernur siapkan Rp2 miliar bangun rumah produksi kelapa di Nias Utara</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:23:09 +0700</t>
+        </is>
+      </c>
+      <c r="D754" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E754" t="inlineStr">
+        <is>
+          <t>Gubernur Sumatera Utara (Sumut) Bobby Nasution menyiapkan anggaran sebesar Rp2 miliar guna membangun rumah produksi ...</t>
+        </is>
+      </c>
+      <c r="F754" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G754" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685772/gubernur-siapkan-rp2-miliar-bangun-rumah-produksi-kelapa-di-nias-utara</t>
+        </is>
+      </c>
+      <c r="H754" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001036490.jpg</t>
+        </is>
+      </c>
+      <c r="I754" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>Peretas Rusia klaim punya bukti NATO terlibat serangan di area Rusia</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:19:07 +0700</t>
+        </is>
+      </c>
+      <c r="D755" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E755" t="inlineStr">
+        <is>
+          <t>Seorang peretas anonim Rusia mengeklaim telah memperoleh bukti tertulis keterlibatan langsung Pakta Pertahanan Atlantik ...</t>
+        </is>
+      </c>
+      <c r="F755" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G755" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685769/peretas-rusia-klaim-punya-bukti-nato-terlibat-serangan-di-area-rusia</t>
+        </is>
+      </c>
+      <c r="H755" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/CjkinzN000015_20260808_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I755" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>Viral Jukir Liar Paksa Pemotor Bayar Parkir di Tambora, Pelaku Ditangkap</t>
+        </is>
+      </c>
+      <c r="C756" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:17:06 +0700</t>
+        </is>
+      </c>
+      <c r="D756" t="inlineStr">
+        <is>
+          <t>Mulia Budi</t>
+        </is>
+      </c>
+      <c r="E756" t="inlineStr">
+        <is>
+          <t>Pria tersebut diduga meminta biaya parkir ke seorang pengendara motor. Namun, ketika pengendara itu meminta karcis parkir justru bang jago tersebut marah.</t>
+        </is>
+      </c>
+      <c r="F756" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G756" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610135/viral-jukir-liar-paksa-pemotor-bayar-parkir-di-tambora-pelaku-ditangkap</t>
+        </is>
+      </c>
+      <c r="H756" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2024/01/10/ilustrasi-media-sosial_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I756" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B757" t="inlineStr">
+        <is>
+          <t>Tim Gabungan Sergap Kapal Bawa 1,3 Ton Ketamin di Perairan Bintan</t>
+        </is>
+      </c>
+      <c r="C757" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:04:21 +0700</t>
+        </is>
+      </c>
+      <c r="D757" t="inlineStr">
+        <is>
+          <t>Wildan Noviansah</t>
+        </is>
+      </c>
+      <c r="E757" t="inlineStr">
+        <is>
+          <t>Tim gabungan Polri, Bea Cukai, BNN, dan TNI AL menggagalkan penyelundupan 1,3 ton ketamin di Bintan. Delapan ABK ditangkap, barang bukti diamankan.</t>
+        </is>
+      </c>
+      <c r="F757" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G757" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610123/tim-gabungan-sergap-kapal-bawa-1-3-ton-ketamin-di-perairan-bintan</t>
+        </is>
+      </c>
+      <c r="H757" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2018/03/06/55f711eb-7f02-4aac-b315-25a07bb80f3b_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I757" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B758" t="inlineStr">
+        <is>
+          <t>Warga Dengar 2 Kali Ledakan Saat Gedung Bapenda DKI Terbakar</t>
+        </is>
+      </c>
+      <c r="C758" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:43:35 +0700</t>
+        </is>
+      </c>
+      <c r="D758" t="inlineStr">
+        <is>
+          <t>Brigitta Belia Permata Sari</t>
+        </is>
+      </c>
+      <c r="E758" t="inlineStr">
+        <is>
+          <t>Kebakaran melanda Gedung Bapenda DKI Jakarta. Warga sempat mendengar ledakan.</t>
+        </is>
+      </c>
+      <c r="F758" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G758" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610114/warga-dengar-2-kali-ledakan-saat-gedung-bapenda-dki-terbakar</t>
+        </is>
+      </c>
+      <c r="H758" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/potret-kobaran-api-mengamuk-di-gedung-bapenda-dki-1786160999187_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I758" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B759" t="inlineStr">
+        <is>
+          <t>Saepul Incar Korban Mutilasi saat Tahu Foto dengan Motor PCX</t>
+        </is>
+      </c>
+      <c r="C759" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:25:38 +0700</t>
+        </is>
+      </c>
+      <c r="D759" t="inlineStr">
+        <is>
+          <t>Mei Amelia Rachmat</t>
+        </is>
+      </c>
+      <c r="E759" t="inlineStr">
+        <is>
+          <t>Polisi ungkap kasus mutilasi di Depok oleh Saepul, yang tergiur motor korban. Pelaku merencanakan kejahatan setelah melihat foto korban di media sosial.</t>
+        </is>
+      </c>
+      <c r="F759" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G759" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610092/saepul-incar-korban-mutilasi-saat-tahu-foto-dengan-motor-pcx</t>
+        </is>
+      </c>
+      <c r="H759" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/potret-saepul-pelaku-mutilasi-pria-inisial-k-51-di-cipayung-kota-depok-1786188316179_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I759" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B760" t="inlineStr">
+        <is>
+          <t>Jelang Musim Tanam, Satgas PRR Kebut Pemulihan Lahan Sawah di Aceh</t>
+        </is>
+      </c>
+      <c r="C760" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:18:22 +0700</t>
+        </is>
+      </c>
+      <c r="D760" t="inlineStr">
+        <is>
+          <t>Dea Duta Aulia</t>
+        </is>
+      </c>
+      <c r="E760" t="inlineStr">
+        <is>
+          <t>Satgas PRR mempercepat pemulihan 57 ribu hektare sawah di Aceh pascabencana. Fokus pada rehabilitasi lahan rusak dan solusi permanen berbasis ilmiah.</t>
+        </is>
+      </c>
+      <c r="F760" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G760" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610084/jelang-musim-tanam-satgas-prr-kebut-pemulihan-lahan-sawah-di-aceh</t>
+        </is>
+      </c>
+      <c r="H760" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/jelang-musim-tanam-satgas-prr-kebut-pemulihan-lahan-sawah-di-aceh-1786187852959_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I760" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B761" t="inlineStr">
+        <is>
+          <t>Kepala Bapanas &amp;amp; Dirut BULOG Turun Langsung Serahkan Bantuan Pangan di Alor</t>
+        </is>
+      </c>
+      <c r="C761" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:13:39 +0700</t>
+        </is>
+      </c>
+      <c r="D761" t="inlineStr">
+        <is>
+          <t>Dea Duta Aulia</t>
+        </is>
+      </c>
+      <c r="E761" t="inlineStr">
+        <is>
+          <t>Pemerintah salurkan bantuan pangan di Kabupaten Alor, NTT, untuk 37.338 penerima. Komitmen memastikan akses pangan merata hingga wilayah kepulauan.</t>
+        </is>
+      </c>
+      <c r="F761" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G761" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610077/kepala-bapanas-dirut-bulog-turun-langsung-serahkan-bantuan-pangan-di-alor</t>
+        </is>
+      </c>
+      <c r="H761" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/kepala-bapanas-dirut-bulog-serahkan-bantuan-pangan-di-alor-1786187534939_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I761" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B762" t="inlineStr">
+        <is>
+          <t>Rumah di Kebon Pala Jaktim Terbakar, 13 Unit Damkar Dikerahkan</t>
+        </is>
+      </c>
+      <c r="C762" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:13:23 +0700</t>
+        </is>
+      </c>
+      <c r="D762" t="inlineStr">
+        <is>
+          <t>Zunita Putri</t>
+        </is>
+      </c>
+      <c r="E762" t="inlineStr">
+        <is>
+          <t>Kebakaran melanda rumah warga di Kebon Pala, Jakarta Timur. 13 unit pemadam kebakaran dikerahkan. Proses pemadaman masih berlangsung, belum ada info korban.</t>
+        </is>
+      </c>
+      <c r="F762" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G762" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610076/rumah-di-kebon-pala-jaktim-terbakar-13-unit-damkar-dikerahkan</t>
+        </is>
+      </c>
+      <c r="H762" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2024/11/13/ilustrasi-api_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I762" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B763" t="inlineStr">
+        <is>
+          <t>Harga Set Panci dan Wajan Cuma Rp 70.000-an Cuma di Transmart Full Day Sale</t>
+        </is>
+      </c>
+      <c r="C763" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:00:18 +0700</t>
+        </is>
+      </c>
+      <c r="D763" t="inlineStr">
+        <is>
+          <t>Aulia Damayanti</t>
+        </is>
+      </c>
+      <c r="E763" t="inlineStr">
+        <is>
+          <t>Transmart Full Day Sale hadir 9 Agustus 2026 dengan diskon hingga 50%+20% untuk alat masak, elektronik, dan perabotan. Hemat jutaan rupiah!</t>
+        </is>
+      </c>
+      <c r="F763" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G763" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8609715/harga-set-panci-dan-wajan-cuma-rp-70-000-an-cuma-di-transmart-full-day-sale</t>
+        </is>
+      </c>
+      <c r="H763" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/transmart-1786167856018.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I763" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B764" t="inlineStr">
+        <is>
+          <t>AS Kucurkan Rp 53,6 T buat Genjot Produksi Baterai dan Mineral Kritis</t>
+        </is>
+      </c>
+      <c r="C764" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:30:55 +0700</t>
+        </is>
+      </c>
+      <c r="D764" t="inlineStr">
+        <is>
+          <t>Ignacio Geordi Oswaldo</t>
+        </is>
+      </c>
+      <c r="E764" t="inlineStr">
+        <is>
+          <t>Amerika Serikat (AS) berencana menginvestasikan US$ 3 miliar atau Rp 53,6 triliun (kurs Rp 17.897) dalam pengembangan mineral penting dan proyek baterai.</t>
+        </is>
+      </c>
+      <c r="F764" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G764" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/industri/d-8609658/as-kucurkan-rp-53-6-t-buat-genjot-produksi-baterai-dan-mineral-kritis</t>
+        </is>
+      </c>
+      <c r="H764" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/17/trump-saat-berpidato-di-gedung-putih-pada-kamis-167-malam-1784277022942_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I764" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B765" t="inlineStr">
+        <is>
+          <t>Masyarakat Alor Jadi Penerima Pertama Bantuan Beras 30 Kg</t>
+        </is>
+      </c>
+      <c r="C765" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:16:09 +0700</t>
+        </is>
+      </c>
+      <c r="D765" t="inlineStr">
+        <is>
+          <t>Heri Purnomo</t>
+        </is>
+      </c>
+      <c r="E765" t="inlineStr">
+        <is>
+          <t>Kabupaten Alor menjadi daerah pertama yang mendapatkan bantuan pangan ini.</t>
+        </is>
+      </c>
+      <c r="F765" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G765" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8610016/masyarakat-alor-jadi-penerima-pertama-bantuan-beras-30-kg</t>
+        </is>
+      </c>
+      <c r="H765" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/menteri-pertanian-mentan-andi-amran-sulaiman-1786178494016_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I765" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B766" t="inlineStr">
+        <is>
+          <t>Pendakian Gede-Pangrango Ditutup Imbas Kebakaran, Tiket Bisa Refund</t>
+        </is>
+      </c>
+      <c r="C766" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:30:46 +0700</t>
+        </is>
+      </c>
+      <c r="D766" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E766" t="inlineStr">
+        <is>
+          <t>Pendakian Gunung Gede-Pangrango ditutup sementara akibat kebakaran lahan. Penutupan berlaku 7-11 Agustus 2026 untuk keselamatan pendaki dan pemulihan kawasan.</t>
+        </is>
+      </c>
+      <c r="F766" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G766" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808131225-20-1390085/pendakian-gede-pangrango-ditutup-imbas-kebakaran-tiket-bisa-refund</t>
+        </is>
+      </c>
+      <c r="H766" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/07/bb-tnggp-tutup-jalur-pendakian-karena-kebakaran-alun-alun-suryakancana-1786099073263_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I766" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B767" t="inlineStr">
+        <is>
+          <t>Anak di Mamuju Sulbar Diperkosa 15 Orang Termasuk 2 Paman Korban</t>
+        </is>
+      </c>
+      <c r="C767" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:20:16 +0700</t>
+        </is>
+      </c>
+      <c r="D767" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E767" t="inlineStr">
+        <is>
+          <t>Polisi menangkap 15 terduga pelaku pemerkosaan anak di Mamuju, termasuk dua paman korban. Kasus ini terungkap setelah keluarga curiga terhadap kondisi korban.</t>
+        </is>
+      </c>
+      <c r="F767" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G767" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808154524-12-1390122/anak-di-mamuju-sulbar-diperkosa-15-orang-termasuk-2-paman-korban</t>
+        </is>
+      </c>
+      <c r="H767" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2018/12/03/55046dbb-b55c-46e0-b27b-7d77d95b5f2c_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I767" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B768" t="inlineStr">
+        <is>
+          <t>Mensos Targetkan 150 Ribu Anak Masuk Sekolah Rakyat pada 2027</t>
+        </is>
+      </c>
+      <c r="C768" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:40:17 +0700</t>
+        </is>
+      </c>
+      <c r="D768" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E768" t="inlineStr">
+        <is>
+          <t>Mensos Saifullah Yusuf menargetkan sedikitnya 150.000 anak mengikuti program Sekolah Rakyat pada 2027.</t>
+        </is>
+      </c>
+      <c r="F768" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G768" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808153540-20-1390120/mensos-targetkan-150-ribu-anak-masuk-sekolah-rakyat-pada-2027</t>
+        </is>
+      </c>
+      <c r="H768" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/saifullah-yusuf-1786177229499_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I768" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B769" t="inlineStr">
+        <is>
+          <t>Korban Pemukulan Direskrimum Kombes TF Melapor ke Polda Sumbar</t>
+        </is>
+      </c>
+      <c r="C769" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:25:10 +0700</t>
+        </is>
+      </c>
+      <c r="D769" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E769" t="inlineStr">
+        <is>
+          <t>Korban dugaan pemukulan oleh Kombes Teddy Fanani melapor ke Polda Sumbar. Keluarga menuntut keadilan, sementara Kapolda perintahkan penyelidikan.</t>
+        </is>
+      </c>
+      <c r="F769" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G769" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808165059-12-1390146/korban-pemukulan-direskrimum-kombes-tf-melapor-ke-polda-sumbar</t>
+        </is>
+      </c>
+      <c r="H769" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2018/08/31/1222ae3b-03ef-4fda-af13-ef2c6b652868_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I769" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B770" t="inlineStr">
+        <is>
+          <t>Savana Gunung Bromo Menghitam Akibat Kebakaran</t>
+        </is>
+      </c>
+      <c r="C770" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:20:32 +0700</t>
+        </is>
+      </c>
+      <c r="D770" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E770" t="inlineStr">
+        <is>
+          <t>Hamparan savana di kawasan wisata Gunung Bromo yang biasanya hijau kini berubah menghitam usai kebakaran hutan dan lahan yang terjadi sejak Senin (3/8) lalu.</t>
+        </is>
+      </c>
+      <c r="F770" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G770" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808112706-20-1390060/savana-gunung-bromo-menghitam-akibat-kebakaran</t>
+        </is>
+      </c>
+      <c r="H770" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/savana-gunung-bromo-menghitam-akibat-diterjang-kebakaran-1786163325629_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I770" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B771" t="inlineStr">
+        <is>
+          <t>Pramono Pastikan Data Pajak Aman Usai Kebakaran Gedung Bapenda</t>
+        </is>
+      </c>
+      <c r="C771" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:50:06 +0700</t>
+        </is>
+      </c>
+      <c r="D771" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E771" t="inlineStr">
+        <is>
+          <t>Gubernur DKI Jakarta Pramono Anung memastikan kebakaran Gedung Bapenda tidak ganggu data perpajakan. Pelayanan publik tetap berjalan meski ada dampak.</t>
+        </is>
+      </c>
+      <c r="F771" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G771" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808145340-20-1390104/pramono-pastikan-data-pajak-aman-usai-kebakaran-gedung-bapenda</t>
+        </is>
+      </c>
+      <c r="H771" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/gedung-bapenda-dki-jakarta-kebakaran-1786149523867_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I771" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B772" t="inlineStr">
+        <is>
+          <t>Penipuan CPNS Mencuat di Jatim, Rugi Ditaksir Tembus Rp20 M</t>
+        </is>
+      </c>
+      <c r="C772" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:24:39 +0700</t>
+        </is>
+      </c>
+      <c r="D772" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E772" t="inlineStr">
+        <is>
+          <t>Kasus penipuan modus penerimaan CPNS yang diduga melibatkan oknum militer aktif mencuat di Jawa Timur. Kerugian ditaksir tembus Rp20 miliar.</t>
+        </is>
+      </c>
+      <c r="F772" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G772" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808161424-12-1390126/penipuan-cpns-mencuat-di-jatim-rugi-ditaksir-tembus-rp20-m</t>
+        </is>
+      </c>
+      <c r="H772" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/penipuan-cpns-libatkan-oknum-militer-mencuat-di-jatim-1786179572617_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I772" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B773" t="inlineStr">
+        <is>
+          <t>1.000 ASN Berkantor di Bapenda Akan Diatur WFH Bergilir Usai Kebakaran</t>
+        </is>
+      </c>
+      <c r="C773" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:40:31 +0700</t>
+        </is>
+      </c>
+      <c r="D773" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E773" t="inlineStr">
+        <is>
+          <t>Pemprov DKI Jakarta siapkan skema WFH untuk 1.000 ASN pascakebakaran di Gedung Bapenda. Layanan publik tetap berjalan dan data perpajakan aman.</t>
+        </is>
+      </c>
+      <c r="F773" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G773" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808142937-20-1390095/1000-asn-berkantor-di-bapenda-akan-diatur-wfh-bergilir-usai-kebakaran</t>
+        </is>
+      </c>
+      <c r="H773" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/gedung-bapenda-dki-jakarta-kebakaran-1786149523991_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I773" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B774" t="inlineStr">
+        <is>
+          <t>Ketua Komite III DPD RI Minta Daerah Termiskin Jadi Prioritas Pendidikan Nasional</t>
+        </is>
+      </c>
+      <c r="C774" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:09:54 +0700</t>
+        </is>
+      </c>
+      <c r="D774" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E774" t="inlineStr">
+        <is>
+          <t>Lima provinsi termiskin yang disebut berada di Papua. DPD meminta kondisi itu menjadi dasar prioritas kebijakan pendidikan nasional.</t>
+        </is>
+      </c>
+      <c r="F774" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G774" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865807/ketua-komite-iii-dpd-ri-minta-daerah-termiskin-jadi-prioritas-pendidikan-nasional</t>
+        </is>
+      </c>
+      <c r="H774" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/EMCLa-6CnWMcSSxKx0BqUCVE21M=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/KASUS-IBU-HAMIL-Ketua-Komite-III-DPD-RI-Filep-Wamafma.jpg</t>
+        </is>
+      </c>
+      <c r="I774" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B775" t="inlineStr">
+        <is>
+          <t>Hasil Kualifikasi MotoGP Inggris 2026: Jorge Martin Pole dan Ukir Rekor, Marc Marquez Start P6</t>
+        </is>
+      </c>
+      <c r="C775" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:55:01 +0700</t>
+        </is>
+      </c>
+      <c r="D775" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E775" t="inlineStr">
+        <is>
+          <t>Jorge Martin pole position MotoGP Inggris 2026 di Sirkuit Silverstone yang diwarnai rekor setelah berhasil jadi yang tercepat pada sesi Kualifikasi.</t>
+        </is>
+      </c>
+      <c r="F775" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G775" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7865806/hasil-kualifikasi-motogp-inggris-2026-jorge-martin-pole-dan-ukir-rekor-marc-marquez-start-p6</t>
+        </is>
+      </c>
+      <c r="H775" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Gp0vMFil6jxZlxLSjbYxP5Smfjk=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Jorge-Martin-di-MotoGP-Ceko-2025.jpg</t>
+        </is>
+      </c>
+      <c r="I775" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B776" t="inlineStr">
+        <is>
+          <t>Marbot Masjid Diserang hingga Tewas saat akan Azan, Pelaku Diduga Gangguan Jiwa, Polisi Lakukan Tes</t>
+        </is>
+      </c>
+      <c r="C776" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:48:17 +0700</t>
+        </is>
+      </c>
+      <c r="D776" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E776" t="inlineStr">
+        <is>
+          <t>Marbot masjid di Purwakarta tewas dibacok saat hendak azan. Polisi berhasil menangkap pelaku yang diduga sakit hati karena disinggung soal ekonomi.</t>
+        </is>
+      </c>
+      <c r="F776" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G776" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865805/marbot-masjid-diserang-hingga-tewas-saat-akan-azan-pelaku-diduga-gangguan-jiwa-polisi-lakukan-tes</t>
+        </is>
+      </c>
+      <c r="H776" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/iVQoFd00f4I54X3zKDiHAJJIyGM=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Marbot-Masjid-Tewas.jpg</t>
+        </is>
+      </c>
+      <c r="I776" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B777" t="inlineStr">
+        <is>
+          <t>Dituding Pengecut, Dokter Tifa: Beli dan Borong Buku Saya, Jangan Cuma Jadi Komentator</t>
+        </is>
+      </c>
+      <c r="C777" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:39:36 +0700</t>
+        </is>
+      </c>
+      <c r="D777" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E777" t="inlineStr">
+        <is>
+          <t>Tifauzia Tyassuma alias Dokter Tifa tak terima disebut pengecut karena memutuskan untuk hijrah dari polemik kasus ijazah palsu Jokowi.</t>
+        </is>
+      </c>
+      <c r="F777" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G777" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865804/dituding-pengecut-dokter-tifa-beli-dan-borong-buku-saya-jangan-cuma-jadi-komentator</t>
+        </is>
+      </c>
+      <c r="H777" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/YZ9m0bUNzYesnOVzFIotI90PixM=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/dokter-tifa-ahli-cls-di-solo-ijazah-jokowi.jpg</t>
+        </is>
+      </c>
+      <c r="I777" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B778" t="inlineStr">
+        <is>
+          <t>16 Atlet Raih Super Tiket Audisi PB Djarum 2026 Makassar: Abidzar Akhirnya Lolos ke Karantina</t>
+        </is>
+      </c>
+      <c r="C778" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:25:24 +0700</t>
+        </is>
+      </c>
+      <c r="D778" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E778" t="inlineStr">
+        <is>
+          <t>Mereka terdiri dari enam atlet yang lolos melalui jalur turnamen dan 10 atlet pilihan tim pencari bakat.</t>
+        </is>
+      </c>
+      <c r="F778" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G778" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7865803/16-atlet-raih-super-tiket-audisi-pb-djarum-2026-makassar-abidzar-akhirnya-lolos-ke-karantina</t>
+        </is>
+      </c>
+      <c r="H778" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/1bNYbOTEuYBxdIdyTVLWaENf7Zs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Super-Tiket-Audisi-umum-Bulutangkis-PB-Djarum-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I778" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B779" t="inlineStr">
+        <is>
+          <t>Gagal di AFF 2026, Herdman Kini Bidik Trofi Pertama di FIFA ASEAN</t>
+        </is>
+      </c>
+      <c r="C779" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:19:29 +0700</t>
+        </is>
+      </c>
+      <c r="D779" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E779" t="inlineStr">
+        <is>
+          <t>Indonesia tersingkir dari AFF 2026, tetapi Herdman langsung membidik FIFA ASEAN sebagai kesempatan mengejar trofi pertama bersama Garuda.</t>
+        </is>
+      </c>
+      <c r="F779" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G779" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865802/gagal-di-aff-2026-herdman-kini-bidik-trofi-pertama-di-fifa-asean</t>
+        </is>
+      </c>
+      <c r="H779" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/LcMPYEsIRuAOvD94-g4gzmdgsBw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Pelatih-Timnas-Indonesia-John-Herdman-bersama-sang-kapten-Rizky-Ridho-3.jpg</t>
+        </is>
+      </c>
+      <c r="I779" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B780" t="inlineStr">
+        <is>
+          <t>Tanda Whatsapp Disadap dari Jauh dan Cara Hentikan</t>
+        </is>
+      </c>
+      <c r="C780" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:00:42 +0700</t>
+        </is>
+      </c>
+      <c r="D780" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E780" t="inlineStr">
+        <is>
+          <t>Penyadapan WhatsApp semakin marak. Kenali tanda-tandanya dan cara melindungi akun Anda, termasuk verifikasi dua langkah dan laporan ke WhatsApp.</t>
+        </is>
+      </c>
+      <c r="F780" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G780" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260808144542-37-757624/tanda-whatsapp-disadap-dari-jauh-dan-cara-hentikan</t>
+        </is>
+      </c>
+      <c r="H780" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2021/03/08/infografis-kasus-phising-email-yang-serang-indonesia-makin-merajalela-2_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I780" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B781" t="inlineStr">
+        <is>
+          <t>Bos Koperasi Dalangi Penyekapan Karyawan di Tangerang</t>
+        </is>
+      </c>
+      <c r="C781" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:23:10 +0700</t>
+        </is>
+      </c>
+      <c r="D781" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E781" t="inlineStr">
+        <is>
+          <t>Polda Banten menangkap 5 pelaku, kasus penyekapan karyawan koperasi diduga didalangi bos.</t>
+        </is>
+      </c>
+      <c r="F781" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G781" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265227/bos-koperasi-dalangi-penyekapan-karyawan-di-tangerang</t>
+        </is>
+      </c>
+      <c r="H781" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/GVPAADbx9t42VHgDnHBhKMRq_aQ=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9314668/original/011114800_1785758460-WhatsApp_Image_2026-08-03_at_18.52.07.jpeg</t>
+        </is>
+      </c>
+      <c r="I781" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" t="inlineStr">
+        <is>
+          <t>Otomotif</t>
+        </is>
+      </c>
+      <c r="B782" t="inlineStr">
+        <is>
+          <t>Hasil Kualifikasi MotoGP Inggris 2026: Martin Pole Position</t>
+        </is>
+      </c>
+      <c r="C782" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:29:39 +0700</t>
+        </is>
+      </c>
+      <c r="D782" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E782" t="inlineStr">
+        <is>
+          <t>Jorge Martin mengamankan pole position pada sesi kualifikasi MotoGP Inggris 2026 yang digelar di Sirkuit Silverstone.</t>
+        </is>
+      </c>
+      <c r="F782" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G782" t="inlineStr">
+        <is>
+          <t>https://otomotif.kompas.com/read/2026/08/08/192511315/hasil-kualifikasi-motogp-inggris-2026-martin-pole-position</t>
+        </is>
+      </c>
+      <c r="H782" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/uj_xl1QLY4XgX1ACRq8qbQnjM78=/0x0:1200x800/1200x675/filters:watermark(data/photo/2026/01/30/697c81750a668.png,0,-0,1)/data/photo/2026/05/10/6a00811ca2c05.jpg</t>
+        </is>
+      </c>
+      <c r="I782" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" t="inlineStr">
+        <is>
+          <t>Edukasi</t>
+        </is>
+      </c>
+      <c r="B783" t="inlineStr">
+        <is>
+          <t>Abdel Achrian Bangga Anaknya Masuk ITB, Cek Jurusan dan Lulusan SMA Mana?</t>
+        </is>
+      </c>
+      <c r="C783" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:29:39 +0700</t>
+        </is>
+      </c>
+      <c r="D783" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E783" t="inlineStr">
+        <is>
+          <t>Anak kedua komedian Abdel Achrian, Latisha Amira berhasil diterima di IUP Manajemen ITB, mulai kuliah pada 2026.</t>
+        </is>
+      </c>
+      <c r="F783" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G783" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/edu/read/2026/08/08/184500071/abdel-achrian-bangga-anaknya-masuk-itb-cek-jurusan-dan-lulusan-sma-mana-</t>
+        </is>
+      </c>
+      <c r="H783" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/ZzgQO-Yvo1vJuut6QvmBgVrMKhs=/0x0:3072x2048/1200x675/filters:watermark(data/photo/2026/01/30/697c819b2dbec.png,0,-0,1)/data/photo/2026/08/08/6a76e4c33d35f.jpg</t>
+        </is>
+      </c>
+      <c r="I783" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" t="inlineStr">
+        <is>
+          <t>Tren</t>
+        </is>
+      </c>
+      <c r="B784" t="inlineStr">
+        <is>
+          <t>Mau Ikut Lelang Mobil Bekas? Simak 4 Hal yang Perlu Disiapkan</t>
+        </is>
+      </c>
+      <c r="C784" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:29:39 +0700</t>
+        </is>
+      </c>
+      <c r="D784" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E784" t="inlineStr">
+        <is>
+          <t>Berikut ini beberapa persiapan ikut lelang mobil bekas agar mendapatkan kendaraan sesuai kebutuhan dan anggaran.</t>
+        </is>
+      </c>
+      <c r="F784" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G784" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/tren/read/2026/08/08/180000165/mau-ikut-lelang-mobil-bekas-simak-4-hal-yang-perlu-disiapkan</t>
+        </is>
+      </c>
+      <c r="H784" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/bpUGLfBlZc-rW9ilHpt0dbndpAU=/0x0:4624x3083/1200x675/filters:watermark(data/photo/2026/01/30/697c818d0ca91.png,0,-0,1)/data/photo/2024/03/19/65f95ee34cb75.jpg</t>
+        </is>
+      </c>
+      <c r="I784" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I716"/>
+  <autoFilter ref="A1:I784"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-08 13:41 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-08.xlsx
+++ b/data/berita_2026-08-08.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$784</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$837</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I784"/>
+  <dimension ref="A1:I837"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -37284,8 +37284,2500 @@
         </is>
       </c>
     </row>
+    <row r="785">
+      <c r="A785" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B785" t="inlineStr">
+        <is>
+          <t>Rektor Unej ajak mahasiswa baru tidak serahkan proses berpikir ke AI</t>
+        </is>
+      </c>
+      <c r="C785" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:32:45 +0700</t>
+        </is>
+      </c>
+      <c r="D785" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E785" t="inlineStr">
+        <is>
+          <t>Rektor Universitas Jember (Unej) Iwan Taruna mengajak mahasiswa baru tidak menyerahkan proses berpikir ke kecerdasan ...</t>
+        </is>
+      </c>
+      <c r="F785" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G785" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685921/rektor-unej-ajak-mahasiswa-baru-tidak-serahkan-proses-berpikir-ke-ai</t>
+        </is>
+      </c>
+      <c r="H785" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/WhatsApp-Image-2026-08-08-at-10.47.49.jpeg</t>
+        </is>
+      </c>
+      <c r="I785" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B786" t="inlineStr">
+        <is>
+          <t>CdM telah identifikasi kebutuhan 18 cabang ke Asian Games 2026</t>
+        </is>
+      </c>
+      <c r="C786" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:28:12 +0700</t>
+        </is>
+      </c>
+      <c r="D786" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E786" t="inlineStr">
+        <is>
+          <t>Chef de Mission (CdM) Tim Indonesia untuk Asian Games Aichi-Nagoya 2026 Todotua Pasaribu telah mengunjungi dan ...</t>
+        </is>
+      </c>
+      <c r="F786" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G786" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685917/cdm-telah-identifikasi-kebutuhan-18-cabang-ke-asian-games-2026</t>
+        </is>
+      </c>
+      <c r="H786" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/1000463087.jpg</t>
+        </is>
+      </c>
+      <c r="I786" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B787" t="inlineStr">
+        <is>
+          <t>Danrem 172: TNI-Polri selidiki KKB pelaku penembakan di Wamena</t>
+        </is>
+      </c>
+      <c r="C787" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:23:11 +0700</t>
+        </is>
+      </c>
+      <c r="D787" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E787" t="inlineStr">
+        <is>
+          <t>Komandan Korem 172/PWY Brigjen TNI Robbi Suryadi mengatakan, TNI-Polri melakukan penyelidikan untuk mengetahui Kelompok ...</t>
+        </is>
+      </c>
+      <c r="F787" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G787" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685916/danrem-172-tni-polri-selidiki-kkb-pelaku-penembakan-di-wamena</t>
+        </is>
+      </c>
+      <c r="H787" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1002606820.jpg</t>
+        </is>
+      </c>
+      <c r="I787" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B788" t="inlineStr">
+        <is>
+          <t>Kemenekraf libatkan pemerintah daerah dalam pengembangan ekosistem gim</t>
+        </is>
+      </c>
+      <c r="C788" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:22:04 +0700</t>
+        </is>
+      </c>
+      <c r="D788" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E788" t="inlineStr">
+        <is>
+          <t>Kementerian Ekonomi Kreatif (Kemenekraf) melibatkan pemerintah daerah dalam upaya untuk menumbuhkan dan mengembangkan ...</t>
+        </is>
+      </c>
+      <c r="F788" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G788" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685915/kemenekraf-libatkan-pemerintah-daerah-dalam-pengembangan-ekosistem-gim</t>
+        </is>
+      </c>
+      <c r="H788" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/20260808_152157.jpg</t>
+        </is>
+      </c>
+      <c r="I788" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>Fhirdan optimistis rebut satu tempat di timnas bola basket</t>
+        </is>
+      </c>
+      <c r="C789" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:19:32 +0700</t>
+        </is>
+      </c>
+      <c r="D789" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E789" t="inlineStr">
+        <is>
+          <t>Pebasket Bogor Hornbills Fhirdan Guntara optimistis untuk memanfaatkan kesempatan seleksi tim nasional (timnas) bola ...</t>
+        </is>
+      </c>
+      <c r="F789" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G789" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685913/fhirdan-optimistis-rebut-satu-tempat-di-timnas-bola-basket</t>
+        </is>
+      </c>
+      <c r="H789" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000476680.jpg</t>
+        </is>
+      </c>
+      <c r="I789" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B790" t="inlineStr">
+        <is>
+          <t>Menko PM: KSEKP pesantren dapat menjadi motor pengentasan kemiskinan</t>
+        </is>
+      </c>
+      <c r="C790" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:15:29 +0700</t>
+        </is>
+      </c>
+      <c r="D790" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E790" t="inlineStr">
+        <is>
+          <t>Menteri Koordinator Pemberdayaan Masyarakat Muhaimin Iskandar mengatakan Kawasan Sosial Ekonomi Khusus Pesantren ...</t>
+        </is>
+      </c>
+      <c r="F790" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G790" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685912/menko-pm-ksekp-pesantren-dapat-menjadi-motor-pengentasan-kemiskinan</t>
+        </is>
+      </c>
+      <c r="H790" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/WhatsApp-Image-2026-08-08-at-20.10.49.jpeg</t>
+        </is>
+      </c>
+      <c r="I790" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B791" t="inlineStr">
+        <is>
+          <t>Pemprov Maluku imbau warga waspadai hoaks lowongan kerja Blok Masela</t>
+        </is>
+      </c>
+      <c r="C791" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:11:34 +0700</t>
+        </is>
+      </c>
+      <c r="D791" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E791" t="inlineStr">
+        <is>
+          <t>Dinas Ketenagakerjaan dan Transmigrasi (Disnakertrans) Provinsi Maluku mengimbau masyarakat, khususnya calon pencari ...</t>
+        </is>
+      </c>
+      <c r="F791" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G791" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685908/pemprov-maluku-imbau-warga-waspadai-hoaks-lowongan-kerja-blok-masela</t>
+        </is>
+      </c>
+      <c r="H791" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/WhatsApp-Image-2026-08-08-at-21.43.58.jpeg</t>
+        </is>
+      </c>
+      <c r="I791" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>Sektor robotika pintar di Tianjin, catat pertumbuhan kuat pada H1 2026</t>
+        </is>
+      </c>
+      <c r="C792" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:10:13 +0700</t>
+        </is>
+      </c>
+      <c r="D792" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E792" t="inlineStr">
+        <is>
+          <t>Kota Tianjin di China utara berhasil menarik sejumlah besar proyek penting di bidang robotika pintar dan kini menjadi ...</t>
+        </is>
+      </c>
+      <c r="F792" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G792" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685904/sektor-robotika-pintar-di-tianjin-catat-pertumbuhan-kuat-pada-h1-2026</t>
+        </is>
+      </c>
+      <c r="H792" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/CjkinzN000010_20260808_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I792" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B793" t="inlineStr">
+        <is>
+          <t>Jorge Martin rebut pole position MotoGP Inggris 2026</t>
+        </is>
+      </c>
+      <c r="C793" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:08:18 +0700</t>
+        </is>
+      </c>
+      <c r="D793" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E793" t="inlineStr">
+        <is>
+          <t>Pembalap Aprilia Racing Jorge Martin merebut pole position MotoGP Inggris 2026 dan menjadi yang tercepat dalam sesi ...</t>
+        </is>
+      </c>
+      <c r="F793" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G793" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685901/jorge-martin-rebut-pole-position-motogp-inggris-2026</t>
+        </is>
+      </c>
+      <c r="H793" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/12/Report-MGP-GP-FR.jpeg</t>
+        </is>
+      </c>
+      <c r="I793" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>BPJS Ketenagakerjaan perluas perlindungan penggerak ekonomi pesantren</t>
+        </is>
+      </c>
+      <c r="C794" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:08:10 +0700</t>
+        </is>
+      </c>
+      <c r="D794" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E794" t="inlineStr">
+        <is>
+          <t>Badan Penyelenggara Jaminan Sosial (BPJS) Ketenagakerjaan memperluas perlindungan jaminan sosial bagi penggerak ...</t>
+        </is>
+      </c>
+      <c r="F794" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G794" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685899/bpjs-ketenagakerjaan-perluas-perlindungan-penggerak-ekonomi-pesantren</t>
+        </is>
+      </c>
+      <c r="H794" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/WhatsApp-Image-2026-08-08-at-19.04.36.jpeg</t>
+        </is>
+      </c>
+      <c r="I794" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>Spanyol kerahkan 300 polisi dan 2.000 tentara cegah gelombang migran</t>
+        </is>
+      </c>
+      <c r="C795" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:06:42 +0700</t>
+        </is>
+      </c>
+      <c r="D795" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E795" t="inlineStr">
+        <is>
+          <t>Spanyol mengerahkan sekitar 300 personel polisi antihuru-hara dan 2.000 tentara di wilayah kantong (enklave) Ceuta ...</t>
+        </is>
+      </c>
+      <c r="F795" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G795" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685897/spanyol-kerahkan-300-polisi-dan-2000-tentara-cegah-gelombang-migran</t>
+        </is>
+      </c>
+      <c r="H795" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/thumbs_b_c_6b5fb18497011384717063ae9e35fd8b.jpg</t>
+        </is>
+      </c>
+      <c r="I795" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>Turkiye bantah perjanjian pertahanan trilateral bertentangan dengan NATO</t>
+        </is>
+      </c>
+      <c r="C796" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:59:23 +0700</t>
+        </is>
+      </c>
+      <c r="D796" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E796" t="inlineStr">
+        <is>
+          <t>Pemerintah Turki pada Jumat (7/8) menepis klaim yang beredar di media sosial bahwa perjanjian pertahanan trilateral ...</t>
+        </is>
+      </c>
+      <c r="F796" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G796" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685896/turkiye-bantah-perjanjian-pertahanan-trilateral-bertentangan-dengan-nato</t>
+        </is>
+      </c>
+      <c r="H796" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/09/NATOMarkasBrusselBelgiaXinhua.jpg</t>
+        </is>
+      </c>
+      <c r="I796" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>Indonesia kalah 0-3 dari Thailand pada Leg 2 SEA V Cup 2026</t>
+        </is>
+      </c>
+      <c r="C797" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:58:27 +0700</t>
+        </is>
+      </c>
+      <c r="D797" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E797" t="inlineStr">
+        <is>
+          <t>Timnas bola voli putri Indonesia kalah 0-3 (18-25, 17-25, 12-25) melawan Thailand dalam pertandingan kedua Leg 2 SEA V ...</t>
+        </is>
+      </c>
+      <c r="F797" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G797" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685895/indonesia-kalah-0-3-dari-thailand-pada-leg-2-sea-v-cup-2026</t>
+        </is>
+      </c>
+      <c r="H797" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/19/IMG-20260719-WA0011.jpg</t>
+        </is>
+      </c>
+      <c r="I797" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>Toyota ingin menambah pilihan kendaraan elektrifikasi</t>
+        </is>
+      </c>
+      <c r="C798" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:54:35 +0700</t>
+        </is>
+      </c>
+      <c r="D798" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/antaranewsdotcom</t>
+        </is>
+      </c>
+      <c r="E798" t="inlineStr">
+        <is>
+          <t>PT Toyota Astra Motor (TAM) ingin menambah pilihan kendaraan elektrifikasi yang sesuai dengan kebutuhan pelanggan dan ...</t>
+        </is>
+      </c>
+      <c r="F798" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G798" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/berita/5685892/toyota-ingin-menambah-pilihan-kendaraan-elektrifikasi</t>
+        </is>
+      </c>
+      <c r="H798" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/2acd857a-1f61-48b1-8428-0eca0082ed36.jpeg</t>
+        </is>
+      </c>
+      <c r="I798" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>Houthi intensifkan serangan rudal-drone terhadap pasukan Yaman</t>
+        </is>
+      </c>
+      <c r="C799" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:53:21 +0700</t>
+        </is>
+      </c>
+      <c r="D799" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E799" t="inlineStr">
+        <is>
+          <t>Kelompok Houthi Yaman pada Jumat menyatakan telah melancarkan serangan besar-besaran menggunakan rudal dan pesawat ...</t>
+        </is>
+      </c>
+      <c r="F799" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G799" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685891/houthi-intensifkan-serangan-rudal-drone-terhadap-pasukan-yaman</t>
+        </is>
+      </c>
+      <c r="H799" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/26/thumbs_b_c_63476bae594e4b11ee5476b7e8611c44.jpg</t>
+        </is>
+      </c>
+      <c r="I799" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B800" t="inlineStr">
+        <is>
+          <t>Seskab Teddy tinjau kesiapan operasional SR Rintisan di Curug</t>
+        </is>
+      </c>
+      <c r="C800" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:52:39 +0700</t>
+        </is>
+      </c>
+      <c r="D800" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E800" t="inlineStr">
+        <is>
+          <t>Sekretaris Kabinet Teddy Indra Wijaya meninjau Sekolah Rakyat (SR) Rintisan di Politeknik Penerbangan Indonesia Curug, ...</t>
+        </is>
+      </c>
+      <c r="F800" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G800" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685887/seskab-teddy-tinjau-kesiapan-operasional-sr-rintisan-di-curug</t>
+        </is>
+      </c>
+      <c r="H800" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG_0999.jpeg</t>
+        </is>
+      </c>
+      <c r="I800" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B801" t="inlineStr">
+        <is>
+          <t>Legislator minta kebijakan naturalisasi dievaluasi usai Piala AFF 2026</t>
+        </is>
+      </c>
+      <c r="C801" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:48:24 +0700</t>
+        </is>
+      </c>
+      <c r="D801" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E801" t="inlineStr">
+        <is>
+          <t>Anggota Komisi XIII DPR RI Franciscus Sibarani meminta kebijakan naturalisasi atlet dievaluasi menyusul kegagalan Tim ...</t>
+        </is>
+      </c>
+      <c r="F801" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G801" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685885/legislator-minta-kebijakan-naturalisasi-dievaluasi-usai-piala-aff-2026</t>
+        </is>
+      </c>
+      <c r="H801" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/HPILtZ8aEAI6W61.jpg</t>
+        </is>
+      </c>
+      <c r="I801" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B802" t="inlineStr">
+        <is>
+          <t>Ismi Ulfaida, siswi Sekolah Rakyat pertama di barisan Paskibraka</t>
+        </is>
+      </c>
+      <c r="C802" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:46:43 +0700</t>
+        </is>
+      </c>
+      <c r="D802" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E802" t="inlineStr">
+        <is>
+          <t>Derap langkah sepatu bersahutan di lapangan Pusat Pengembangan Sumber Daya Manusia Kementerian Pendidikan Dasar dan ...</t>
+        </is>
+      </c>
+      <c r="F802" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G802" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685883/ismi-ulfaida-siswi-sekolah-rakyat-pertama-di-barisan-paskibraka</t>
+        </is>
+      </c>
+      <c r="H802" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000035128.jpg</t>
+        </is>
+      </c>
+      <c r="I802" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B803" t="inlineStr">
+        <is>
+          <t>Kasus pembobolan properti di Prancis naik 5,8 Persen pada Juli 2026</t>
+        </is>
+      </c>
+      <c r="C803" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:45:42 +0700</t>
+        </is>
+      </c>
+      <c r="D803" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E803" t="inlineStr">
+        <is>
+          <t>Jumlah kasus perampokan, khususnya pembobolan properti di Prancis pada Juli 2026 meningkat sekitar 1.500 kasus ...</t>
+        </is>
+      </c>
+      <c r="F803" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G803" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685880/kasus-pembobolan-properti-di-prancis-naik-58-persen-pada-juli-2026</t>
+        </is>
+      </c>
+      <c r="H803" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/12/11/Ukraina.jpg</t>
+        </is>
+      </c>
+      <c r="I803" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>Kebakaran lahan mengancam permukiman padat di Palembang</t>
+        </is>
+      </c>
+      <c r="C804" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:44:59 +0700</t>
+        </is>
+      </c>
+      <c r="D804" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E804" t="inlineStr">
+        <is>
+          <t>Warga berlari menghindari asap saat kebakaran lahan di dekat permukiman padat penduduk di Kemas Rindo, Kertapati, ...</t>
+        </is>
+      </c>
+      <c r="F804" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G804" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5685877/kebakaran-lahan-mengancam-permukiman-padat-di-palembang</t>
+        </is>
+      </c>
+      <c r="H804" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/Kebakaran-lahan-di-Kertapati-Palembang-080826-Lmo-12A.jpg</t>
+        </is>
+      </c>
+      <c r="I804" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>LRT Sumsel layani 96 perjalanan dukung CFN selama Agustus 2026</t>
+        </is>
+      </c>
+      <c r="C805" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:43:22 +0700</t>
+        </is>
+      </c>
+      <c r="D805" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E805" t="inlineStr">
+        <is>
+          <t>PT Kereta Api Indonesia (Persero) Divisi Regional III Palembang bersama Balai Pengelola Kereta Api Ringan Sumatera ...</t>
+        </is>
+      </c>
+      <c r="F805" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G805" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685875/lrt-sumsel-layani-96-perjalanan-dukung-cfn-selama-agustus-2026</t>
+        </is>
+      </c>
+      <c r="H805" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/74915aa1-a76f-4382-9592-adfa09f680c5.jpeg</t>
+        </is>
+      </c>
+      <c r="I805" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>PMI Probolinggo bantu padamkan karhutla Gunung Bromo</t>
+        </is>
+      </c>
+      <c r="C806" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:43:00 +0700</t>
+        </is>
+      </c>
+      <c r="D806" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E806" t="inlineStr">
+        <is>
+          <t>Palang Merah Indonesia (PMI) Kabupaten Probolinggo ikut membantu memadamkan kebakaran hutan dan lahan (karhutla) yang ...</t>
+        </is>
+      </c>
+      <c r="F806" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G806" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685872/pmi-probolinggo-bantu-padamkan-karhutla-gunung-bromo</t>
+        </is>
+      </c>
+      <c r="H806" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/WhatsApp-Image-2026-08-07-at-21.20.38-1200x630.jpeg</t>
+        </is>
+      </c>
+      <c r="I806" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B807" t="inlineStr">
+        <is>
+          <t>Slovakia tetapkan status darurat akibat krisis air dan gelombang panas</t>
+        </is>
+      </c>
+      <c r="C807" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:39:18 +0700</t>
+        </is>
+      </c>
+      <c r="D807" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E807" t="inlineStr">
+        <is>
+          <t>Status darurat telah ditetapkan di dua permukiman di Slovakia timur akibat krisis air minum dan gelombang panas ekstrem ...</t>
+        </is>
+      </c>
+      <c r="F807" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G807" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685869/slovakia-tetapkan-status-darurat-akibat-krisis-air-dan-gelombang-panas</t>
+        </is>
+      </c>
+      <c r="H807" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/27/7325.jpg</t>
+        </is>
+      </c>
+      <c r="I807" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B808" t="inlineStr">
+        <is>
+          <t>Pekalongan pastikan penempatan ASN berdasar kompetensi pasca-OTT</t>
+        </is>
+      </c>
+      <c r="C808" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:36:47 +0700</t>
+        </is>
+      </c>
+      <c r="D808" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E808" t="inlineStr">
+        <is>
+          <t>Pemerintah Kabupaten Pekalongan, Jawa Tengah, memastikan penempatan aparatur sipil negara (ASN) mengacu pada kompetensi ...</t>
+        </is>
+      </c>
+      <c r="F808" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G808" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685865/pekalongan-pastikan-penempatan-asn-berdasar-kompetensi-pasca-ott</t>
+        </is>
+      </c>
+      <c r="H808" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/Plt-Bupati-Sukirman-pascaOTT-Bupati-Fadia.jpg</t>
+        </is>
+      </c>
+      <c r="I808" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B809" t="inlineStr">
+        <is>
+          <t>Banteng Jakarta FC siapkan 23 pemain dalam Soekarno Cup 2026</t>
+        </is>
+      </c>
+      <c r="C809" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:35:47 +0700</t>
+        </is>
+      </c>
+      <c r="D809" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E809" t="inlineStr">
+        <is>
+          <t>Tim sepak bola Banteng Jakarta FC menyiapkan 23 pemain mewakili DKI Jakarta dalam turnamen untuk usia ...</t>
+        </is>
+      </c>
+      <c r="F809" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G809" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685864/banteng-jakarta-fc-siapkan-23-pemain-dalam-soekarno-cup-2026</t>
+        </is>
+      </c>
+      <c r="H809" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/5858173f-4275-4814-b5c6-b9c6e6bcd82d.jpeg</t>
+        </is>
+      </c>
+      <c r="I809" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>Sophia KATSEYE untuk sementara akan absen dari aktivitas grup</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:32:49 +0700</t>
+        </is>
+      </c>
+      <c r="D810" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E810" t="inlineStr">
+        <is>
+          <t>Vokalis grup KATSEYE, Sophia, untuk sementara akan absen dari berbagai aktivitas grup karena alasan kesehatan.
+HYBE ...</t>
+        </is>
+      </c>
+      <c r="F810" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G810" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685860/sophia-katseye-untuk-sementara-akan-absen-dari-aktivitas-grup</t>
+        </is>
+      </c>
+      <c r="H810" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/07/09/IMG-20250709-WA0001.jpg</t>
+        </is>
+      </c>
+      <c r="I810" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B811" t="inlineStr">
+        <is>
+          <t>Anies Baswedan kenang sosok Habib Saggaf ulama perekat umat</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:23:36 +0700</t>
+        </is>
+      </c>
+      <c r="D811" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E811" t="inlineStr">
+        <is>
+          <t>Gubernur DKI Jakarta Periode 2017-2022 Anies Rasyid Baswedan mengenang sosok Habib Saggaf bin Muhammad Aljufri, sebagai ...</t>
+        </is>
+      </c>
+      <c r="F811" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G811" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685859/anies-baswedan-kenang-sosok-habib-saggaf-ulama-perekat-umat</t>
+        </is>
+      </c>
+      <c r="H811" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/ANIES-dan-HABIB-SAGGAF.jpg</t>
+        </is>
+      </c>
+      <c r="I811" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B812" t="inlineStr">
+        <is>
+          <t>Transmart Full Day Sale Balik Lagi, Beli TV 43 di Semurah Ini</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:30:28 +0700</t>
+        </is>
+      </c>
+      <c r="D812" t="inlineStr">
+        <is>
+          <t>Ignacio Geordi Oswaldo</t>
+        </is>
+      </c>
+      <c r="E812" t="inlineStr">
+        <is>
+          <t>Transmart Full Day Sale hadir dengan diskon hingga 50+20% untuk berbagai produk. Nikmati promo menarik mulai 9/8/2026, syarat dan ketentuan berlaku.</t>
+        </is>
+      </c>
+      <c r="F812" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G812" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8609722/transmart-full-day-sale-balik-lagi-beli-tv-43-di-semurah-ini</t>
+        </is>
+      </c>
+      <c r="H812" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/transmart-full-day-sale-balik-lagi-beli-tv-43-di-semurah-ini-1786168152940.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I812" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B813" t="inlineStr">
+        <is>
+          <t>Hindari Defisit Belanja, Negara Ini Terpaksa Jual Saham BUMN</t>
+        </is>
+      </c>
+      <c r="C813" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:15:57 +0700</t>
+        </is>
+      </c>
+      <c r="D813" t="inlineStr">
+        <is>
+          <t>Ignacio Geordi Oswaldo</t>
+        </is>
+      </c>
+      <c r="E813" t="inlineStr">
+        <is>
+          <t>Defisit fiskal yang terus berlangsung selama beberapa tahun terakhir mendorong pemerintah India untuk mengambil langkah agresif untuk mencari dana.</t>
+        </is>
+      </c>
+      <c r="F813" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G813" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8609924/hindari-defisit-belanja-negara-ini-terpaksa-jual-saham-bumn</t>
+        </is>
+      </c>
+      <c r="H813" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2024/07/12/dolar-as-masih-di-atas-rp-16100-hari-ini-3_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I813" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B814" t="inlineStr">
+        <is>
+          <t>Tempat Makan dan Minum di Transmart Full Day Sale Diobral!</t>
+        </is>
+      </c>
+      <c r="C814" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:00:58 +0700</t>
+        </is>
+      </c>
+      <c r="D814" t="inlineStr">
+        <is>
+          <t>Aulia Damayanti</t>
+        </is>
+      </c>
+      <c r="E814" t="inlineStr">
+        <is>
+          <t>Transmart menggelar Full Day Sale dengan diskon hingga 50%+20% untuk peralatan makan dan minum. Promo mulai Rp 12.000, berlaku hingga pukul 22.00.</t>
+        </is>
+      </c>
+      <c r="F814" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G814" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8609718/tempat-makan-dan-minum-di-transmart-full-day-sale-diobral</t>
+        </is>
+      </c>
+      <c r="H814" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/tempat-makan-dan-minum-di-transmart-full-day-sale-diobral-1786167962984.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I814" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B815" t="inlineStr">
+        <is>
+          <t>Trump Mau Pecat Bos The Fed Lisa Cook</t>
+        </is>
+      </c>
+      <c r="C815" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:30:55 +0700</t>
+        </is>
+      </c>
+      <c r="D815" t="inlineStr">
+        <is>
+          <t>Ignacio Geordi Oswaldo</t>
+        </is>
+      </c>
+      <c r="E815" t="inlineStr">
+        <is>
+          <t>Presiden Amerika Serikat (AS) Donald Trump mempertimbangkan untuk memecat Gubernur Dewan Federal Reserve, Lisa Cook.</t>
+        </is>
+      </c>
+      <c r="F815" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G815" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/moneter/d-8609711/trump-mau-pecat-bos-the-fed-lisa-cook</t>
+        </is>
+      </c>
+      <c r="H815" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2023/02/02/bank-sentral-as-the-fed-naikkan-suku-bunga-sebesar-025-3_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I815" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B816" t="inlineStr">
+        <is>
+          <t>Pertamina Marine Gandeng China, Peluang Kerja Pelaut RI Makin Luas</t>
+        </is>
+      </c>
+      <c r="C816" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:13:32 +0700</t>
+        </is>
+      </c>
+      <c r="D816" t="inlineStr">
+        <is>
+          <t>Ignacio Geordi Oswaldo</t>
+        </is>
+      </c>
+      <c r="E816" t="inlineStr">
+        <is>
+          <t>Salah satu peluang terbesar yang dapat dimanfaatkan adalah meningkatnya kebutuhan tenaga pelaut di China seiring keterbatasan ketersediaan awak kapal.</t>
+        </is>
+      </c>
+      <c r="F816" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G816" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8610133/pertamina-marine-gandeng-china-peluang-kerja-pelaut-ri-makin-luas</t>
+        </is>
+      </c>
+      <c r="H816" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2023/08/02/ilustrasi-kapal-kargo_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I816" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B817" t="inlineStr">
+        <is>
+          <t>Catheez Tak Terburu-buru Menikah Meski Vior dan Meyden Sudah Berumah Tangga</t>
+        </is>
+      </c>
+      <c r="C817" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:26:37 +0700</t>
+        </is>
+      </c>
+      <c r="D817" t="inlineStr">
+        <is>
+          <t>Muhammad Ahsan Nurrijal</t>
+        </is>
+      </c>
+      <c r="E817" t="inlineStr">
+        <is>
+          <t>Catheez, anggota 'Bocah Kosong' yang lajang, memilih fokus pada karier meski sahabatnya sudah menikah. Ia menunggu pasangan yang sesuai tanpa terburu-buru.</t>
+        </is>
+      </c>
+      <c r="F817" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G817" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8610083/catheez-tak-terburu-buru-menikah-meski-vior-dan-meyden-sudah-berumah-tangga</t>
+        </is>
+      </c>
+      <c r="H817" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/10/08/catheez-1759898630170_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I817" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B818" t="inlineStr">
+        <is>
+          <t>Lionel Messi Berkabung, sang Ayah Meninggal Dunia di Usia 68 Tahun</t>
+        </is>
+      </c>
+      <c r="C818" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:37:21 +0700</t>
+        </is>
+      </c>
+      <c r="D818" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E818" t="inlineStr">
+        <is>
+          <t>Ayah Lionel Messi, Jorge, meninggal dunia di usia 68 tahun setelah berjuang melawan sakit berkepanjangan.</t>
+        </is>
+      </c>
+      <c r="F818" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G818" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865821/lionel-messi-berkabung-sang-ayah-meninggal-dunia-di-usia-68-tahun</t>
+        </is>
+      </c>
+      <c r="H818" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/28UKf7vWQ9VAeH0o7NdVBK71qYo=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Lionel-Messi-dan-Omar-Souto.jpg</t>
+        </is>
+      </c>
+      <c r="I818" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B819" t="inlineStr">
+        <is>
+          <t>Profil Ade Darmawan yang Prediksinya 100 Persen Akurat soal Roy Suryo Ajukan Praperadilan ke-4</t>
+        </is>
+      </c>
+      <c r="C819" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:34:47 +0700</t>
+        </is>
+      </c>
+      <c r="D819" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E819" t="inlineStr">
+        <is>
+          <t>Berikut ini adalah profil Sekjen Peradi Bersatu Ade Darmawan yang prediksinya 100 persen akurat soal Roy Suryo ajukan praperadilan ke-4.</t>
+        </is>
+      </c>
+      <c r="F819" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G819" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865820/profil-ade-darmawan-yang-prediksinya-100-persen-akurat-soal-roy-suryo-ajukan-praperadilan-ke-4</t>
+        </is>
+      </c>
+      <c r="H819" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/JL0q5vOW6zgsnndMoQ0aVBaSY-c=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ade-jokowi-dan-roy-suryo.jpg</t>
+        </is>
+      </c>
+      <c r="I819" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B820" t="inlineStr">
+        <is>
+          <t>Live Sprint Race MotoGP Inggris 2026: Start Jam 22.00 WIB, Kans Marc Marquez Tembus 200 Poin</t>
+        </is>
+      </c>
+      <c r="C820" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:27:31 +0700</t>
+        </is>
+      </c>
+      <c r="D820" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E820" t="inlineStr">
+        <is>
+          <t>Marc Marquez bisa menembus 200 poin di tabel klasemen MotoGP 2026 jika memenangkan sprint race MotoGP Inggris 2026 di Silverstone.</t>
+        </is>
+      </c>
+      <c r="F820" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G820" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7865819/live-sprint-race-motogp-inggris-2026-start-jam-2200-wib-kans-marc-marquez-tembus-200-poin</t>
+        </is>
+      </c>
+      <c r="H820" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/QWRdNYbbfG5s6YXga5PrKpnEFfo=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Sprint-Race-MotoGP-Amerika-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I820" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B821" t="inlineStr">
+        <is>
+          <t>Prakiraan Cuaca Provinsi Sulawesi Selatan, Minggu 9 Agustus 2026: Mayoritas Cerah Berawan</t>
+        </is>
+      </c>
+      <c r="C821" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:23:10 +0700</t>
+        </is>
+      </c>
+      <c r="D821" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E821" t="inlineStr">
+        <is>
+          <t>Berikut ini prakiraan cuaca Sulawesi Selatan yang dirilis BMKG untuk Minggu (9/8/2026).  Waspada angin kencang di sejumlah daerah</t>
+        </is>
+      </c>
+      <c r="F821" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G821" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865818/prakiraan-cuaca-provinsi-sulawesi-selatan-minggu-9-agustus-2026-mayoritas-cerah-berawan</t>
+        </is>
+      </c>
+      <c r="H821" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/lDgUVS5zQ1sLN8t3mHbweeriZkY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/cuaca-cerah-berawan-xx.jpg</t>
+        </is>
+      </c>
+      <c r="I821" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B822" t="inlineStr">
+        <is>
+          <t>Potensi Cuaca Daerah di Indonesia, Minggu 9 Agustus 2026: Sejumlah Provinsi Angin Kencang</t>
+        </is>
+      </c>
+      <c r="C822" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:06:23 +0700</t>
+        </is>
+      </c>
+      <c r="D822" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E822" t="inlineStr">
+        <is>
+          <t>Berikut potensi cuaca ekstrem dari BMKG untuk seluruh wilayah di Indonesia pada Minggu (9/8/2026). Waspada angin kencang</t>
+        </is>
+      </c>
+      <c r="F822" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G822" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865817/potensi-cuaca-daerah-di-indonesia-minggu-9-agustus-2026-sejumlah-provinsi-angin-kencang</t>
+        </is>
+      </c>
+      <c r="H822" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/HOrGXDZKm8k3YyRuq5WWYoksQMU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/pesisir-manado-yang-diterjang-angin-kencang-senin-852023121.jpg</t>
+        </is>
+      </c>
+      <c r="I822" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>Pendakian Berujung Duka, Pendaki asal Sumenep Meninggal di Gunung Argopuro seusai Alami Hipotermia</t>
+        </is>
+      </c>
+      <c r="C823" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:05:43 +0700</t>
+        </is>
+      </c>
+      <c r="D823" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E823" t="inlineStr">
+        <is>
+          <t>Jailani sempat mengalami hipotermia sebelum akhirnya dinyatakan meninggal dunia.</t>
+        </is>
+      </c>
+      <c r="F823" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G823" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865816/pendakian-berujung-duka-pendaki-asal-sumenep-meninggal-di-gunung-argopuro-seusai-alami-hipotermia</t>
+        </is>
+      </c>
+      <c r="H823" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/N86l72lvs3Vqh6Pkby9cyrbjr7Q=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/PENDAKI-MENINGGAL-Gunung-Argopuro-Kabupaten-Probolinggo.jpg</t>
+        </is>
+      </c>
+      <c r="I823" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B824" t="inlineStr">
+        <is>
+          <t>Kepala BPS: Sensus Ekonomi 2026 Guna Mutakhirkan Peta Perekonomian Pascapandemi Covid-19</t>
+        </is>
+      </c>
+      <c r="C824" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:59:07 +0700</t>
+        </is>
+      </c>
+      <c r="D824" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E824" t="inlineStr">
+        <is>
+          <t>Sensus Ekonomi merupakan kegiatan rutin dan amanat undang-undang statistik yang diselenggarakan sepuluh tahun sekali</t>
+        </is>
+      </c>
+      <c r="F824" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G824" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865815/kepala-bps-sensus-ekonomi-2026-guna-mutakhirkan-peta-perekonomian-pascapandemi-covid-19</t>
+        </is>
+      </c>
+      <c r="H824" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/PGFrThAVQSR98E2814RfldS-CzI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Kepala-BPS-Amalia-Adininggar-Widyasanti-Podcast-di-Tribunnews_20260808_161645.jpg</t>
+        </is>
+      </c>
+      <c r="I824" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B825" t="inlineStr">
+        <is>
+          <t>Ketangguhan Alex Eala Kunci Tiket 16 Besar Kanada Open, Cedera Engkel Terlupakan Sejenak</t>
+        </is>
+      </c>
+      <c r="C825" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:56:08 +0700</t>
+        </is>
+      </c>
+      <c r="D825" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E825" t="inlineStr">
+        <is>
+          <t>Alex Eala berhasil melangkah ke babak 16 besar tenis Kanada Open 2026 meski sempat mengalami cedera engkel di gim kedua.</t>
+        </is>
+      </c>
+      <c r="F825" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G825" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7865814/ketangguhan-alex-eala-kunci-tiket-16-besar-kanada-open-cedera-engkel-terlupakan-sejenak</t>
+        </is>
+      </c>
+      <c r="H825" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/0fq3TCb3sGuyya0TZ8FScanSb4k=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Alex-Eala-Janice-Tjen-Abu-Dhabi-Open-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I825" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B826" t="inlineStr">
+        <is>
+          <t>Beri Ruang Anak Berekspresi, Seni Bisa Jadi Medium Bangun Kepercayaan Diri</t>
+        </is>
+      </c>
+      <c r="C826" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:55:22 +0700</t>
+        </is>
+      </c>
+      <c r="D826" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E826" t="inlineStr">
+        <is>
+          <t>Karya itu dirancang agar anak-anak dapat membayangkan kota versinya sendiri, sekaligus menempatkan diri dan berinteraksi di dalam ruang tersebut.</t>
+        </is>
+      </c>
+      <c r="F826" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G826" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865813/beri-ruang-anak-berekspresi-seni-bisa-jadi-medium-bangun-kepercayaan-diri</t>
+        </is>
+      </c>
+      <c r="H826" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Y09EQ3wkC5OxVIs82XcQxFRdYdg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/INSTALASI-SENI-Instalasi-seni-interaktif.jpg</t>
+        </is>
+      </c>
+      <c r="I826" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B827" t="inlineStr">
+        <is>
+          <t>300 Anak Meninggal di Gaza dalam 300 Hari Gencatan Senjata</t>
+        </is>
+      </c>
+      <c r="C827" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:54:27 +0700</t>
+        </is>
+      </c>
+      <c r="D827" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E827" t="inlineStr">
+        <is>
+          <t>UNICEF melaporkan sedikitnya 300 anak meninggal di Gaza dalam 300 hari sejak gencatan senjata diumumkan pada Oktober 2025.</t>
+        </is>
+      </c>
+      <c r="F827" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G827" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7865812/300-anak-meninggal-di-gaza-dalam-300-hari-gencatan-senjata</t>
+        </is>
+      </c>
+      <c r="H827" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/pWp_b6B09_hjskkY8LP_JI_G8Tw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/SITUASI-DI-GAZA-qewqe.jpg</t>
+        </is>
+      </c>
+      <c r="I827" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B828" t="inlineStr">
+        <is>
+          <t>Rara Tinggalkan Porprov, Christopher Kurangi Nongkrong demi Paskibraka</t>
+        </is>
+      </c>
+      <c r="C828" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:39:31 +0700</t>
+        </is>
+      </c>
+      <c r="D828" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E828" t="inlineStr">
+        <is>
+          <t>Rara melepas Porprov dan olimpiade, sementara Christopher mengurangi nongkrong demi mengejar Paskibraka Nasional di Istana.</t>
+        </is>
+      </c>
+      <c r="F828" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G828" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865811/rara-tinggalkan-porprov-christopher-kurangi-nongkrong-demi-paskibraka</t>
+        </is>
+      </c>
+      <c r="H828" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/EWHbUEdMD1Ec8BkzGfywykMUXHY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Paskibraka-Christopher-Leon-Bringga-Tabuni-Papua-dan-Raudah-Mabrura-Riau.jpg</t>
+        </is>
+      </c>
+      <c r="I828" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>Malaysia Laporkan Filipina ke PBB, Tak Terima Wilayah Maritim Sabah Dicaplok Manila</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:36:37 +0700</t>
+        </is>
+      </c>
+      <c r="D829" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E829" t="inlineStr">
+        <is>
+          <t>Langkah tegas ini diambil Malaysia sebagai bentuk penolakan atas klaim perluasan landas kontinen Filipina.</t>
+        </is>
+      </c>
+      <c r="F829" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G829" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7865810/malaysia-laporkan-filipina-ke-pbb-tak-terima-wilayah-maritim-sabah-dicaplok-manila</t>
+        </is>
+      </c>
+      <c r="H829" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/DwLaymIH_CDpb55bBNGOep-3OJU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/MENLU-MALAYSIA-Menteri-Luar-Negeri-Malaysia-Datuk-Seri-Mohamad-Hasan-Ambalat-Indonesia.jpg</t>
+        </is>
+      </c>
+      <c r="I829" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>Fakta Pembunuhan Marbot Masjid di Purwakarta: Pelaku Disebut Sering Resahkan Warga</t>
+        </is>
+      </c>
+      <c r="C830" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:33:14 +0700</t>
+        </is>
+      </c>
+      <c r="D830" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E830" t="inlineStr">
+        <is>
+          <t>Marbot masjid di Purwakarta tewas dibunuh pelaku yang tersinggung soal ekonomi. Pelaku yang kerap meresahkan warga tersebut kini telah ditangkap.</t>
+        </is>
+      </c>
+      <c r="F830" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G830" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865809/fakta-pembunuhan-marbot-masjid-di-purwakarta-pelaku-disebut-sering-resahkan-warga</t>
+        </is>
+      </c>
+      <c r="H830" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/iVQoFd00f4I54X3zKDiHAJJIyGM=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Marbot-Masjid-Tewas.jpg</t>
+        </is>
+      </c>
+      <c r="I830" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B831" t="inlineStr">
+        <is>
+          <t>Pikap yang Fleksibel, Isuzu Traga Disulap Jadi Armada Salon Keliling di GIIAS 2026</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:29:36 +0700</t>
+        </is>
+      </c>
+      <c r="D831" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E831" t="inlineStr">
+        <is>
+          <t>Salon keliling ini hasil kerja sama Isuzu dengan Putri Hair Choice dari ParagonCorp dan Karoseri Delima Mandiri, Bogor.</t>
+        </is>
+      </c>
+      <c r="F831" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G831" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/otomotif/7865808/pikap-yang-fleksibel-isuzu-traga-disulap-jadi-armada-salon-keliling-di-giias-2026</t>
+        </is>
+      </c>
+      <c r="H831" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/_hEhvARFMgAMB6Ql_QUJ_d9_E2Y=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Salon-keliling-Isuzu-Traga-GIIAS-2026-OK.jpg</t>
+        </is>
+      </c>
+      <c r="I831" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B832" t="inlineStr">
+        <is>
+          <t>Kondisi Kampung Walesi Papua Pascapenembakan di Festival Lembah Baliem</t>
+        </is>
+      </c>
+      <c r="C832" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:10:08 +0700</t>
+        </is>
+      </c>
+      <c r="D832" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E832" t="inlineStr">
+        <is>
+          <t>Penembakan dilakukan dari arah depan pintu masuk festival.</t>
+        </is>
+      </c>
+      <c r="F832" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G832" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265242/kondisi-kampung-walesi-papua-pascapenembakan-di-festival-lembah-baliem</t>
+        </is>
+      </c>
+      <c r="H832" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/Lq-D7C_bNeBvJmZRsKm9Dz2iBZg=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9319184/original/076078900_1786194252-WhatsApp-Image-2026-08-08-at-18.14.19.jpeg</t>
+        </is>
+      </c>
+      <c r="I832" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>Sudah 20 Tahun, Aturan Polusi Jakarta Didorong Direvisi</t>
+        </is>
+      </c>
+      <c r="C833" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:47:25 +0700</t>
+        </is>
+      </c>
+      <c r="D833" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E833" t="inlineStr">
+        <is>
+          <t>Polusi udara Jakarta makin kompleks, aturan lama dinilai tak lagi memadai.</t>
+        </is>
+      </c>
+      <c r="F833" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G833" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265237/sudah-20-tahun-aturan-polusi-jakarta-didorong-direvisi</t>
+        </is>
+      </c>
+      <c r="H833" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/Dxb3oVe0p-JqteJfoTmcpR-NJnQ=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/4516753/original/082794300_1690458364-Polusi-Udara-Jakarta-6.jpg</t>
+        </is>
+      </c>
+      <c r="I833" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B834" t="inlineStr">
+        <is>
+          <t>Energi Bersih Masuk Sawah Bantu Petani Atasi Masalah Pascapanen</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:40:41 +0700</t>
+        </is>
+      </c>
+      <c r="D834" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E834" t="inlineStr">
+        <is>
+          <t>Mesin bertenaga surya ini membawa cara baru mengolah hasil panen jagung.</t>
+        </is>
+      </c>
+      <c r="F834" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G834" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265229/energi-bersih-masuk-sawah-bantu-petani-atasi-masalah-pascapanen</t>
+        </is>
+      </c>
+      <c r="H834" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/BIkVp5tCgSqDiwprCJzukcG_0FM=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9319172/original/081140100_1786192013-WhatsApp_Image_2026-08-07_at_11.56.53_AM.jpeg</t>
+        </is>
+      </c>
+      <c r="I834" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" t="inlineStr">
+        <is>
+          <t>Otomotif</t>
+        </is>
+      </c>
+      <c r="B835" t="inlineStr">
+        <is>
+          <t>Hasil Kualifikasi Moto3 Silverstone: Veda Pratama Start Posisi 16</t>
+        </is>
+      </c>
+      <c r="C835" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:41:29 +0700</t>
+        </is>
+      </c>
+      <c r="D835" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E835" t="inlineStr">
+        <is>
+          <t>Veda Ega Pratama harus puas mengawali balapan Moto3 Silverstone dari posisi ke-16 usai mencatatkan waktu 2 menit 10,910 detik pada Q2</t>
+        </is>
+      </c>
+      <c r="F835" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G835" t="inlineStr">
+        <is>
+          <t>https://otomotif.kompas.com/read/2026/08/08/204104815/hasil-kualifikasi-moto3-silverstone-veda-pratama-start-posisi-16</t>
+        </is>
+      </c>
+      <c r="H835" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/qX_kW7KvheqAfued2WwRubyuIFk=/0x0:3751x2501/1200x675/filters:watermark(data/photo/2026/01/30/697c81750a668.png,0,-0,1)/data/photo/2026/07/13/6a54088886ae4.jpg</t>
+        </is>
+      </c>
+      <c r="I835" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" t="inlineStr">
+        <is>
+          <t>Tren</t>
+        </is>
+      </c>
+      <c r="B836" t="inlineStr">
+        <is>
+          <t>Benarkah Penampilan Paw Bisa Tandai Kondisi Kesehatan Kucing?</t>
+        </is>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:41:29 +0700</t>
+        </is>
+      </c>
+      <c r="D836" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E836" t="inlineStr">
+        <is>
+          <t>Sebuah unggahan menyebut bahwa penampilan paw bisa menandai kondisi kesehatan kucing, viral di media sosial.</t>
+        </is>
+      </c>
+      <c r="F836" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G836" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/tren/read/2026/08/08/200000065/benarkah-penampilan-paw-bisa-tandai-kondisi-kesehatan-kucing-</t>
+        </is>
+      </c>
+      <c r="H836" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/gyr1Ab21kC_wwAm86mx2dXFQkFY=/0x105:640x532/1200x675/filters:watermark(data/photo/2026/01/30/697c818d0ca91.png,0,-0,1)/data/photo/2026/01/15/69686fe294503.jpg</t>
+        </is>
+      </c>
+      <c r="I836" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B837" t="inlineStr">
+        <is>
+          <t>Mentan Amran Kunjungi Alor Usai Terima Keluhan Harga Beras Tembus Rp 30.000 Per Kg</t>
+        </is>
+      </c>
+      <c r="C837" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:41:29 +0700</t>
+        </is>
+      </c>
+      <c r="D837" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E837" t="inlineStr">
+        <is>
+          <t>Mentan Amran langsung terbang ke Alor usai ada keluhan harga beras, batalkan rapat. Ia pastikan ketersediaan pangan dan solusi.</t>
+        </is>
+      </c>
+      <c r="F837" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G837" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/08/08/191924178/mentan-amran-kunjungi-alor-usai-terima-keluhan-harga-beras-tembus-rp-30000</t>
+        </is>
+      </c>
+      <c r="H837" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/6XnE8Hx5StfwqFRaGwM_UM-XvA8=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/08/6a7719cf2cd28.jpg</t>
+        </is>
+      </c>
+      <c r="I837" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I784"/>
+  <autoFilter ref="A1:I837"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-08 14:26 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-08.xlsx
+++ b/data/berita_2026-08-08.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$837</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$895</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I837"/>
+  <dimension ref="A1:I895"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -39776,8 +39776,2734 @@
         </is>
       </c>
     </row>
+    <row r="838">
+      <c r="A838" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B838" t="inlineStr">
+        <is>
+          <t>Posmeti gelar Turnamen Merpati Tinggi Tomprang sambut HUT RI</t>
+        </is>
+      </c>
+      <c r="C838" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:19:55 +0700</t>
+        </is>
+      </c>
+      <c r="D838" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E838" t="inlineStr">
+        <is>
+          <t>Perkumpulan Olahraga Seni Merpati Terbang Tinggi (Posmeti) menggelar Turnamen Merpati Tinggi Tomprang dalam rangka ...</t>
+        </is>
+      </c>
+      <c r="F838" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G838" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685959/posmeti-gelar-turnamen-merpati-tinggi-tomprang-sambut-hut-ri</t>
+        </is>
+      </c>
+      <c r="H838" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000302419.jpg</t>
+        </is>
+      </c>
+      <c r="I838" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B839" t="inlineStr">
+        <is>
+          <t>Wapres Turkiye: Pakta pertahanan tak ditujukan untuk lawan Iran</t>
+        </is>
+      </c>
+      <c r="C839" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:18:18 +0700</t>
+        </is>
+      </c>
+      <c r="D839" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E839" t="inlineStr">
+        <is>
+          <t>Wakil Presiden Turkiye Cevdet Yilmaz pada Sabtu mengatakan bahwa perjanjian pertahanan Turki dengan Arab Saudi dan ...</t>
+        </is>
+      </c>
+      <c r="F839" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G839" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685955/wapres-turkiye-pakta-pertahanan-tak-ditujukan-untuk-lawan-iran</t>
+        </is>
+      </c>
+      <c r="H839" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IranBenderadiMabesPBBXinhua_LiMuzi_am.jpg</t>
+        </is>
+      </c>
+      <c r="I839" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B840" t="inlineStr">
+        <is>
+          <t>DPP Perbasi perbarui data pemain dan klub</t>
+        </is>
+      </c>
+      <c r="C840" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:14:56 +0700</t>
+        </is>
+      </c>
+      <c r="D840" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E840" t="inlineStr">
+        <is>
+          <t>Dewan Pengurus Pusat Persatuan Bola Basket Seluruh Indonesia (DPP Perbasi) melakukan pembaruan data pemain, klub, ...</t>
+        </is>
+      </c>
+      <c r="F840" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G840" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685952/dpp-perbasi-perbarui-data-pemain-dan-klub</t>
+        </is>
+      </c>
+      <c r="H840" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000476713.jpg</t>
+        </is>
+      </c>
+      <c r="I840" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B841" t="inlineStr">
+        <is>
+          <t>Indonesia dan India perkuat kerja sama pelestarian warisan budaya</t>
+        </is>
+      </c>
+      <c r="C841" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:09:22 +0700</t>
+        </is>
+      </c>
+      <c r="D841" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E841" t="inlineStr">
+        <is>
+          <t>Pemerintah Indonesia dan India memperkuat kerja sama dalam upaya pelestarian warisan budaya, pertukaran budaya, dan ...</t>
+        </is>
+      </c>
+      <c r="F841" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G841" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685949/indonesia-dan-india-perkuat-kerja-sama-pelestarian-warisan-budaya</t>
+        </is>
+      </c>
+      <c r="H841" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/WhatsApp-Image-2026-08-08-at-20.03.57.jpeg</t>
+        </is>
+      </c>
+      <c r="I841" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B842" t="inlineStr">
+        <is>
+          <t>Waka DPR dorong Agustusan dikemas untuk tanamkan nasionalisme gen Alfa</t>
+        </is>
+      </c>
+      <c r="C842" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:09:19 +0700</t>
+        </is>
+      </c>
+      <c r="D842" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E842" t="inlineStr">
+        <is>
+          <t>Wakil Ketua DPR RI Cucun Ahmad Syamsurijal mendorong Agustusan atau tradisi perayaan HUT kemerdekaan RI di tingkat ...</t>
+        </is>
+      </c>
+      <c r="F842" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G842" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685948/waka-dpr-dorong-agustusan-dikemas-untuk-tanamkan-nasionalisme-gen-alfa</t>
+        </is>
+      </c>
+      <c r="H842" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/WhatsApp-Image-2026-08-08-at-19.53.13.jpeg</t>
+        </is>
+      </c>
+      <c r="I842" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B843" t="inlineStr">
+        <is>
+          <t>Wapres Turkiye: Mesir berpotensi bergabung dengan pakta pertahanan</t>
+        </is>
+      </c>
+      <c r="C843" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:07:47 +0700</t>
+        </is>
+      </c>
+      <c r="D843" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E843" t="inlineStr">
+        <is>
+          <t>Wakil Presiden Turkiye Cevdet Yilmaz pada Sabtu mengatakan bahwa Mesir berpotensi bergabung dalam perjanjian pertahanan ...</t>
+        </is>
+      </c>
+      <c r="F843" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G843" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685947/wapres-turkiye-mesir-berpotensi-bergabung-dengan-pakta-pertahanan</t>
+        </is>
+      </c>
+      <c r="H843" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/MesirSuasanaSungaiNilXinhuaAhmedGomaa_aa.jpg</t>
+        </is>
+      </c>
+      <c r="I843" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B844" t="inlineStr">
+        <is>
+          <t>Task Foce Hanura targetkan struktur partai 100 persen se-Indonesia</t>
+        </is>
+      </c>
+      <c r="C844" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:01:49 +0700</t>
+        </is>
+      </c>
+      <c r="D844" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E844" t="inlineStr">
+        <is>
+          <t>Ketua Tim Task Force DPP Partai Hanura Rio Capella mengatakan pihaknya menargetkan penguatan struktur partai hingga ...</t>
+        </is>
+      </c>
+      <c r="F844" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G844" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685943/task-foce-hanura-targetkan-struktur-partai-100-persen-se-indonesia</t>
+        </is>
+      </c>
+      <c r="H844" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000582569.jpg</t>
+        </is>
+      </c>
+      <c r="I844" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B845" t="inlineStr">
+        <is>
+          <t>Kedubes Palestina percantik kawasan Jakarta, apresiasi dukungan RI</t>
+        </is>
+      </c>
+      <c r="C845" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:01:28 +0700</t>
+        </is>
+      </c>
+      <c r="D845" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E845" t="inlineStr">
+        <is>
+          <t>Kedutaan Besar Negara Palestina di Jakarta, Sabtu, menggelar kerja sukarela bersama komunitas dan pelajar Palestina ...</t>
+        </is>
+      </c>
+      <c r="F845" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G845" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685939/kedubes-palestina-percantik-kawasan-jakarta-apresiasi-dukungan-ri</t>
+        </is>
+      </c>
+      <c r="H845" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000011258.jpg</t>
+        </is>
+      </c>
+      <c r="I845" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B846" t="inlineStr">
+        <is>
+          <t>Tim pendahulu petakan tantangan arena dan transportasi Asian Games</t>
+        </is>
+      </c>
+      <c r="C846" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:57:50 +0700</t>
+        </is>
+      </c>
+      <c r="D846" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E846" t="inlineStr">
+        <is>
+          <t>Tim pendahulu Chef de Mission (CdM) Indonesia telah berada di Nagoya, Jepang, untuk mematangkan berbagai kebutuhan ...</t>
+        </is>
+      </c>
+      <c r="F846" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G846" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685936/tim-pendahulu-petakan-tantangan-arena-dan-transportasi-asian-games</t>
+        </is>
+      </c>
+      <c r="H846" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/21/cdm-asian-games-tinjau-pelatnas-wushu-2825484.jpg</t>
+        </is>
+      </c>
+      <c r="I846" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>Calon Paskibraka jalani latihan gabungan untuk upacara HUT ke-81 RI</t>
+        </is>
+      </c>
+      <c r="C847" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:49:10 +0700</t>
+        </is>
+      </c>
+      <c r="D847" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E847" t="inlineStr">
+        <is>
+          <t>ANTARA - Calon Pasukan Pengibar Bendera Pusaka (Paskibraka) tinkat pusat menjalani latihan gabungan bersama TNI, Polri ...</t>
+        </is>
+      </c>
+      <c r="F847" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G847" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5685925/calon-paskibraka-jalani-latihan-gabungan-untuk-upacara-hut-ke-81-ri</t>
+        </is>
+      </c>
+      <c r="H847" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/CALON-PASKIRBARAKA-JALANI-LATIHAN-GABUNGAN-UNTUK-UPACARA-HUT-KE-81-RI.jpg</t>
+        </is>
+      </c>
+      <c r="I847" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B848" t="inlineStr">
+        <is>
+          <t>Erdogan: Pakta Turkiye-Saudi-Pakistan perkuat perang melawan terorisme</t>
+        </is>
+      </c>
+      <c r="C848" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:48:10 +0700</t>
+        </is>
+      </c>
+      <c r="D848" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E848" t="inlineStr">
+        <is>
+          <t>Presiden Turkiye Recep Tayyip Erdogan menyatakan bahwa Kesepakatan Mekkah, yang ditandatangani oleh Turkiye, Arab ...</t>
+        </is>
+      </c>
+      <c r="F848" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G848" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685933/erdogan-pakta-turkiye-saudi-pakistan-perkuat-perang-melawan-terorisme</t>
+        </is>
+      </c>
+      <c r="H848" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/ErdoganRecepTayyipPresTurkiIstanaKepresBogorRabu120225ALiviaKristianti.jpg</t>
+        </is>
+      </c>
+      <c r="I848" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>Pemerintah berhati-hati dalam merevisi peraturan tentang industri gim</t>
+        </is>
+      </c>
+      <c r="C849" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:45:56 +0700</t>
+        </is>
+      </c>
+      <c r="D849" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E849" t="inlineStr">
+        <is>
+          <t>Menteri Ekonomi Kreatif Teuku Riefky Harsya menyampaikan bahwa pemerintah berhati-hati dalam menyusun ...</t>
+        </is>
+      </c>
+      <c r="F849" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G849" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685929/pemerintah-berhati-hati-dalam-merevisi-peraturan-tentang-industri-gim</t>
+        </is>
+      </c>
+      <c r="H849" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG-20260808-WA0248.jpg</t>
+        </is>
+      </c>
+      <c r="I849" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>Pimpinan MPR Ziarah ke Makam Bung Hatta, Kenang Perjuangan Pendiri Bangsa</t>
+        </is>
+      </c>
+      <c r="C850" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:02:36 +0700</t>
+        </is>
+      </c>
+      <c r="D850" t="inlineStr">
+        <is>
+          <t>Fara Difa Alfeni</t>
+        </is>
+      </c>
+      <c r="E850" t="inlineStr">
+        <is>
+          <t>Pimpinan MPR RI ziarah ke makam Bung Hatta menjelang HUT ke-81 Kemerdekaan RI. Ini momentum mengenang jasa dan semangat perjuangan para pendiri bangsa.</t>
+        </is>
+      </c>
+      <c r="F850" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G850" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610227/pimpinan-mpr-ziarah-ke-makam-bung-hatta-kenang-perjuangan-pendiri-bangsa</t>
+        </is>
+      </c>
+      <c r="H850" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/ziarah-ke-makam-bung-hatta-muzani-ingatkan-perjuangan-pendiri-bangsa-1786196487570_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I850" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>Pria Bunuh Wanita Open BO di Pinrang Sulsel, Dipicu Cekcok Masalah Tarif</t>
+        </is>
+      </c>
+      <c r="C851" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:49:13 +0700</t>
+        </is>
+      </c>
+      <c r="D851" t="inlineStr">
+        <is>
+          <t>Muchlis Abduh</t>
+        </is>
+      </c>
+      <c r="E851" t="inlineStr">
+        <is>
+          <t>Polisi menangkap pria inisial MB usai membunuh wanita inisial IN (28) saat open booking (BO) di kamar kos daerah Kabupaten Pinrang, Sulawesi Selatan (Sulsel)</t>
+        </is>
+      </c>
+      <c r="F851" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G851" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610223/pria-bunuh-wanita-open-bo-di-pinrang-sulsel-dipicu-cekcok-masalah-tarif</t>
+        </is>
+      </c>
+      <c r="H851" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/pria-berinisial-mb-29-ditangkap-gegara-membunuh-wanita-inisial-in-1786186106452_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I851" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B852" t="inlineStr">
+        <is>
+          <t>2 Lantai Ini Diduga Jadi Titik Awal Kebakaran Gedung Bapenda DKI</t>
+        </is>
+      </c>
+      <c r="C852" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:19:18 +0700</t>
+        </is>
+      </c>
+      <c r="D852" t="inlineStr">
+        <is>
+          <t>Brigitta Belia Permata Sari</t>
+        </is>
+      </c>
+      <c r="E852" t="inlineStr">
+        <is>
+          <t>Polisi masih menyelidiki penyebab kebakaran Gedung Badan Pendapatan Daerah (Bapenda) DKI Jakarta. Dugaan sementara, api berasal dari lantai 11 atau lantai 12.</t>
+        </is>
+      </c>
+      <c r="F852" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G852" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610202/2-lantai-ini-diduga-jadi-titik-awal-kebakaran-gedung-bapenda-dki</t>
+        </is>
+      </c>
+      <c r="H852" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/potret-kobaran-api-mengamuk-di-gedung-bapenda-dki-1786160999264_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I852" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>Olah TKP Kebakaran Gedung Bapenda DKI, Polisi Ambil Sampel Abu dari 3 Lantai</t>
+        </is>
+      </c>
+      <c r="C853" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:54:35 +0700</t>
+        </is>
+      </c>
+      <c r="D853" t="inlineStr">
+        <is>
+          <t>Brigitta Belia Permata Sari</t>
+        </is>
+      </c>
+      <c r="E853" t="inlineStr">
+        <is>
+          <t>Polisi bersama Puslabfor Polri melakukan olah tempat kejadian perkara (TKP) dan mengambil sejumlah sampel dari tiga lantai gedung yang terbakar.</t>
+        </is>
+      </c>
+      <c r="F853" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G853" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610177/olah-tkp-kebakaran-gedung-bapenda-dki-polisi-ambil-sampel-abu-dari-3-lantai</t>
+        </is>
+      </c>
+      <c r="H853" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/kasat-reskrim-polres-metro-jakarta-pusat-akbp-roby-heri-saputra-beliadetikcom-1786193582821_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I853" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B854" t="inlineStr">
+        <is>
+          <t>Hendak Antar Paket ke Lantai 13, Kurir Baru Tahu Gedung Bapenda DKI Terbakar</t>
+        </is>
+      </c>
+      <c r="C854" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:47:06 +0700</t>
+        </is>
+      </c>
+      <c r="D854" t="inlineStr">
+        <is>
+          <t>Brigitta Belia Permata Sari</t>
+        </is>
+      </c>
+      <c r="E854" t="inlineStr">
+        <is>
+          <t>Kurir Muhaimin terkejut saat tiba di Gedung Bapenda DKI Jakarta dan menemukan kebakaran. Paket yang dibawanya berisi dekorasi untuk 17 Agustus.</t>
+        </is>
+      </c>
+      <c r="F854" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G854" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610173/hendak-antar-paket-ke-lantai-13-kurir-baru-tahu-gedung-bapenda-dki-terbakar</t>
+        </is>
+      </c>
+      <c r="H854" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/kurir-bernama-muhaimin-40-1786193079492_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I854" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>Ibu-Anak Tewas di Hutan Kalbar Diduga Dibunuh Perampok, Duit Rp 135 Juta Raib</t>
+        </is>
+      </c>
+      <c r="C855" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:34:35 +0700</t>
+        </is>
+      </c>
+      <c r="D855" t="inlineStr">
+        <is>
+          <t>Ocsya Ade CP</t>
+        </is>
+      </c>
+      <c r="E855" t="inlineStr">
+        <is>
+          <t>Kematian ibu dan balita yang jasadnya ditemukan di sebuah hutan daerah Kabupaten Landak, Kalimantan Barat (Kalbar), mengarah pada dugaan perampokan.</t>
+        </is>
+      </c>
+      <c r="F855" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G855" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610156/ibu-anak-tewas-di-hutan-kalbar-diduga-dibunuh-perampok-duit-rp-135-juta-raib</t>
+        </is>
+      </c>
+      <c r="H855" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/jenazah-ibu-dan-balitanya-yang-tewas-terikat-di-hutan-landak-1786178167460_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I855" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>Sespimma Polri 76 Salurkan Bantuan-Ajak Warga Bandung Jaga Kamtibmas</t>
+        </is>
+      </c>
+      <c r="C856" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:22:45 +0700</t>
+        </is>
+      </c>
+      <c r="D856" t="inlineStr">
+        <is>
+          <t>Wildan Noviansah</t>
+        </is>
+      </c>
+      <c r="E856" t="inlineStr">
+        <is>
+          <t>Sespimma Polri Angkatan 76 TA 2026 menggelar bakti sosial di Bandung, menyalurkan bantuan dan mengajak masyarakat menjaga keamanan serta ketertiban.</t>
+        </is>
+      </c>
+      <c r="F856" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G856" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610146/sespimma-polri-76-salurkan-bantuan-ajak-warga-bandung-jaga-kamtibmas</t>
+        </is>
+      </c>
+      <c r="H856" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/sespimma-polri-angkatan-76-ta-2026-menggelar-bakti-sosial-di-bandung-dokistimewa-1786191710707_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I856" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>Polisi Ungkap Saepul Pelaku Mutilasi Punya Basic Tukang Daging</t>
+        </is>
+      </c>
+      <c r="C857" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:20:15 +0700</t>
+        </is>
+      </c>
+      <c r="D857" t="inlineStr">
+        <is>
+          <t>Mei Amelia R</t>
+        </is>
+      </c>
+      <c r="E857" t="inlineStr">
+        <is>
+          <t>Polisi mengungkap Saepul (26) yang membunuh dan memutilasi K (51) di Depok. Motifnya adalah merampok motor korban setelah berkenalan di media sosial.</t>
+        </is>
+      </c>
+      <c r="F857" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G857" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610152/polisi-ungkap-saepul-pelaku-mutilasi-punya-basic-tukang-daging</t>
+        </is>
+      </c>
+      <c r="H857" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/saepul-26-pelaku-mutilasi-pria-inisial-k-di-depok-diperiksa-di-polda-metro-jaya-1786191209681_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I857" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B858" t="inlineStr">
+        <is>
+          <t>Beli AC Split 1PK di Transmart Full Day Sale Dapat Diskon Hingga Rp 1,7 Juta!</t>
+        </is>
+      </c>
+      <c r="C858" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:00:50 +0700</t>
+        </is>
+      </c>
+      <c r="D858" t="inlineStr">
+        <is>
+          <t>Ignacio Geordi Oswaldo</t>
+        </is>
+      </c>
+      <c r="E858" t="inlineStr">
+        <is>
+          <t>Transmart menggelar Full Day Sale pada 9 Agustus 2026, dengan diskon hingga 50+20% untuk berbagai produk, termasuk AC Polytron. Jangan lewatkan.</t>
+        </is>
+      </c>
+      <c r="F858" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G858" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8609720/beli-ac-split-1pk-di-transmart-full-day-sale-dapat-diskon-hingga-rp-1-7-juta</t>
+        </is>
+      </c>
+      <c r="H858" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/beli-ac-split-1pk-di-transmart-full-day-sale-dapat-diskon-hingga-rp-17-juta-1786168062463.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I858" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B859" t="inlineStr">
+        <is>
+          <t>Pengadilan AS Minta Trump Setop Pembangunan Ballroom Rp 7,16 T di Gedung Putih</t>
+        </is>
+      </c>
+      <c r="C859" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:45:53 +0700</t>
+        </is>
+      </c>
+      <c r="D859" t="inlineStr">
+        <is>
+          <t>Aulia Damayanti</t>
+        </is>
+      </c>
+      <c r="E859" t="inlineStr">
+        <is>
+          <t>Pengadilan banding federal Amerika Serikat (AS) meminta Presiden AS Donald Trump untuk menghentikan pembangunan ballroom di sisi timur Gedung Putih.</t>
+        </is>
+      </c>
+      <c r="F859" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G859" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/infrastruktur/d-8609913/pengadilan-as-minta-trump-setop-pembangunan-ballroom-rp-7-16-t-di-gedung-putih</t>
+        </is>
+      </c>
+      <c r="H859" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/presiden-as-donald-trump-saat-seremoni-penandatanganan-perintah-eksekutif-membatasi-hak-kewarganegaraan-berdasarkan-tempat-kel-1786086100834_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I859" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B860" t="inlineStr">
+        <is>
+          <t>Ruben Onsu Kangen Dipanggil 'Ayah' Anak-anak, Pilih Tak Larut dalam Sedih</t>
+        </is>
+      </c>
+      <c r="C860" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:29:46 +0700</t>
+        </is>
+      </c>
+      <c r="D860" t="inlineStr">
+        <is>
+          <t>Muhammad Ahsan Nurrijal</t>
+        </is>
+      </c>
+      <c r="E860" t="inlineStr">
+        <is>
+          <t>Ruben Onsu mengungkap kerinduan akan panggilan 'Ayah' dari anak-anaknya di tengah proses hukum hak asuh. Ia berusaha tetap positif dan menerima keadaan.</t>
+        </is>
+      </c>
+      <c r="F860" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G860" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8610087/ruben-onsu-kangen-dipanggil-ayah-anak-anak-pilih-tak-larut-dalam-sedih</t>
+        </is>
+      </c>
+      <c r="H860" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/ruben-onsu-dan-sarwendah-1785990958341_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I860" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t>Siap-Siap, Besok Ada Gebyar Diskon Gede di Transmart Full Day Sale</t>
+        </is>
+      </c>
+      <c r="C861" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D861" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E861" t="inlineStr">
+        <is>
+          <t>Siap-siap, soalnya Transmart Full Day Sale bakal balik lagi besok, Minggu (9/8), sambil bawa diskon gede-gedean 50 persen plus 20 persen.</t>
+        </is>
+      </c>
+      <c r="F861" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G861" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260807124334-97-1389674/siap-siap-besok-ada-gebyar-diskon-gede-di-transmart-full-day-sale</t>
+        </is>
+      </c>
+      <c r="H861" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2023/10/08/warga-berbelanja-di-transmart-kota-kasablanka-13_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I861" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>4 Titik di Tol Jakarta-Cikampek Diperbaiki hingga Pekan Depan</t>
+        </is>
+      </c>
+      <c r="C862" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:45:51 +0700</t>
+        </is>
+      </c>
+      <c r="D862" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E862" t="inlineStr">
+        <is>
+          <t>PT Jasamarga Transjawa Tol (JTT) kembali melakukan pemeliharaan di sejumlah titik ruas Tol Jakarta-Cikampek hingga pekan depan.</t>
+        </is>
+      </c>
+      <c r="F862" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G862" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260808201357-92-1390183/4-titik-di-tol-jakarta-cikampek-diperbaiki-hingga-pekan-depan</t>
+        </is>
+      </c>
+      <c r="H862" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/03/24/pt-jasamarga-transjawa-tol-jtt-mendukung-pemberlakuan-rekayasa-lalu-lintas-berupa-contraflow-satu-lajur-dari-km-70-sd-km-47-ar-1774349147847_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I862" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>FOTO: Menyulap Sampah Jadi Paving Block</t>
+        </is>
+      </c>
+      <c r="C863" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:18:15 +0700</t>
+        </is>
+      </c>
+      <c r="D863" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E863" t="inlineStr">
+        <is>
+          <t>Sampah plastik tertolak dimanfaatkan sebagai bahan baku pembuatan paving block yang ramah lingkungan di kawasan Kebayoran Lama, Jakarta Selatan.</t>
+        </is>
+      </c>
+      <c r="F863" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G863" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260807175918-94-1389856/foto-menyulap-sampah-jadi-paving-block</t>
+        </is>
+      </c>
+      <c r="H863" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/07/mengubah-sampah-menjadi-paving-blok-1786098440328_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I863" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>Alat Masak Rp70 Ribuan Cuma di Transmart Full Day Sale, Serbu Bun!</t>
+        </is>
+      </c>
+      <c r="C864" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D864" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E864" t="inlineStr">
+        <is>
+          <t>Siap-siap, soalnya Transmart Full Day Sale bakal balik lagi besok, Minggu (9/8), sambil bawa diskon gede-gedean 50 persen plus 20 persen.</t>
+        </is>
+      </c>
+      <c r="F864" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G864" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260807125115-97-1389681/alat-masak-rp70-ribuan-cuma-di-transmart-full-day-sale-serbu-bun</t>
+        </is>
+      </c>
+      <c r="H864" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2023/11/12/pengunjung-ramai-serbu-transmart-full-day-sale-di-transmart-cilandak-3_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I864" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B865" t="inlineStr">
+        <is>
+          <t>Kepala Bapanas dan Dirut Bulog Serahkan Bantuan Pangan Perdana di Alor</t>
+        </is>
+      </c>
+      <c r="C865" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:31:14 +0700</t>
+        </is>
+      </c>
+      <c r="D865" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E865" t="inlineStr">
+        <is>
+          <t>Kepala Bapanas dan Dirut Bulog kunjungi Alor untuk pastikan bantuan pangan tiga bulan diterima 37.338 penerima, komitmen ketahanan pangan.</t>
+        </is>
+      </c>
+      <c r="F865" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G865" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260808190414-97-1390176/kepala-bapanas-dan-dirut-bulog-serahkan-bantuan-pangan-perdana-di-alor</t>
+        </is>
+      </c>
+      <c r="H865" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/bulog-1786190836313_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I865" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B866" t="inlineStr">
+        <is>
+          <t>Alat Elektronik Lagi Diskon di Transmart Full Day Sale, Cek Daftarnya</t>
+        </is>
+      </c>
+      <c r="C866" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D866" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E866" t="inlineStr">
+        <is>
+          <t>Siap-siap, soalnya Transmart Full Day Sale bakal balik lagi besok, Minggu (9/8), sambil bawa diskon gede-gedean 50 persen plus 20 persen.</t>
+        </is>
+      </c>
+      <c r="F866" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G866" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260807123224-97-1389671/alat-elektronik-lagi-diskon-di-transmart-full-day-sale-cek-daftarnya</t>
+        </is>
+      </c>
+      <c r="H866" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2025/04/27/transmart-full-day-sale-di-kokas-diserbu-pengunjung-tv-dan-ac-jadi-incaran-1745751864041_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I866" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B867" t="inlineStr">
+        <is>
+          <t>Sambut Hari Merdeka, Transmart Full Day Sale Besok Diskon 50% + 20%</t>
+        </is>
+      </c>
+      <c r="C867" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D867" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E867" t="inlineStr">
+        <is>
+          <t>Dalam rangka menyambut hari kemerdekaan RI, Transmart bakal tebar diskon seharian penuh hingga 50% + 20% pada Minggu (9/8).</t>
+        </is>
+      </c>
+      <c r="F867" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G867" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260807130017-97-1389684/sambut-hari-merdeka-transmart-full-day-sale-besok-diskon-50-20</t>
+        </is>
+      </c>
+      <c r="H867" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/04/05/transmart-full-day-sale-1775380942036_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I867" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B868" t="inlineStr">
+        <is>
+          <t>Mentan Respons Curhatan Adriano: Aspirasi Riil untuk Masyarakat Alor</t>
+        </is>
+      </c>
+      <c r="C868" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:29:11 +0700</t>
+        </is>
+      </c>
+      <c r="D868" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E868" t="inlineStr">
+        <is>
+          <t>Usai mendapat aspirasi tentang distribusi beras di Alor, Mentan membatalkan agenda rapat di Jakarta dan segera terbang ke NTT untuk melihat situasi di lapangan.</t>
+        </is>
+      </c>
+      <c r="F868" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G868" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260808144735-97-1390102/mentan-respons-curhatan-adriano-aspirasi-riil-untuk-masyarakat-alor</t>
+        </is>
+      </c>
+      <c r="H868" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/kementan-1786175594903_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I868" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B869" t="inlineStr">
+        <is>
+          <t>Respons Bahlil Usai Kinerja Dipuji Prabowo: Harus Jawab dengan Kerja</t>
+        </is>
+      </c>
+      <c r="C869" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:23:29 +0700</t>
+        </is>
+      </c>
+      <c r="D869" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E869" t="inlineStr">
+        <is>
+          <t>Menteri Energi dan Sumber Daya Mineral (ESDM) Bahlil Lahadalia memilih merendah usai Presiden Prabowo Subianto mengaku puas terhadap kinerjanya.</t>
+        </is>
+      </c>
+      <c r="F869" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G869" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260808151745-85-1390117/respons-bahlil-usai-kinerja-dipuji-prabowo-harus-jawab-dengan-kerja</t>
+        </is>
+      </c>
+      <c r="H869" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/07/peluncuran-sepuluh-buku-karya-nyata-untuk-negeri-bahlil-lahadalia-1786099773572_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I869" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B870" t="inlineStr">
+        <is>
+          <t>Daftar Perbaikan Tata Kelola MBG di Bawah Komando Sudaryono</t>
+        </is>
+      </c>
+      <c r="C870" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:50:13 +0700</t>
+        </is>
+      </c>
+      <c r="D870" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E870" t="inlineStr">
+        <is>
+          <t>Kepala BGN Sudaryono melakukan sejumlah perbaikan pelaksanaan program Makan Bergizi Gratis (MBG). Berikut daftarnya.</t>
+        </is>
+      </c>
+      <c r="F870" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G870" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260808141250-92-1390091/daftar-perbaikan-tata-kelola-mbg-di-bawah-komando-sudaryono</t>
+        </is>
+      </c>
+      <c r="H870" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/07/15/libur-telah-usai-mbg-kembali-dsalurkan-ke-sekolah-1784084515528_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I870" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B871" t="inlineStr">
+        <is>
+          <t>Perkuat Pengawasan MBG, Pejabat Eselon BGN Akan Berkantor di Daerah</t>
+        </is>
+      </c>
+      <c r="C871" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:42:30 +0700</t>
+        </is>
+      </c>
+      <c r="D871" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E871" t="inlineStr">
+        <is>
+          <t>Kepala Badan Gizi Nasional (BGN) Sudaryono akan mewajibkan pejabat eselon I hingga II di lembaganya untuk berkantor di daerah.</t>
+        </is>
+      </c>
+      <c r="F871" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G871" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260808115113-92-1390063/perkuat-pengawasan-mbg-pejabat-eselon-bgn-akan-berkantor-di-daerah</t>
+        </is>
+      </c>
+      <c r="H871" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/07/29/bgn-tutup-833-dapur-sppg-bermasalah-1785317578257_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I871" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B872" t="inlineStr">
+        <is>
+          <t>Niat Nabung Tinggi Tapi Kantong Tipis, Sinyal Daya Beli Lemah?</t>
+        </is>
+      </c>
+      <c r="C872" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 12:35:42 +0700</t>
+        </is>
+      </c>
+      <c r="D872" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E872" t="inlineStr">
+        <is>
+          <t>Ekonom mengingatkan soal risiko pelemahan daya beli di tengah tingginya minat menabung masyarakat yang tak dibarengi dengan kapasitas finansial.</t>
+        </is>
+      </c>
+      <c r="F872" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G872" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260808121353-78-1390076/niat-nabung-tinggi-tapi-kantong-tipis-sinyal-daya-beli-lemah</t>
+        </is>
+      </c>
+      <c r="H872" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2022/04/23/ilustrasi-dompet-berisi-uang-rupiah_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I872" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B873" t="inlineStr">
+        <is>
+          <t>Drone Jatuh Timpa Rumah Warga Sukoharjo Jateng, Plt Bupati Ikut Padamkan Api</t>
+        </is>
+      </c>
+      <c r="C873" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:13:30 +0700</t>
+        </is>
+      </c>
+      <c r="D873" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E873" t="inlineStr">
+        <is>
+          <t>Sapto dalam momen itu terlihat mengenakan baju putih dan menaiki tangga kayu yang disandarkan ke bagian atap rumah.</t>
+        </is>
+      </c>
+      <c r="F873" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G873" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865827/drone-jatuh-timpa-rumah-warga-sukoharjo-jatengplt-bupati-ikut-padamkan-api</t>
+        </is>
+      </c>
+      <c r="H873" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/qhC2SKjK-wHYSpZ-l6juG3pMRC8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Wakil-Bupati-terpilih-Sukoharjo-2024-Eko-Sapto-Purnomo.jpg</t>
+        </is>
+      </c>
+      <c r="I873" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B874" t="inlineStr">
+        <is>
+          <t>Chelsea Bungkam AC Milan 3-0 di SUGBK, The Blues Angkat Trofi Indonesia Super Cup 2026</t>
+        </is>
+      </c>
+      <c r="C874" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:08:12 +0700</t>
+        </is>
+      </c>
+      <c r="D874" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E874" t="inlineStr">
+        <is>
+          <t>Chelsea mengalahkan AC Milan dengan skor 3-0 pada ajang Indonesia Super Cup 2026 di Stadion Utama Gelora Bung Karno pada Sabtu (8/8/2026).</t>
+        </is>
+      </c>
+      <c r="F874" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G874" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865826/chelsea-bungkam-ac-milan-3-0-di-sugbk-the-blues-angkat-trofi-indonesia-super-cup-2026</t>
+        </is>
+      </c>
+      <c r="H874" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/RjKVan-JihQxMePaSto9HU0bRnE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Joao-Pedro-Chelsea-AC-Milan-GBK.jpg</t>
+        </is>
+      </c>
+      <c r="I874" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B875" t="inlineStr">
+        <is>
+          <t>Pembunuhan Marbot Masjid di Purwakarta, Pelaku Diduga Tersinggung Soal Ekonomi</t>
+        </is>
+      </c>
+      <c r="C875" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:58:36 +0700</t>
+        </is>
+      </c>
+      <c r="D875" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E875" t="inlineStr">
+        <is>
+          <t>Polisi menyita sebilah pedang, celurit, serta pakaian yang diduga digunakan pelaku saat melakukan aksi.</t>
+        </is>
+      </c>
+      <c r="F875" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G875" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865825/pembunuhan-marbot-masjid-di-purwakarta-pelaku-diduga-tersinggung-soal-ekonomi</t>
+        </is>
+      </c>
+      <c r="H875" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/iVQoFd00f4I54X3zKDiHAJJIyGM=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Marbot-Masjid-Tewas.jpg</t>
+        </is>
+      </c>
+      <c r="I875" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B876" t="inlineStr">
+        <is>
+          <t>Terjemahan Lirik With or Without You - U2: See The Stone Set In Your Eyes</t>
+        </is>
+      </c>
+      <c r="C876" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:48:43 +0700</t>
+        </is>
+      </c>
+      <c r="D876" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E876" t="inlineStr">
+        <is>
+          <t>Bono, sang vokalis, menulis lagu ini berdasarkan konflik kisah cinta dan kehidupan sebagai musisi.</t>
+        </is>
+      </c>
+      <c r="F876" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G876" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/musik/7865824/terjemahan-lirik-with-or-without-you-u2-see-the-stone-set-in-your-eyes</t>
+        </is>
+      </c>
+      <c r="H876" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/zLN77GXG_MWcQ27NDqNvGgp-QJs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-musik-ilustrasi-lirik-ilustrasi-terjemahan-lirik-lagu.jpg</t>
+        </is>
+      </c>
+      <c r="I876" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B877" t="inlineStr">
+        <is>
+          <t>Ditpolairud Polda Metro Ungkap Dugaan Penyelundupan 150 Kg Pasir Timah Asal Babel, Begini Modusnya</t>
+        </is>
+      </c>
+      <c r="C877" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:45:35 +0700</t>
+        </is>
+      </c>
+      <c r="D877" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E877" t="inlineStr">
+        <is>
+          <t>Satu karung ditemukan di bawah kursi pengemudi, sedangkan dua karung lainnya berada di bagian atas truk yang ditutupi terpal</t>
+        </is>
+      </c>
+      <c r="F877" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G877" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865823/ditpolairud-polda-metro-ungkap-dugaan-penyelundupan-150-kg-pasir-timah-asal-babel-begini-modusnya</t>
+        </is>
+      </c>
+      <c r="H877" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/gWFEBzmQSvObD1Pag6j0eWwbwJY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Petugas-Ditpolairud-Polda-Metro-Jaya-ekspedisi.jpg</t>
+        </is>
+      </c>
+      <c r="I877" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B878" t="inlineStr">
+        <is>
+          <t>Terjemahan Lirik Lagu Accidentally in Love - Counting Crows: Ost Film Shrek 2</t>
+        </is>
+      </c>
+      <c r="C878" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:42:42 +0700</t>
+        </is>
+      </c>
+      <c r="D878" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E878" t="inlineStr">
+        <is>
+          <t>Lagu ini kala itu langsung menjadi hit global karena nuansa romantis dan ringan serta berkaitan dengan film animasi yang saat itu populer.</t>
+        </is>
+      </c>
+      <c r="F878" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G878" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/musik/7865822/terjemahan-lirik-lagu-accidentally-in-love-counting-crows-ost-film-shrek-2</t>
+        </is>
+      </c>
+      <c r="H878" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/8ofGbaRMpqu_gFPWYkenF6qEE2Y=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Potret-ilustrasi-lirik-lagu-terjemahan-musik-mendengarkan-musik.jpg</t>
+        </is>
+      </c>
+      <c r="I878" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B879" t="inlineStr">
+        <is>
+          <t>Kabar Baik! Husein Sastranegara Kembali Layani Penerbangan</t>
+        </is>
+      </c>
+      <c r="C879" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:10:16 +0700</t>
+        </is>
+      </c>
+      <c r="D879" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E879" t="inlineStr">
+        <is>
+          <t>Bandara Husein Sastranegara Bandung siap melayani penerbangan jet berbadan sedang mulai 14 Agustus 2026.</t>
+        </is>
+      </c>
+      <c r="F879" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G879" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260808181710-7-757652/kabar-baik-husein-sastranegara-kembali-layani-penerbangan</t>
+        </is>
+      </c>
+      <c r="H879" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/08/pt-angkasa-pura-indonesia-persero-atau-injourney-airports-telah-mendapat-persetujuan-dari-kementerian-perhubungan-ri-kemenhub--1786187820102_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I879" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B880" t="inlineStr">
+        <is>
+          <t>Petaka Cuaca Kepung New York, Panas Sampai 38 Derajat Celsius</t>
+        </is>
+      </c>
+      <c r="C880" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:30:37 +0700</t>
+        </is>
+      </c>
+      <c r="D880" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E880" t="inlineStr">
+        <is>
+          <t>Panas ekstrem dan badai petir melanda New York hingga akhir pekan. Suhu terasa tembus 37,8 Celsius Derajat, sementara hujan deras berisiko memicu banjir.</t>
+        </is>
+      </c>
+      <c r="F880" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G880" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260808170927-7-757640/petaka-cuaca-kepung-new-york-panas-sampai-38-derajat-celsius</t>
+        </is>
+      </c>
+      <c r="H880" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/08/seorang-pejalan-kaki-menggunakan-kipas-tangan-saat-gelombang-panas-melanda-new-york-city-as-pada-7-agustus-2026-1786183761571_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I880" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B881" t="inlineStr">
+        <is>
+          <t>Bupati Bandung dan KPK Perkuat Sinergi Tata Kelola Pemerintahan Bersih</t>
+        </is>
+      </c>
+      <c r="C881" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:22:43 +0700</t>
+        </is>
+      </c>
+      <c r="D881" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E881" t="inlineStr">
+        <is>
+          <t>Bupati Dadang Supriatna menekankan pentingnya transparansi dan akuntabilitas dalam pelayanan publik.</t>
+        </is>
+      </c>
+      <c r="F881" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G881" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260808195852-4-757682/bupati-bandung-kpk-perkuat-sinergi-tata-kelola-pemerintahan-bersih</t>
+        </is>
+      </c>
+      <c r="H881" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/04/27/bupati-kabupaten-bandung-dadang-supriatna-dalam-acara-cnbc-indonesia-food-summit-2026-di-menara-bank-mega-jakarta-senin-274202-1777273449670_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I881" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B882" t="inlineStr">
+        <is>
+          <t>Foto Topan Dolphin Mengamuk, Jepang Diterjang Angin 198 Km per Jam</t>
+        </is>
+      </c>
+      <c r="C882" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:10:00 +0700</t>
+        </is>
+      </c>
+      <c r="D882" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E882" t="inlineStr">
+        <is>
+          <t>Topan Dolphin menerjang selatan Jepang dengan angin hingga 198 km/jam, memicu evakuasi 260.000 warga, pembatalan 500 penerbangan, dan penutupan pabrik.</t>
+        </is>
+      </c>
+      <c r="F882" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G882" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260808165223-7-757633/foto-topan-dolphin-mengamuk-jepang-diterjang-angin-198-km-per-jam</t>
+        </is>
+      </c>
+      <c r="H882" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/08/topan-dolphin-membawa-angin-kencang-hujan-deras-dan-gelombang-tinggi-ke-wilayah-selatan-jepang-pada-jumat-782026-1786182740417_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I882" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B883" t="inlineStr">
+        <is>
+          <t>Transmart Banting Harga Elektronik Besok, Jangan Lupa Merapat!</t>
+        </is>
+      </c>
+      <c r="C883" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:30:16 +0700</t>
+        </is>
+      </c>
+      <c r="D883" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E883" t="inlineStr">
+        <is>
+          <t>Transmart menggelar Full Day Sale dengan diskon hingga 50% + 20% untuk produk elektronik. Dapatkan harga murah untuk TV, kulkas, dan AC pada 9 Agustus 2026.</t>
+        </is>
+      </c>
+      <c r="F883" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G883" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260808110404-4-757597/transmart-banting-harga-elektronik-besok-jangan-lupa-merapat</t>
+        </is>
+      </c>
+      <c r="H883" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/01/18/booth-elektronik-di-transmart-kokas-minggu-181-cnbc-indonesiaelga-1768724093084_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I883" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B884" t="inlineStr">
+        <is>
+          <t>Video: Ekspansi Kendaraan Listrik di Tambang, Infrastruktur Jadi PR</t>
+        </is>
+      </c>
+      <c r="C884" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:00:44 +0700</t>
+        </is>
+      </c>
+      <c r="D884" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E884" t="inlineStr">
+        <is>
+          <t>Ekspansi Kendaraan Listrik di Tambang, Infrastruktur Charging - Bengkel Jadi Tantangan</t>
+        </is>
+      </c>
+      <c r="F884" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G884" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260805090318-8-756636/video-ekspansi-kendaraan-listrik-di-tambang-infrastruktur-jadi-pr</t>
+        </is>
+      </c>
+      <c r="H884" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/06/ekspansi-kendaraan-listrik-di-tambang-infrastruktur-charging-bengkel-jadi-tantangan-1785984234651_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I884" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B885" t="inlineStr">
+        <is>
+          <t>Diskon Gede-Gedean, Harga Sepeda Listrik di Transmart Cuma Segini!</t>
+        </is>
+      </c>
+      <c r="C885" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:30:34 +0700</t>
+        </is>
+      </c>
+      <c r="D885" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E885" t="inlineStr">
+        <is>
+          <t>Transmart menggelar Full Day Sale pada 9 Agustus 2026, menawarkan diskon besar untuk sepeda listrik dan produk lainnya. Jangan lewatkan!</t>
+        </is>
+      </c>
+      <c r="F885" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G885" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260808113209-4-757600/diskon-gede-gedean-harga-sepeda-listrik-di-transmart-cuma-segini</t>
+        </is>
+      </c>
+      <c r="H885" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2025/06/06/cek-transmart-moms-sepeda-listrik-banting-harga-1749195439237_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I885" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B886" t="inlineStr">
+        <is>
+          <t>Ada Diskon 50%+20%, Beli Kasur di Transmart Tidur Makin Nyenyak</t>
+        </is>
+      </c>
+      <c r="C886" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:30:43 +0700</t>
+        </is>
+      </c>
+      <c r="D886" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E886" t="inlineStr">
+        <is>
+          <t>Transmart menggelar Full Day Sale dengan diskon hingga 50% + 20% pada 9 Agustus 2026. Dapatkan kasur berkualitas dan berbagai produk lainnya.</t>
+        </is>
+      </c>
+      <c r="F886" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G886" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260808112244-4-757598/ada-diskon-50-20-beli-kasur-di-transmart-tidur-makin-nyenyak</t>
+        </is>
+      </c>
+      <c r="H886" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2025/03/23/diskon-transmart-fullday-sale-kembali-lagi-dengan-berbagai-macam-tawaran-diskon-hingga-5020-melalui-program-transmart-full-day-1742720587517_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I886" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B887" t="inlineStr">
+        <is>
+          <t>Tanda Kiamat Muncul dari Sikat Gigi</t>
+        </is>
+      </c>
+      <c r="C887" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:00:25 +0700</t>
+        </is>
+      </c>
+      <c r="D887" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E887" t="inlineStr">
+        <is>
+          <t>Sikat gigi, barang sepele, ternyata berkontribusi pada perubahan iklim. Penggunaan plastik dalam sikat gigi modern jadi masalah lingkungan serius.</t>
+        </is>
+      </c>
+      <c r="F887" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G887" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260808153825-37-757629/tanda-kiamat-muncul-dari-sikat-gigi</t>
+        </is>
+      </c>
+      <c r="H887" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2023/03/24/ilustrasi-sikat-gigi_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I887" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B888" t="inlineStr">
+        <is>
+          <t>Seberapa Panas Bumi di Masa Depan? Ini Prediksi Ilmuwan</t>
+        </is>
+      </c>
+      <c r="C888" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:40:01 +0700</t>
+        </is>
+      </c>
+      <c r="D888" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E888" t="inlineStr">
+        <is>
+          <t>Suhu bumi diperkirakan terus meningkat akibat pemanasan global. Rekor suhu ekstrem 2023 menunjukkan dampak nyata perubahan iklim yang harus diatasi.</t>
+        </is>
+      </c>
+      <c r="F888" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G888" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260808161201-37-757630/seberapa-panas-bumi-di-masa-depan-ini-prediksi-ilmuwan</t>
+        </is>
+      </c>
+      <c r="H888" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/07/16/sebuah-patung-es-yang-menggambarkan-kurir-sepeda-salah-satu-kelompok-pekerja-yang-paling-rentan-terhadap-gelombang-panas-yang--1784170974162_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I888" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B889" t="inlineStr">
+        <is>
+          <t>AS Mulai Gelisah, RI Sudah Duluan Bikin Aturan</t>
+        </is>
+      </c>
+      <c r="C889" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:00:32 +0700</t>
+        </is>
+      </c>
+      <c r="D889" t="inlineStr">
+        <is>
+          <t>Redaksi</t>
+        </is>
+      </c>
+      <c r="E889" t="inlineStr">
+        <is>
+          <t>Dukungan larangan penggunaan HP di sekolah meningkat di AS, dengan 77% warga setuju. Indonesia telah lebih dulu menerapkan pembatasan gawai untuk belajar.</t>
+        </is>
+      </c>
+      <c r="F889" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G889" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260808153032-37-757627/as-mulai-gelisah-ri-sudah-duluan-bikin-aturan</t>
+        </is>
+      </c>
+      <c r="H889" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/07/09/ilustrasi-bermain-hp-1783573433198_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I889" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" t="inlineStr">
+        <is>
+          <t>Finansial</t>
+        </is>
+      </c>
+      <c r="B890" t="inlineStr">
+        <is>
+          <t>Telkom Rampungkan Spin-Off InfraCo Tahap 2, InfraNexia Jadi Pilar Bisnis Wholesale Connectivity</t>
+        </is>
+      </c>
+      <c r="C890" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:06:53 +0700</t>
+        </is>
+      </c>
+      <c r="D890" t="inlineStr">
+        <is>
+          <t>Dwi Murdaningsih</t>
+        </is>
+      </c>
+      <c r="E890" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA - Pasca penyelesaian Spin-Off InfraCo Tahap 1 yang efektif berlaku sejak Januari 2026, PT Telkom Infrastruktur Indonesia (InfraNexia) memperkuat posisinya sebagai penyedia infrastruktur digital wholesale yang netral, andal,...</t>
+        </is>
+      </c>
+      <c r="F890" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G890" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjgf7h368/telkom-rampungkan-spinoff-infraco-tahap-2-infranexia-jadi-pilar-bisnis-wholesale-connectivity</t>
+        </is>
+      </c>
+      <c r="H890" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/infranexia-terus-mencatatkan-pertumbuhan-bisnis-yang-positif-memperluas-kolaborasi_260808210240-908.jpeg</t>
+        </is>
+      </c>
+      <c r="I890" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B891" t="inlineStr">
+        <is>
+          <t>Mimpi Anak Petani, Ismi Ulfaida Jadi Paskibraka Pertama dari Sekolah Rakyat</t>
+        </is>
+      </c>
+      <c r="C891" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:09:26 +0700</t>
+        </is>
+      </c>
+      <c r="D891" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E891" t="inlineStr">
+        <is>
+          <t>Sejak SMP, Ismi punya mimpi bergabung dalam Paskibraka.</t>
+        </is>
+      </c>
+      <c r="F891" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G891" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265281/mimpi-anak-petani-ismi-ulfaida-jadi-paskibraka-pertama-dari-sekolah-rakyat</t>
+        </is>
+      </c>
+      <c r="H891" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/Org3rO1VQTK8cpLTcGih0_gXhUw=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9319208/original/038562100_1786198164-1000035126.jpg</t>
+        </is>
+      </c>
+      <c r="I891" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B892" t="inlineStr">
+        <is>
+          <t>Motif Penyiksaan dan Penyekapan Karyawan Koperasi di Tangerang</t>
+        </is>
+      </c>
+      <c r="C892" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:39:25 +0700</t>
+        </is>
+      </c>
+      <c r="D892" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E892" t="inlineStr">
+        <is>
+          <t>Polda Banten menangkap 5 pelaku, kasus penyekapan karyawan koperasi diduga didalangi bos.</t>
+        </is>
+      </c>
+      <c r="F892" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G892" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265227/motif-penyiksaan-dan-penyekapan-karyawan-koperasi-di-tangerang</t>
+        </is>
+      </c>
+      <c r="H892" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/GVPAADbx9t42VHgDnHBhKMRq_aQ=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9314668/original/011114800_1785758460-WhatsApp_Image_2026-08-03_at_18.52.07.jpeg</t>
+        </is>
+      </c>
+      <c r="I892" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B893" t="inlineStr">
+        <is>
+          <t>Truk Polisi Bawa Siswa SMA 79 Kecelakaan di Cawang, Sopir Diduga Mengantuk</t>
+        </is>
+      </c>
+      <c r="C893" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:26:00 +0700</t>
+        </is>
+      </c>
+      <c r="D893" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E893" t="inlineStr">
+        <is>
+          <t>Dua truk kepolisian yang membawa siswa dan guru SMA Negeri 79 kecelakaan di Cawang. Sopir truk depan diduga mengantuk.</t>
+        </is>
+      </c>
+      <c r="F893" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G893" t="inlineStr">
+        <is>
+          <t>https://megapolitan.kompas.com/read/2026/08/08/21222541/truk-polisi-bawa-siswa-sma-79-kecelakaan-di-cawang-sopir-diduga-mengantuk</t>
+        </is>
+      </c>
+      <c r="H893" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/ppB9jeT7U_sEMM9RXUrUTzuxtYM=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/08/6a773473ce84b.jpeg</t>
+        </is>
+      </c>
+      <c r="I893" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B894" t="inlineStr">
+        <is>
+          <t>Soal 995 Senjata di Sekolah, Menteri PPPA Ingatkan Dampak Psikologis pada Anak</t>
+        </is>
+      </c>
+      <c r="C894" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:26:00 +0700</t>
+        </is>
+      </c>
+      <c r="D894" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E894" t="inlineStr">
+        <is>
+          <t>Menteri PPPA Arifah Fauzi menyoroti temuan 995 senjata di sekolah swasta Jakarta Selatan. Ia mendesak pihak sekolah menjamin keamanan dan psikologis anak.</t>
+        </is>
+      </c>
+      <c r="F894" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G894" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/08/08/20240371/soal-995-senjata-di-sekolah-menteri-pppa-ingatkan-dampak-psikologis-pada</t>
+        </is>
+      </c>
+      <c r="H894" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/Oef8EvPI2mVevWJdhzRZS3433Lc=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/07/22/6a60389ab0b20.jpeg</t>
+        </is>
+      </c>
+      <c r="I894" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" t="inlineStr">
+        <is>
+          <t>Bola</t>
+        </is>
+      </c>
+      <c r="B895" t="inlineStr">
+        <is>
+          <t>Live Chelsea Vs AC Milan 1-0: Joao Pedro Bawa The Blues Unggul</t>
+        </is>
+      </c>
+      <c r="C895" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:26:00 +0700</t>
+        </is>
+      </c>
+      <c r="D895" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E895" t="inlineStr">
+        <is>
+          <t>Laga pramusim Chelsea vs AC Milan digelar di Stadion Utama Gelora Bung Karno, Jakarta pada hari Sabtu (8/8/2026) malam WIB.</t>
+        </is>
+      </c>
+      <c r="F895" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G895" t="inlineStr">
+        <is>
+          <t>https://bola.kompas.com/read/2026/08/08/19534828/live-chelsea-vs-ac-milan-1-0-joao-pedro-bawa-the-blues-unggul</t>
+        </is>
+      </c>
+      <c r="H895" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/Pc5UlBR-n495yTuiC-KI1-PxP3E=/413x0:3791x2252/1200x675/filters:watermark(data/photo/2026/01/30/697c8163c3944.png,0,-0,1)/data/photo/2026/08/08/6a771fe7b1f4b.jpg</t>
+        </is>
+      </c>
+      <c r="I895" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I837"/>
+  <autoFilter ref="A1:I895"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-08 15:23 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-08.xlsx
+++ b/data/berita_2026-08-08.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$895</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$944</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I895"/>
+  <dimension ref="A1:I944"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -42502,8 +42502,2312 @@
         </is>
       </c>
     </row>
+    <row r="896">
+      <c r="A896" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B896" t="inlineStr">
+        <is>
+          <t>Zelensky klaim AS janji pasok rudal ke Ukraina setiap bulan</t>
+        </is>
+      </c>
+      <c r="C896" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:15:45 +0700</t>
+        </is>
+      </c>
+      <c r="D896" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E896" t="inlineStr">
+        <is>
+          <t>Presiden Vladimir Zelensky pada Sabtu mengeklaim bahwa Ukraina telah membuat kesepakatan dengan Amerika ...</t>
+        </is>
+      </c>
+      <c r="F896" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G896" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686045/zelensky-klaim-as-janji-pasok-rudal-ke-ukraina-setiap-bulan</t>
+        </is>
+      </c>
+      <c r="H896" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/02/AA-20260801-42116676-42116666-9_KILLED_27_INJURED_IN_RUSSIAN_MISSILE_ATTACKS_ON_KYIV.jpg</t>
+        </is>
+      </c>
+      <c r="I896" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B897" t="inlineStr">
+        <is>
+          <t>Seskab: Mutu Sekolah Rakyat tak kalah dari sekolah lain</t>
+        </is>
+      </c>
+      <c r="C897" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:14:01 +0700</t>
+        </is>
+      </c>
+      <c r="D897" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E897" t="inlineStr">
+        <is>
+          <t>Sekretaris Kabinet (Seskab) Teddy Indra Wijaya menegaskan bahwa Sekolah Rakyat tidak kalah dari sekolah lainnya dalam ...</t>
+        </is>
+      </c>
+      <c r="F897" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G897" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686041/seskab-mutu-sekolah-rakyat-tak-kalah-dari-sekolah-lain</t>
+        </is>
+      </c>
+      <c r="H897" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG_1004.jpeg</t>
+        </is>
+      </c>
+      <c r="I897" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B898" t="inlineStr">
+        <is>
+          <t>Pertamina Patra Niaga Kalimantan raih 10 Penghargaan ISRA 2026</t>
+        </is>
+      </c>
+      <c r="C898" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:12:23 +0700</t>
+        </is>
+      </c>
+      <c r="D898" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E898" t="inlineStr">
+        <is>
+          <t>PT Pertamina Patra Niaga Regional Kalimantan meraih 10 penghargaan Indonesia Social Responsibility Award (ISRA) 2026 ...</t>
+        </is>
+      </c>
+      <c r="F898" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G898" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686035/pertamina-patra-niaga-kalimantan-raih-10-penghargaan-isra-2026</t>
+        </is>
+      </c>
+      <c r="H898" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG_20260808_213954.jpg</t>
+        </is>
+      </c>
+      <c r="I898" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B899" t="inlineStr">
+        <is>
+          <t>Kapendam: Penembakan di FBLB  kelompok KKB Kodap III Ndugama</t>
+        </is>
+      </c>
+      <c r="C899" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:09:25 +0700</t>
+        </is>
+      </c>
+      <c r="D899" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E899" t="inlineStr">
+        <is>
+          <t>2026 adalah kelompok KKB dari Kodap III Ndugama.
+Memang dari hasil penyelidikan terungkap pelaku penembakan ...</t>
+        </is>
+      </c>
+      <c r="F899" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G899" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686031/kapendam-penembakan-di-fblb-kelompok-kkb-kodap-iii-ndugama</t>
+        </is>
+      </c>
+      <c r="H899" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1002607642.jpg</t>
+        </is>
+      </c>
+      <c r="I899" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B900" t="inlineStr">
+        <is>
+          <t>Gubernur Sumut minta kepala daerah se-Nias percepat usulan BKP 2027</t>
+        </is>
+      </c>
+      <c r="C900" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:08:04 +0700</t>
+        </is>
+      </c>
+      <c r="D900" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E900" t="inlineStr">
+        <is>
+          <t>Gubernur Sumatera Utara (Sumut) Bobby Nasution meminta kepala daerah se-Kepulauan Nias segera mengusulkan Bantuan ...</t>
+        </is>
+      </c>
+      <c r="F900" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G900" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686029/gubernur-sumut-minta-kepala-daerah-se-nias-percepat-usulan-bkp-2027</t>
+        </is>
+      </c>
+      <c r="H900" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001036900.jpg</t>
+        </is>
+      </c>
+      <c r="I900" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B901" t="inlineStr">
+        <is>
+          <t>Piala Interkontinental FIBA 2026 adu enam tim di China</t>
+        </is>
+      </c>
+      <c r="C901" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:04:44 +0700</t>
+        </is>
+      </c>
+      <c r="D901" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E901" t="inlineStr">
+        <is>
+          <t>Piala Interkontinental Federasi Bola Basket Internasional (FIBA) 2026 akan mengadu enam tim dari lima benua yang ...</t>
+        </is>
+      </c>
+      <c r="F901" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G901" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686027/piala-interkontinental-fiba-2026-adu-enam-tim-di-china</t>
+        </is>
+      </c>
+      <c r="H901" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000476811.jpg</t>
+        </is>
+      </c>
+      <c r="I901" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B902" t="inlineStr">
+        <is>
+          <t>DJP Jatim dan GP Ansor perkuat edukasi perpajakan</t>
+        </is>
+      </c>
+      <c r="C902" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:04:34 +0700</t>
+        </is>
+      </c>
+      <c r="D902" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E902" t="inlineStr">
+        <is>
+          <t>Direktorat Jenderal Pajak (DJP) Jawa Timur dan Pimpinan Wilayah (PW) Gerakan Pemuda (GP) Ansor Jawa Timur ...</t>
+        </is>
+      </c>
+      <c r="F902" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G902" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686025/djp-jatim-dan-gp-ansor-perkuat-edukasi-perpajakan</t>
+        </is>
+      </c>
+      <c r="H902" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/ANTARA-2026-08-07T182849.643.jpg.jpeg</t>
+        </is>
+      </c>
+      <c r="I902" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B903" t="inlineStr">
+        <is>
+          <t>Sekum Perhumas: Humas harus bertransformasi jadi pengambil keputusan</t>
+        </is>
+      </c>
+      <c r="C903" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:04:06 +0700</t>
+        </is>
+      </c>
+      <c r="D903" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E903" t="inlineStr">
+        <is>
+          <t>Sekretaris Umum (Sekum) Persatuan Hubungan Masyarakat (Perhumas) Indonesia Benny Siga Butar Butar menyebut Humas harus ...</t>
+        </is>
+      </c>
+      <c r="F903" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G903" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686023/sekum-perhumas-humas-harus-bertransformasi-jadi-pengambil-keputusan</t>
+        </is>
+      </c>
+      <c r="H903" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1002920195.jpg</t>
+        </is>
+      </c>
+      <c r="I903" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B904" t="inlineStr">
+        <is>
+          <t>Jalan Abdul Muis dibuka pascakebakaran Gedung Bapenda DKI</t>
+        </is>
+      </c>
+      <c r="C904" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:01:32 +0700</t>
+        </is>
+      </c>
+      <c r="D904" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E904" t="inlineStr">
+        <is>
+          <t>ANTARA - Jalan Abdul Muis yang sempat ditutup imbas kebakaran Gedung Badan Pendapatan Daerah (Bapenda) DKI Jakarta kini ...</t>
+        </is>
+      </c>
+      <c r="F904" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G904" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686004/jalan-abdul-muis-dibuka-pascakebakaran-gedung-bapenda-dki</t>
+        </is>
+      </c>
+      <c r="H904" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/JALAN-ABDUL-MUIS-DIBUKA-PASCAKEBAKARAN-GEDUNG-BAPENDA-DKI.jpg</t>
+        </is>
+      </c>
+      <c r="I904" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B905" t="inlineStr">
+        <is>
+          <t>Rasio desa berlistrik di Gorontalo Utara capai 100 persen</t>
+        </is>
+      </c>
+      <c r="C905" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:00:16 +0700</t>
+        </is>
+      </c>
+      <c r="D905" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E905" t="inlineStr">
+        <is>
+          <t>Rasio desa berlistrik di Kabupaten Gorontalo Utara, Provinsi Gorontalo, telah mencapai 100 persen dari total jumlah ...</t>
+        </is>
+      </c>
+      <c r="F905" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G905" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686019/rasio-desa-berlistrik-di-gorontalo-utara-capai-100-persen</t>
+        </is>
+      </c>
+      <c r="H905" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/784422.jpg</t>
+        </is>
+      </c>
+      <c r="I905" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B906" t="inlineStr">
+        <is>
+          <t>Pemerintah dorong akses pasar lebih luas untuk gim buatan Indonesia</t>
+        </is>
+      </c>
+      <c r="C906" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:59:14 +0700</t>
+        </is>
+      </c>
+      <c r="D906" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E906" t="inlineStr">
+        <is>
+          <t>ANTARA - Menteri Ekonomi Kreatif Teuku Riefky Harsya mengatakan pemerintah berkomitmen memberikan akses pasar lebih ...</t>
+        </is>
+      </c>
+      <c r="F906" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G906" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5685981/pemerintah-dorong-akses-pasar-lebih-luas-untuk-gim-buatan-indonesia</t>
+        </is>
+      </c>
+      <c r="H906" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/PEMERINTAH-DORONG-AKSES-PASAR-LEBIH-LUAS-UNTUK-GIM-BUATAN-INDONESIA.jpg</t>
+        </is>
+      </c>
+      <c r="I906" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B907" t="inlineStr">
+        <is>
+          <t>DPP Perbasi imbau seluruh DPD manfaatkan basis data untuk pembinaan</t>
+        </is>
+      </c>
+      <c r="C907" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:57:32 +0700</t>
+        </is>
+      </c>
+      <c r="D907" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E907" t="inlineStr">
+        <is>
+          <t>Ketua Bidang Database Dewan Pengurus Pusat Persatuan Bola Basket Seluruh Indonesia (DPP Perbasi) Jamin Mattotoran ...</t>
+        </is>
+      </c>
+      <c r="F907" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G907" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686017/dpp-perbasi-imbau-seluruh-dpd-manfaatkan-basis-data-untuk-pembinaan</t>
+        </is>
+      </c>
+      <c r="H907" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000476776.jpg</t>
+        </is>
+      </c>
+      <c r="I907" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B908" t="inlineStr">
+        <is>
+          <t>Kalsel gelar lomba masak serba ikan untuk pencegahan stunting</t>
+        </is>
+      </c>
+      <c r="C908" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:57:27 +0700</t>
+        </is>
+      </c>
+      <c r="D908" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E908" t="inlineStr">
+        <is>
+          <t>ANTARA - Dinas Kelautan dan Perikanan Provinsi Kalimantan Selatan bersama Tim Penggerak PKK setempat, menggelar lomba ...</t>
+        </is>
+      </c>
+      <c r="F908" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G908" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5685975/kalsel-gelar-lomba-masak-serba-ikan-untuk-pencegahan-stunting</t>
+        </is>
+      </c>
+      <c r="H908" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/KALSEL-GELAR-LOMBA-MASAK-SERBA-IKAN-UNTUK-PENCEGAHAN-STUNTING.jpg</t>
+        </is>
+      </c>
+      <c r="I908" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B909" t="inlineStr">
+        <is>
+          <t>Hanura siap ganti pengurus daerah yang lambat jalankan instruksi</t>
+        </is>
+      </c>
+      <c r="C909" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:56:25 +0700</t>
+        </is>
+      </c>
+      <c r="D909" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E909" t="inlineStr">
+        <is>
+          <t>Ketua Tim Task Force DPP Partai Hanura Rio Capella mengatakan pihaknya siap mengganti pengurus daerah yang lambat ...</t>
+        </is>
+      </c>
+      <c r="F909" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G909" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686016/hanura-siap-ganti-pengurus-daerah-yang-lambat-jalankan-instruksi</t>
+        </is>
+      </c>
+      <c r="H909" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000582623.jpg</t>
+        </is>
+      </c>
+      <c r="I909" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B910" t="inlineStr">
+        <is>
+          <t>Disbud Bantul: Serapan Danais lampaui 60 persen</t>
+        </is>
+      </c>
+      <c r="C910" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:56:02 +0700</t>
+        </is>
+      </c>
+      <c r="D910" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E910" t="inlineStr">
+        <is>
+          <t>Dinas Kebudayaan (Disbud) Kabupaten Bantul, Daerah Istimewa Yogyakarta (DIY), menyebut serapan Dana Keistimewaan ...</t>
+        </is>
+      </c>
+      <c r="F910" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G910" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686015/disbud-bantul-serapan-danais-lampaui-60-persen</t>
+        </is>
+      </c>
+      <c r="H910" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/2ac020c4-a5b8-46f9-85f1-a7f4c2d4fcc4-1_all_1112.jpg</t>
+        </is>
+      </c>
+      <c r="I910" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B911" t="inlineStr">
+        <is>
+          <t>Rekonstruksi daerah aliran sungai Krueng Meureubo Aceh Barat selesai</t>
+        </is>
+      </c>
+      <c r="C911" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:54:24 +0700</t>
+        </is>
+      </c>
+      <c r="D911" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E911" t="inlineStr">
+        <is>
+          <t>ANTARA - Rekonstruksi Daerah Aliran Sungai (DAS) Krueng Meureubo, Kecamatan Pante Ceureumen, Aceh Barat, Aceh, dalam ...</t>
+        </is>
+      </c>
+      <c r="F911" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G911" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5685963/rekonstruksi-daerah-aliran-sungai-krueng-meureubo-aceh-barat-selesai</t>
+        </is>
+      </c>
+      <c r="H911" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/REKONSTRUKSI-DAERAH-ALIRAN-SUNGAI-KRUENG-MEUREUBO-ACEH-BARAT-SELESAI.jpg</t>
+        </is>
+      </c>
+      <c r="I911" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B912" t="inlineStr">
+        <is>
+          <t>Tim gabungan padamkan karhutla 12,5 ha di dua lokasi di Bengkalis Riau</t>
+        </is>
+      </c>
+      <c r="C912" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:52:47 +0700</t>
+        </is>
+      </c>
+      <c r="D912" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E912" t="inlineStr">
+        <is>
+          <t>Tim Gabungan Kepolisian Resor Bengkalis Provinsi Riau bersama TNI, Badan Penanggulangan Bencana Daerah, Manggala Agni, ...</t>
+        </is>
+      </c>
+      <c r="F912" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G912" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686013/tim-gabungan-padamkan-karhutla-125-ha-di-dua-lokasi-di-bengkalis-riau</t>
+        </is>
+      </c>
+      <c r="H912" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000701281.jpg</t>
+        </is>
+      </c>
+      <c r="I912" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B913" t="inlineStr">
+        <is>
+          <t>Warga sulap jalan desa jadi gemerlap jelang HUT Ke-81 RI</t>
+        </is>
+      </c>
+      <c r="C913" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:51:12 +0700</t>
+        </is>
+      </c>
+      <c r="D913" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E913" t="inlineStr">
+        <is>
+          <t>Foto udara ornamen lampu hias berbentuk lambang Garuda di Desa Kandang, Kecamatan Comal, Kabupaten Pemalang, Jawa ...</t>
+        </is>
+      </c>
+      <c r="F913" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G913" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5686012/warga-sulap-jalan-desa-jadi-gemerlap-jelang-hut-ke-81-ri</t>
+        </is>
+      </c>
+      <c r="H913" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/Ornamen-lampu-hias-tematik-sambut-HUT-RI-080826-hpp-1A.jpg</t>
+        </is>
+      </c>
+      <c r="I913" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B914" t="inlineStr">
+        <is>
+          <t>Menteri PPN: i-Sentra @Lamongan perkuat hilirisasi industri</t>
+        </is>
+      </c>
+      <c r="C914" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:49:26 +0700</t>
+        </is>
+      </c>
+      <c r="D914" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E914" t="inlineStr">
+        <is>
+          <t>Menteri Perencanaan Pembangunan Nasional/ Kepala Bappenas Rachmat Pambudy menyatakan i-Sentra @Lamongan yang merupakan ...</t>
+        </is>
+      </c>
+      <c r="F914" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G914" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686008/menteri-ppn-i-sentra-lamongan-perkuat-hilirisasi-industri</t>
+        </is>
+      </c>
+      <c r="H914" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/5a22a984-324c-4e05-903b-32bae3e30f63.jpeg</t>
+        </is>
+      </c>
+      <c r="I914" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B915" t="inlineStr">
+        <is>
+          <t>Ayah Lionel Messi, Jorge Messi meninggal dunia pada usia 68 tahun</t>
+        </is>
+      </c>
+      <c r="C915" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:47:18 +0700</t>
+        </is>
+      </c>
+      <c r="D915" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E915" t="inlineStr">
+        <is>
+          <t>Ayah megabintang sepak bola Lionel Messi, Jorge Messi meninggal dunia pada Jumat (7/8) malam waktu setempat atau Sabtu ...</t>
+        </is>
+      </c>
+      <c r="F915" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G915" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686001/ayah-lionel-messi-jorge-messi-meninggal-dunia-pada-usia-68-tahun</t>
+        </is>
+      </c>
+      <c r="H915" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000043186.jpg</t>
+        </is>
+      </c>
+      <c r="I915" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B916" t="inlineStr">
+        <is>
+          <t>Chelsea menang telak 3-0 atas AC Milan di GBK</t>
+        </is>
+      </c>
+      <c r="C916" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:45:42 +0700</t>
+        </is>
+      </c>
+      <c r="D916" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E916" t="inlineStr">
+        <is>
+          <t>Pesepak bola AC Milan Rafael Leao (kiri) berusaha menghindari tekel pesepak bola Chelsea Josh Acheampong (kanan) dalam ...</t>
+        </is>
+      </c>
+      <c r="F916" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G916" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5685997/chelsea-menang-telak-3-0-atas-ac-milan-di-gbk</t>
+        </is>
+      </c>
+      <c r="H916" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/Chelsea-melawan-AC-Milan-080826-03A.jpg</t>
+        </is>
+      </c>
+      <c r="I916" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B917" t="inlineStr">
+        <is>
+          <t>Dewa United Horus pinjamkan Ikal ke EVOS Divine</t>
+        </is>
+      </c>
+      <c r="C917" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:44:07 +0700</t>
+        </is>
+      </c>
+      <c r="D917" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E917" t="inlineStr">
+        <is>
+          <t>Dewa United Horus resmi meminjamkan pemainnya, Muhammad "Ikal" Haikal, kepada EVOS Divine hingga akhir musim ...</t>
+        </is>
+      </c>
+      <c r="F917" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G917" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685995/dewa-united-horus-pinjamkan-ikal-ke-evos-divine</t>
+        </is>
+      </c>
+      <c r="H917" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/27/du_image_20260426221814338651_du_image_LKMN6221-1.jpg</t>
+        </is>
+      </c>
+      <c r="I917" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B918" t="inlineStr">
+        <is>
+          <t>BPS: Sensus Ekonomi 2026 perbarui data struktur perekonomian nasional</t>
+        </is>
+      </c>
+      <c r="C918" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:43:41 +0700</t>
+        </is>
+      </c>
+      <c r="D918" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E918" t="inlineStr">
+        <is>
+          <t>Badan Pusat Statistik (BPS) menyatakan Sensus Ekonomi 2026 menjadi bagian dari upaya pemerintah memperbarui data ...</t>
+        </is>
+      </c>
+      <c r="F918" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G918" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685993/bps-sensus-ekonomi-2026-perbarui-data-struktur-perekonomian-nasional</t>
+        </is>
+      </c>
+      <c r="H918" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000502077.jpg</t>
+        </is>
+      </c>
+      <c r="I918" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B919" t="inlineStr">
+        <is>
+          <t>Kesbangpol Bangka Selatan bagikan bendera ke sekolah</t>
+        </is>
+      </c>
+      <c r="C919" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:42:54 +0700</t>
+        </is>
+      </c>
+      <c r="D919" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E919" t="inlineStr">
+        <is>
+          <t>Badan Kesatuan Bangsa dan Politik (Kesbangpol) Kabupaten Bangka Selatan, Kepulauan Bangka Belitung, membagikan ribuan ...</t>
+        </is>
+      </c>
+      <c r="F919" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G919" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685992/kesbangpol-bangka-selatan-bagikan-bendera-ke-sekolah</t>
+        </is>
+      </c>
+      <c r="H919" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001631308.jpg</t>
+        </is>
+      </c>
+      <c r="I919" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B920" t="inlineStr">
+        <is>
+          <t>Pramusim: Inter Milan tekuk Juventus 2-1 di Australia</t>
+        </is>
+      </c>
+      <c r="C920" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:36:05 +0700</t>
+        </is>
+      </c>
+      <c r="D920" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E920" t="inlineStr">
+        <is>
+          <t>Inter Milan menekuk Juventus dengan skor 2-1 dalam laga pramusim yang digelar di Perth Stadium, Australia, pada Sabtu ...</t>
+        </is>
+      </c>
+      <c r="F920" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G920" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685987/pramusim-inter-milan-tekuk-juventus-2-1-di-australia</t>
+        </is>
+      </c>
+      <c r="H920" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000043183.jpg</t>
+        </is>
+      </c>
+      <c r="I920" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B921" t="inlineStr">
+        <is>
+          <t>Akademisi tekankan pentingnya pengembangan kasus eks Jampidsus</t>
+        </is>
+      </c>
+      <c r="C921" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:34:53 +0700</t>
+        </is>
+      </c>
+      <c r="D921" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E921" t="inlineStr">
+        <is>
+          <t>Dosen Fakultas Hukum Bisnis Universitas Bina Nusantara, Muhammad Reza Syarifuddin Zaki, menekankan pentingnya ...</t>
+        </is>
+      </c>
+      <c r="F921" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G921" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685985/akademisi-tekankan-pentingnya-pengembangan-kasus-eks-jampidsus</t>
+        </is>
+      </c>
+      <c r="H921" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000582589.jpg</t>
+        </is>
+      </c>
+      <c r="I921" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B922" t="inlineStr">
+        <is>
+          <t>Veda Ega Pratama start ke-16 pada Moto3 Inggris 2026</t>
+        </is>
+      </c>
+      <c r="C922" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:32:11 +0700</t>
+        </is>
+      </c>
+      <c r="D922" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E922" t="inlineStr">
+        <is>
+          <t>Pembalap Indonesia Veda Ega Pratama akan memulai balapan Moto3 Grand Prix Inggris 2026 dari posisi ke-16 setelah ...</t>
+        </is>
+      </c>
+      <c r="F922" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G922" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685979/veda-ega-pratama-start-ke-16-pada-moto3-inggris-2026</t>
+        </is>
+      </c>
+      <c r="H922" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/20/Pratama-wp_large.jpg</t>
+        </is>
+      </c>
+      <c r="I922" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B923" t="inlineStr">
+        <is>
+          <t>Seskab Teddy motivasi siswa Sekolah Rakyat berani bermimpi besar</t>
+        </is>
+      </c>
+      <c r="C923" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:30:08 +0700</t>
+        </is>
+      </c>
+      <c r="D923" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E923" t="inlineStr">
+        <is>
+          <t>Sekretaris Kabinet Teddy Indra Wijaya memotivasi siswa dan calon siswa Sekolah Rakyat untuk berani bermimpi dan ...</t>
+        </is>
+      </c>
+      <c r="F923" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G923" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685973/seskab-teddy-motivasi-siswa-sekolah-rakyat-berani-bermimpi-besar</t>
+        </is>
+      </c>
+      <c r="H923" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000035131.jpg</t>
+        </is>
+      </c>
+      <c r="I923" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B924" t="inlineStr">
+        <is>
+          <t>Kemenekraf: Pendampingan akselerasi jaga industri gim berkelanjutan</t>
+        </is>
+      </c>
+      <c r="C924" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:28:43 +0700</t>
+        </is>
+      </c>
+      <c r="D924" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E924" t="inlineStr">
+        <is>
+          <t>Kementerian Ekonomi Kreatif (Kemenekraf) mengungkap pendampingan dalam bentuk program akselerasi penting bagi pelaku ...</t>
+        </is>
+      </c>
+      <c r="F924" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G924" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685972/kemenekraf-pendampingan-akselerasi-jaga-industri-gim-berkelanjutan</t>
+        </is>
+      </c>
+      <c r="H924" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/20260808_152205.jpg</t>
+        </is>
+      </c>
+      <c r="I924" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B925" t="inlineStr">
+        <is>
+          <t>LPS: Jumlah rekening simpanan Jatim raih top tiga nasional</t>
+        </is>
+      </c>
+      <c r="C925" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:27:24 +0700</t>
+        </is>
+      </c>
+      <c r="D925" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E925" t="inlineStr">
+        <is>
+          <t>Lembaga Penjamin Simpanan (LPS) mencatat Jawa Timur menempati posisi top tiga untuk jumlah rekening terbanyak secara ...</t>
+        </is>
+      </c>
+      <c r="F925" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G925" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685971/lps-jumlah-rekening-simpanan-jatim-raih-top-tiga-nasional</t>
+        </is>
+      </c>
+      <c r="H925" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/WhatsApp-Image-2026-08-08-at-20.51.49.jpeg</t>
+        </is>
+      </c>
+      <c r="I925" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B926" t="inlineStr">
+        <is>
+          <t>BI Jatim dan TNI AL perkuat kedaulatan rupiah di kepulauan lewat ERB</t>
+        </is>
+      </c>
+      <c r="C926" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:25:55 +0700</t>
+        </is>
+      </c>
+      <c r="D926" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E926" t="inlineStr">
+        <is>
+          <t>Kantor Perwakilan Bank Indonesia Provinsi Jawa Timur bersama Pemerintah Provinsi Jawa Timur dan Tentara Nasional ...</t>
+        </is>
+      </c>
+      <c r="F926" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G926" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685969/bi-jatim-dan-tni-al-perkuat-kedaulatan-rupiah-di-kepulauan-lewat-erb</t>
+        </is>
+      </c>
+      <c r="H926" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG_6691-1.jpg.jpeg</t>
+        </is>
+      </c>
+      <c r="I926" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B927" t="inlineStr">
+        <is>
+          <t>Wigi Pratama kembali perkuat Deltras FC</t>
+        </is>
+      </c>
+      <c r="C927" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:25:20 +0700</t>
+        </is>
+      </c>
+      <c r="D927" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E927" t="inlineStr">
+        <is>
+          <t>Wigi Pratama kembali memperkuat Deltras FC untuk kompetisi Liga 2 (Pegadaian Championship) Musim 2026/27 dan ...</t>
+        </is>
+      </c>
+      <c r="F927" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G927" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685968/wigi-pratama-kembali-perkuat-deltras-fc</t>
+        </is>
+      </c>
+      <c r="H927" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/ANTARA-2026-08-08T195349.780.jpg.jpeg</t>
+        </is>
+      </c>
+      <c r="I927" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B928" t="inlineStr">
+        <is>
+          <t>Anggota DPR puji kerja cepat polisi ungkap pembunuhan bocah di Tapsel</t>
+        </is>
+      </c>
+      <c r="C928" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:22:11 +0700</t>
+        </is>
+      </c>
+      <c r="D928" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E928" t="inlineStr">
+        <is>
+          <t>Anggota Komisi III DPR RI, Soedeson Tandra, mengapresiasi kerja cepat Kapolres Tapanuli Selatan (Tapsel) AKBP Anton ...</t>
+        </is>
+      </c>
+      <c r="F928" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G928" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685967/anggota-dpr-puji-kerja-cepat-polisi-ungkap-pembunuhan-bocah-di-tapsel</t>
+        </is>
+      </c>
+      <c r="H928" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000582388.jpg</t>
+        </is>
+      </c>
+      <c r="I928" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B929" t="inlineStr">
+        <is>
+          <t>Raksasa Minyak AS Raup Untung Besar-besaran, Kantongi Rp 2,8 T/Hari</t>
+        </is>
+      </c>
+      <c r="C929" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:00:12 +0700</t>
+        </is>
+      </c>
+      <c r="D929" t="inlineStr">
+        <is>
+          <t>Ignacio Geordi Oswaldo</t>
+        </is>
+      </c>
+      <c r="E929" t="inlineStr">
+        <is>
+          <t>Sebanyak dua perusahaan minyak terbesar asal Amerika Serikat (AS), ExxonMobil dan Chevron melaporkan keuntungan sangat besar berkat lonjakan harga minyak.</t>
+        </is>
+      </c>
+      <c r="F929" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G929" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8609641/raksasa-minyak-as-raup-untung-besar-besaran-kantongi-rp-2-8-t-hari</t>
+        </is>
+      </c>
+      <c r="H929" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2016/04/18/26b2f8ef-da0f-40f3-b37d-a4c4464064a8_169.jpg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I929" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B930" t="inlineStr">
+        <is>
+          <t>RI Lepas 100 Kapal Ekspor Mineral Senilai Rp 2,2 Triliun</t>
+        </is>
+      </c>
+      <c r="C930" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:30:54 +0700</t>
+        </is>
+      </c>
+      <c r="D930" t="inlineStr">
+        <is>
+          <t>Ignacio Geordi Oswaldo</t>
+        </is>
+      </c>
+      <c r="E930" t="inlineStr">
+        <is>
+          <t>Kantor Staf Presiden (KSP) bersama kementerian dan lembaga (K/L) terkait menyelesaikan hambatan ekspor mineral setelah terganjal kandungan logam tanah jarang.</t>
+        </is>
+      </c>
+      <c r="F930" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G930" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8609967/ri-lepas-100-kapal-ekspor-mineral-senilai-rp-2-2-triliun</t>
+        </is>
+      </c>
+      <c r="H930" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2021/10/09/logam-tanah-jarang-ini-jadi-harta-karun-yang-diincar-dunia_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I930" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B931" t="inlineStr">
+        <is>
+          <t>BPK Beri WTP ke ESDM, Tapi Soroti Pengelolaan Denda Tambang</t>
+        </is>
+      </c>
+      <c r="C931" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:59:02 +0700</t>
+        </is>
+      </c>
+      <c r="D931" t="inlineStr">
+        <is>
+          <t>Fadhly Fauzi Rachman</t>
+        </is>
+      </c>
+      <c r="E931" t="inlineStr">
+        <is>
+          <t>BPK memberikan opini WTP untuk Kementerian ESDM, namun soroti pengelolaan denda tambang dan rekomendasi perbaikan keuangan.</t>
+        </is>
+      </c>
+      <c r="F931" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G931" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8610275/bpk-beri-wtp-ke-esdm-tapi-soroti-pengelolaan-denda-tambang</t>
+        </is>
+      </c>
+      <c r="H931" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2016/08/05/9051b9fc-d12e-41a5-9dc0-96e2360c3c68_169.jpg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I931" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B932" t="inlineStr">
+        <is>
+          <t>Bangga! Putri Tommy Kurniawan Sabet Medali Emas Kompetisi di London</t>
+        </is>
+      </c>
+      <c r="C932" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:46:54 +0700</t>
+        </is>
+      </c>
+      <c r="D932" t="inlineStr">
+        <is>
+          <t>Mauludi Rismoyo</t>
+        </is>
+      </c>
+      <c r="E932" t="inlineStr">
+        <is>
+          <t>Aktor dan politisi Tommy Kurniawan lagi berbahagia. Putrinya, Nuaira Syabila Azzahra Kurniawan, baru saja mengukir prestasi gemilang di kancah internasional.</t>
+        </is>
+      </c>
+      <c r="F932" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G932" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8610255/bangga-putri-tommy-kurniawan-sabet-medali-emas-kompetisi-di-london</t>
+        </is>
+      </c>
+      <c r="H932" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/nuaira-syabila-1786182084930_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I932" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B933" t="inlineStr">
+        <is>
+          <t>IAEI dan KNEKS Siap Perkuat Masterplan Ekononomi Syariah RI</t>
+        </is>
+      </c>
+      <c r="C933" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:00:13 +0700</t>
+        </is>
+      </c>
+      <c r="D933" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E933" t="inlineStr">
+        <is>
+          <t>Ketua Harian IAEI Muhammad Syakir Sula mengatakan Indonesia memiliki modal besar untuk menjadi pemimpin ekonomi syariah global.</t>
+        </is>
+      </c>
+      <c r="F933" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G933" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/ekonomi/20260808215555-625-1390193/iaei-dan-kneks-siap-perkuat-masterplan-ekononomi-syariah-ri</t>
+        </is>
+      </c>
+      <c r="H933" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2022/04/13/ilustrasi-alquran-1_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I933" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B934" t="inlineStr">
+        <is>
+          <t>Kebakaran di Surya Kencana, Kemenhut Tutup Sementara Jalur Pendakian Gunung Gede Pangrango</t>
+        </is>
+      </c>
+      <c r="C934" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:11:55 +0700</t>
+        </is>
+      </c>
+      <c r="D934" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E934" t="inlineStr">
+        <is>
+          <t>Calon pendaki pada tanggal tersebut mendapatkan fasilitas refund penuh yang dikirimkan via WhatsApp resmi BBTNGGP.</t>
+        </is>
+      </c>
+      <c r="F934" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G934" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865831/kebakaran-di-surya-kencana-kemenhut-tutup-sementara-jalur-pendakian-gunung-gede-pangrango</t>
+        </is>
+      </c>
+      <c r="H934" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Ei2eg7JfnmoKlvZ3ctGCDIzrInc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/pemadaman-di-tngoo.jpg</t>
+        </is>
+      </c>
+      <c r="I934" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B935" t="inlineStr">
+        <is>
+          <t>16 Besar Kanada Open 2026: Alex Eala Jumpa Unggulan, Sabalenka Lawan Alexandrova</t>
+        </is>
+      </c>
+      <c r="C935" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:09:18 +0700</t>
+        </is>
+      </c>
+      <c r="D935" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E935" t="inlineStr">
+        <is>
+          <t>Babak 16 besar Kanada Open 2026 akan menjadi panggung dari Alex Eala yang akan berhadapan dengan Belinda Bencic, Sabalenka jumpa Alexandrova</t>
+        </is>
+      </c>
+      <c r="F935" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G935" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7865830/16-besar-kanada-open-2026-alex-eala-jumpa-unggulan-sabalenka-lawan-alexandrova</t>
+        </is>
+      </c>
+      <c r="H935" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/dfoxn2WJQ1kbXsIyUEsZE34UFOU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Aryna-Sabalenka-WTA-Finals-2025-1.jpg</t>
+        </is>
+      </c>
+      <c r="I935" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B936" t="inlineStr">
+        <is>
+          <t>Teddy, Purbaya, dan Bahlil Menteri dengan Kinerja Terbaik Menurut Survei Terbaru IPO</t>
+        </is>
+      </c>
+      <c r="C936" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:04:28 +0700</t>
+        </is>
+      </c>
+      <c r="D936" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E936" t="inlineStr">
+        <is>
+          <t>Survei IPO menempatkan Sekretaris Kabinet Teddy Indra Wijaya, Menteri Keuangan Purbaya Yudhi Sadewa, dan Menteri ESDM Bahlil Lahadalia.</t>
+        </is>
+      </c>
+      <c r="F936" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G936" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865829/teddy-purbaya-dan-bahlil-menteri-dengan-kinerja-terbaik-menurut-survei-terbaru-ipo</t>
+        </is>
+      </c>
+      <c r="H936" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/4bdwaC2lq6Y4EP7wiEAVVPorg2k=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/menteri-kinerja-123.jpg</t>
+        </is>
+      </c>
+      <c r="I936" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B937" t="inlineStr">
+        <is>
+          <t>Penembakan di Festival Lembah Baliem, Dua Warga Jadi Korban, Ini Kondisinya</t>
+        </is>
+      </c>
+      <c r="C937" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:59:42 +0700</t>
+        </is>
+      </c>
+      <c r="D937" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E937" t="inlineStr">
+        <is>
+          <t>Penembakan terjadi saat Festival Lembah Baliem berlangsung. Dua warga terluka dan kini menjalani perawatan di RSUD Wamena.</t>
+        </is>
+      </c>
+      <c r="F937" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G937" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865828/penembakan-di-festival-lembah-baliem-dua-warga-jadi-korban-ini-kondisinya</t>
+        </is>
+      </c>
+      <c r="H937" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/qEyJ1F8EbobD-Yt2hKPIYq9rr5k=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Penembakan-di-Festival-Budaya-Lembah-Baliem-Jayawijaya-Papua-Pegunungan.jpg</t>
+        </is>
+      </c>
+      <c r="I937" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B938" t="inlineStr">
+        <is>
+          <t>Bank Besar Mau PHK Massal, Ini Biang Keroknya</t>
+        </is>
+      </c>
+      <c r="C938" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:20:32 +0700</t>
+        </is>
+      </c>
+      <c r="D938" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E938" t="inlineStr">
+        <is>
+          <t>Standard Chartered rencanakan PHK 7.000 karyawan dalam empat tahun, fokus pada efisiensi melalui AI.</t>
+        </is>
+      </c>
+      <c r="F938" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G938" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260808153532-17-757628/bank-besar-mau-phk-massal-ini-biang-keroknya</t>
+        </is>
+      </c>
+      <c r="H938" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2018/02/27/cbf85bcb-e5b2-480d-828e-480df6f0f99c_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I938" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B939" t="inlineStr">
+        <is>
+          <t>Saat Raja Ritel Indonesia Tumbang, Diambil Alih Keluarga Konglomerat</t>
+        </is>
+      </c>
+      <c r="C939" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:45:19 +0700</t>
+        </is>
+      </c>
+      <c r="D939" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E939" t="inlineStr">
+        <is>
+          <t>Matahari, ritel ikonik Indonesia, berawal dari toko Micky Mouse. Didirikan Hari Darmawan, kini memiliki 155 gerai. Simak perjalanan suksesnya!</t>
+        </is>
+      </c>
+      <c r="F939" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G939" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260808150918-17-757625/saat-raja-ritel-indonesia-tumbang-diambil-alih-keluarga-konglomerat</t>
+        </is>
+      </c>
+      <c r="H939" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2018/01/31/aee647ba-570f-443e-9e65-4be398016f5c_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I939" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940" t="inlineStr">
+        <is>
+          <t>Pertanian</t>
+        </is>
+      </c>
+      <c r="B940" t="inlineStr">
+        <is>
+          <t>Ekspor CPO Meningkat, GAPKI Dorong Peremajaan Kebun Rakyat</t>
+        </is>
+      </c>
+      <c r="C940" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:40:52 +0700</t>
+        </is>
+      </c>
+      <c r="D940" t="inlineStr">
+        <is>
+          <t>Satria K Yudha</t>
+        </is>
+      </c>
+      <c r="E940" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA – Gabungan Pengusaha Kelapa Sawit Indonesia (GAPKI) menilai peningkatan produktivitas petani plasma dan swadaya menjadi kunci untuk menjaga pasokan sawit nasional di tengah meningkatnya permintaan domestik dan pasar...</t>
+        </is>
+      </c>
+      <c r="F940" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G940" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjggo4416/ekspor-cpo-meningkat-gapki-dorong-peremajaan-kebun-rakyat</t>
+        </is>
+      </c>
+      <c r="H940" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/_260808214007-397.png</t>
+        </is>
+      </c>
+      <c r="I940" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="941">
+      <c r="A941" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B941" t="inlineStr">
+        <is>
+          <t>TNI-Polri Selidiki KKB Pelaku Penembakan di Festival Lembah Baliem</t>
+        </is>
+      </c>
+      <c r="C941" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:01:11 +0700</t>
+        </is>
+      </c>
+      <c r="D941" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E941" t="inlineStr">
+        <is>
+          <t>TNI-Polri masih menyelidiki kelompok penembak 2 warga di sekitar Festival Lembah Baliem.</t>
+        </is>
+      </c>
+      <c r="F941" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G941" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265291/tni-polri-selidiki-kkb-pelaku-penembakan-di-festival-lembah-baliem</t>
+        </is>
+      </c>
+      <c r="H941" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/7xl6WO2Vyt6ayedPBYX0n-dLKko=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9319217/original/056142800_1786200165-Anatarara.webp</t>
+        </is>
+      </c>
+      <c r="I941" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" t="inlineStr">
+        <is>
+          <t>Bola</t>
+        </is>
+      </c>
+      <c r="B942" t="inlineStr">
+        <is>
+          <t>Duka Lionel Messi, Kehilangan Sosok yang Paling Berjasa dalam Kariernya</t>
+        </is>
+      </c>
+      <c r="C942" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:23:52 +0700</t>
+        </is>
+      </c>
+      <c r="D942" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E942" t="inlineStr">
+        <is>
+          <t>Jorge Messi meninggal dunia pada usia 68 tahun, sosok penting di balik karier La Pulga.</t>
+        </is>
+      </c>
+      <c r="F942" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G942" t="inlineStr">
+        <is>
+          <t>https://bola.kompas.com/read/2026/08/08/22215328/duka-lionel-messi-kehilangan-sosok-yang-paling-berjasa-dalam-kariernya</t>
+        </is>
+      </c>
+      <c r="H942" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/636cVPHtw_W2W8NFctqlVw-4bSo=/240x160:1200x800/1200x675/filters:watermark(data/photo/2026/01/30/697c8163c3944.png,0,-0,1)/data/photo/2026/07/20/6a5d5aa6d90e3.jpg</t>
+        </is>
+      </c>
+      <c r="I942" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B943" t="inlineStr">
+        <is>
+          <t>Menag: Rp 4,1 Triliun BOS Madrasah dan BOP Raudlatul Athfal Tahap II Segera Cair</t>
+        </is>
+      </c>
+      <c r="C943" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:23:52 +0700</t>
+        </is>
+      </c>
+      <c r="D943" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E943" t="inlineStr">
+        <is>
+          <t>Kemenag siap salurkan dana BOS Madrasah dan BOP RA Tahap II 2026 sebesar Rp 4,1 triliun demi pendidikan. Pastikan madrasah aman, nyaman, dan tingkatkan mutu!</t>
+        </is>
+      </c>
+      <c r="F943" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G943" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/08/08/21091281/menag-rp-41-triliun-bos-madrasah-dan-bop-raudlatul-athfal-tahap-ii-segera</t>
+        </is>
+      </c>
+      <c r="H943" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/Pi0KFxjY_8rglX0tW9R-jmaG2W0=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/01/6a6df97f37e23.jpg</t>
+        </is>
+      </c>
+      <c r="I943" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" t="inlineStr">
+        <is>
+          <t>Jawa Tengah</t>
+        </is>
+      </c>
+      <c r="B944" t="inlineStr">
+        <is>
+          <t>Jadwal KRL Jogja-Solo Minggu 9 Agustus 2026 Lengkap, Cek Jam Berangkat dari Semua Stasiun</t>
+        </is>
+      </c>
+      <c r="C944" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:23:52 +0700</t>
+        </is>
+      </c>
+      <c r="D944" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E944" t="inlineStr">
+        <is>
+          <t>Simak jadwal KRL Jogja-Solo Minggu (9/8/2026). Commuter Line Yogyakarta-Palur beroperasi dari pagi hingga malam.</t>
+        </is>
+      </c>
+      <c r="F944" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G944" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/jawa-tengah/read/2026/08/08/201700488/jadwal-krl-jogja-solo-minggu-9-agustus-2026-lengkap-cek-jam</t>
+        </is>
+      </c>
+      <c r="H944" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/LtWWzbsAqb3XDnyWPqxuth_zcZ8=/0x0:1106x737/1200x675/data/photo/2024/10/31/6723b38cc74a7.jpg</t>
+        </is>
+      </c>
+      <c r="I944" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I895"/>
+  <autoFilter ref="A1:I944"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-08 16:24 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-08.xlsx
+++ b/data/berita_2026-08-08.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$944</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$965</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I944"/>
+  <dimension ref="A1:I965"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -44806,8 +44806,995 @@
         </is>
       </c>
     </row>
+    <row r="945">
+      <c r="A945" t="inlineStr">
+        <is>
+          <t>Top News</t>
+        </is>
+      </c>
+      <c r="B945" t="inlineStr">
+        <is>
+          <t>Joao Pedro cetak dua gol Chelsea untuk bungkam Milan di GBK</t>
+        </is>
+      </c>
+      <c r="C945" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:35:06 +0700</t>
+        </is>
+      </c>
+      <c r="D945" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E945" t="inlineStr">
+        <is>
+          <t>Pemain Chelsea Joao Pedro mencetak dua gol untuk membungkam AC Milan dengan skor akhir 3-0 dalam laga ...</t>
+        </is>
+      </c>
+      <c r="F945" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G945" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686069/joao-pedro-cetak-dua-gol-chelsea-untuk-bungkam-milan-di-gbk</t>
+        </is>
+      </c>
+      <c r="H945" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/Chelsea-kalahkan-AC-Milan-080826-02A.jpg</t>
+        </is>
+      </c>
+      <c r="I945" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B946" t="inlineStr">
+        <is>
+          <t>Kebakaran Meluas, Kawasan Wisata Bromo Ditutup Total</t>
+        </is>
+      </c>
+      <c r="C946" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 23:08:04 +0700</t>
+        </is>
+      </c>
+      <c r="D946" t="inlineStr">
+        <is>
+          <t>M Rofiq</t>
+        </is>
+      </c>
+      <c r="E946" t="inlineStr">
+        <is>
+          <t>Penutupan tersebut mencakup akses dari empat wilayah, yakni Kabupaten Lumajang, Malang, Pasuruan, dan Kabupaten Probolinggo.</t>
+        </is>
+      </c>
+      <c r="F946" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G946" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610330/kebakaran-meluas-kawasan-wisata-bromo-ditutup-total</t>
+        </is>
+      </c>
+      <c r="H946" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/kebakaran-bromo-yang-makin-meluas-1786195878372_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I946" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="947">
+      <c r="A947" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B947" t="inlineStr">
+        <is>
+          <t>Bareskrim Bongkar 'Pabrik' Vape Etomidate di Kamar Kos Kemang</t>
+        </is>
+      </c>
+      <c r="C947" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:40:58 +0700</t>
+        </is>
+      </c>
+      <c r="D947" t="inlineStr">
+        <is>
+          <t>Yogi Ernes</t>
+        </is>
+      </c>
+      <c r="E947" t="inlineStr">
+        <is>
+          <t>Para pelaku mengaku mendapatkan tawaran memproduksi vape etomidate itu dari seseorang di Facebook. Mereka dijanjikan upah jutaan rupiah per harinya.</t>
+        </is>
+      </c>
+      <c r="F947" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G947" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610310/bareskrim-bongkar-pabrik-vape-etomidate-di-kamar-kos-kemang</t>
+        </is>
+      </c>
+      <c r="H947" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/barang-bukti-vape-etomidate-ditemukan-dalam-kamar-kos-di-kemang-dokbareskrim-1786203531890_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I947" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="948">
+      <c r="A948" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B948" t="inlineStr">
+        <is>
+          <t>Penampakan Kapal Pengangkut 1,3 Ton Ketamin yang Disergap di Bintan</t>
+        </is>
+      </c>
+      <c r="C948" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:27:50 +0700</t>
+        </is>
+      </c>
+      <c r="D948" t="inlineStr">
+        <is>
+          <t>Mei Amelia R</t>
+        </is>
+      </c>
+      <c r="E948" t="inlineStr">
+        <is>
+          <t>Tim gabungan Bareskrim, Bea Cukai, BNN, dan TNI AL menyergap kapal Tanzania yang menyelundupkan 1,3 ton ketamin di perairan Bintan. Delapan ABK diamankan.</t>
+        </is>
+      </c>
+      <c r="F948" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G948" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610301/penampakan-kapal-pengangkut-1-3-ton-ketamin-yang-disergap-di-bintan</t>
+        </is>
+      </c>
+      <c r="H948" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/kapal-mv-king-sun-pengangkut-13-ton-ketamin-disergap-di-perairan-bintan-1786202843343_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I948" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B949" t="inlineStr">
+        <is>
+          <t>Residivis Kambuhan di Bogor: Hunting Masjid Sepi, Kotak Amal Jadi Incaran</t>
+        </is>
+      </c>
+      <c r="C949" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:06:23 +0700</t>
+        </is>
+      </c>
+      <c r="D949" t="inlineStr">
+        <is>
+          <t>Tim detikcom</t>
+        </is>
+      </c>
+      <c r="E949" t="inlineStr">
+        <is>
+          <t>Seorang residivis kembali berulah di Bogor, dengan membobol kotak amal di sejumlah masjid. Pelaku terlebih dahulu mencari masjid sepi untuk memuluskan aksinya.</t>
+        </is>
+      </c>
+      <c r="F949" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G949" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610290/residivis-kambuhan-di-bogor-hunting-masjid-sepi-kotak-amal-jadi-incaran</t>
+        </is>
+      </c>
+      <c r="H949" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/residivis-ditangkap-lagi-usai-bobol-4-kotak-amal-di-bogor-1786011251674_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I949" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B950" t="inlineStr">
+        <is>
+          <t>Ahmad Muzani Bicara Relevansi Qanun Asasi dalam Perkuat Persatuan Bangsa</t>
+        </is>
+      </c>
+      <c r="C950" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:51:44 +0700</t>
+        </is>
+      </c>
+      <c r="D950" t="inlineStr">
+        <is>
+          <t>Dea Duta Aulia</t>
+        </is>
+      </c>
+      <c r="E950" t="inlineStr">
+        <is>
+          <t>Ketua MPR RI Ahmad Muzani menekankan pentingnya Empat Pilar kebangsaan untuk persatuan dan pembangunan menuju Indonesia Emas 2045 dalam Halaqah Kebangsaan.</t>
+        </is>
+      </c>
+      <c r="F950" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G950" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610267/ahmad-muzani-bicara-relevansi-qanun-asasi-dalam-perkuat-persatuan-bangsa</t>
+        </is>
+      </c>
+      <c r="H950" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/ahmad-muzani-bicara-relevansi-qanun-asasi-memperkuat-persatuan-bangsa-1786200590451_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I950" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B951" t="inlineStr">
+        <is>
+          <t>Pencuri di Jakbar Sempat Mau Balikin Motor Curian Saat Tahu Wajahnya Viral</t>
+        </is>
+      </c>
+      <c r="C951" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:40:34 +0700</t>
+        </is>
+      </c>
+      <c r="D951" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E951" t="inlineStr">
+        <is>
+          <t>DMJ rupanya sempat mendatangi Polsek Ciputat Timur untuk meminta tolong menghubungi SY dengan alasan ingin mengembalikan motor yang sempat dibawanya tersebut.</t>
+        </is>
+      </c>
+      <c r="F951" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G951" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610252/pencuri-di-jakbar-sempat-mau-balikin-motor-curian-saat-tahu-wajahnya-viral</t>
+        </is>
+      </c>
+      <c r="H951" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/seorang-pria-menjadi-korban-curanmor-di-kembangan-jakbar-sepeda-motor-pria-itu-diduga-dibawa-wanita-saat-pertemuan-pertama-fir-1785999460503_43.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I951" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B952" t="inlineStr">
+        <is>
+          <t>Polda Metro Gagalkan Penyelundupan 150 Kg Pasir Timah dalam Truk Ekspedisi</t>
+        </is>
+      </c>
+      <c r="C952" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:29:34 +0700</t>
+        </is>
+      </c>
+      <c r="D952" t="inlineStr">
+        <is>
+          <t>Audrey Santoso</t>
+        </is>
+      </c>
+      <c r="E952" t="inlineStr">
+        <is>
+          <t>Subdit Gakkum Ditpolairud Polda Metro Jaya ungkap penyelundupan pasir timah 150 kg dari Bangka Belitung. Penyelidikan masih berlanjut.</t>
+        </is>
+      </c>
+      <c r="F952" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G952" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8610245/polda-metro-gagalkan-penyelundupan-150-kg-pasir-timah-dalam-truk-ekspedisi</t>
+        </is>
+      </c>
+      <c r="H952" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/08/penyelundupan-150-kg-pasir-timah-1786199309175_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I952" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B953" t="inlineStr">
+        <is>
+          <t>Pasar Properti Melejit via Program 3 Juta Rumah, Asuransi Jadi Kunci Mitigasi Risiko</t>
+        </is>
+      </c>
+      <c r="C953" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 23:19:00 +0700</t>
+        </is>
+      </c>
+      <c r="D953" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E953" t="inlineStr">
+        <is>
+          <t>Momentum dorongan kepemilikan rumah melalui Program 3 Juta Rumah pemerintah pun dinilai perlu diimbangi dengan kesadaran asuransi yang kuat.</t>
+        </is>
+      </c>
+      <c r="F953" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G953" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/properti/7865841/pasar-properti-melejit-via-program-3-juta-rumah-asuransi-jadi-kunci-mitigasi-risiko</t>
+        </is>
+      </c>
+      <c r="H953" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/DZyaGIghm_iveJP5kKNnUc8d9tA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/BTN-Dukung-Program-3-Juta-Rumah_20250207_220150.jpg</t>
+        </is>
+      </c>
+      <c r="I953" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B954" t="inlineStr">
+        <is>
+          <t>Modus Ajak Menikah, Pria di Blitar Tipu Pekerja Migran di Hongkong Rp622 Juta</t>
+        </is>
+      </c>
+      <c r="C954" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 23:18:27 +0700</t>
+        </is>
+      </c>
+      <c r="D954" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E954" t="inlineStr">
+        <is>
+          <t>S menjadi korban penipuan seorang laki-laki berinisial IS (43), warga Desa Slumbung, Kecamatan Gandusari, Kabupaten Blitar.</t>
+        </is>
+      </c>
+      <c r="F954" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G954" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7865840/modus-ajak-menikah-pria-di-blitar-tipu-pekerja-migran-di-hongkong-rp622-juta</t>
+        </is>
+      </c>
+      <c r="H954" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/424KEBvmFB6GDIqpWyU284w89U0=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ILUSTRASI-LOVE-SCAMMING-32432sdfsd.jpg</t>
+        </is>
+      </c>
+      <c r="I954" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="955">
+      <c r="A955" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B955" t="inlineStr">
+        <is>
+          <t>Pimpinan DPR Dorong Tradisi Agustusan untuk Edukasi Nasionalisme Gen Alpha</t>
+        </is>
+      </c>
+      <c r="C955" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 23:16:03 +0700</t>
+        </is>
+      </c>
+      <c r="D955" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E955" t="inlineStr">
+        <is>
+          <t>Wakil Ketua DPR RI Cucun Ahmad Syamsurijal mendorong perayaan HUT RI di tingkat kampung dikemas edukatif untuk mengenalkan nilai sejarah.</t>
+        </is>
+      </c>
+      <c r="F955" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G955" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865839/pimpinan-dpr-dorong-tradisi-agustusan-untuk-edukasi-nasionalisme-gen-alpha</t>
+        </is>
+      </c>
+      <c r="H955" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/sI2m_aWyzxcjIc0zJCqMqo08_A0=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/cucun-wakil-ketua-dopr.jpg</t>
+        </is>
+      </c>
+      <c r="I955" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B956" t="inlineStr">
+        <is>
+          <t>MA Koreksi Kerugian Negara Kasus Korupsi Timah, Sebut Nilainya Bukan Rp 300 Triliun</t>
+        </is>
+      </c>
+      <c r="C956" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 23:12:03 +0700</t>
+        </is>
+      </c>
+      <c r="D956" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E956" t="inlineStr">
+        <is>
+          <t>Lewat putusan kasasinya, MA menyatakan angka kerugian negara dalam kasus ini bukanlah Rp 300 triliun, melainkan sekitar Rp 28 triliun.</t>
+        </is>
+      </c>
+      <c r="F956" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G956" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865838/ma-koreksi-kerugian-negara-kasus-korupsi-timah-sebut-nilainya-bukan-rp-300-triliun</t>
+        </is>
+      </c>
+      <c r="H956" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/rUdvae9c2OX3wT_OZbSuRb7ObfU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Gedung-Mahkamah-Agung-ilustrasi-CPNS.jpg</t>
+        </is>
+      </c>
+      <c r="I956" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B957" t="inlineStr">
+        <is>
+          <t>Talenta Terpilih dari Batam Berpeluang Lanjut ke Akademi Garudayaksa</t>
+        </is>
+      </c>
+      <c r="C957" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 23:10:20 +0700</t>
+        </is>
+      </c>
+      <c r="D957" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E957" t="inlineStr">
+        <is>
+          <t>Talenta-talenta muda yang teridentifikasi memiliki potensi disiapkan untuk mengikuti tahapan pembinaan lanjutan melalui ajang International Series</t>
+        </is>
+      </c>
+      <c r="F957" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G957" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865837/talenta-terpilih-dari-batam-berpeluang-lanjut-ke-akademi-garudayaksa</t>
+        </is>
+      </c>
+      <c r="H957" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/TP6J7DpuEt73fs1KHzlSzMSnpck=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/TURNAMEN-USIA-DINI-Turnamen-sepakbola-usia-dini-Batam-Prime-International.jpg</t>
+        </is>
+      </c>
+      <c r="I957" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B958" t="inlineStr">
+        <is>
+          <t>Pengalaman Pengunjung GIIAS 2026 Test Drive SUV Deepal S05 REEV dan Nevo Q05</t>
+        </is>
+      </c>
+      <c r="C958" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:58:29 +0700</t>
+        </is>
+      </c>
+      <c r="D958" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E958" t="inlineStr">
+        <is>
+          <t>Nevo Q05 merupakan SUV terbaru dari Changan yang rilis perdana di GIIAS 2026 dan diklaim punya wheelbase terpanjang di kelasnya.</t>
+        </is>
+      </c>
+      <c r="F958" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G958" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/otomotif/7865836/pengalaman-pengunjung-giias-2026-test-drive-suv-deepal-s05-reev-dan-nevo-q05</t>
+        </is>
+      </c>
+      <c r="H958" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/osJAII6LWEwrq-YnPnNx3HbzwIE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Sesi-test-drive-Changan-Nevo-Q05-di-GIIAS-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I958" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B959" t="inlineStr">
+        <is>
+          <t>Anggota DPR Bambang Haryo Minta Sistem Keselamatan dan Penyelamatan Diperkuat</t>
+        </is>
+      </c>
+      <c r="C959" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:51:58 +0700</t>
+        </is>
+      </c>
+      <c r="D959" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E959" t="inlineStr">
+        <is>
+          <t>Bambang Haryo meminta keselamatan pelayaran diperkuat dari pemeriksaan kapal hingga kemampuan SAR saat kecelakaan terjadi.</t>
+        </is>
+      </c>
+      <c r="F959" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G959" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865835/anggota-dpr-bambang-haryo-minta-sistem-keselamatan-dan-penyelamatan-diperkuat</t>
+        </is>
+      </c>
+      <c r="H959" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/MqtBI4UIq6Mjg-s0FOiJY17JfaA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Anggota-DPR-Bambang-Haryo-Soekartono-korban-kebakaran-KMP-Mutiara-Sentosa-II.jpg</t>
+        </is>
+      </c>
+      <c r="I959" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B960" t="inlineStr">
+        <is>
+          <t>Mengapa Rusia Menjual Cadangan Emasnya?</t>
+        </is>
+      </c>
+      <c r="C960" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:42:25 +0700</t>
+        </is>
+      </c>
+      <c r="D960" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E960" t="inlineStr">
+        <is>
+          <t>Selama setahun terakhir, Rusia telah menjadi penjual emas terbesar di dunia. Ini adalah cara negara tersebut meningkatkan pendapatannya…</t>
+        </is>
+      </c>
+      <c r="F960" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G960" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7865834/mengapa-rusia-menjual-cadangan-emasnya</t>
+        </is>
+      </c>
+      <c r="H960" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/hYrs7hunOiK36vJGLJREVRzwCn8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/BDeutsche-Welle77474131_403.jpg.jpg</t>
+        </is>
+      </c>
+      <c r="I960" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B961" t="inlineStr">
+        <is>
+          <t>Dari Pelaksana ke Pencipta Nilai, Ini Strategi Alih Profesi bagi Purna Ajudan</t>
+        </is>
+      </c>
+      <c r="C961" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:31:05 +0700</t>
+        </is>
+      </c>
+      <c r="D961" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E961" t="inlineStr">
+        <is>
+          <t>Setiap insan Narasraya harus mempersiapkan diri dalam rangka mempersiapkan karier selanjutnya setelah purna tugas.</t>
+        </is>
+      </c>
+      <c r="F961" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G961" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865833/dari-pelaksana-ke-pencipta-nilai-ini-strategi-alih-profesi-bagi-purna-ajudan</t>
+        </is>
+      </c>
+      <c r="H961" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/6Eyn-I96gj3NWCk1FSt3IlptQJs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Syam-Basrijal-1.jpg</t>
+        </is>
+      </c>
+      <c r="I961" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="962">
+      <c r="A962" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B962" t="inlineStr">
+        <is>
+          <t>Bertemu Dasco di DPR, Pengurus Gerakan Muda untuk Rakyat Dorong Penguatan AI dan Keamanan Siber</t>
+        </is>
+      </c>
+      <c r="C962" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:21:37 +0700</t>
+        </is>
+      </c>
+      <c r="D962" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E962" t="inlineStr">
+        <is>
+          <t>DPP GEMURA menilai kolaborasi pemuda dan pemerintah kunci menghadapi tantangan Artificial Intelligence dan keamanan siber.</t>
+        </is>
+      </c>
+      <c r="F962" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G962" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865832/bertemu-dasco-di-dpr-pengurus-gerakan-muda-untuk-rakyat-dorong-penguatan-ai-dan-keamanan-siber</t>
+        </is>
+      </c>
+      <c r="H962" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/XBRYklAupnoUt6hJJ_BvbSRbQ2M=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Gerakan-Muda-untuk-Rakyat-1.jpg</t>
+        </is>
+      </c>
+      <c r="I962" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="963">
+      <c r="A963" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B963" t="inlineStr">
+        <is>
+          <t>Perempuan Lansia Ditemukan Tewas Penuh Luka di Dasar Sumur di Kuningan</t>
+        </is>
+      </c>
+      <c r="C963" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 23:24:01 +0700</t>
+        </is>
+      </c>
+      <c r="D963" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E963" t="inlineStr">
+        <is>
+          <t>Lansia 77 tahun ditemukan tewas di dasar sumur di Kuningan dengan luka-luka. Polisi mendalami kasus penemuan jenazah yang gegerkan warga.</t>
+        </is>
+      </c>
+      <c r="F963" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G963" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/08/08/232303978/perempuan-lansia-ditemukan-tewas-penuh-luka-di-dasar-sumur-di-kuningan</t>
+        </is>
+      </c>
+      <c r="H963" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/9t5a_uqZ3txufv1t6NJnBw0GHbI=/0x0:750x500/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/03/13/69b3ba491a15a.jpg</t>
+        </is>
+      </c>
+      <c r="I963" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="964">
+      <c r="A964" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B964" t="inlineStr">
+        <is>
+          <t>Motif Utama Pemutilasi di Depok Ingin Kuasai Motor PCX Milik Korban</t>
+        </is>
+      </c>
+      <c r="C964" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 23:24:01 +0700</t>
+        </is>
+      </c>
+      <c r="D964" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E964" t="inlineStr">
+        <is>
+          <t>Polisi mengungkap motif utama pemutilasi di Depok. Pelaku disebut ingin menguasai motor PCX milik korban karena desakan ekonomi.</t>
+        </is>
+      </c>
+      <c r="F964" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G964" t="inlineStr">
+        <is>
+          <t>https://megapolitan.kompas.com/read/2026/08/08/21362311/motif-utama-pemutilasi-di-depok-ingin-kuasai-motor-pcx-milik-korban</t>
+        </is>
+      </c>
+      <c r="H964" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/Z-D46xurFbbXdOBDXSnv4NnIOGM=/72x0:1314x828/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/05/6a72f482dae12.jpeg</t>
+        </is>
+      </c>
+      <c r="I964" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B965" t="inlineStr">
+        <is>
+          <t>Motif Perampokan dan Pembunuhan Bos Royal Phone Ambarawa Murni Ekonomi, Polisi: Tak Ada Dendam</t>
+        </is>
+      </c>
+      <c r="C965" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 23:24:01 +0700</t>
+        </is>
+      </c>
+      <c r="D965" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E965" t="inlineStr">
+        <is>
+          <t>Polisi mengungkap motif perampokan konter Royal Phone yang menewaskan pemiliknya di Kelurahan Pojoksari, Kecamatan Ambarawa, Kabupaten Semarang</t>
+        </is>
+      </c>
+      <c r="F965" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G965" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/08/08/202521378/motif-perampokan-dan-pembunuhan-bos-royal-phone-ambarawa-murni-ekonomi</t>
+        </is>
+      </c>
+      <c r="H965" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/SWBRQMx6T9AMLfJ4k1h0L2KjIsk=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/08/6a76f0b78810c.jpg</t>
+        </is>
+      </c>
+      <c r="I965" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I944"/>
+  <autoFilter ref="A1:I965"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-08 17:24 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-08.xlsx
+++ b/data/berita_2026-08-08.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$965</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1000</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I965"/>
+  <dimension ref="A1:I1000"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -45793,8 +45793,1654 @@
         </is>
       </c>
     </row>
+    <row r="966">
+      <c r="A966" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B966" t="inlineStr">
+        <is>
+          <t>Tournament of Flowers TIFF 2026, kolaborasi perkuat pariwisata Tomohon</t>
+        </is>
+      </c>
+      <c r="C966" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 23:42:18 +0700</t>
+        </is>
+      </c>
+      <c r="D966" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E966" t="inlineStr">
+        <is>
+          <t>ANTARA - Pemerintah kota Tomohon, Sulawesi Utara menggelar Tournament of Flowers (TOF) sebagai bagian dari rangkaian ...</t>
+        </is>
+      </c>
+      <c r="F966" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G966" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686115/tournament-of-flowers-tiff-2026-kolaborasi-perkuat-pariwisata-tomohon</t>
+        </is>
+      </c>
+      <c r="H966" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_TOURNAMENT-OF-FLOWERS-TIFF-2026-KOLABORASI-PERKUAT-PARIWISATA-TOMOHON.jpg</t>
+        </is>
+      </c>
+      <c r="I966" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="967">
+      <c r="A967" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B967" t="inlineStr">
+        <is>
+          <t>Pemuda Pekalongan bentangkan kain merah putih 200 meter sambut HUT RI</t>
+        </is>
+      </c>
+      <c r="C967" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 23:38:57 +0700</t>
+        </is>
+      </c>
+      <c r="D967" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E967" t="inlineStr">
+        <is>
+          <t>ANTARA - Berbagai cara dilakukan masyarakat untuk memeriahkan Hari Ulang Tahun ke-8 Republik Indonesia, ...</t>
+        </is>
+      </c>
+      <c r="F967" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G967" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686112/pemuda-pekalongan-bentangkan-kain-merah-putih-200-meter-sambut-hut-ri</t>
+        </is>
+      </c>
+      <c r="H967" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_PEMUDA-PEKALONGAN-BENTANGKAN-KAIN-MERAH-PUTIH-200-METER-SAMBUT-HUT-RI_1.jpg</t>
+        </is>
+      </c>
+      <c r="I967" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="968">
+      <c r="A968" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B968" t="inlineStr">
+        <is>
+          <t>Ferran Torres minta dijual ke PSG seusai capai persyaratan personal</t>
+        </is>
+      </c>
+      <c r="C968" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 23:38:31 +0700</t>
+        </is>
+      </c>
+      <c r="D968" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E968" t="inlineStr">
+        <is>
+          <t>Penyerang Barcelona Ferran Torres telah menyampaikan keinginan kepada pihak klub untuk bergabung dengan Paris ...</t>
+        </is>
+      </c>
+      <c r="F968" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G968" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686117/ferran-torres-minta-dijual-ke-psg-seusai-capai-persyaratan-personal</t>
+        </is>
+      </c>
+      <c r="H968" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/20/Spain-v-Argentina-Final-FIFA-World-Cup-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I968" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="969">
+      <c r="A969" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B969" t="inlineStr">
+        <is>
+          <t>Momentum positif Mario Aji terhenti saat Q2 Moto2 Inggris</t>
+        </is>
+      </c>
+      <c r="C969" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 23:29:20 +0700</t>
+        </is>
+      </c>
+      <c r="D969" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E969" t="inlineStr">
+        <is>
+          <t>Momentum positif pembalap Indonesia Mario Suryo Aji terhenti setelah terlibat tabrakan dengan Zonta van den Goorbergh ...</t>
+        </is>
+      </c>
+      <c r="F969" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G969" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686113/momentum-positif-mario-aji-terhenti-saat-q2-moto2-inggris</t>
+        </is>
+      </c>
+      <c r="H969" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/21/Latihan-pembalap-nasional-Moto2-dan-Moto3-di-Mandalika-210726-AS-8.jpg</t>
+        </is>
+      </c>
+      <c r="I969" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="970">
+      <c r="A970" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B970" t="inlineStr">
+        <is>
+          <t>Mentan percepat intervensi pertanian untuk tekan kemiskinan di Alor</t>
+        </is>
+      </c>
+      <c r="C970" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 23:19:18 +0700</t>
+        </is>
+      </c>
+      <c r="D970" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E970" t="inlineStr">
+        <is>
+          <t>Menteri Pertanian Andi Amran Sulaiman mempercepat intervensi pertanian di Alor, Nusa Tenggara Timur (NTT) melalui ...</t>
+        </is>
+      </c>
+      <c r="F970" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G970" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686109/mentan-percepat-intervensi-pertanian-untuk-tekan-kemiskinan-di-alor</t>
+        </is>
+      </c>
+      <c r="H970" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/83871AAC-4AC3-4A63-ABE1-F68F81B23725.jpeg</t>
+        </is>
+      </c>
+      <c r="I970" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="971">
+      <c r="A971" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B971" t="inlineStr">
+        <is>
+          <t>Xabi Alonso sebut dukungan penggemar Chelsea menakjubkan di GBK</t>
+        </is>
+      </c>
+      <c r="C971" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 23:18:36 +0700</t>
+        </is>
+      </c>
+      <c r="D971" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E971" t="inlineStr">
+        <is>
+          <t>Manajer Chelsea Xabi Alonso menyebut penggemar Chelsea menunjukkan dukungan yang menakjubkan dalam laga pramusim ...</t>
+        </is>
+      </c>
+      <c r="F971" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G971" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686107/xabi-alonso-sebut-dukungan-penggemar-chelsea-menakjubkan-di-gbk</t>
+        </is>
+      </c>
+      <c r="H971" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/65c3991c-4f05-473d-80c4-08c88de490fd.jpeg</t>
+        </is>
+      </c>
+      <c r="I971" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="972">
+      <c r="A972" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B972" t="inlineStr">
+        <is>
+          <t>Melihat keseruan dolanan lempung di Museum Radya Pustaka Solo</t>
+        </is>
+      </c>
+      <c r="C972" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 23:17:27 +0700</t>
+        </is>
+      </c>
+      <c r="D972" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E972" t="inlineStr">
+        <is>
+          <t>ANTARA - Museum Radya Pustaka di Kota Solo menghadirkan inovasi, salah satunya melalui kegiatan edukatif kelas dolanan ...</t>
+        </is>
+      </c>
+      <c r="F972" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G972" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686103/melihat-keseruan-dolanan-lempung-di-museum-radya-pustaka-solo</t>
+        </is>
+      </c>
+      <c r="H972" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_MELIHAT-KESERUAN-DOLANAN-LEMPUNG-DI-MUSEUM-RADYA-PUSTAKA-SOLO.jpg</t>
+        </is>
+      </c>
+      <c r="I972" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="973">
+      <c r="A973" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B973" t="inlineStr">
+        <is>
+          <t>WNBPA tegaskan inklusi hadapi polemik atlet transgender</t>
+        </is>
+      </c>
+      <c r="C973" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 23:03:59 +0700</t>
+        </is>
+      </c>
+      <c r="D973" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E973" t="inlineStr">
+        <is>
+          <t>Asosiasi Pemain Bola Basket Nasional Perempuan di AS (Women’s National Basketball Players Association/WNBPA) ...</t>
+        </is>
+      </c>
+      <c r="F973" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G973" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686100/wnbpa-tegaskan-inklusi-hadapi-polemik-atlet-transgender</t>
+        </is>
+      </c>
+      <c r="H973" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2020/04/04/wnba.jpg</t>
+        </is>
+      </c>
+      <c r="I973" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="974">
+      <c r="A974" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B974" t="inlineStr">
+        <is>
+          <t>Ruben Amorim kagumi dukungan penggemar AC Milan di Indonesia</t>
+        </is>
+      </c>
+      <c r="C974" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:53:37 +0700</t>
+        </is>
+      </c>
+      <c r="D974" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E974" t="inlineStr">
+        <is>
+          <t>Pelatih AC Milan Ruben Amorim mengagumi dukungan dari penggemar AC Milan di Indonesia selama tim tersebut menjalani ...</t>
+        </is>
+      </c>
+      <c r="F974" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G974" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686096/ruben-amorim-kagumi-dukungan-penggemar-ac-milan-di-indonesia</t>
+        </is>
+      </c>
+      <c r="H974" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/2aa53dff-80c5-4b25-9493-0ff161d54ac9.jpeg</t>
+        </is>
+      </c>
+      <c r="I974" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="975">
+      <c r="A975" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B975" t="inlineStr">
+        <is>
+          <t>KDM minta LPM bantu dorong percepatan pembangunan desa</t>
+        </is>
+      </c>
+      <c r="C975" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:49:47 +0700</t>
+        </is>
+      </c>
+      <c r="D975" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E975" t="inlineStr">
+        <is>
+          <t>Gubernur Jawa Barat Dedi Mulyadi meminta Lembaga Pemberdayaan Masyarakat (LPM) membantu mendorong percepatan ...</t>
+        </is>
+      </c>
+      <c r="F975" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G975" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686095/kdm-minta-lpm-bantu-dorong-percepatan-pembangunan-desa</t>
+        </is>
+      </c>
+      <c r="H975" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1002083943.jpg</t>
+        </is>
+      </c>
+      <c r="I975" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="976">
+      <c r="A976" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B976" t="inlineStr">
+        <is>
+          <t>Thailand dan Malaysia tembus semifinal Piala AFF 2026</t>
+        </is>
+      </c>
+      <c r="C976" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:48:45 +0700</t>
+        </is>
+      </c>
+      <c r="D976" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E976" t="inlineStr">
+        <is>
+          <t>Thailand memastikan diri sebagai juara Grup B Piala AFF 2026 dan lolos semifinal setelah menutup fase grup dengan ...</t>
+        </is>
+      </c>
+      <c r="F976" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G976" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686092/thailand-dan-malaysia-tembus-semifinal-piala-aff-2026</t>
+        </is>
+      </c>
+      <c r="H976" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/07/26/semifinal-piala-aff-u-23-indonesia-lawan-thailand-2583629.jpg</t>
+        </is>
+      </c>
+      <c r="I976" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="977">
+      <c r="A977" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B977" t="inlineStr">
+        <is>
+          <t>Menteri PPPA: Festival Egrang perkuat komitmen ruang aman anak Jember</t>
+        </is>
+      </c>
+      <c r="C977" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:46:57 +0700</t>
+        </is>
+      </c>
+      <c r="D977" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E977" t="inlineStr">
+        <is>
+          <t>Menteri Pemberdayaan Perempuan dan Perlindungan Anak (PPPA) Arifatul Choiri Fauzi mengatakan Festival Egrang dapat ...</t>
+        </is>
+      </c>
+      <c r="F977" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G977" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686091/menteri-pppa-festival-egrang-perkuat-komitmen-ruang-aman-anak-jember</t>
+        </is>
+      </c>
+      <c r="H977" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/WhatsApp-Image-2026-08-08-at-21.55.38.jpeg</t>
+        </is>
+      </c>
+      <c r="I977" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="978">
+      <c r="A978" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B978" t="inlineStr">
+        <is>
+          <t>Tim rescue Australia banyak belajar dengan tim Indonesia</t>
+        </is>
+      </c>
+      <c r="C978" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:46:39 +0700</t>
+        </is>
+      </c>
+      <c r="D978" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E978" t="inlineStr">
+        <is>
+          <t>Tim rescue Northern Star Resources (NTR) dari Australia mengapresiasi kemampuan para rescuer atau penyelamat Indonesia ...</t>
+        </is>
+      </c>
+      <c r="F978" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G978" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686089/tim-rescue-australia-banyak-belajar-dengan-tim-indonesia</t>
+        </is>
+      </c>
+      <c r="H978" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG_3686.jpeg</t>
+        </is>
+      </c>
+      <c r="I978" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="979">
+      <c r="A979" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B979" t="inlineStr">
+        <is>
+          <t>Kemkomdigi ungkap "3C" jadi fokus untuk sokong industri gim nasional</t>
+        </is>
+      </c>
+      <c r="C979" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:43:32 +0700</t>
+        </is>
+      </c>
+      <c r="D979" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E979" t="inlineStr">
+        <is>
+          <t>Staf Khusus Menteri Komunikasi dan Digital bidang Pemuda dan Startup Alfreno Kautsar mengatakan Kementerian Komunikasi ...</t>
+        </is>
+      </c>
+      <c r="F979" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G979" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686087/kemkomdigi-ungkap-3c-jadi-fokus-untuk-sokong-industri-gim-nasional</t>
+        </is>
+      </c>
+      <c r="H979" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/20260808_145434.jpg</t>
+        </is>
+      </c>
+      <c r="I979" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="980">
+      <c r="A980" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B980" t="inlineStr">
+        <is>
+          <t>Jembatan Perintis Sikundo Aceh Barat mulai dibangun</t>
+        </is>
+      </c>
+      <c r="C980" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:41:33 +0700</t>
+        </is>
+      </c>
+      <c r="D980" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E980" t="inlineStr">
+        <is>
+          <t>ANTARA - Pembangunan jembatan perintis di Desa Sikundo, Kecamatan Pante Ceureumen, Kabupaten Aceh Barat, Aceh, mulai ...</t>
+        </is>
+      </c>
+      <c r="F980" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G980" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686061/jembatan-perintis-sikundo-aceh-barat-mulai-dibangun</t>
+        </is>
+      </c>
+      <c r="H980" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/JEMBATAN-PERINTIS-SIKUNDO-ACEH-BARAT-MULAI-DIBANGUN.jpg</t>
+        </is>
+      </c>
+      <c r="I980" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="981">
+      <c r="A981" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B981" t="inlineStr">
+        <is>
+          <t>Kebakaran di Samarinda hanguskan enam bangunan, 20 jiwa terdampak</t>
+        </is>
+      </c>
+      <c r="C981" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:40:23 +0700</t>
+        </is>
+      </c>
+      <c r="D981" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E981" t="inlineStr">
+        <is>
+          <t>Pemadam Kebakaran dan Penyelamatan (Disdamkar) Kota Samarinda, Kalimantan Timur, bersama tim relawan gabungan bergerak ...</t>
+        </is>
+      </c>
+      <c r="F981" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G981" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686083/kebakaran-di-samarinda-hanguskan-enam-bangunan-20-jiwa-terdampak</t>
+        </is>
+      </c>
+      <c r="H981" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1001893456.jpg</t>
+        </is>
+      </c>
+      <c r="I981" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="982">
+      <c r="A982" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B982" t="inlineStr">
+        <is>
+          <t>Meriahkan HUT Ke-81 RI, warga Dayak Dusmala lomba tangkap anak babi</t>
+        </is>
+      </c>
+      <c r="C982" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:39:31 +0700</t>
+        </is>
+      </c>
+      <c r="D982" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E982" t="inlineStr">
+        <is>
+          <t>ANTARA - Dalam rangka memeriahkan HUT ke-81 Republik Indonesia (RI), Kerukunan Warga Dayak Dusun Maanyan dan Lawangan ...</t>
+        </is>
+      </c>
+      <c r="F982" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G982" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5686037/meriahkan-hut-ke-81-ri-warga-dayak-dusmala-lomba-tangkap-anak-babi</t>
+        </is>
+      </c>
+      <c r="H982" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/MERIAHKAN-HUT-KE-81-RI-WARGA-DAYAK-DUSMALA-LOMBA-TANGKAP-ANAK-BABI.jpg</t>
+        </is>
+      </c>
+      <c r="I982" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="983">
+      <c r="A983" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B983" t="inlineStr">
+        <is>
+          <t>Kemenhut tutup seluruh pintu masuk wisata Bromo akibat kebakaran hutan</t>
+        </is>
+      </c>
+      <c r="C983" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:39:30 +0700</t>
+        </is>
+      </c>
+      <c r="D983" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E983" t="inlineStr">
+        <is>
+          <t>Kementerian Kehutanan melalui Balai Besar Taman Nasional Bromo Tengger Semeru (TNBTS) mengumumkan penutupan secara ...</t>
+        </is>
+      </c>
+      <c r="F983" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G983" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686081/kemenhut-tutup-seluruh-pintu-masuk-wisata-bromo-akibat-kebakaran-hutan</t>
+        </is>
+      </c>
+      <c r="H983" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG-20260808-WA0025_1.jpg</t>
+        </is>
+      </c>
+      <c r="I983" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="984">
+      <c r="A984" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B984" t="inlineStr">
+        <is>
+          <t>Polresta Bandung kerahkan 350 personel patroli guna antisipasi begal</t>
+        </is>
+      </c>
+      <c r="C984" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:38:15 +0700</t>
+        </is>
+      </c>
+      <c r="D984" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E984" t="inlineStr">
+        <is>
+          <t>Polresta Bandung bersama TNI dan Pemerintah Kabupaten Bandung, Jawa Barat, mengerahkan sekitar 350 personel dalam ...</t>
+        </is>
+      </c>
+      <c r="F984" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G984" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686077/polresta-bandung-kerahkan-350-personel-patroli-guna-antisipasi-begal</t>
+        </is>
+      </c>
+      <c r="H984" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/487604.jpg</t>
+        </is>
+      </c>
+      <c r="I984" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="985">
+      <c r="A985" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B985" t="inlineStr">
+        <is>
+          <t>Satgas Yonif 511/DY bagi alat tulis bagi 50 siswa SD Popome</t>
+        </is>
+      </c>
+      <c r="C985" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:36:23 +0700</t>
+        </is>
+      </c>
+      <c r="D985" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E985" t="inlineStr">
+        <is>
+          <t>Satuan Tugas (Satgas) Pengamanan Perbatasan (Pamtas) Yonif 511/DY membagikan alat tulis bagi 50 siswa SD Popome, ...</t>
+        </is>
+      </c>
+      <c r="F985" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G985" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686076/satgas-yonif-511-dy-bagi-alat-tulis-bagi-50-siswa-sd-popome</t>
+        </is>
+      </c>
+      <c r="H985" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/WhatsApp-Image-2026-08-06-at-13.50.42.jpeg</t>
+        </is>
+      </c>
+      <c r="I985" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="986">
+      <c r="A986" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B986" t="inlineStr">
+        <is>
+          <t>Kebakaran rumah dekat Terminal UKI diduga akibat korsleting listrik</t>
+        </is>
+      </c>
+      <c r="C986" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:36:19 +0700</t>
+        </is>
+      </c>
+      <c r="D986" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E986" t="inlineStr">
+        <is>
+          <t>Suku Dinas Penanggulangan Kebakaran dan Penyelamatan (Sudin Gulkarmat) Jakarta Timur mengungkapkan kebakaran rumah ...</t>
+        </is>
+      </c>
+      <c r="F986" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G986" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686072/kebakaran-rumah-dekat-terminal-uki-diduga-akibat-korsleting-listrik</t>
+        </is>
+      </c>
+      <c r="H986" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/InShot_20260808_221844676.jpg</t>
+        </is>
+      </c>
+      <c r="I986" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="987">
+      <c r="A987" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B987" t="inlineStr">
+        <is>
+          <t>Sekjen ASEAN tekankan pentingnya prinsip TAC di tengah gejolak global</t>
+        </is>
+      </c>
+      <c r="C987" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:32:09 +0700</t>
+        </is>
+      </c>
+      <c r="D987" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E987" t="inlineStr">
+        <is>
+          <t>Sekretaris Jenderal Perhimpunan Bangsa-Bangsa Asia Tenggara (ASEAN) Kao Kim Hourn menekankan pentingnya prinsip-prinsip ...</t>
+        </is>
+      </c>
+      <c r="F987" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G987" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686068/sekjen-asean-tekankan-pentingnya-prinsip-tac-di-tengah-gejolak-global</t>
+        </is>
+      </c>
+      <c r="H987" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1000679935.jpg</t>
+        </is>
+      </c>
+      <c r="I987" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="988">
+      <c r="A988" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B988" t="inlineStr">
+        <is>
+          <t>Lanal Tual Maluku perkuat program Taruna Bakti di Sekolah Rakyat</t>
+        </is>
+      </c>
+      <c r="C988" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:29:03 +0700</t>
+        </is>
+      </c>
+      <c r="D988" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E988" t="inlineStr">
+        <is>
+          <t>Pangkalan TNI Angkatan Laut (Lanal) Tual, Maluku, memperkuat pelaksanaan Program Taruna Bhakti Akademi TNI Tahun 2026 ...</t>
+        </is>
+      </c>
+      <c r="F988" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G988" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686065/lanal-tual-maluku-perkuat-program-taruna-bakti-di-sekolah-rakyat</t>
+        </is>
+      </c>
+      <c r="H988" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/WhatsApp-Image-2026-08-08-at-21.27.57.jpeg</t>
+        </is>
+      </c>
+      <c r="I988" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B989" t="inlineStr">
+        <is>
+          <t>Disparbud usulkan tiga ciri khas Garut untuk ditetapkan jadi WBTB</t>
+        </is>
+      </c>
+      <c r="C989" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:24:43 +0700</t>
+        </is>
+      </c>
+      <c r="D989" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E989" t="inlineStr">
+        <is>
+          <t>Dinas Pariwisata dan Kebudayaan (Disparbud) Kabupaten Garut, Jawa Barat sudah mengusulkan tiga ciri khas hasil budaya ...</t>
+        </is>
+      </c>
+      <c r="F989" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G989" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686057/disparbud-usulkan-tiga-ciri-khas-garut-untuk-ditetapkan-jadi-wbtb</t>
+        </is>
+      </c>
+      <c r="H989" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/IMG_20260808_211612.jpg</t>
+        </is>
+      </c>
+      <c r="I989" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B990" t="inlineStr">
+        <is>
+          <t>Weekend Naik Kereta Api, KAI Ingatkan Pelanggan Cek Barang Bawaan Sebelum Turun</t>
+        </is>
+      </c>
+      <c r="C990" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:21:02 +0700</t>
+        </is>
+      </c>
+      <c r="D990" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E990" t="inlineStr">
+        <is>
+          <t>Memasuki akhir pekan, PT Kereta Api Indonesia (Persero) mengingatkan pelanggan untuk kembali memeriksa seluruh barang ...</t>
+        </is>
+      </c>
+      <c r="F990" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G990" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686053/weekend-naik-kereta-api-kai-ingatkan-pelanggan-cek-barang-bawaan-sebelum-turun</t>
+        </is>
+      </c>
+      <c r="H990" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/KAI-Ingatkan-Pelanggan-Cek-Bawaan.jpg</t>
+        </is>
+      </c>
+      <c r="I990" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B991" t="inlineStr">
+        <is>
+          <t>Kendari gelar Karnaval Juang sambut HUT ke-81 RI</t>
+        </is>
+      </c>
+      <c r="C991" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:19:10 +0700</t>
+        </is>
+      </c>
+      <c r="D991" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E991" t="inlineStr">
+        <is>
+          <t>Pemerintah Kota (Pemkot) Kendari, Sulawesi Tenggara (Sultra(, menggelar kegiatan karnaval juang dan gerak jalan santai ...</t>
+        </is>
+      </c>
+      <c r="F991" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G991" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686051/kendari-gelar-karnaval-juang-sambut-hut-ke-81-ri</t>
+        </is>
+      </c>
+      <c r="H991" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/010209ca-3369-4d7d-935f-73313ffc75ca.jpeg</t>
+        </is>
+      </c>
+      <c r="I991" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="992">
+      <c r="A992" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B992" t="inlineStr">
+        <is>
+          <t>Di Tengah Lintas Sumatra, Rumah Singgah KAI Membawa Nuansa Rumah Limas bagi Pekerja</t>
+        </is>
+      </c>
+      <c r="C992" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:19:02 +0700</t>
+        </is>
+      </c>
+      <c r="D992" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E992" t="inlineStr">
+        <is>
+          <t>Di sejumlah lintas kereta api Sumatera Selatan dan Lampung, terdapat stasiun yang berada cukup jauh dari kawasan ...</t>
+        </is>
+      </c>
+      <c r="F992" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G992" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686048/di-tengah-lintas-sumatra-rumah-singgah-kai-membawa-nuansa-rumah-limas-bagi-pekerja</t>
+        </is>
+      </c>
+      <c r="H992" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/ruang-tunggu-KAI.jpg</t>
+        </is>
+      </c>
+      <c r="I992" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="993">
+      <c r="A993" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B993" t="inlineStr">
+        <is>
+          <t>Kapendam: Penembakan di Baliem kelompok KKB Kodap III Ndugama</t>
+        </is>
+      </c>
+      <c r="C993" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:09:25 +0700</t>
+        </is>
+      </c>
+      <c r="D993" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E993" t="inlineStr">
+        <is>
+          <t>2026 adalah kelompok KKB dari Kodap III Ndugama.
+Memang dari hasil penyelidikan terungkap pelaku penembakan ...</t>
+        </is>
+      </c>
+      <c r="F993" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G993" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5686031/kapendam-penembakan-di-baliem-kelompok-kkb-kodap-iii-ndugama</t>
+        </is>
+      </c>
+      <c r="H993" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/1002607642.jpg</t>
+        </is>
+      </c>
+      <c r="I993" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B994" t="inlineStr">
+        <is>
+          <t>Bayi Prematur Tak Bisa Langsung Dibandingkan dengan Bayi Cukup Bulan, Kenali Usia Koreksi</t>
+        </is>
+      </c>
+      <c r="C994" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 23:59:15 +0700</t>
+        </is>
+      </c>
+      <c r="D994" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E994" t="inlineStr">
+        <is>
+          <t>Bayi prematur memerlukan pemantauan tumbuh kembang secara berkala dan tidak bisa langsung dibandingkan dengan bayi cukup bulan</t>
+        </is>
+      </c>
+      <c r="F994" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G994" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7865846/bayi-prematur-tak-bisa-langsung-dibandingkan-dengan-bayi-cukup-bulan-kenali-usia-koreksi</t>
+        </is>
+      </c>
+      <c r="H994" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/JeCwcDq4yQnZbv5mGEnPU4UDADI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/bunda-1.jpg</t>
+        </is>
+      </c>
+      <c r="I994" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="995">
+      <c r="A995" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B995" t="inlineStr">
+        <is>
+          <t>BRIN dan Kementan Soroti Dampak Batas Nikotin 1 mg, Tembakau Lokal Petani Berisiko Tak Terserap</t>
+        </is>
+      </c>
+      <c r="C995" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 23:37:49 +0700</t>
+        </is>
+      </c>
+      <c r="D995" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E995" t="inlineStr">
+        <is>
+          <t>BRIN dan Kementan menilai pembatasan nikotin maksimal 1 mg dan tar 10 mg per batang berisiko mengurangi penyerapan tembakau lokal petani.</t>
+        </is>
+      </c>
+      <c r="F995" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G995" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865845/brin-dan-kementan-soroti-dampak-batas-nikotin-1-mg-tembakau-lokal-petani-berisiko-tak-terserap</t>
+        </is>
+      </c>
+      <c r="H995" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/dStV0qFddyxxWn7yf-Z4L8m_7Ss=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-nikotin-123.jpg</t>
+        </is>
+      </c>
+      <c r="I995" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B996" t="inlineStr">
+        <is>
+          <t>Banteng Jakarta FC Siapkan 23 Pemain U-17 Hadapi Soekarno Cup 2026</t>
+        </is>
+      </c>
+      <c r="C996" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 23:31:57 +0700</t>
+        </is>
+      </c>
+      <c r="D996" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E996" t="inlineStr">
+        <is>
+          <t>Banteng Jakarta FC menyiapkan 23 pemain hasil kolaborasi dengan PPOP DKI dan ditangani eks pemain Persija, Agus Suprianto, untuk Soekarno Cup 2026.</t>
+        </is>
+      </c>
+      <c r="F996" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G996" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7865844/banteng-jakarta-fc-siapkan-23-pemain-u-17-hadapi-soekarno-cup-2026</t>
+        </is>
+      </c>
+      <c r="H996" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/dRJ94OKVFLxEIbggWiVhd_2RU-I=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Banteng-Jakarta-FC-menyiapkan-23-pemain-U-17.jpg</t>
+        </is>
+      </c>
+      <c r="I996" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="997">
+      <c r="A997" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B997" t="inlineStr">
+        <is>
+          <t>Konsolidasi di Banten, Hanura Instruksikan Pemasangan Papan Merek di Rumah Pengurus</t>
+        </is>
+      </c>
+      <c r="C997" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 23:26:54 +0700</t>
+        </is>
+      </c>
+      <c r="D997" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E997" t="inlineStr">
+        <is>
+          <t>Rio Capella mengungkapkan alasan strategis dipilihnya Banten sebagai lokasi pertama penataan kelembagaan partai.</t>
+        </is>
+      </c>
+      <c r="F997" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G997" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865843/konsolidasi-di-banten-hanura-instruksikan-pemasangan-papan-merek-di-rumah-pengurus</t>
+        </is>
+      </c>
+      <c r="H997" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Js8gvAYutNljCayWdzDdclXKftk=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/KONSOLIDASI-SATGAS.jpg</t>
+        </is>
+      </c>
+      <c r="I997" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B998" t="inlineStr">
+        <is>
+          <t>Sosok Burhanuddin Abdullah, Eks Gubernur BI yang Lebih Sering Membaca Buku Non-Ekonomi</t>
+        </is>
+      </c>
+      <c r="C998" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 23:24:13 +0700</t>
+        </is>
+      </c>
+      <c r="D998" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E998" t="inlineStr">
+        <is>
+          <t>Burhanuddin Abdullah mengaku lebih banyak membaca buku-buku yang berada di luar bidang ekonomi.</t>
+        </is>
+      </c>
+      <c r="F998" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G998" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7865842/sosok-burhanuddin-abdullah-eks-gubernur-bi-yang-lebih-sering-membaca-buku-non-ekonomi</t>
+        </is>
+      </c>
+      <c r="H998" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/pfci_aut8HHsXUD9KDKsy9_hXcY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Dr-HC-Ir-Burhanuddin-Abdullah-Harahap-MA.jpg</t>
+        </is>
+      </c>
+      <c r="I998" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" t="inlineStr">
+        <is>
+          <t>Bisnis</t>
+        </is>
+      </c>
+      <c r="B999" t="inlineStr">
+        <is>
+          <t>Pengusaha Bengkel Las Bentuk Asosiasi, Perkuat Kompetensi dan Akses Pasar</t>
+        </is>
+      </c>
+      <c r="C999" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 23:30:00 +0700</t>
+        </is>
+      </c>
+      <c r="D999" t="inlineStr">
+        <is>
+          <t>Satria K Yudha</t>
+        </is>
+      </c>
+      <c r="E999" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA – Industri pengelasan nasional didorong meningkatkan profesionalisme, kompetensi, dan daya saing agar mampu mendukung pertumbuhan ekonomi serta pembangunan infrastruktur di Indonesia. Penguatan pelaku usaha, khususnya bengkel las dan...</t>
+        </is>
+      </c>
+      <c r="F999" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G999" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjgkg0416/pengusaha-bengkel-las-bentuk-asosiasi-perkuat-kompetensi-dan-akses-pasar</t>
+        </is>
+      </c>
+      <c r="H999" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/_260808230252-314.png</t>
+        </is>
+      </c>
+      <c r="I999" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1000" t="inlineStr">
+        <is>
+          <t>Kamar Kos di Kemang Disulap Jadi Pabrik Vape Narkoba</t>
+        </is>
+      </c>
+      <c r="C1000" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 23:39:46 +0700</t>
+        </is>
+      </c>
+      <c r="D1000" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1000" t="inlineStr">
+        <is>
+          <t>Polisi menggerebek kamar kos di Kemang yang dijadikan tempat produksi vape diduga mengandung narkotika jenis etomidate.</t>
+        </is>
+      </c>
+      <c r="F1000" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1000" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265341/kamar-kos-di-kemang-disulap-jadi-pabrik-vape-narkoba</t>
+        </is>
+      </c>
+      <c r="H1000" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/kerQqXGejHezgmzrCCExr0UQHjs=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9319248/original/079248700_1786207173-8d22f8f3-7542-4f42-b3fb-cb9e04a17908.jpg</t>
+        </is>
+      </c>
+      <c r="I1000" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I965"/>
+  <autoFilter ref="A1:I1000"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-08 20:20 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-08.xlsx
+++ b/data/berita_2026-08-08.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1000</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1004</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1000"/>
+  <dimension ref="A1:I1004"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -47439,8 +47439,196 @@
         </is>
       </c>
     </row>
+    <row r="1001">
+      <c r="A1001" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1001" t="inlineStr">
+        <is>
+          <t>Karhutla di Bangka Tengah Tembus 118 Hektare Selama Juli-Agustus 2026</t>
+        </is>
+      </c>
+      <c r="C1001" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 23:00:35 +0700</t>
+        </is>
+      </c>
+      <c r="D1001" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1001" t="inlineStr">
+        <is>
+          <t>Kepala BPBD Kabupaten Bangka Tengah, Yudi Shabara, mengonfirmasi bahwa luasan tersebut merupakan akumulasi dari seluruh penanganan insiden kebakaran lahan.</t>
+        </is>
+      </c>
+      <c r="F1001" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1001" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808215415-20-1390194/karhutla-di-bangka-tengah-tembus-118-hektare-selama-juli-agustus-2026</t>
+        </is>
+      </c>
+      <c r="H1001" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/06/pemadaman-kebakaran-kawasan-hutan-di-boyolali-1785974493274_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1001" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1002" t="inlineStr">
+        <is>
+          <t>TNI-Polri Usut KKB Pelaku Penembakan Warga di Festival Lembah Baliem</t>
+        </is>
+      </c>
+      <c r="C1002" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:30:06 +0700</t>
+        </is>
+      </c>
+      <c r="D1002" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1002" t="inlineStr">
+        <is>
+          <t>Serangan mendadak tersebut menyasar warga sipil yang hendak menyaksikan gelaran Festival Budaya Lembah Baliem (FBLB) 2026 di Distrik Walesi, Papua Pegunungan.</t>
+        </is>
+      </c>
+      <c r="F1002" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1002" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808211301-20-1390190/tni-polri-usut-kkb-pelaku-penembakan-warga-di-festival-lembah-baliem</t>
+        </is>
+      </c>
+      <c r="H1002" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/festival-lembah-baliem-1786174634223_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1002" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1003" t="inlineStr">
+        <is>
+          <t>Lansia 70 Tahun Diduga Disekap di Apartemen Serpong, Mobil-HP Raib</t>
+        </is>
+      </c>
+      <c r="C1003" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:50:16 +0700</t>
+        </is>
+      </c>
+      <c r="D1003" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1003" t="inlineStr">
+        <is>
+          <t>Seorang lansia mengaku menjadi korban penyekapan dan perampokan di apartemen Serpong. Ia kehilangan mobil, handphone, dan dokumen penting.</t>
+        </is>
+      </c>
+      <c r="F1003" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1003" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808183647-12-1390166/lansia-70-tahun-diduga-disekap-di-apartemen-serpong-mobil-hp-raib</t>
+        </is>
+      </c>
+      <c r="H1003" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2023/05/30/ilustrasi-perdagangan-manusia-2_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1003" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1004" t="inlineStr">
+        <is>
+          <t>Polisi Tangkap 5 Pelaku Aniaya-Paksa Pria Masturbasi di Tangerang</t>
+        </is>
+      </c>
+      <c r="C1004" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:50:09 +0700</t>
+        </is>
+      </c>
+      <c r="D1004" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1004" t="inlineStr">
+        <is>
+          <t>Polresta Tangerang menangkap lima tersangka penyiksaan dan pelecehan seksual terhadap karyawan bank keliling.</t>
+        </is>
+      </c>
+      <c r="F1004" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1004" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260808163417-12-1390141/polisi-tangkap-5-pelaku-aniaya-paksa-pria-masturbasi-di-tangerang</t>
+        </is>
+      </c>
+      <c r="H1004" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2023/08/10/ilustrasi-penganiayaan-1_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1004" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I1000"/>
+  <autoFilter ref="A1:I1004"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-09 04:13 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-08.xlsx
+++ b/data/berita_2026-08-08.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1004</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1022</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1004"/>
+  <dimension ref="A1:I1022"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -47627,8 +47627,854 @@
         </is>
       </c>
     </row>
+    <row r="1005">
+      <c r="A1005" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1005" t="inlineStr">
+        <is>
+          <t>Iran: Pasukan Asing Harus Pergi dari Timteng demi Stabilitas Keamanan</t>
+        </is>
+      </c>
+      <c r="C1005" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 22:00:34 +0700</t>
+        </is>
+      </c>
+      <c r="D1005" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1005" t="inlineStr">
+        <is>
+          <t>Penasihat Senior Pemimpin Tertinggi Iran, Ali Akbar Velayati, menyebut ketiadaan intervensi asing adalah kunci stabilitas keamanan Timur Tengah.</t>
+        </is>
+      </c>
+      <c r="F1005" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1005" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260808205614-120-1390187/iran-pasukan-asing-harus-pergi-dari-timteng-demi-stabilitas-keamanan</t>
+        </is>
+      </c>
+      <c r="H1005" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2022/03/03/invasi-rusia-menggila-as-kirim-pasukan-ke-jerman_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1005" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1006" t="inlineStr">
+        <is>
+          <t>Diamuk Gelombang Panas, Korea Utara Sarankan Warga Makan Daging Anjing</t>
+        </is>
+      </c>
+      <c r="C1006" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 21:00:11 +0700</t>
+        </is>
+      </c>
+      <c r="D1006" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1006" t="inlineStr">
+        <is>
+          <t>Korea Utara menyarankan warganya untuk mengonsumsi sup daging anjing demi mengatasi gelombang panas yang melanda Semenanjung Korea.</t>
+        </is>
+      </c>
+      <c r="F1006" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1006" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260808153002-113-1390118/diamuk-gelombang-panas-korea-utara-sarankan-warga-makan-daging-anjing</t>
+        </is>
+      </c>
+      <c r="H1006" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2017/12/04/a1d4db93-f011-4f3d-9bbb-0ed30b293338_169.jpg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1006" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1007" t="inlineStr">
+        <is>
+          <t>Malaysia Airlines Wajibkan Semua Pilot Tes Urine, Buntut Kasus Narkoba</t>
+        </is>
+      </c>
+      <c r="C1007" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:22:14 +0700</t>
+        </is>
+      </c>
+      <c r="D1007" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1007" t="inlineStr">
+        <is>
+          <t>Malaysia Aviation Group (MAG), yang mengoperasikan Malaysia Airlines, bakal mewajibkan tes urine untuk semua pilot di semua maskapai penerbangannya.</t>
+        </is>
+      </c>
+      <c r="F1007" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1007" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260808102704-106-1390040/malaysia-airlines-wajibkan-semua-pilot-tes-urine-buntut-kasus-narkoba</t>
+        </is>
+      </c>
+      <c r="H1007" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2021/12/02/malaysia-airlines_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1007" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1008" t="inlineStr">
+        <is>
+          <t>Wakil Menteri Perang AS Akan Kunjungi Indonesia, Ada Apa?</t>
+        </is>
+      </c>
+      <c r="C1008" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:07:41 +0700</t>
+        </is>
+      </c>
+      <c r="D1008" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1008" t="inlineStr">
+        <is>
+          <t>Wakil Menteri Perang AS untuk Kebijakan Elbridge Colby dan Asisten Menteri Perang AS untuk Keamanan Indo-Pasifik John Noh akan mengunjungi Indonesia.</t>
+        </is>
+      </c>
+      <c r="F1008" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1008" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260616085545-106-1369606/wakil-menteri-perang-as-akan-kunjungi-indonesia-ada-apa</t>
+        </is>
+      </c>
+      <c r="H1008" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/elbridge-colby-1786182720274_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1008" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1009" t="inlineStr">
+        <is>
+          <t>Topan Dolphin Terjang Jepang, Ancam Pesisir China dan Taiwan</t>
+        </is>
+      </c>
+      <c r="C1009" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 20:00:20 +0700</t>
+        </is>
+      </c>
+      <c r="D1009" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1009" t="inlineStr">
+        <is>
+          <t>Topan Dolphin menerjang kawasan Okinawa di selatan Jepang pada Sabtu (8/8) dan mengancam pesisir China hingga Taiwan.</t>
+        </is>
+      </c>
+      <c r="F1009" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1009" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260808160611-113-1390124/topan-dolphin-terjang-jepang-ancam-pesisir-china-dan-taiwan</t>
+        </is>
+      </c>
+      <c r="H1009" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/ilustrasi-topan-dolphin-1786179514553_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1009" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1010" t="inlineStr">
+        <is>
+          <t>FOTO: Arab Saudi, Pakistan, dan Turki Teken Pakta Pertahanan Bersama</t>
+        </is>
+      </c>
+      <c r="C1010" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:51:20 +0700</t>
+        </is>
+      </c>
+      <c r="D1010" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1010" t="inlineStr">
+        <is>
+          <t>Arab Saudi, Pakistan, dan Turki meneken pakta pertahanan bersama pada Jumat (7/8).</t>
+        </is>
+      </c>
+      <c r="F1010" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1010" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260808175852-122-1390155/foto-arab-saudi-pakistan-dan-turki-teken-pakta-pertahanan-bersama</t>
+        </is>
+      </c>
+      <c r="H1010" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/arab-saudi-pakistan-dan-turki-teken-pakta-pertahanan-bersama-1786186718870_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1010" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1011" t="inlineStr">
+        <is>
+          <t>Hillary Clinton Komentari Dekorasi Gedung Putih ala Trump: Norak!</t>
+        </is>
+      </c>
+      <c r="C1011" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:30:11 +0700</t>
+        </is>
+      </c>
+      <c r="D1011" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1011" t="inlineStr">
+        <is>
+          <t>Mantan Menteri Luar Negeri Amerika Serikat (AS) Hillary Clinton mengomentari perombakan Presiden AS Donald Trump terhadap dekorasi Gedung Putih.</t>
+        </is>
+      </c>
+      <c r="F1011" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1011" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260808105130-134-1390043/hillary-clinton-komentari-dekorasi-gedung-putih-ala-trump-norak</t>
+        </is>
+      </c>
+      <c r="H1011" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2022/09/01/hillary-clinton-1_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1011" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1012" t="inlineStr">
+        <is>
+          <t>Saudi, Pakistan, dan Turki Teken Pakta Pertahanan Serupa NATO</t>
+        </is>
+      </c>
+      <c r="C1012" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 19:10:21 +0700</t>
+        </is>
+      </c>
+      <c r="D1012" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1012" t="inlineStr">
+        <is>
+          <t>Arab Saudi, Pakistan, Turki meneken pakta pertahanan bersama yang menetapkan serangan terhadap salah satu akan dianggap sebagai serangan terhadap mereka semua.</t>
+        </is>
+      </c>
+      <c r="F1012" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1012" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260808150424-124-1390107/saudi-pakistan-dan-turki-teken-pakta-pertahanan-serupa-nato</t>
+        </is>
+      </c>
+      <c r="H1012" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/thumbnail-video-1786176414951_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1012" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1013" t="inlineStr">
+        <is>
+          <t>Kapal Tanker Terbakar di Jalur Selatan Selat Hormuz</t>
+        </is>
+      </c>
+      <c r="C1013" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:48:25 +0700</t>
+        </is>
+      </c>
+      <c r="D1013" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1013" t="inlineStr">
+        <is>
+          <t>Sebuah kapal yang diduga kuat sebagai tanker minyak dilaporkan terbakar di koridor selatan Selat Hormuz pada Sabtu (8/8), menurut laporan media lokal Iran.</t>
+        </is>
+      </c>
+      <c r="F1013" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1013" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260808183651-120-1390165/kapal-tanker-terbakar-di-jalur-selatan-selat-hormuz</t>
+        </is>
+      </c>
+      <c r="H1013" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2024/08/27/kapal-tanker-minyak-diserang-houthi-di-laut-merah_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1013" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1014" t="inlineStr">
+        <is>
+          <t>Hillary Clinton Samakan Trump dengan Saddam Husein</t>
+        </is>
+      </c>
+      <c r="C1014" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 18:40:07 +0700</t>
+        </is>
+      </c>
+      <c r="D1014" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1014" t="inlineStr">
+        <is>
+          <t>Mantan Menteri Luar Negeri Amerika Serikat (AS) Hillary Clinton menyamakan Presiden AS Donald Trump dengan mantan diktator Irak, Saddam Hussein.</t>
+        </is>
+      </c>
+      <c r="F1014" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1014" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260808173033-134-1390152/hillary-clinton-samakan-trump-dengan-saddam-husein</t>
+        </is>
+      </c>
+      <c r="H1014" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2022/09/01/hillary-clinton-1_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1014" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1015" t="inlineStr">
+        <is>
+          <t>Jumlah Anak Palestina di Penjara Israel Meningkat 8 Kali Lipat</t>
+        </is>
+      </c>
+      <c r="C1015" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:50:20 +0700</t>
+        </is>
+      </c>
+      <c r="D1015" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1015" t="inlineStr">
+        <is>
+          <t>Jumlah anak Palestina di bawah umur yang ditahan secara administratif di Israel selama lebih dari satu tahun meningkat lebih dari delapan kali lipat.</t>
+        </is>
+      </c>
+      <c r="F1015" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1015" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260807190638-120-1389899/jumlah-anak-palestina-di-penjara-israel-meningkat-8-kali-lipat</t>
+        </is>
+      </c>
+      <c r="H1015" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2022/11/25/ilustrasi-penjara_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1015" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1016" t="inlineStr">
+        <is>
+          <t>Penembakan di Sekolah, PM Thailand Janji Rilis UU Kepemilikan Senjata</t>
+        </is>
+      </c>
+      <c r="C1016" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:30:25 +0700</t>
+        </is>
+      </c>
+      <c r="D1016" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1016" t="inlineStr">
+        <is>
+          <t>Perdana Menteri Thailand Anutin Charnvirakul berjanji akan segera menerbitkan undang-undang pengawasan senjata api yang baru pada Jumat (7/8).</t>
+        </is>
+      </c>
+      <c r="F1016" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1016" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260808153748-106-1390119/penembakan-di-sekolah-pm-thailand-janji-rilis-uu-kepemilikan-senjata</t>
+        </is>
+      </c>
+      <c r="H1016" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/07/penembakan-sekolah-di-thailand-1786075379384_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1016" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1017" t="inlineStr">
+        <is>
+          <t>Berada dalam Satu Negara, Apa Beda Pasukan Houthi dan Militer Yaman?</t>
+        </is>
+      </c>
+      <c r="C1017" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:15:23 +0700</t>
+        </is>
+      </c>
+      <c r="D1017" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1017" t="inlineStr">
+        <is>
+          <t>Pasukan Houthi menyerang kamp militer di Yaman bagian tengah pada Kamis (6/8) malam, menewaskan 30 personel pasukan pemerintah Yaman dan melukai 11 warga sipil.</t>
+        </is>
+      </c>
+      <c r="F1017" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1017" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260807202510-120-1389947/berada-dalam-satu-negara-apa-beda-pasukan-houthi-militer-yaman</t>
+        </is>
+      </c>
+      <c r="H1017" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/01/05/pasukan-yaman-rebut-kota-hadramaut-dari-kelompok-separatis-1767586913790_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1017" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1018" t="inlineStr">
+        <is>
+          <t>Ukraina Kembali Serang Dua Kilang Minyak Rusia</t>
+        </is>
+      </c>
+      <c r="C1018" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:12:48 +0700</t>
+        </is>
+      </c>
+      <c r="D1018" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1018" t="inlineStr">
+        <is>
+          <t>Militer Ukraina menyerang kilang minyak di Ilsky dan Syzran milik Rusia pada Sabtu (8/8) dini hari waktu setempat.</t>
+        </is>
+      </c>
+      <c r="F1018" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1018" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260808170047-134-1390147/ukraina-kembali-serang-dua-kilang-minyak-rusia</t>
+        </is>
+      </c>
+      <c r="H1018" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2022/12/07/ilustrasi-ledakan-atau-bom_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1018" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1019" t="inlineStr">
+        <is>
+          <t>Trump-Netanyahu Mulai Retak, Israel Akan Perangi Iran Sendirian?</t>
+        </is>
+      </c>
+      <c r="C1019" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 17:00:17 +0700</t>
+        </is>
+      </c>
+      <c r="D1019" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1019" t="inlineStr">
+        <is>
+          <t>Para pengamat buka suara mengenai potensi Israel perangi Iran sendirian menyusul retaknya hubungan Trump dan Netanyahu.</t>
+        </is>
+      </c>
+      <c r="F1019" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1019" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260808161934-120-1390137/trump-netanyahu-mulai-retak-israel-akan-perangi-iran-sendirian</t>
+        </is>
+      </c>
+      <c r="H1019" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/05/21/benjamin-netanyahu-dan-donald-trump-1779324448748_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1019" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1020" t="inlineStr">
+        <is>
+          <t>Abelardo De la Espriella Dilantik Jadi Presiden Kolombia</t>
+        </is>
+      </c>
+      <c r="C1020" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:30:26 +0700</t>
+        </is>
+      </c>
+      <c r="D1020" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1020" t="inlineStr">
+        <is>
+          <t>Abelardo de la Espriella, tokoh sayap kanan yang didukung Amerika Serikat (AS), resmi dilantik sebagai Presiden Kolombia, Jumat (7/8).</t>
+        </is>
+      </c>
+      <c r="F1020" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1020" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260808092336-134-1390027/abelardo-de-la-espriella-dilantik-jadi-presiden-kolombia</t>
+        </is>
+      </c>
+      <c r="H1020" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/abelardo-de-la-espriella-1786157649493_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1020" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1021" t="inlineStr">
+        <is>
+          <t>Horor Insiden Penembakan Massal di Idaho AS, 3 Tewas 7 Terluka</t>
+        </is>
+      </c>
+      <c r="C1021" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:50:27 +0700</t>
+        </is>
+      </c>
+      <c r="D1021" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1021" t="inlineStr">
+        <is>
+          <t>Insiden penembakan massal terjadi di sebuah restoran cepat saji di Twin Falls, Idaho, AS. Polisi baru saja merilis kondisi horor insiden penembakan tersebut.</t>
+        </is>
+      </c>
+      <c r="F1021" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1021" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260808122039-134-1390075/horor-insiden-penembakan-massal-di-idaho-as-3-tewas-7-terluka</t>
+        </is>
+      </c>
+      <c r="H1021" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2025/09/04/ilustrasi-penembakan-1756966587846_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1021" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1022" t="inlineStr">
+        <is>
+          <t>Alasan Mossad Pecat 2 Pejabat Senior usai Gagal di Iran</t>
+        </is>
+      </c>
+      <c r="C1022" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 15:30:15 +0700</t>
+        </is>
+      </c>
+      <c r="D1022" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1022" t="inlineStr">
+        <is>
+          <t>Badan intelijen Israel Mossad memecat dua pejabat senior mereka buntut kegagalan Negeri Zionis menggulingkan rezim Iran.</t>
+        </is>
+      </c>
+      <c r="F1022" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1022" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260808142441-120-1390094/alasan-mossad-pecat-2-pejabat-senior-usai-gagal-di-iran</t>
+        </is>
+      </c>
+      <c r="H1022" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/08/logo-mossad-1786174991130_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1022" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I1004"/>
+  <autoFilter ref="A1:I1022"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-09 09:33 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-08.xlsx
+++ b/data/berita_2026-08-08.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1022</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1023</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1022"/>
+  <dimension ref="A1:I1023"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -48473,8 +48473,55 @@
         </is>
       </c>
     </row>
+    <row r="1023">
+      <c r="A1023" t="inlineStr">
+        <is>
+          <t>Top News</t>
+        </is>
+      </c>
+      <c r="B1023" t="inlineStr">
+        <is>
+          <t>DKI siap hadirkan bus rute Bundaran Senayan-Ancol saat "car free day"</t>
+        </is>
+      </c>
+      <c r="C1023" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 16:39:33 +0700</t>
+        </is>
+      </c>
+      <c r="D1023" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1023" t="inlineStr">
+        <is>
+          <t>Pemerintah Provinsi DKI Jakarta menghadirkan layanan shuttle bus Transjakarta rute Bundaran ...</t>
+        </is>
+      </c>
+      <c r="F1023" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1023" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5685736/dki-siap-hadirkan-bus-rute-bundaran-senayan-ancol-saat-car-free-day</t>
+        </is>
+      </c>
+      <c r="H1023" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/12/1000303145_1.jpg</t>
+        </is>
+      </c>
+      <c r="I1023" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I1022"/>
+  <autoFilter ref="A1:I1023"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-10 00:50 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-08.xlsx
+++ b/data/berita_2026-08-08.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1023</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1024</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1023"/>
+  <dimension ref="A1:I1024"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -48520,8 +48520,55 @@
         </is>
       </c>
     </row>
+    <row r="1024">
+      <c r="A1024" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1024" t="inlineStr">
+        <is>
+          <t>Jalan Hidup Caregiver: Orang Sakit Tak Hanya Butuh Obat, Mereka Perlu Teman</t>
+        </is>
+      </c>
+      <c r="C1024" t="inlineStr">
+        <is>
+          <t>Sat, 08 Aug 2026 14:36:05 +0700</t>
+        </is>
+      </c>
+      <c r="D1024" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1024" t="inlineStr">
+        <is>
+          <t>Sebagai caregiver, kebutuhan pasiennya bukan hanya soal bantuan fisik, melainkan juga membantu secara emosional.</t>
+        </is>
+      </c>
+      <c r="F1024" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1024" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8265044/jalan-hidup-caregiver-orang-sakit-tak-hanya-butuh-obat-mereka-perlu-teman</t>
+        </is>
+      </c>
+      <c r="H1024" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/E2y__8T2jwmTzRFnP2eqmgu16TI=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9318972/original/052714900_1786174560-DSC00537.jpg</t>
+        </is>
+      </c>
+      <c r="I1024" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I1023"/>
+  <autoFilter ref="A1:I1024"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>